<commit_message>
ARSO Kranj zajem 2026-07-16 17:30 UTC
</commit_message>
<xml_diff>
--- a/tabela_vremena/ARSO_Kranj.xlsx
+++ b/tabela_vremena/ARSO_Kranj.xlsx
@@ -8492,7 +8492,36 @@
         <v>0.0</v>
       </c>
     </row>
+    <row r="291">
+      <c r="A291" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:20</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D291" s="2">
+        <v>28.8</v>
+      </c>
+      <c r="E291" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F291" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G291" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G290"/>
+  <autoFilter ref="A1:G291"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ARSO Kranj zajem 2026-07-16 22:34 UTC
</commit_message>
<xml_diff>
--- a/tabela_vremena/ARSO_Kranj.xlsx
+++ b/tabela_vremena/ARSO_Kranj.xlsx
@@ -8521,7 +8521,877 @@
         <v>0.0</v>
       </c>
     </row>
+    <row r="292">
+      <c r="A292" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:30</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D292" s="2">
+        <v>28.5</v>
+      </c>
+      <c r="E292" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F292" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G292" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:40</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D293" s="2">
+        <v>28.4</v>
+      </c>
+      <c r="E293" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F293" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G293" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:50</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D294" s="2">
+        <v>28.4</v>
+      </c>
+      <c r="E294" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F294" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G294" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:00</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D295" s="2">
+        <v>28.2</v>
+      </c>
+      <c r="E295" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F295" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G295" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:10</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D296" s="2">
+        <v>28.1</v>
+      </c>
+      <c r="E296" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F296" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G296" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:20</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D297" s="2">
+        <v>27.9</v>
+      </c>
+      <c r="E297" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F297" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G297" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:30</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D298" s="2">
+        <v>27.7</v>
+      </c>
+      <c r="E298" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F298" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G298" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:40</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D299" s="2">
+        <v>27.5</v>
+      </c>
+      <c r="E299" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F299" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G299" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:50</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D300" s="2">
+        <v>27.3</v>
+      </c>
+      <c r="E300" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F300" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G300" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:00</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D301" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="E301" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F301" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G301" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:10</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D302" s="2">
+        <v>26.7</v>
+      </c>
+      <c r="E302" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F302" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G302" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:20</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D303" s="2">
+        <v>26.2</v>
+      </c>
+      <c r="E303" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F303" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G303" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:30</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D304" s="2">
+        <v>25.8</v>
+      </c>
+      <c r="E304" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F304" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G304" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:40</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D305" s="2">
+        <v>25.4</v>
+      </c>
+      <c r="E305" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F305" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G305" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:50</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D306" s="2">
+        <v>24.9</v>
+      </c>
+      <c r="E306" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F306" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G306" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:00</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D307" s="2">
+        <v>24.6</v>
+      </c>
+      <c r="E307" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F307" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G307" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:10</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D308" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="E308" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F308" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G308" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:20</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D309" s="2">
+        <v>23.8</v>
+      </c>
+      <c r="E309" s="2">
+        <v>72.0</v>
+      </c>
+      <c r="F309" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G309" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:30</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D310" s="2">
+        <v>23.4</v>
+      </c>
+      <c r="E310" s="2">
+        <v>74.0</v>
+      </c>
+      <c r="F310" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G310" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:40</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D311" s="2">
+        <v>23.1</v>
+      </c>
+      <c r="E311" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F311" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G311" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:50</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D312" s="2">
+        <v>22.9</v>
+      </c>
+      <c r="E312" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F312" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G312" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:00</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D313" s="2">
+        <v>22.8</v>
+      </c>
+      <c r="E313" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F313" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G313" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:10</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D314" s="2">
+        <v>22.6</v>
+      </c>
+      <c r="E314" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F314" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G314" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:20</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D315" s="2">
+        <v>22.4</v>
+      </c>
+      <c r="E315" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F315" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G315" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:30</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D316" s="2">
+        <v>22.2</v>
+      </c>
+      <c r="E316" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F316" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G316" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:40</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D317" s="2">
+        <v>22.2</v>
+      </c>
+      <c r="E317" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F317" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G317" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16.07.2026</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:50</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D318" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="E318" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F318" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G318" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:00</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D319" s="2">
+        <v>21.8</v>
+      </c>
+      <c r="E319" s="2">
+        <v>83.0</v>
+      </c>
+      <c r="F319" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G319" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:10</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D320" s="2">
+        <v>21.6</v>
+      </c>
+      <c r="E320" s="2">
+        <v>83.0</v>
+      </c>
+      <c r="F320" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G320" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:20</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D321" s="2">
+        <v>21.5</v>
+      </c>
+      <c r="E321" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F321" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G321" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G291"/>
+  <autoFilter ref="A1:G321"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ARSO Kranj zajem 2026-07-17 01:16 UTC
</commit_message>
<xml_diff>
--- a/tabela_vremena/ARSO_Kranj.xlsx
+++ b/tabela_vremena/ARSO_Kranj.xlsx
@@ -9391,7 +9391,471 @@
         <v>0.0</v>
       </c>
     </row>
+    <row r="322">
+      <c r="A322" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:30</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D322" s="2">
+        <v>21.5</v>
+      </c>
+      <c r="E322" s="2">
+        <v>83.0</v>
+      </c>
+      <c r="F322" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G322" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:40</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D323" s="2">
+        <v>21.3</v>
+      </c>
+      <c r="E323" s="2">
+        <v>83.0</v>
+      </c>
+      <c r="F323" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G323" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:50</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D324" s="2">
+        <v>21.2</v>
+      </c>
+      <c r="E324" s="2">
+        <v>84.0</v>
+      </c>
+      <c r="F324" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G324" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:00</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D325" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="E325" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F325" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G325" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:10</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D326" s="2">
+        <v>20.9</v>
+      </c>
+      <c r="E326" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F326" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G326" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:20</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D327" s="2">
+        <v>20.8</v>
+      </c>
+      <c r="E327" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F327" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G327" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:30</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D328" s="2">
+        <v>20.8</v>
+      </c>
+      <c r="E328" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F328" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G328" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:40</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D329" s="2">
+        <v>20.7</v>
+      </c>
+      <c r="E329" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F329" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G329" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:50</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D330" s="2">
+        <v>20.6</v>
+      </c>
+      <c r="E330" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F330" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G330" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:00</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D331" s="2">
+        <v>20.6</v>
+      </c>
+      <c r="E331" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F331" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G331" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:10</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D332" s="2">
+        <v>20.6</v>
+      </c>
+      <c r="E332" s="2">
+        <v>84.0</v>
+      </c>
+      <c r="F332" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G332" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:20</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D333" s="2">
+        <v>20.5</v>
+      </c>
+      <c r="E333" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F333" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G333" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:30</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D334" s="2">
+        <v>20.4</v>
+      </c>
+      <c r="E334" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F334" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G334" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:40</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D335" s="2">
+        <v>20.3</v>
+      </c>
+      <c r="E335" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F335" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G335" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:50</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D336" s="2">
+        <v>20.2</v>
+      </c>
+      <c r="E336" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F336" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G336" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:00</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D337" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="E337" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F337" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G337" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G321"/>
+  <autoFilter ref="A1:G337"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ARSO Kranj zajem 2026-07-17 06:30 UTC
</commit_message>
<xml_diff>
--- a/tabela_vremena/ARSO_Kranj.xlsx
+++ b/tabela_vremena/ARSO_Kranj.xlsx
@@ -9855,7 +9855,906 @@
         <v>0.0</v>
       </c>
     </row>
+    <row r="338">
+      <c r="A338" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:10</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D338" s="2">
+        <v>19.8</v>
+      </c>
+      <c r="E338" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F338" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G338" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:20</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D339" s="2">
+        <v>19.7</v>
+      </c>
+      <c r="E339" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F339" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G339" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:30</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D340" s="2">
+        <v>19.7</v>
+      </c>
+      <c r="E340" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F340" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G340" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:40</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D341" s="2">
+        <v>19.8</v>
+      </c>
+      <c r="E341" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F341" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G341" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:50</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D342" s="2">
+        <v>19.8</v>
+      </c>
+      <c r="E342" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F342" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G342" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:00</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D343" s="2">
+        <v>19.9</v>
+      </c>
+      <c r="E343" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F343" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G343" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:10</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D344" s="2">
+        <v>19.9</v>
+      </c>
+      <c r="E344" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F344" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G344" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:20</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D345" s="2">
+        <v>19.7</v>
+      </c>
+      <c r="E345" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F345" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G345" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:30</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D346" s="2">
+        <v>19.6</v>
+      </c>
+      <c r="E346" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F346" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G346" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:40</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D347" s="2">
+        <v>19.4</v>
+      </c>
+      <c r="E347" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F347" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G347" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:50</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D348" s="2">
+        <v>19.4</v>
+      </c>
+      <c r="E348" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F348" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G348" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:00</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D349" s="2">
+        <v>19.5</v>
+      </c>
+      <c r="E349" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F349" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G349" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:10</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D350" s="2">
+        <v>19.4</v>
+      </c>
+      <c r="E350" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F350" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G350" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:20</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D351" s="2">
+        <v>19.3</v>
+      </c>
+      <c r="E351" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F351" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G351" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:30</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D352" s="2">
+        <v>19.2</v>
+      </c>
+      <c r="E352" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F352" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G352" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:40</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D353" s="2">
+        <v>19.2</v>
+      </c>
+      <c r="E353" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F353" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G353" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:50</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D354" s="2">
+        <v>19.2</v>
+      </c>
+      <c r="E354" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F354" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G354" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:00</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D355" s="2">
+        <v>19.3</v>
+      </c>
+      <c r="E355" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F355" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G355" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:10</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D356" s="2">
+        <v>19.3</v>
+      </c>
+      <c r="E356" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F356" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G356" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:20</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D357" s="2">
+        <v>19.4</v>
+      </c>
+      <c r="E357" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F357" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G357" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:30</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D358" s="2">
+        <v>19.6</v>
+      </c>
+      <c r="E358" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F358" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G358" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:40</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D359" s="2">
+        <v>19.8</v>
+      </c>
+      <c r="E359" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F359" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G359" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:50</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D360" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="E360" s="2">
+        <v>83.0</v>
+      </c>
+      <c r="F360" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G360" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:00</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D361" s="2">
+        <v>20.3</v>
+      </c>
+      <c r="E361" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F361" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G361" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:10</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D362" s="2">
+        <v>20.8</v>
+      </c>
+      <c r="E362" s="2">
+        <v>81.0</v>
+      </c>
+      <c r="F362" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G362" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:20</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D363" s="2">
+        <v>20.8</v>
+      </c>
+      <c r="E363" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F363" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G363" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:30</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D364" s="2">
+        <v>20.9</v>
+      </c>
+      <c r="E364" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F364" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G364" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:40</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D365" s="2">
+        <v>21.2</v>
+      </c>
+      <c r="E365" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F365" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G365" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:50</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D366" s="2">
+        <v>21.6</v>
+      </c>
+      <c r="E366" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F366" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G366" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:00</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D367" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="E367" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F367" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G367" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:10</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D368" s="2">
+        <v>22.3</v>
+      </c>
+      <c r="E368" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F368" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G368" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G337"/>
+  <autoFilter ref="A1:G368"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ARSO Kranj zajem 2026-07-17 08:44 Europe/Ljubljana
</commit_message>
<xml_diff>
--- a/tabela_vremena/ARSO_Kranj.xlsx
+++ b/tabela_vremena/ARSO_Kranj.xlsx
@@ -10754,7 +10754,65 @@
         <v>0.0</v>
       </c>
     </row>
+    <row r="369">
+      <c r="A369" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:20</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D369" s="2">
+        <v>22.5</v>
+      </c>
+      <c r="E369" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="F369" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G369" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:30</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D370" s="2">
+        <v>22.3</v>
+      </c>
+      <c r="E370" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F370" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G370" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G368"/>
+  <autoFilter ref="A1:G370"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ARSO Kranj zajem 2026-07-17 08:59 Europe/Ljubljana
</commit_message>
<xml_diff>
--- a/tabela_vremena/ARSO_Kranj.xlsx
+++ b/tabela_vremena/ARSO_Kranj.xlsx
@@ -10812,7 +10812,36 @@
         <v>0.0</v>
       </c>
     </row>
+    <row r="371">
+      <c r="A371" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:40</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D371" s="2">
+        <v>22.3</v>
+      </c>
+      <c r="E371" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F371" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G371" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G370"/>
+  <autoFilter ref="A1:G371"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ARSO Kranj zajem 2026-07-17 11:19 Europe/Ljubljana
</commit_message>
<xml_diff>
--- a/tabela_vremena/ARSO_Kranj.xlsx
+++ b/tabela_vremena/ARSO_Kranj.xlsx
@@ -10841,7 +10841,413 @@
         <v>0.0</v>
       </c>
     </row>
+    <row r="372">
+      <c r="A372" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:50</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D372" s="2">
+        <v>22.3</v>
+      </c>
+      <c r="E372" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F372" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G372" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:00</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D373" s="2">
+        <v>22.5</v>
+      </c>
+      <c r="E373" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F373" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G373" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:10</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D374" s="2">
+        <v>22.9</v>
+      </c>
+      <c r="E374" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="F374" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G374" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:20</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D375" s="2">
+        <v>23.3</v>
+      </c>
+      <c r="E375" s="2">
+        <v>72.0</v>
+      </c>
+      <c r="F375" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G375" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:30</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D376" s="2">
+        <v>23.5</v>
+      </c>
+      <c r="E376" s="2">
+        <v>72.0</v>
+      </c>
+      <c r="F376" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G376" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:40</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D377" s="2">
+        <v>23.6</v>
+      </c>
+      <c r="E377" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F377" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G377" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:50</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D378" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="E378" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F378" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G378" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:00</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D379" s="2">
+        <v>24.3</v>
+      </c>
+      <c r="E379" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F379" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G379" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:10</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D380" s="2">
+        <v>24.2</v>
+      </c>
+      <c r="E380" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F380" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G380" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:20</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D381" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="E381" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F381" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G381" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:30</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D382" s="2">
+        <v>23.2</v>
+      </c>
+      <c r="E382" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F382" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G382" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:40</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D383" s="2">
+        <v>22.8</v>
+      </c>
+      <c r="E383" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F383" s="2">
+        <v>0.8</v>
+      </c>
+      <c r="G383" s="2">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:50</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D384" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="E384" s="2">
+        <v>81.0</v>
+      </c>
+      <c r="F384" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G384" s="2">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:00</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D385" s="2">
+        <v>22.9</v>
+      </c>
+      <c r="E385" s="2">
+        <v>81.0</v>
+      </c>
+      <c r="F385" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G385" s="2">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G371"/>
+  <autoFilter ref="A1:G385"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ARSO Kranj zajem 2026-07-18 00:35 Europe/Ljubljana
</commit_message>
<xml_diff>
--- a/tabela_vremena/ARSO_Kranj.xlsx
+++ b/tabela_vremena/ARSO_Kranj.xlsx
@@ -11247,7 +11247,2327 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="386">
+      <c r="A386" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:10</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D386" s="2">
+        <v>22.5</v>
+      </c>
+      <c r="E386" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F386" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G386" s="2">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:20</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D387" s="2">
+        <v>21.7</v>
+      </c>
+      <c r="E387" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F387" s="2">
+        <v>0.3</v>
+      </c>
+      <c r="G387" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:30</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D388" s="2">
+        <v>21.7</v>
+      </c>
+      <c r="E388" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F388" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G388" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:40</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D389" s="2">
+        <v>21.7</v>
+      </c>
+      <c r="E389" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F389" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G389" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:50</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D390" s="2">
+        <v>22.1</v>
+      </c>
+      <c r="E390" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F390" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G390" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:00</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D391" s="2">
+        <v>22.6</v>
+      </c>
+      <c r="E391" s="2">
+        <v>74.0</v>
+      </c>
+      <c r="F391" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G391" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:10</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D392" s="2">
+        <v>23.1</v>
+      </c>
+      <c r="E392" s="2">
+        <v>72.0</v>
+      </c>
+      <c r="F392" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G392" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:20</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D393" s="2">
+        <v>23.3</v>
+      </c>
+      <c r="E393" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F393" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G393" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:30</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D394" s="2">
+        <v>23.6</v>
+      </c>
+      <c r="E394" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F394" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G394" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:40</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D395" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="E395" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F395" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G395" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:50</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D396" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="E396" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F396" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G396" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:00</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D397" s="2">
+        <v>24.2</v>
+      </c>
+      <c r="E397" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F397" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G397" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:10</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D398" s="2">
+        <v>24.4</v>
+      </c>
+      <c r="E398" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F398" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G398" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:20</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D399" s="2">
+        <v>24.5</v>
+      </c>
+      <c r="E399" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F399" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G399" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:30</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D400" s="2">
+        <v>24.5</v>
+      </c>
+      <c r="E400" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F400" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G400" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:40</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D401" s="2">
+        <v>24.8</v>
+      </c>
+      <c r="E401" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F401" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G401" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:50</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D402" s="2">
+        <v>25.4</v>
+      </c>
+      <c r="E402" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F402" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G402" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:00</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D403" s="2">
+        <v>25.8</v>
+      </c>
+      <c r="E403" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F403" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G403" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:10</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D404" s="2">
+        <v>25.5</v>
+      </c>
+      <c r="E404" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F404" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G404" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:20</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D405" s="2">
+        <v>25.7</v>
+      </c>
+      <c r="E405" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F405" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G405" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:30</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D406" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="E406" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F406" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G406" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:40</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D407" s="2">
+        <v>26.9</v>
+      </c>
+      <c r="E407" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F407" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G407" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:50</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D408" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="E408" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F408" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G408" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:00</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D409" s="2">
+        <v>27.3</v>
+      </c>
+      <c r="E409" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F409" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G409" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:10</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D410" s="2">
+        <v>27.6</v>
+      </c>
+      <c r="E410" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F410" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G410" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:20</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D411" s="2">
+        <v>27.8</v>
+      </c>
+      <c r="E411" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F411" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G411" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:30</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D412" s="2">
+        <v>28.2</v>
+      </c>
+      <c r="E412" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F412" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G412" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:40</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D413" s="2">
+        <v>28.6</v>
+      </c>
+      <c r="E413" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F413" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G413" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:50</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D414" s="2">
+        <v>28.1</v>
+      </c>
+      <c r="E414" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F414" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G414" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:00</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D415" s="2">
+        <v>28.3</v>
+      </c>
+      <c r="E415" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F415" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G415" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:10</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D416" s="2">
+        <v>28.4</v>
+      </c>
+      <c r="E416" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F416" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G416" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:20</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D417" s="2">
+        <v>28.1</v>
+      </c>
+      <c r="E417" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F417" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G417" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:30</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D418" s="2">
+        <v>28.3</v>
+      </c>
+      <c r="E418" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F418" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G418" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:40</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D419" s="2">
+        <v>28.8</v>
+      </c>
+      <c r="E419" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F419" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G419" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:50</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D420" s="2">
+        <v>28.4</v>
+      </c>
+      <c r="E420" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F420" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G420" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:00</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D421" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="E421" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F421" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G421" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:10</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D422" s="2">
+        <v>29.3</v>
+      </c>
+      <c r="E422" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F422" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G422" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:20</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D423" s="2">
+        <v>29.7</v>
+      </c>
+      <c r="E423" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F423" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G423" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:30</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D424" s="2">
+        <v>29.9</v>
+      </c>
+      <c r="E424" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F424" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G424" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:40</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D425" s="2">
+        <v>30.2</v>
+      </c>
+      <c r="E425" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F425" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G425" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:50</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D426" s="2">
+        <v>30.3</v>
+      </c>
+      <c r="E426" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F426" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G426" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:00</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D427" s="2">
+        <v>30.8</v>
+      </c>
+      <c r="E427" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F427" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G427" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:10</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D428" s="2">
+        <v>30.6</v>
+      </c>
+      <c r="E428" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F428" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G428" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:20</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D429" s="2">
+        <v>30.6</v>
+      </c>
+      <c r="E429" s="2">
+        <v>37.0</v>
+      </c>
+      <c r="F429" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G429" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:30</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D430" s="2">
+        <v>30.6</v>
+      </c>
+      <c r="E430" s="2">
+        <v>37.0</v>
+      </c>
+      <c r="F430" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G430" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:40</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D431" s="2">
+        <v>30.6</v>
+      </c>
+      <c r="E431" s="2">
+        <v>38.0</v>
+      </c>
+      <c r="F431" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G431" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:50</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D432" s="2">
+        <v>30.7</v>
+      </c>
+      <c r="E432" s="2">
+        <v>38.0</v>
+      </c>
+      <c r="F432" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G432" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:00</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D433" s="2">
+        <v>30.8</v>
+      </c>
+      <c r="E433" s="2">
+        <v>38.0</v>
+      </c>
+      <c r="F433" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G433" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:10</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D434" s="2">
+        <v>30.2</v>
+      </c>
+      <c r="E434" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F434" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G434" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:20</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D435" s="2">
+        <v>29.7</v>
+      </c>
+      <c r="E435" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F435" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G435" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:30</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D436" s="2">
+        <v>29.2</v>
+      </c>
+      <c r="E436" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F436" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G436" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:40</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D437" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="E437" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F437" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G437" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:50</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D438" s="2">
+        <v>28.7</v>
+      </c>
+      <c r="E438" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F438" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G438" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:00</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D439" s="2">
+        <v>28.5</v>
+      </c>
+      <c r="E439" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F439" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G439" s="2">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:10</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D440" s="2">
+        <v>28.1</v>
+      </c>
+      <c r="E440" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F440" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G440" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:20</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D441" s="2">
+        <v>27.9</v>
+      </c>
+      <c r="E441" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F441" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G441" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:30</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D442" s="2">
+        <v>27.7</v>
+      </c>
+      <c r="E442" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F442" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G442" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:40</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D443" s="2">
+        <v>27.3</v>
+      </c>
+      <c r="E443" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F443" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G443" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:50</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D444" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="E444" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F444" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G444" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:00</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D445" s="2">
+        <v>26.8</v>
+      </c>
+      <c r="E445" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F445" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G445" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:10</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D446" s="2">
+        <v>26.5</v>
+      </c>
+      <c r="E446" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F446" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G446" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:20</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D447" s="2">
+        <v>25.9</v>
+      </c>
+      <c r="E447" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F447" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G447" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:30</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D448" s="2">
+        <v>25.5</v>
+      </c>
+      <c r="E448" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F448" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G448" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:40</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D449" s="2">
+        <v>24.8</v>
+      </c>
+      <c r="E449" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F449" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G449" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:50</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D450" s="2">
+        <v>24.4</v>
+      </c>
+      <c r="E450" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F450" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G450" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:00</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D451" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="E451" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F451" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G451" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:10</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D452" s="2">
+        <v>23.5</v>
+      </c>
+      <c r="E452" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F452" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G452" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:20</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D453" s="2">
+        <v>23.2</v>
+      </c>
+      <c r="E453" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F453" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G453" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:30</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D454" s="2">
+        <v>22.9</v>
+      </c>
+      <c r="E454" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F454" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G454" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:40</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D455" s="2">
+        <v>22.5</v>
+      </c>
+      <c r="E455" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F455" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G455" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:50</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D456" s="2">
+        <v>22.3</v>
+      </c>
+      <c r="E456" s="2">
+        <v>69.0</v>
+      </c>
+      <c r="F456" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G456" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:00</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D457" s="2">
+        <v>22.2</v>
+      </c>
+      <c r="E457" s="2">
+        <v>72.0</v>
+      </c>
+      <c r="F457" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G457" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:10</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D458" s="2">
+        <v>21.8</v>
+      </c>
+      <c r="E458" s="2">
+        <v>74.0</v>
+      </c>
+      <c r="F458" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G458" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:20</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D459" s="2">
+        <v>21.5</v>
+      </c>
+      <c r="E459" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F459" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G459" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:30</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D460" s="2">
+        <v>21.2</v>
+      </c>
+      <c r="E460" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F460" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G460" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:40</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D461" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="E461" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F461" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G461" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17.07.2026</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:50</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D462" s="2">
+        <v>20.8</v>
+      </c>
+      <c r="E462" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F462" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G462" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:00</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D463" s="2">
+        <v>20.7</v>
+      </c>
+      <c r="E463" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F463" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G463" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:10</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D464" s="2">
+        <v>20.5</v>
+      </c>
+      <c r="E464" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F464" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G464" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:20</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D465" s="2">
+        <v>20.4</v>
+      </c>
+      <c r="E465" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F465" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G465" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G385"/>
+  <autoFilter ref="A1:G465"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ARSO Kranj zajem 2026-07-19 00:34 Europe/Ljubljana
</commit_message>
<xml_diff>
--- a/tabela_vremena/ARSO_Kranj.xlsx
+++ b/tabela_vremena/ARSO_Kranj.xlsx
@@ -13567,7 +13567,4183 @@
         <v>0.0</v>
       </c>
     </row>
+    <row r="466">
+      <c r="A466" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:30</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D466" s="2">
+        <v>20.4</v>
+      </c>
+      <c r="E466" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F466" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G466" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:40</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D467" s="2">
+        <v>20.9</v>
+      </c>
+      <c r="E467" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F467" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G467" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:50</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D468" s="2">
+        <v>21.2</v>
+      </c>
+      <c r="E468" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="F468" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G468" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:00</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D469" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="E469" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F469" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G469" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:10</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D470" s="2">
+        <v>20.7</v>
+      </c>
+      <c r="E470" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F470" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G470" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:20</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D471" s="2">
+        <v>20.9</v>
+      </c>
+      <c r="E471" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F471" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G471" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:30</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D472" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="E472" s="2">
+        <v>74.0</v>
+      </c>
+      <c r="F472" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G472" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:40</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D473" s="2">
+        <v>21.1</v>
+      </c>
+      <c r="E473" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="F473" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G473" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:50</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D474" s="2">
+        <v>21.5</v>
+      </c>
+      <c r="E474" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F474" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G474" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:00</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D475" s="2">
+        <v>21.6</v>
+      </c>
+      <c r="E475" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F475" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G475" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:10</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D476" s="2">
+        <v>21.6</v>
+      </c>
+      <c r="E476" s="2">
+        <v>69.0</v>
+      </c>
+      <c r="F476" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G476" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:20</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D477" s="2">
+        <v>21.5</v>
+      </c>
+      <c r="E477" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F477" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G477" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:30</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D478" s="2">
+        <v>21.8</v>
+      </c>
+      <c r="E478" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F478" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G478" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:40</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D479" s="2">
+        <v>21.9</v>
+      </c>
+      <c r="E479" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F479" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G479" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:50</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D480" s="2">
+        <v>22.2</v>
+      </c>
+      <c r="E480" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F480" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G480" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:00</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D481" s="2">
+        <v>22.4</v>
+      </c>
+      <c r="E481" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F481" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G481" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:10</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D482" s="2">
+        <v>22.6</v>
+      </c>
+      <c r="E482" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F482" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G482" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:20</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D483" s="2">
+        <v>22.7</v>
+      </c>
+      <c r="E483" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F483" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G483" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:30</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D484" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="E484" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F484" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G484" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:40</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D485" s="2">
+        <v>23.4</v>
+      </c>
+      <c r="E485" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F485" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G485" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:50</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D486" s="2">
+        <v>23.5</v>
+      </c>
+      <c r="E486" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F486" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G486" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:00</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D487" s="2">
+        <v>23.4</v>
+      </c>
+      <c r="E487" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F487" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G487" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:10</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D488" s="2">
+        <v>23.3</v>
+      </c>
+      <c r="E488" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F488" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G488" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:20</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D489" s="2">
+        <v>23.2</v>
+      </c>
+      <c r="E489" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F489" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G489" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:30</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D490" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="E490" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F490" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G490" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:40</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D491" s="2">
+        <v>22.8</v>
+      </c>
+      <c r="E491" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F491" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G491" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:50</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D492" s="2">
+        <v>22.7</v>
+      </c>
+      <c r="E492" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F492" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G492" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:00</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D493" s="2">
+        <v>22.5</v>
+      </c>
+      <c r="E493" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F493" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G493" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:10</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D494" s="2">
+        <v>22.4</v>
+      </c>
+      <c r="E494" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F494" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G494" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:20</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D495" s="2">
+        <v>22.2</v>
+      </c>
+      <c r="E495" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F495" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G495" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:30</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D496" s="2">
+        <v>21.9</v>
+      </c>
+      <c r="E496" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F496" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G496" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:40</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D497" s="2">
+        <v>21.6</v>
+      </c>
+      <c r="E497" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F497" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G497" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:50</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D498" s="2">
+        <v>21.5</v>
+      </c>
+      <c r="E498" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F498" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G498" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:00</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D499" s="2">
+        <v>21.4</v>
+      </c>
+      <c r="E499" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F499" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G499" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:10</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D500" s="2">
+        <v>21.5</v>
+      </c>
+      <c r="E500" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F500" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G500" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:20</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D501" s="2">
+        <v>21.6</v>
+      </c>
+      <c r="E501" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F501" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G501" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:30</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D502" s="2">
+        <v>21.6</v>
+      </c>
+      <c r="E502" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F502" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G502" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:40</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D503" s="2">
+        <v>21.7</v>
+      </c>
+      <c r="E503" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F503" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G503" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:50</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D504" s="2">
+        <v>21.9</v>
+      </c>
+      <c r="E504" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F504" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G504" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:00</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D505" s="2">
+        <v>21.9</v>
+      </c>
+      <c r="E505" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F505" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G505" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:10</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D506" s="2">
+        <v>21.9</v>
+      </c>
+      <c r="E506" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F506" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G506" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:20</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D507" s="2">
+        <v>22.1</v>
+      </c>
+      <c r="E507" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F507" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G507" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:30</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D508" s="2">
+        <v>22.7</v>
+      </c>
+      <c r="E508" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F508" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G508" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:40</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D509" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="E509" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F509" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G509" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:50</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D510" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="E510" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F510" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G510" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:00</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D511" s="2">
+        <v>23.2</v>
+      </c>
+      <c r="E511" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F511" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G511" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:10</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D512" s="2">
+        <v>23.3</v>
+      </c>
+      <c r="E512" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F512" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G512" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:20</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D513" s="2">
+        <v>23.3</v>
+      </c>
+      <c r="E513" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F513" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G513" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:30</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D514" s="2">
+        <v>23.3</v>
+      </c>
+      <c r="E514" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F514" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G514" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:40</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D515" s="2">
+        <v>23.5</v>
+      </c>
+      <c r="E515" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F515" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G515" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:50</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D516" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="E516" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F516" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G516" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:00</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D517" s="2">
+        <v>24.7</v>
+      </c>
+      <c r="E517" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F517" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G517" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:10</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D518" s="2">
+        <v>25.2</v>
+      </c>
+      <c r="E518" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F518" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G518" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:20</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D519" s="2">
+        <v>25.7</v>
+      </c>
+      <c r="E519" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F519" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G519" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:30</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D520" s="2">
+        <v>26.1</v>
+      </c>
+      <c r="E520" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F520" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G520" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:40</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D521" s="2">
+        <v>26.7</v>
+      </c>
+      <c r="E521" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F521" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G521" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:50</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D522" s="2">
+        <v>26.5</v>
+      </c>
+      <c r="E522" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F522" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G522" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:00</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D523" s="2">
+        <v>27.3</v>
+      </c>
+      <c r="E523" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F523" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G523" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:10</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D524" s="2">
+        <v>27.5</v>
+      </c>
+      <c r="E524" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F524" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G524" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:20</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D525" s="2">
+        <v>26.9</v>
+      </c>
+      <c r="E525" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F525" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G525" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:30</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D526" s="2">
+        <v>26.7</v>
+      </c>
+      <c r="E526" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F526" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G526" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:40</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D527" s="2">
+        <v>27.2</v>
+      </c>
+      <c r="E527" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F527" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G527" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:50</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D528" s="2">
+        <v>27.8</v>
+      </c>
+      <c r="E528" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F528" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G528" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:00</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D529" s="2">
+        <v>28.4</v>
+      </c>
+      <c r="E529" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F529" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G529" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:10</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D530" s="2">
+        <v>28.8</v>
+      </c>
+      <c r="E530" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F530" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G530" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:20</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D531" s="2">
+        <v>28.8</v>
+      </c>
+      <c r="E531" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F531" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G531" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:30</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D532" s="2">
+        <v>29.7</v>
+      </c>
+      <c r="E532" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F532" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G532" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:40</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D533" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="E533" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F533" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G533" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:50</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D534" s="2">
+        <v>30.3</v>
+      </c>
+      <c r="E534" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F534" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G534" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:00</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D535" s="2">
+        <v>30.4</v>
+      </c>
+      <c r="E535" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F535" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G535" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:10</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D536" s="2">
+        <v>30.6</v>
+      </c>
+      <c r="E536" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F536" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G536" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:20</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D537" s="2">
+        <v>30.6</v>
+      </c>
+      <c r="E537" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F537" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G537" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:30</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D538" s="2">
+        <v>30.7</v>
+      </c>
+      <c r="E538" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F538" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G538" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:40</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D539" s="2">
+        <v>30.9</v>
+      </c>
+      <c r="E539" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F539" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G539" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:50</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D540" s="2">
+        <v>30.9</v>
+      </c>
+      <c r="E540" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F540" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G540" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:00</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D541" s="2">
+        <v>31.3</v>
+      </c>
+      <c r="E541" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F541" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G541" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:10</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D542" s="2">
+        <v>31.5</v>
+      </c>
+      <c r="E542" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F542" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G542" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:20</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D543" s="2">
+        <v>31.8</v>
+      </c>
+      <c r="E543" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F543" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G543" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:30</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D544" s="2">
+        <v>31.9</v>
+      </c>
+      <c r="E544" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F544" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G544" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:40</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D545" s="2">
+        <v>31.7</v>
+      </c>
+      <c r="E545" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F545" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G545" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:50</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D546" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="E546" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F546" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G546" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:00</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D547" s="2">
+        <v>32.3</v>
+      </c>
+      <c r="E547" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F547" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G547" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:10</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D548" s="2">
+        <v>32.3</v>
+      </c>
+      <c r="E548" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F548" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G548" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:20</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D549" s="2">
+        <v>32.3</v>
+      </c>
+      <c r="E549" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F549" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G549" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:30</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D550" s="2">
+        <v>31.9</v>
+      </c>
+      <c r="E550" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F550" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G550" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:40</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D551" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="E551" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F551" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G551" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:50</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D552" s="2">
+        <v>32.6</v>
+      </c>
+      <c r="E552" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F552" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G552" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:00</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D553" s="2">
+        <v>32.9</v>
+      </c>
+      <c r="E553" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="F553" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G553" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:10</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D554" s="2">
+        <v>32.8</v>
+      </c>
+      <c r="E554" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F554" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G554" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:20</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D555" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="E555" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="F555" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G555" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:30</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D556" s="2">
+        <v>33.1</v>
+      </c>
+      <c r="E556" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F556" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G556" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:40</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D557" s="2">
+        <v>32.7</v>
+      </c>
+      <c r="E557" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F557" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G557" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:50</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D558" s="2">
+        <v>32.3</v>
+      </c>
+      <c r="E558" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F558" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G558" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:00</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D559" s="2">
+        <v>32.8</v>
+      </c>
+      <c r="E559" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F559" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G559" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:10</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D560" s="2">
+        <v>31.7</v>
+      </c>
+      <c r="E560" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="F560" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G560" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:20</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D561" s="2">
+        <v>30.5</v>
+      </c>
+      <c r="E561" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F561" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G561" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:30</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D562" s="2">
+        <v>29.5</v>
+      </c>
+      <c r="E562" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F562" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G562" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:40</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D563" s="2">
+        <v>28.8</v>
+      </c>
+      <c r="E563" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F563" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G563" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:50</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D564" s="2">
+        <v>27.8</v>
+      </c>
+      <c r="E564" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F564" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G564" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:00</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D565" s="2">
+        <v>25.6</v>
+      </c>
+      <c r="E565" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F565" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G565" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:10</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D566" s="2">
+        <v>22.8</v>
+      </c>
+      <c r="E566" s="2">
+        <v>81.0</v>
+      </c>
+      <c r="F566" s="2">
+        <v>1.3</v>
+      </c>
+      <c r="G566" s="2">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:20</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D567" s="2">
+        <v>22.4</v>
+      </c>
+      <c r="E567" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F567" s="2">
+        <v>0.9</v>
+      </c>
+      <c r="G567" s="2">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:30</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D568" s="2">
+        <v>20.5</v>
+      </c>
+      <c r="E568" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F568" s="2">
+        <v>0.3</v>
+      </c>
+      <c r="G568" s="2">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:40</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D569" s="2">
+        <v>19.6</v>
+      </c>
+      <c r="E569" s="2">
+        <v>91.0</v>
+      </c>
+      <c r="F569" s="2">
+        <v>2.7</v>
+      </c>
+      <c r="G569" s="2">
+        <v>5.2</v>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:50</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D570" s="2">
+        <v>19.4</v>
+      </c>
+      <c r="E570" s="2">
+        <v>93.0</v>
+      </c>
+      <c r="F570" s="2">
+        <v>0.3</v>
+      </c>
+      <c r="G570" s="2">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:00</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D571" s="2">
+        <v>19.1</v>
+      </c>
+      <c r="E571" s="2">
+        <v>91.0</v>
+      </c>
+      <c r="F571" s="2">
+        <v>0.6</v>
+      </c>
+      <c r="G571" s="2">
+        <v>6.1</v>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:10</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D572" s="2">
+        <v>18.7</v>
+      </c>
+      <c r="E572" s="2">
+        <v>90.0</v>
+      </c>
+      <c r="F572" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="G572" s="2">
+        <v>6.3</v>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:20</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D573" s="2">
+        <v>18.9</v>
+      </c>
+      <c r="E573" s="2">
+        <v>90.0</v>
+      </c>
+      <c r="F573" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="G573" s="2">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:30</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D574" s="2">
+        <v>19.1</v>
+      </c>
+      <c r="E574" s="2">
+        <v>90.0</v>
+      </c>
+      <c r="F574" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G574" s="2">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:40</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D575" s="2">
+        <v>19.4</v>
+      </c>
+      <c r="E575" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F575" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G575" s="2">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:50</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D576" s="2">
+        <v>19.5</v>
+      </c>
+      <c r="E576" s="2">
+        <v>92.0</v>
+      </c>
+      <c r="F576" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G576" s="2">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:00</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D577" s="2">
+        <v>19.5</v>
+      </c>
+      <c r="E577" s="2">
+        <v>90.0</v>
+      </c>
+      <c r="F577" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G577" s="2">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:10</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D578" s="2">
+        <v>19.6</v>
+      </c>
+      <c r="E578" s="2">
+        <v>89.0</v>
+      </c>
+      <c r="F578" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G578" s="2">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:20</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D579" s="2">
+        <v>19.7</v>
+      </c>
+      <c r="E579" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F579" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G579" s="2">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:30</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D580" s="2">
+        <v>19.7</v>
+      </c>
+      <c r="E580" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F580" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G580" s="2">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:40</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D581" s="2">
+        <v>19.8</v>
+      </c>
+      <c r="E581" s="2">
+        <v>90.0</v>
+      </c>
+      <c r="F581" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G581" s="2">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:50</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D582" s="2">
+        <v>19.7</v>
+      </c>
+      <c r="E582" s="2">
+        <v>91.0</v>
+      </c>
+      <c r="F582" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G582" s="2">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:00</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D583" s="2">
+        <v>19.6</v>
+      </c>
+      <c r="E583" s="2">
+        <v>93.0</v>
+      </c>
+      <c r="F583" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="G583" s="2">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:10</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D584" s="2">
+        <v>19.6</v>
+      </c>
+      <c r="E584" s="2">
+        <v>93.0</v>
+      </c>
+      <c r="F584" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G584" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:20</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D585" s="2">
+        <v>19.5</v>
+      </c>
+      <c r="E585" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F585" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G585" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:30</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D586" s="2">
+        <v>19.4</v>
+      </c>
+      <c r="E586" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F586" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G586" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:40</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D587" s="2">
+        <v>19.4</v>
+      </c>
+      <c r="E587" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F587" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G587" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:50</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D588" s="2">
+        <v>19.4</v>
+      </c>
+      <c r="E588" s="2">
+        <v>95.0</v>
+      </c>
+      <c r="F588" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G588" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:00</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D589" s="2">
+        <v>19.3</v>
+      </c>
+      <c r="E589" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F589" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G589" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:10</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D590" s="2">
+        <v>19.3</v>
+      </c>
+      <c r="E590" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F590" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G590" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:20</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D591" s="2">
+        <v>19.2</v>
+      </c>
+      <c r="E591" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F591" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G591" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:30</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D592" s="2">
+        <v>19.2</v>
+      </c>
+      <c r="E592" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F592" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G592" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:40</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D593" s="2">
+        <v>19.3</v>
+      </c>
+      <c r="E593" s="2">
+        <v>95.0</v>
+      </c>
+      <c r="F593" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G593" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:50</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D594" s="2">
+        <v>19.3</v>
+      </c>
+      <c r="E594" s="2">
+        <v>95.0</v>
+      </c>
+      <c r="F594" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G594" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:00</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D595" s="2">
+        <v>19.4</v>
+      </c>
+      <c r="E595" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F595" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G595" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:10</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D596" s="2">
+        <v>19.3</v>
+      </c>
+      <c r="E596" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F596" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G596" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:20</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D597" s="2">
+        <v>19.4</v>
+      </c>
+      <c r="E597" s="2">
+        <v>93.0</v>
+      </c>
+      <c r="F597" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="G597" s="2">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:30</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D598" s="2">
+        <v>19.2</v>
+      </c>
+      <c r="E598" s="2">
+        <v>93.0</v>
+      </c>
+      <c r="F598" s="2">
+        <v>0.4</v>
+      </c>
+      <c r="G598" s="2">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:40</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D599" s="2">
+        <v>18.8</v>
+      </c>
+      <c r="E599" s="2">
+        <v>90.0</v>
+      </c>
+      <c r="F599" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="G599" s="2">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:50</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D600" s="2">
+        <v>18.5</v>
+      </c>
+      <c r="E600" s="2">
+        <v>91.0</v>
+      </c>
+      <c r="F600" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="G600" s="2">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:00</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D601" s="2">
+        <v>18.3</v>
+      </c>
+      <c r="E601" s="2">
+        <v>93.0</v>
+      </c>
+      <c r="F601" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="G601" s="2">
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:10</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D602" s="2">
+        <v>18.3</v>
+      </c>
+      <c r="E602" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F602" s="2">
+        <v>0.3</v>
+      </c>
+      <c r="G602" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:20</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D603" s="2">
+        <v>18.3</v>
+      </c>
+      <c r="E603" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F603" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G603" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:30</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D604" s="2">
+        <v>18.3</v>
+      </c>
+      <c r="E604" s="2">
+        <v>93.0</v>
+      </c>
+      <c r="F604" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G604" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:40</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D605" s="2">
+        <v>18.2</v>
+      </c>
+      <c r="E605" s="2">
+        <v>92.0</v>
+      </c>
+      <c r="F605" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G605" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18.07.2026</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:50</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D606" s="2">
+        <v>18.2</v>
+      </c>
+      <c r="E606" s="2">
+        <v>93.0</v>
+      </c>
+      <c r="F606" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G606" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:00</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D607" s="2">
+        <v>18.1</v>
+      </c>
+      <c r="E607" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F607" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G607" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:10</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D608" s="2">
+        <v>18.0</v>
+      </c>
+      <c r="E608" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F608" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G608" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:20</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D609" s="2">
+        <v>17.9</v>
+      </c>
+      <c r="E609" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F609" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G609" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G465"/>
+  <autoFilter ref="A1:G609"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ARSO Kranj zajem 2026-07-20 00:36 Europe/Ljubljana
</commit_message>
<xml_diff>
--- a/tabela_vremena/ARSO_Kranj.xlsx
+++ b/tabela_vremena/ARSO_Kranj.xlsx
@@ -17743,7 +17743,4183 @@
         <v>3.6</v>
       </c>
     </row>
+    <row r="610">
+      <c r="A610" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:30</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D610" s="2">
+        <v>17.8</v>
+      </c>
+      <c r="E610" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F610" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G610" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:40</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D611" s="2">
+        <v>17.7</v>
+      </c>
+      <c r="E611" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F611" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G611" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:50</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D612" s="2">
+        <v>17.6</v>
+      </c>
+      <c r="E612" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F612" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G612" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:00</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D613" s="2">
+        <v>17.5</v>
+      </c>
+      <c r="E613" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F613" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G613" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:10</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D614" s="2">
+        <v>17.6</v>
+      </c>
+      <c r="E614" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F614" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G614" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:20</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D615" s="2">
+        <v>17.6</v>
+      </c>
+      <c r="E615" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F615" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G615" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:30</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D616" s="2">
+        <v>17.6</v>
+      </c>
+      <c r="E616" s="2">
+        <v>93.0</v>
+      </c>
+      <c r="F616" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G616" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:40</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D617" s="2">
+        <v>17.5</v>
+      </c>
+      <c r="E617" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F617" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G617" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:50</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D618" s="2">
+        <v>17.5</v>
+      </c>
+      <c r="E618" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F618" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G618" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:00</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D619" s="2">
+        <v>17.4</v>
+      </c>
+      <c r="E619" s="2">
+        <v>93.0</v>
+      </c>
+      <c r="F619" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G619" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:10</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D620" s="2">
+        <v>17.3</v>
+      </c>
+      <c r="E620" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F620" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G620" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:20</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D621" s="2">
+        <v>17.3</v>
+      </c>
+      <c r="E621" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F621" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G621" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:30</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D622" s="2">
+        <v>17.3</v>
+      </c>
+      <c r="E622" s="2">
+        <v>92.0</v>
+      </c>
+      <c r="F622" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G622" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:40</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D623" s="2">
+        <v>17.2</v>
+      </c>
+      <c r="E623" s="2">
+        <v>92.0</v>
+      </c>
+      <c r="F623" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G623" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:50</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D624" s="2">
+        <v>17.2</v>
+      </c>
+      <c r="E624" s="2">
+        <v>92.0</v>
+      </c>
+      <c r="F624" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G624" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:00</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D625" s="2">
+        <v>17.0</v>
+      </c>
+      <c r="E625" s="2">
+        <v>93.0</v>
+      </c>
+      <c r="F625" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G625" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:10</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D626" s="2">
+        <v>17.0</v>
+      </c>
+      <c r="E626" s="2">
+        <v>93.0</v>
+      </c>
+      <c r="F626" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G626" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:20</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D627" s="2">
+        <v>17.0</v>
+      </c>
+      <c r="E627" s="2">
+        <v>93.0</v>
+      </c>
+      <c r="F627" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G627" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:30</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D628" s="2">
+        <v>17.1</v>
+      </c>
+      <c r="E628" s="2">
+        <v>93.0</v>
+      </c>
+      <c r="F628" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G628" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:40</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D629" s="2">
+        <v>17.0</v>
+      </c>
+      <c r="E629" s="2">
+        <v>92.0</v>
+      </c>
+      <c r="F629" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G629" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:50</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D630" s="2">
+        <v>16.9</v>
+      </c>
+      <c r="E630" s="2">
+        <v>92.0</v>
+      </c>
+      <c r="F630" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G630" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:00</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D631" s="2">
+        <v>16.9</v>
+      </c>
+      <c r="E631" s="2">
+        <v>92.0</v>
+      </c>
+      <c r="F631" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G631" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:10</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D632" s="2">
+        <v>16.7</v>
+      </c>
+      <c r="E632" s="2">
+        <v>92.0</v>
+      </c>
+      <c r="F632" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G632" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:20</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D633" s="2">
+        <v>16.7</v>
+      </c>
+      <c r="E633" s="2">
+        <v>93.0</v>
+      </c>
+      <c r="F633" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G633" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:30</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D634" s="2">
+        <v>16.5</v>
+      </c>
+      <c r="E634" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F634" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G634" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:40</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D635" s="2">
+        <v>16.3</v>
+      </c>
+      <c r="E635" s="2">
+        <v>93.0</v>
+      </c>
+      <c r="F635" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G635" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:50</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D636" s="2">
+        <v>16.1</v>
+      </c>
+      <c r="E636" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F636" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G636" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:00</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D637" s="2">
+        <v>16.0</v>
+      </c>
+      <c r="E637" s="2">
+        <v>95.0</v>
+      </c>
+      <c r="F637" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G637" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:10</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D638" s="2">
+        <v>15.9</v>
+      </c>
+      <c r="E638" s="2">
+        <v>95.0</v>
+      </c>
+      <c r="F638" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G638" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:20</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D639" s="2">
+        <v>15.8</v>
+      </c>
+      <c r="E639" s="2">
+        <v>95.0</v>
+      </c>
+      <c r="F639" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G639" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:30</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D640" s="2">
+        <v>15.6</v>
+      </c>
+      <c r="E640" s="2">
+        <v>95.0</v>
+      </c>
+      <c r="F640" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G640" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:40</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D641" s="2">
+        <v>15.6</v>
+      </c>
+      <c r="E641" s="2">
+        <v>95.0</v>
+      </c>
+      <c r="F641" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G641" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:50</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D642" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="E642" s="2">
+        <v>95.0</v>
+      </c>
+      <c r="F642" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G642" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:00</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D643" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="E643" s="2">
+        <v>95.0</v>
+      </c>
+      <c r="F643" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G643" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:10</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D644" s="2">
+        <v>15.4</v>
+      </c>
+      <c r="E644" s="2">
+        <v>95.0</v>
+      </c>
+      <c r="F644" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G644" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:20</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D645" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="E645" s="2">
+        <v>95.0</v>
+      </c>
+      <c r="F645" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G645" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:30</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D646" s="2">
+        <v>15.8</v>
+      </c>
+      <c r="E646" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F646" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G646" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:40</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D647" s="2">
+        <v>15.9</v>
+      </c>
+      <c r="E647" s="2">
+        <v>92.0</v>
+      </c>
+      <c r="F647" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G647" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:50</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D648" s="2">
+        <v>16.4</v>
+      </c>
+      <c r="E648" s="2">
+        <v>91.0</v>
+      </c>
+      <c r="F648" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G648" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:00</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D649" s="2">
+        <v>17.1</v>
+      </c>
+      <c r="E649" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F649" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G649" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:10</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D650" s="2">
+        <v>17.1</v>
+      </c>
+      <c r="E650" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F650" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G650" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:20</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D651" s="2">
+        <v>17.6</v>
+      </c>
+      <c r="E651" s="2">
+        <v>83.0</v>
+      </c>
+      <c r="F651" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G651" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:30</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D652" s="2">
+        <v>18.0</v>
+      </c>
+      <c r="E652" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F652" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G652" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:40</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D653" s="2">
+        <v>18.3</v>
+      </c>
+      <c r="E653" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F653" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G653" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:50</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D654" s="2">
+        <v>18.7</v>
+      </c>
+      <c r="E654" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F654" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G654" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:00</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D655" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="E655" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F655" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G655" s="2">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:10</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D656" s="2">
+        <v>19.5</v>
+      </c>
+      <c r="E656" s="2">
+        <v>74.0</v>
+      </c>
+      <c r="F656" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G656" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:20</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D657" s="2">
+        <v>19.6</v>
+      </c>
+      <c r="E657" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F657" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G657" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:30</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D658" s="2">
+        <v>19.6</v>
+      </c>
+      <c r="E658" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F658" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G658" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:40</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D659" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="E659" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="F659" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G659" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:50</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D660" s="2">
+        <v>20.2</v>
+      </c>
+      <c r="E660" s="2">
+        <v>74.0</v>
+      </c>
+      <c r="F660" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G660" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:00</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D661" s="2">
+        <v>20.7</v>
+      </c>
+      <c r="E661" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F661" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G661" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:10</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D662" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="E662" s="2">
+        <v>69.0</v>
+      </c>
+      <c r="F662" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G662" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:20</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D663" s="2">
+        <v>21.4</v>
+      </c>
+      <c r="E663" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F663" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G663" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:30</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D664" s="2">
+        <v>21.6</v>
+      </c>
+      <c r="E664" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F664" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G664" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:40</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D665" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="E665" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F665" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G665" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:50</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D666" s="2">
+        <v>22.7</v>
+      </c>
+      <c r="E666" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F666" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G666" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:00</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D667" s="2">
+        <v>22.8</v>
+      </c>
+      <c r="E667" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F667" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G667" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:10</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D668" s="2">
+        <v>23.5</v>
+      </c>
+      <c r="E668" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F668" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G668" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:20</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D669" s="2">
+        <v>23.8</v>
+      </c>
+      <c r="E669" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F669" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G669" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:30</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D670" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="E670" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F670" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G670" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:40</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D671" s="2">
+        <v>24.5</v>
+      </c>
+      <c r="E671" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F671" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G671" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:50</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D672" s="2">
+        <v>24.8</v>
+      </c>
+      <c r="E672" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F672" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G672" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:00</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D673" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="E673" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F673" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G673" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:10</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D674" s="2">
+        <v>25.4</v>
+      </c>
+      <c r="E674" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F674" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G674" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:20</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D675" s="2">
+        <v>25.3</v>
+      </c>
+      <c r="E675" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F675" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G675" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:30</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D676" s="2">
+        <v>25.7</v>
+      </c>
+      <c r="E676" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F676" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G676" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:40</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D677" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="E677" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F677" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G677" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:50</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D678" s="2">
+        <v>25.9</v>
+      </c>
+      <c r="E678" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F678" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G678" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:00</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D679" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="E679" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F679" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G679" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:10</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D680" s="2">
+        <v>26.4</v>
+      </c>
+      <c r="E680" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F680" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G680" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:20</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D681" s="2">
+        <v>26.4</v>
+      </c>
+      <c r="E681" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F681" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G681" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:30</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D682" s="2">
+        <v>26.8</v>
+      </c>
+      <c r="E682" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F682" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G682" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:40</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D683" s="2">
+        <v>27.6</v>
+      </c>
+      <c r="E683" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F683" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G683" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:50</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D684" s="2">
+        <v>27.4</v>
+      </c>
+      <c r="E684" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F684" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G684" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:00</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D685" s="2">
+        <v>27.2</v>
+      </c>
+      <c r="E685" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F685" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G685" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:10</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D686" s="2">
+        <v>27.7</v>
+      </c>
+      <c r="E686" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F686" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G686" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:20</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D687" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="E687" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F687" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G687" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:30</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D688" s="2">
+        <v>28.2</v>
+      </c>
+      <c r="E688" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F688" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G688" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:40</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D689" s="2">
+        <v>28.3</v>
+      </c>
+      <c r="E689" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F689" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G689" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:50</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D690" s="2">
+        <v>28.7</v>
+      </c>
+      <c r="E690" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F690" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G690" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:00</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D691" s="2">
+        <v>28.5</v>
+      </c>
+      <c r="E691" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F691" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G691" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:10</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D692" s="2">
+        <v>28.4</v>
+      </c>
+      <c r="E692" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F692" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G692" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:20</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D693" s="2">
+        <v>28.6</v>
+      </c>
+      <c r="E693" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F693" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G693" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:30</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D694" s="2">
+        <v>29.3</v>
+      </c>
+      <c r="E694" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F694" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G694" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:40</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D695" s="2">
+        <v>29.2</v>
+      </c>
+      <c r="E695" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F695" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G695" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:50</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D696" s="2">
+        <v>29.3</v>
+      </c>
+      <c r="E696" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F696" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G696" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:00</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D697" s="2">
+        <v>29.5</v>
+      </c>
+      <c r="E697" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F697" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G697" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:10</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D698" s="2">
+        <v>29.7</v>
+      </c>
+      <c r="E698" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F698" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G698" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:20</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D699" s="2">
+        <v>29.3</v>
+      </c>
+      <c r="E699" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F699" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G699" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:30</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D700" s="2">
+        <v>29.3</v>
+      </c>
+      <c r="E700" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F700" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G700" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:40</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D701" s="2">
+        <v>29.6</v>
+      </c>
+      <c r="E701" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F701" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G701" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:50</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D702" s="2">
+        <v>29.4</v>
+      </c>
+      <c r="E702" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F702" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G702" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:00</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D703" s="2">
+        <v>29.5</v>
+      </c>
+      <c r="E703" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F703" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G703" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:10</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D704" s="2">
+        <v>29.4</v>
+      </c>
+      <c r="E704" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F704" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G704" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:20</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D705" s="2">
+        <v>29.2</v>
+      </c>
+      <c r="E705" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F705" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G705" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:30</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D706" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="E706" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F706" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G706" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:40</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D707" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="E707" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F707" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G707" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:50</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D708" s="2">
+        <v>28.2</v>
+      </c>
+      <c r="E708" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F708" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G708" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B709" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:00</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D709" s="2">
+        <v>26.7</v>
+      </c>
+      <c r="E709" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F709" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G709" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:10</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D710" s="2">
+        <v>24.3</v>
+      </c>
+      <c r="E710" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F710" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G710" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:20</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D711" s="2">
+        <v>24.2</v>
+      </c>
+      <c r="E711" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F711" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G711" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:30</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D712" s="2">
+        <v>24.2</v>
+      </c>
+      <c r="E712" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F712" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G712" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:40</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D713" s="2">
+        <v>23.6</v>
+      </c>
+      <c r="E713" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F713" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G713" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:50</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D714" s="2">
+        <v>22.2</v>
+      </c>
+      <c r="E714" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F714" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G714" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:00</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D715" s="2">
+        <v>22.1</v>
+      </c>
+      <c r="E715" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F715" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G715" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B716" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:10</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D716" s="2">
+        <v>22.2</v>
+      </c>
+      <c r="E716" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F716" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G716" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B717" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:20</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D717" s="2">
+        <v>22.2</v>
+      </c>
+      <c r="E717" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F717" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G717" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B718" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:30</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D718" s="2">
+        <v>22.2</v>
+      </c>
+      <c r="E718" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F718" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G718" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B719" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:40</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D719" s="2">
+        <v>22.2</v>
+      </c>
+      <c r="E719" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F719" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G719" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:50</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D720" s="2">
+        <v>22.3</v>
+      </c>
+      <c r="E720" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F720" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G720" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:00</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D721" s="2">
+        <v>22.2</v>
+      </c>
+      <c r="E721" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F721" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G721" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:10</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D722" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="E722" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F722" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G722" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:20</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D723" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="E723" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F723" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G723" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:30</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D724" s="2">
+        <v>21.9</v>
+      </c>
+      <c r="E724" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F724" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G724" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:40</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D725" s="2">
+        <v>21.9</v>
+      </c>
+      <c r="E725" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F725" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G725" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:50</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D726" s="2">
+        <v>21.8</v>
+      </c>
+      <c r="E726" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F726" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G726" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:00</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D727" s="2">
+        <v>21.9</v>
+      </c>
+      <c r="E727" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F727" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G727" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:10</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D728" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="E728" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F728" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G728" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:20</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D729" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="E729" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F729" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G729" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:30</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D730" s="2">
+        <v>22.1</v>
+      </c>
+      <c r="E730" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F730" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G730" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:40</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D731" s="2">
+        <v>22.1</v>
+      </c>
+      <c r="E731" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F731" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G731" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:50</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D732" s="2">
+        <v>21.9</v>
+      </c>
+      <c r="E732" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F732" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G732" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:00</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D733" s="2">
+        <v>21.6</v>
+      </c>
+      <c r="E733" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F733" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G733" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:10</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D734" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="E734" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F734" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G734" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:20</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D735" s="2">
+        <v>20.4</v>
+      </c>
+      <c r="E735" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F735" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G735" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:30</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D736" s="2">
+        <v>20.2</v>
+      </c>
+      <c r="E736" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F736" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G736" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:40</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D737" s="2">
+        <v>19.9</v>
+      </c>
+      <c r="E737" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F737" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G737" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:50</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D738" s="2">
+        <v>19.6</v>
+      </c>
+      <c r="E738" s="2">
+        <v>72.0</v>
+      </c>
+      <c r="F738" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G738" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:00</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D739" s="2">
+        <v>19.4</v>
+      </c>
+      <c r="E739" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="F739" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G739" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:10</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D740" s="2">
+        <v>19.1</v>
+      </c>
+      <c r="E740" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F740" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G740" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:20</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D741" s="2">
+        <v>18.8</v>
+      </c>
+      <c r="E741" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F741" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G741" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:30</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D742" s="2">
+        <v>18.5</v>
+      </c>
+      <c r="E742" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F742" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G742" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:40</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D743" s="2">
+        <v>18.3</v>
+      </c>
+      <c r="E743" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F743" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G743" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:50</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D744" s="2">
+        <v>18.0</v>
+      </c>
+      <c r="E744" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F744" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G744" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:00</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D745" s="2">
+        <v>17.7</v>
+      </c>
+      <c r="E745" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F745" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G745" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:10</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D746" s="2">
+        <v>17.6</v>
+      </c>
+      <c r="E746" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F746" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G746" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:20</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D747" s="2">
+        <v>17.4</v>
+      </c>
+      <c r="E747" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F747" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G747" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:30</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D748" s="2">
+        <v>17.7</v>
+      </c>
+      <c r="E748" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F748" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G748" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:40</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D749" s="2">
+        <v>17.7</v>
+      </c>
+      <c r="E749" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F749" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G749" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19.07.2026</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:50</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D750" s="2">
+        <v>17.7</v>
+      </c>
+      <c r="E750" s="2">
+        <v>81.0</v>
+      </c>
+      <c r="F750" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G750" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:00</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D751" s="2">
+        <v>17.6</v>
+      </c>
+      <c r="E751" s="2">
+        <v>81.0</v>
+      </c>
+      <c r="F751" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G751" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:10</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D752" s="2">
+        <v>17.2</v>
+      </c>
+      <c r="E752" s="2">
+        <v>83.0</v>
+      </c>
+      <c r="F752" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G752" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:20</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D753" s="2">
+        <v>16.9</v>
+      </c>
+      <c r="E753" s="2">
+        <v>84.0</v>
+      </c>
+      <c r="F753" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G753" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G609"/>
+  <autoFilter ref="A1:G753"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ARSO Kranj zajem 2026-07-21 00:42 Europe/Ljubljana
</commit_message>
<xml_diff>
--- a/tabela_vremena/ARSO_Kranj.xlsx
+++ b/tabela_vremena/ARSO_Kranj.xlsx
@@ -21919,7 +21919,4096 @@
         <v>0.0</v>
       </c>
     </row>
+    <row r="754">
+      <c r="A754" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:30</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D754" s="2">
+        <v>16.6</v>
+      </c>
+      <c r="E754" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F754" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G754" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:40</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D755" s="2">
+        <v>16.5</v>
+      </c>
+      <c r="E755" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F755" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G755" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B756" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:50</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D756" s="2">
+        <v>16.3</v>
+      </c>
+      <c r="E756" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F756" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G756" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B757" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:00</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D757" s="2">
+        <v>16.0</v>
+      </c>
+      <c r="E757" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F757" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G757" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B758" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:10</t>
+        </is>
+      </c>
+      <c r="C758" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D758" s="2">
+        <v>15.8</v>
+      </c>
+      <c r="E758" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F758" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G758" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B759" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:20</t>
+        </is>
+      </c>
+      <c r="C759" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D759" s="2">
+        <v>15.6</v>
+      </c>
+      <c r="E759" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F759" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G759" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B760" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:30</t>
+        </is>
+      </c>
+      <c r="C760" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D760" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="E760" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F760" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G760" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B761" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:40</t>
+        </is>
+      </c>
+      <c r="C761" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D761" s="2">
+        <v>15.4</v>
+      </c>
+      <c r="E761" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F761" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G761" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B762" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:50</t>
+        </is>
+      </c>
+      <c r="C762" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D762" s="2">
+        <v>15.2</v>
+      </c>
+      <c r="E762" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F762" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G762" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B763" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:00</t>
+        </is>
+      </c>
+      <c r="C763" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D763" s="2">
+        <v>15.1</v>
+      </c>
+      <c r="E763" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F763" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G763" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B764" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:10</t>
+        </is>
+      </c>
+      <c r="C764" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D764" s="2">
+        <v>15.0</v>
+      </c>
+      <c r="E764" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F764" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G764" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B765" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:20</t>
+        </is>
+      </c>
+      <c r="C765" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D765" s="2">
+        <v>14.9</v>
+      </c>
+      <c r="E765" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F765" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G765" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B766" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:30</t>
+        </is>
+      </c>
+      <c r="C766" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D766" s="2">
+        <v>14.8</v>
+      </c>
+      <c r="E766" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F766" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G766" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B767" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:40</t>
+        </is>
+      </c>
+      <c r="C767" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D767" s="2">
+        <v>14.7</v>
+      </c>
+      <c r="E767" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F767" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G767" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B768" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:50</t>
+        </is>
+      </c>
+      <c r="C768" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D768" s="2">
+        <v>14.5</v>
+      </c>
+      <c r="E768" s="2">
+        <v>89.0</v>
+      </c>
+      <c r="F768" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G768" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B769" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:00</t>
+        </is>
+      </c>
+      <c r="C769" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D769" s="2">
+        <v>14.5</v>
+      </c>
+      <c r="E769" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F769" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G769" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B770" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:10</t>
+        </is>
+      </c>
+      <c r="C770" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D770" s="2">
+        <v>14.5</v>
+      </c>
+      <c r="E770" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F770" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G770" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B771" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:20</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D771" s="2">
+        <v>14.4</v>
+      </c>
+      <c r="E771" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F771" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G771" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B772" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:30</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D772" s="2">
+        <v>14.4</v>
+      </c>
+      <c r="E772" s="2">
+        <v>89.0</v>
+      </c>
+      <c r="F772" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G772" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B773" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:40</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D773" s="2">
+        <v>14.3</v>
+      </c>
+      <c r="E773" s="2">
+        <v>89.0</v>
+      </c>
+      <c r="F773" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G773" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B774" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:50</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D774" s="2">
+        <v>14.3</v>
+      </c>
+      <c r="E774" s="2">
+        <v>89.0</v>
+      </c>
+      <c r="F774" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G774" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B775" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:00</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D775" s="2">
+        <v>14.3</v>
+      </c>
+      <c r="E775" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F775" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G775" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B776" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:10</t>
+        </is>
+      </c>
+      <c r="C776" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D776" s="2">
+        <v>14.2</v>
+      </c>
+      <c r="E776" s="2">
+        <v>89.0</v>
+      </c>
+      <c r="F776" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G776" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B777" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:20</t>
+        </is>
+      </c>
+      <c r="C777" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D777" s="2">
+        <v>14.1</v>
+      </c>
+      <c r="E777" s="2">
+        <v>89.0</v>
+      </c>
+      <c r="F777" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G777" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B778" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:30</t>
+        </is>
+      </c>
+      <c r="C778" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D778" s="2">
+        <v>14.1</v>
+      </c>
+      <c r="E778" s="2">
+        <v>89.0</v>
+      </c>
+      <c r="F778" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G778" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B779" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:40</t>
+        </is>
+      </c>
+      <c r="C779" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D779" s="2">
+        <v>14.1</v>
+      </c>
+      <c r="E779" s="2">
+        <v>89.0</v>
+      </c>
+      <c r="F779" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G779" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B780" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:50</t>
+        </is>
+      </c>
+      <c r="C780" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D780" s="2">
+        <v>14.1</v>
+      </c>
+      <c r="E780" s="2">
+        <v>89.0</v>
+      </c>
+      <c r="F780" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G780" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B781" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:00</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D781" s="2">
+        <v>14.2</v>
+      </c>
+      <c r="E781" s="2">
+        <v>89.0</v>
+      </c>
+      <c r="F781" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G781" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B782" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:10</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D782" s="2">
+        <v>14.3</v>
+      </c>
+      <c r="E782" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F782" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G782" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B783" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:20</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D783" s="2">
+        <v>14.4</v>
+      </c>
+      <c r="E783" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F783" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G783" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B784" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:30</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D784" s="2">
+        <v>14.4</v>
+      </c>
+      <c r="E784" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F784" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G784" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B785" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:40</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D785" s="2">
+        <v>14.6</v>
+      </c>
+      <c r="E785" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F785" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G785" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B786" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:50</t>
+        </is>
+      </c>
+      <c r="C786" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D786" s="2">
+        <v>14.8</v>
+      </c>
+      <c r="E786" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F786" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G786" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B787" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:00</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D787" s="2">
+        <v>14.8</v>
+      </c>
+      <c r="E787" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F787" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G787" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B788" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:10</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D788" s="2">
+        <v>14.9</v>
+      </c>
+      <c r="E788" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F788" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G788" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B789" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:20</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D789" s="2">
+        <v>15.0</v>
+      </c>
+      <c r="E789" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F789" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G789" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B790" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:30</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D790" s="2">
+        <v>15.1</v>
+      </c>
+      <c r="E790" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F790" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G790" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B791" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:40</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D791" s="2">
+        <v>15.1</v>
+      </c>
+      <c r="E791" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F791" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G791" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B792" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:50</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D792" s="2">
+        <v>15.1</v>
+      </c>
+      <c r="E792" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F792" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G792" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B793" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:00</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D793" s="2">
+        <v>15.1</v>
+      </c>
+      <c r="E793" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F793" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="G793" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B794" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:10</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D794" s="2">
+        <v>15.1</v>
+      </c>
+      <c r="E794" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F794" s="2">
+        <v>0.3</v>
+      </c>
+      <c r="G794" s="2">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B795" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:20</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D795" s="2">
+        <v>15.2</v>
+      </c>
+      <c r="E795" s="2">
+        <v>89.0</v>
+      </c>
+      <c r="F795" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G795" s="2">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B796" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:30</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D796" s="2">
+        <v>15.3</v>
+      </c>
+      <c r="E796" s="2">
+        <v>89.0</v>
+      </c>
+      <c r="F796" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G796" s="2">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B797" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:40</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D797" s="2">
+        <v>15.4</v>
+      </c>
+      <c r="E797" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F797" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G797" s="2">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B798" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:50</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D798" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="E798" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F798" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G798" s="2">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B799" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:00</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D799" s="2">
+        <v>15.7</v>
+      </c>
+      <c r="E799" s="2">
+        <v>89.0</v>
+      </c>
+      <c r="F799" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G799" s="2">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B800" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:10</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D800" s="2">
+        <v>16.1</v>
+      </c>
+      <c r="E800" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F800" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G800" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B801" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:20</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D801" s="2">
+        <v>16.2</v>
+      </c>
+      <c r="E801" s="2">
+        <v>84.0</v>
+      </c>
+      <c r="F801" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G801" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B802" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:30</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D802" s="2">
+        <v>16.6</v>
+      </c>
+      <c r="E802" s="2">
+        <v>84.0</v>
+      </c>
+      <c r="F802" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G802" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B803" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:40</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D803" s="2">
+        <v>17.2</v>
+      </c>
+      <c r="E803" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F803" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G803" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B804" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:50</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D804" s="2">
+        <v>17.7</v>
+      </c>
+      <c r="E804" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F804" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G804" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B805" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:00</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D805" s="2">
+        <v>17.8</v>
+      </c>
+      <c r="E805" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F805" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G805" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B806" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:10</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D806" s="2">
+        <v>18.1</v>
+      </c>
+      <c r="E806" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F806" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G806" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B807" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:20</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D807" s="2">
+        <v>18.4</v>
+      </c>
+      <c r="E807" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F807" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G807" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B808" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:30</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D808" s="2">
+        <v>18.4</v>
+      </c>
+      <c r="E808" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F808" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G808" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B809" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:40</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D809" s="2">
+        <v>18.5</v>
+      </c>
+      <c r="E809" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="F809" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G809" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B810" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:30</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D810" s="2">
+        <v>20.9</v>
+      </c>
+      <c r="E810" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F810" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G810" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B811" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:40</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D811" s="2">
+        <v>20.9</v>
+      </c>
+      <c r="E811" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F811" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G811" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B812" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:50</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D812" s="2">
+        <v>20.6</v>
+      </c>
+      <c r="E812" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F812" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G812" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B813" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:00</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D813" s="2">
+        <v>20.7</v>
+      </c>
+      <c r="E813" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F813" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G813" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B814" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:10</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D814" s="2">
+        <v>20.8</v>
+      </c>
+      <c r="E814" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F814" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G814" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B815" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:20</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D815" s="2">
+        <v>21.1</v>
+      </c>
+      <c r="E815" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F815" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G815" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B816" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:30</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D816" s="2">
+        <v>21.6</v>
+      </c>
+      <c r="E816" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F816" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G816" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B817" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:40</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D817" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="E817" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F817" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G817" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B818" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:50</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D818" s="2">
+        <v>22.5</v>
+      </c>
+      <c r="E818" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F818" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G818" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B819" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:00</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D819" s="2">
+        <v>22.7</v>
+      </c>
+      <c r="E819" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F819" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G819" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B820" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:10</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D820" s="2">
+        <v>22.4</v>
+      </c>
+      <c r="E820" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F820" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G820" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B821" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:20</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D821" s="2">
+        <v>22.6</v>
+      </c>
+      <c r="E821" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F821" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G821" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B822" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:30</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D822" s="2">
+        <v>23.2</v>
+      </c>
+      <c r="E822" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F822" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G822" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B823" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:40</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D823" s="2">
+        <v>23.8</v>
+      </c>
+      <c r="E823" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F823" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G823" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B824" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:50</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D824" s="2">
+        <v>23.9</v>
+      </c>
+      <c r="E824" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F824" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G824" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B825" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:00</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D825" s="2">
+        <v>24.1</v>
+      </c>
+      <c r="E825" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F825" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G825" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B826" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:10</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D826" s="2">
+        <v>24.7</v>
+      </c>
+      <c r="E826" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F826" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G826" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B827" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:20</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D827" s="2">
+        <v>24.2</v>
+      </c>
+      <c r="E827" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F827" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G827" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B828" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:30</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D828" s="2">
+        <v>24.9</v>
+      </c>
+      <c r="E828" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F828" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G828" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B829" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:40</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D829" s="2">
+        <v>25.3</v>
+      </c>
+      <c r="E829" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F829" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G829" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B830" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:50</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D830" s="2">
+        <v>25.3</v>
+      </c>
+      <c r="E830" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F830" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G830" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B831" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:00</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D831" s="2">
+        <v>25.5</v>
+      </c>
+      <c r="E831" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F831" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G831" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B832" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:10</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D832" s="2">
+        <v>25.3</v>
+      </c>
+      <c r="E832" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F832" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G832" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B833" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:20</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D833" s="2">
+        <v>25.2</v>
+      </c>
+      <c r="E833" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F833" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G833" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B834" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:30</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D834" s="2">
+        <v>25.8</v>
+      </c>
+      <c r="E834" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F834" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G834" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B835" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:40</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D835" s="2">
+        <v>25.5</v>
+      </c>
+      <c r="E835" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F835" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G835" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B836" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:50</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D836" s="2">
+        <v>25.1</v>
+      </c>
+      <c r="E836" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F836" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G836" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B837" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:00</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D837" s="2">
+        <v>25.4</v>
+      </c>
+      <c r="E837" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F837" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G837" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B838" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:10</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D838" s="2">
+        <v>25.5</v>
+      </c>
+      <c r="E838" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F838" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G838" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B839" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:20</t>
+        </is>
+      </c>
+      <c r="C839" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D839" s="2">
+        <v>25.8</v>
+      </c>
+      <c r="E839" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F839" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G839" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B840" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:30</t>
+        </is>
+      </c>
+      <c r="C840" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D840" s="2">
+        <v>25.2</v>
+      </c>
+      <c r="E840" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F840" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G840" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B841" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:40</t>
+        </is>
+      </c>
+      <c r="C841" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D841" s="2">
+        <v>25.3</v>
+      </c>
+      <c r="E841" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F841" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G841" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B842" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:50</t>
+        </is>
+      </c>
+      <c r="C842" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D842" s="2">
+        <v>25.2</v>
+      </c>
+      <c r="E842" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F842" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G842" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B843" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:00</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D843" s="2">
+        <v>24.8</v>
+      </c>
+      <c r="E843" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F843" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G843" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B844" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:10</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D844" s="2">
+        <v>24.9</v>
+      </c>
+      <c r="E844" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F844" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G844" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B845" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:20</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D845" s="2">
+        <v>24.6</v>
+      </c>
+      <c r="E845" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F845" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G845" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:30</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D846" s="2">
+        <v>24.9</v>
+      </c>
+      <c r="E846" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F846" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G846" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:40</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D847" s="2">
+        <v>24.5</v>
+      </c>
+      <c r="E847" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F847" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G847" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B848" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:50</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D848" s="2">
+        <v>25.1</v>
+      </c>
+      <c r="E848" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F848" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G848" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:00</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D849" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="E849" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F849" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G849" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:10</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D850" s="2">
+        <v>25.1</v>
+      </c>
+      <c r="E850" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F850" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G850" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B851" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:20</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D851" s="2">
+        <v>25.2</v>
+      </c>
+      <c r="E851" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F851" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G851" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B852" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:30</t>
+        </is>
+      </c>
+      <c r="C852" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D852" s="2">
+        <v>25.2</v>
+      </c>
+      <c r="E852" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F852" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G852" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:40</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D853" s="2">
+        <v>25.8</v>
+      </c>
+      <c r="E853" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F853" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G853" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B854" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:50</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D854" s="2">
+        <v>26.1</v>
+      </c>
+      <c r="E854" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F854" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G854" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:00</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D855" s="2">
+        <v>25.9</v>
+      </c>
+      <c r="E855" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F855" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G855" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:10</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D856" s="2">
+        <v>25.8</v>
+      </c>
+      <c r="E856" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F856" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G856" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:20</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D857" s="2">
+        <v>25.8</v>
+      </c>
+      <c r="E857" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F857" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G857" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B858" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:30</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D858" s="2">
+        <v>25.8</v>
+      </c>
+      <c r="E858" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F858" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G858" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B859" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:40</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D859" s="2">
+        <v>25.5</v>
+      </c>
+      <c r="E859" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F859" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G859" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B860" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:50</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D860" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="E860" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F860" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G860" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B861" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:00</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D861" s="2">
+        <v>25.4</v>
+      </c>
+      <c r="E861" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F861" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G861" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B862" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:10</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D862" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="E862" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F862" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G862" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B863" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:20</t>
+        </is>
+      </c>
+      <c r="C863" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D863" s="2">
+        <v>24.6</v>
+      </c>
+      <c r="E863" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F863" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G863" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B864" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:30</t>
+        </is>
+      </c>
+      <c r="C864" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D864" s="2">
+        <v>24.4</v>
+      </c>
+      <c r="E864" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F864" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G864" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B865" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:40</t>
+        </is>
+      </c>
+      <c r="C865" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D865" s="2">
+        <v>24.5</v>
+      </c>
+      <c r="E865" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F865" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G865" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B866" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:50</t>
+        </is>
+      </c>
+      <c r="C866" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D866" s="2">
+        <v>24.1</v>
+      </c>
+      <c r="E866" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F866" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G866" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B867" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:00</t>
+        </is>
+      </c>
+      <c r="C867" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D867" s="2">
+        <v>23.7</v>
+      </c>
+      <c r="E867" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F867" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G867" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B868" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:10</t>
+        </is>
+      </c>
+      <c r="C868" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D868" s="2">
+        <v>23.5</v>
+      </c>
+      <c r="E868" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F868" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G868" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B869" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:20</t>
+        </is>
+      </c>
+      <c r="C869" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D869" s="2">
+        <v>23.3</v>
+      </c>
+      <c r="E869" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F869" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G869" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B870" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:30</t>
+        </is>
+      </c>
+      <c r="C870" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D870" s="2">
+        <v>23.1</v>
+      </c>
+      <c r="E870" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F870" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G870" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B871" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:40</t>
+        </is>
+      </c>
+      <c r="C871" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D871" s="2">
+        <v>22.8</v>
+      </c>
+      <c r="E871" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F871" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G871" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B872" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:50</t>
+        </is>
+      </c>
+      <c r="C872" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D872" s="2">
+        <v>22.6</v>
+      </c>
+      <c r="E872" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F872" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G872" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B873" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:00</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D873" s="2">
+        <v>22.3</v>
+      </c>
+      <c r="E873" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F873" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G873" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B874" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:10</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D874" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="E874" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F874" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G874" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B875" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:20</t>
+        </is>
+      </c>
+      <c r="C875" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D875" s="2">
+        <v>21.8</v>
+      </c>
+      <c r="E875" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F875" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G875" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B876" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:30</t>
+        </is>
+      </c>
+      <c r="C876" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D876" s="2">
+        <v>21.4</v>
+      </c>
+      <c r="E876" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F876" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G876" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B877" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:40</t>
+        </is>
+      </c>
+      <c r="C877" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D877" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="E877" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F877" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G877" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B878" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:50</t>
+        </is>
+      </c>
+      <c r="C878" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D878" s="2">
+        <v>20.5</v>
+      </c>
+      <c r="E878" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F878" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G878" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B879" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:00</t>
+        </is>
+      </c>
+      <c r="C879" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D879" s="2">
+        <v>20.1</v>
+      </c>
+      <c r="E879" s="2">
+        <v>69.0</v>
+      </c>
+      <c r="F879" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G879" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B880" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:10</t>
+        </is>
+      </c>
+      <c r="C880" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D880" s="2">
+        <v>19.9</v>
+      </c>
+      <c r="E880" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F880" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G880" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B881" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:20</t>
+        </is>
+      </c>
+      <c r="C881" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D881" s="2">
+        <v>19.5</v>
+      </c>
+      <c r="E881" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="F881" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G881" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B882" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:30</t>
+        </is>
+      </c>
+      <c r="C882" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D882" s="2">
+        <v>19.3</v>
+      </c>
+      <c r="E882" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F882" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G882" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B883" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:40</t>
+        </is>
+      </c>
+      <c r="C883" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D883" s="2">
+        <v>19.1</v>
+      </c>
+      <c r="E883" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F883" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G883" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B884" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:50</t>
+        </is>
+      </c>
+      <c r="C884" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D884" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="E884" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F884" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G884" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B885" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:00</t>
+        </is>
+      </c>
+      <c r="C885" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D885" s="2">
+        <v>18.8</v>
+      </c>
+      <c r="E885" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F885" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G885" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B886" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:10</t>
+        </is>
+      </c>
+      <c r="C886" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D886" s="2">
+        <v>18.6</v>
+      </c>
+      <c r="E886" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F886" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G886" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B887" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:20</t>
+        </is>
+      </c>
+      <c r="C887" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D887" s="2">
+        <v>18.4</v>
+      </c>
+      <c r="E887" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F887" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G887" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B888" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:30</t>
+        </is>
+      </c>
+      <c r="C888" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D888" s="2">
+        <v>18.2</v>
+      </c>
+      <c r="E888" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F888" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G888" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B889" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:40</t>
+        </is>
+      </c>
+      <c r="C889" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D889" s="2">
+        <v>18.1</v>
+      </c>
+      <c r="E889" s="2">
+        <v>81.0</v>
+      </c>
+      <c r="F889" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G889" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20.07.2026</t>
+        </is>
+      </c>
+      <c r="B890" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:50</t>
+        </is>
+      </c>
+      <c r="C890" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D890" s="2">
+        <v>18.0</v>
+      </c>
+      <c r="E890" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F890" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G890" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21.07.2026</t>
+        </is>
+      </c>
+      <c r="B891" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:00</t>
+        </is>
+      </c>
+      <c r="C891" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D891" s="2">
+        <v>17.9</v>
+      </c>
+      <c r="E891" s="2">
+        <v>81.0</v>
+      </c>
+      <c r="F891" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G891" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21.07.2026</t>
+        </is>
+      </c>
+      <c r="B892" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:10</t>
+        </is>
+      </c>
+      <c r="C892" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D892" s="2">
+        <v>17.8</v>
+      </c>
+      <c r="E892" s="2">
+        <v>81.0</v>
+      </c>
+      <c r="F892" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G892" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21.07.2026</t>
+        </is>
+      </c>
+      <c r="B893" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:20</t>
+        </is>
+      </c>
+      <c r="C893" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D893" s="2">
+        <v>17.8</v>
+      </c>
+      <c r="E893" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F893" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G893" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21.07.2026</t>
+        </is>
+      </c>
+      <c r="B894" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:30</t>
+        </is>
+      </c>
+      <c r="C894" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D894" s="2">
+        <v>17.6</v>
+      </c>
+      <c r="E894" s="2">
+        <v>83.0</v>
+      </c>
+      <c r="F894" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G894" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G753"/>
+  <autoFilter ref="A1:G894"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ARSO Kranj zajem 2026-07-24 00:41 Europe/Ljubljana
</commit_message>
<xml_diff>
--- a/tabela_vremena/ARSO_Kranj.xlsx
+++ b/tabela_vremena/ARSO_Kranj.xlsx
@@ -34476,7 +34476,4154 @@
         <v>0.0</v>
       </c>
     </row>
+    <row r="1187">
+      <c r="A1187" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1187" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:40</t>
+        </is>
+      </c>
+      <c r="C1187" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1187" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="E1187" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F1187" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1187" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1188" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:50</t>
+        </is>
+      </c>
+      <c r="C1188" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1188" s="2">
+        <v>15.3</v>
+      </c>
+      <c r="E1188" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F1188" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1188" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1189" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:00</t>
+        </is>
+      </c>
+      <c r="C1189" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1189" s="2">
+        <v>15.1</v>
+      </c>
+      <c r="E1189" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F1189" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1189" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1190" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:10</t>
+        </is>
+      </c>
+      <c r="C1190" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1190" s="2">
+        <v>15.0</v>
+      </c>
+      <c r="E1190" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F1190" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1190" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1191" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:20</t>
+        </is>
+      </c>
+      <c r="C1191" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1191" s="2">
+        <v>15.0</v>
+      </c>
+      <c r="E1191" s="2">
+        <v>72.0</v>
+      </c>
+      <c r="F1191" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1191" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1192" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:30</t>
+        </is>
+      </c>
+      <c r="C1192" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1192" s="2">
+        <v>15.0</v>
+      </c>
+      <c r="E1192" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F1192" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1192" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1193">
+      <c r="A1193" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1193" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:40</t>
+        </is>
+      </c>
+      <c r="C1193" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1193" s="2">
+        <v>14.9</v>
+      </c>
+      <c r="E1193" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F1193" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1193" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1194" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:50</t>
+        </is>
+      </c>
+      <c r="C1194" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1194" s="2">
+        <v>14.8</v>
+      </c>
+      <c r="E1194" s="2">
+        <v>72.0</v>
+      </c>
+      <c r="F1194" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1194" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1195" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:00</t>
+        </is>
+      </c>
+      <c r="C1195" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1195" s="2">
+        <v>14.7</v>
+      </c>
+      <c r="E1195" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="F1195" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1195" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1196" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:10</t>
+        </is>
+      </c>
+      <c r="C1196" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1196" s="2">
+        <v>14.7</v>
+      </c>
+      <c r="E1196" s="2">
+        <v>72.0</v>
+      </c>
+      <c r="F1196" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1196" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1197" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:20</t>
+        </is>
+      </c>
+      <c r="C1197" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1197" s="2">
+        <v>14.6</v>
+      </c>
+      <c r="E1197" s="2">
+        <v>74.0</v>
+      </c>
+      <c r="F1197" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1197" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1198">
+      <c r="A1198" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1198" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:30</t>
+        </is>
+      </c>
+      <c r="C1198" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1198" s="2">
+        <v>14.4</v>
+      </c>
+      <c r="E1198" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F1198" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1198" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1199">
+      <c r="A1199" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1199" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:40</t>
+        </is>
+      </c>
+      <c r="C1199" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1199" s="2">
+        <v>14.2</v>
+      </c>
+      <c r="E1199" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F1199" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1199" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1200">
+      <c r="A1200" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1200" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:50</t>
+        </is>
+      </c>
+      <c r="C1200" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1200" s="2">
+        <v>14.2</v>
+      </c>
+      <c r="E1200" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F1200" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1200" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1201">
+      <c r="A1201" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1201" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:00</t>
+        </is>
+      </c>
+      <c r="C1201" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1201" s="2">
+        <v>14.2</v>
+      </c>
+      <c r="E1201" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F1201" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1201" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1202">
+      <c r="A1202" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1202" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:10</t>
+        </is>
+      </c>
+      <c r="C1202" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1202" s="2">
+        <v>14.3</v>
+      </c>
+      <c r="E1202" s="2">
+        <v>74.0</v>
+      </c>
+      <c r="F1202" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1202" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1203" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:20</t>
+        </is>
+      </c>
+      <c r="C1203" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1203" s="2">
+        <v>14.3</v>
+      </c>
+      <c r="E1203" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F1203" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1203" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1204" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:30</t>
+        </is>
+      </c>
+      <c r="C1204" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1204" s="2">
+        <v>14.2</v>
+      </c>
+      <c r="E1204" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F1204" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1204" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1205" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:40</t>
+        </is>
+      </c>
+      <c r="C1205" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1205" s="2">
+        <v>14.1</v>
+      </c>
+      <c r="E1205" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F1205" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1205" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1206" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:50</t>
+        </is>
+      </c>
+      <c r="C1206" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1206" s="2">
+        <v>13.9</v>
+      </c>
+      <c r="E1206" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F1206" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1206" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1207" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:00</t>
+        </is>
+      </c>
+      <c r="C1207" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1207" s="2">
+        <v>14.0</v>
+      </c>
+      <c r="E1207" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F1207" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1207" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1208" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:10</t>
+        </is>
+      </c>
+      <c r="C1208" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1208" s="2">
+        <v>13.9</v>
+      </c>
+      <c r="E1208" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F1208" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1208" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1209" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:20</t>
+        </is>
+      </c>
+      <c r="C1209" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1209" s="2">
+        <v>13.8</v>
+      </c>
+      <c r="E1209" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F1209" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1209" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1210" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:30</t>
+        </is>
+      </c>
+      <c r="C1210" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1210" s="2">
+        <v>13.8</v>
+      </c>
+      <c r="E1210" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F1210" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1210" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1211" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:40</t>
+        </is>
+      </c>
+      <c r="C1211" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1211" s="2">
+        <v>13.8</v>
+      </c>
+      <c r="E1211" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F1211" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1211" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1212" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:50</t>
+        </is>
+      </c>
+      <c r="C1212" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1212" s="2">
+        <v>13.7</v>
+      </c>
+      <c r="E1212" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F1212" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1212" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1213" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:00</t>
+        </is>
+      </c>
+      <c r="C1213" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1213" s="2">
+        <v>13.7</v>
+      </c>
+      <c r="E1213" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F1213" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1213" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1214" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:10</t>
+        </is>
+      </c>
+      <c r="C1214" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1214" s="2">
+        <v>13.6</v>
+      </c>
+      <c r="E1214" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F1214" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1214" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1215" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:20</t>
+        </is>
+      </c>
+      <c r="C1215" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1215" s="2">
+        <v>13.5</v>
+      </c>
+      <c r="E1215" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F1215" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1215" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1216" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:30</t>
+        </is>
+      </c>
+      <c r="C1216" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1216" s="2">
+        <v>13.4</v>
+      </c>
+      <c r="E1216" s="2">
+        <v>81.0</v>
+      </c>
+      <c r="F1216" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1216" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1217" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:40</t>
+        </is>
+      </c>
+      <c r="C1217" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1217" s="2">
+        <v>13.3</v>
+      </c>
+      <c r="E1217" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F1217" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1217" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1218" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:50</t>
+        </is>
+      </c>
+      <c r="C1218" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1218" s="2">
+        <v>13.3</v>
+      </c>
+      <c r="E1218" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F1218" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1218" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1219" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:00</t>
+        </is>
+      </c>
+      <c r="C1219" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1219" s="2">
+        <v>13.2</v>
+      </c>
+      <c r="E1219" s="2">
+        <v>81.0</v>
+      </c>
+      <c r="F1219" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1219" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1220" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:10</t>
+        </is>
+      </c>
+      <c r="C1220" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1220" s="2">
+        <v>13.2</v>
+      </c>
+      <c r="E1220" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F1220" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1220" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1221" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:20</t>
+        </is>
+      </c>
+      <c r="C1221" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1221" s="2">
+        <v>13.3</v>
+      </c>
+      <c r="E1221" s="2">
+        <v>81.0</v>
+      </c>
+      <c r="F1221" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1221" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1222" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:30</t>
+        </is>
+      </c>
+      <c r="C1222" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1222" s="2">
+        <v>13.4</v>
+      </c>
+      <c r="E1222" s="2">
+        <v>81.0</v>
+      </c>
+      <c r="F1222" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1222" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1223" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:40</t>
+        </is>
+      </c>
+      <c r="C1223" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1223" s="2">
+        <v>13.5</v>
+      </c>
+      <c r="E1223" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F1223" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1223" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1224" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:50</t>
+        </is>
+      </c>
+      <c r="C1224" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1224" s="2">
+        <v>13.7</v>
+      </c>
+      <c r="E1224" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F1224" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1224" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1225" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:00</t>
+        </is>
+      </c>
+      <c r="C1225" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1225" s="2">
+        <v>14.0</v>
+      </c>
+      <c r="E1225" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F1225" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1225" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1226" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:10</t>
+        </is>
+      </c>
+      <c r="C1226" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1226" s="2">
+        <v>14.2</v>
+      </c>
+      <c r="E1226" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F1226" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1226" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1227" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:20</t>
+        </is>
+      </c>
+      <c r="C1227" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1227" s="2">
+        <v>14.4</v>
+      </c>
+      <c r="E1227" s="2">
+        <v>74.0</v>
+      </c>
+      <c r="F1227" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1227" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1228" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:30</t>
+        </is>
+      </c>
+      <c r="C1228" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1228" s="2">
+        <v>14.6</v>
+      </c>
+      <c r="E1228" s="2">
+        <v>72.0</v>
+      </c>
+      <c r="F1228" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1228" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1229" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:40</t>
+        </is>
+      </c>
+      <c r="C1229" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1229" s="2">
+        <v>14.8</v>
+      </c>
+      <c r="E1229" s="2">
+        <v>72.0</v>
+      </c>
+      <c r="F1229" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1229" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1230" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:50</t>
+        </is>
+      </c>
+      <c r="C1230" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1230" s="2">
+        <v>15.1</v>
+      </c>
+      <c r="E1230" s="2">
+        <v>72.0</v>
+      </c>
+      <c r="F1230" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1230" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1231" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:00</t>
+        </is>
+      </c>
+      <c r="C1231" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1231" s="2">
+        <v>15.6</v>
+      </c>
+      <c r="E1231" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F1231" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1231" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1232">
+      <c r="A1232" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1232" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:10</t>
+        </is>
+      </c>
+      <c r="C1232" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1232" s="2">
+        <v>16.2</v>
+      </c>
+      <c r="E1232" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F1232" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1232" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1233" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:20</t>
+        </is>
+      </c>
+      <c r="C1233" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1233" s="2">
+        <v>16.7</v>
+      </c>
+      <c r="E1233" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F1233" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1233" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1234">
+      <c r="A1234" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1234" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:30</t>
+        </is>
+      </c>
+      <c r="C1234" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1234" s="2">
+        <v>16.9</v>
+      </c>
+      <c r="E1234" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F1234" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1234" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1235" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:40</t>
+        </is>
+      </c>
+      <c r="C1235" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1235" s="2">
+        <v>17.4</v>
+      </c>
+      <c r="E1235" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F1235" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1235" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1236" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:50</t>
+        </is>
+      </c>
+      <c r="C1236" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1236" s="2">
+        <v>17.9</v>
+      </c>
+      <c r="E1236" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F1236" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1236" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1237">
+      <c r="A1237" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1237" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:00</t>
+        </is>
+      </c>
+      <c r="C1237" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1237" s="2">
+        <v>18.7</v>
+      </c>
+      <c r="E1237" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F1237" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1237" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="A1238" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1238" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:10</t>
+        </is>
+      </c>
+      <c r="C1238" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1238" s="2">
+        <v>18.8</v>
+      </c>
+      <c r="E1238" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F1238" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1238" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="A1239" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1239" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:20</t>
+        </is>
+      </c>
+      <c r="C1239" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1239" s="2">
+        <v>19.4</v>
+      </c>
+      <c r="E1239" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F1239" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1239" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="A1240" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1240" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:30</t>
+        </is>
+      </c>
+      <c r="C1240" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1240" s="2">
+        <v>19.8</v>
+      </c>
+      <c r="E1240" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F1240" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1240" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1241" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:40</t>
+        </is>
+      </c>
+      <c r="C1241" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1241" s="2">
+        <v>20.3</v>
+      </c>
+      <c r="E1241" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F1241" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1241" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="A1242" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1242" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:50</t>
+        </is>
+      </c>
+      <c r="C1242" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1242" s="2">
+        <v>20.5</v>
+      </c>
+      <c r="E1242" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F1242" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1242" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="A1243" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1243" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:00</t>
+        </is>
+      </c>
+      <c r="C1243" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1243" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="E1243" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F1243" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1243" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1244" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:10</t>
+        </is>
+      </c>
+      <c r="C1244" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1244" s="2">
+        <v>21.5</v>
+      </c>
+      <c r="E1244" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F1244" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1244" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1245">
+      <c r="A1245" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1245" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:20</t>
+        </is>
+      </c>
+      <c r="C1245" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1245" s="2">
+        <v>21.8</v>
+      </c>
+      <c r="E1245" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F1245" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1245" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="A1246" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1246" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:30</t>
+        </is>
+      </c>
+      <c r="C1246" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1246" s="2">
+        <v>21.9</v>
+      </c>
+      <c r="E1246" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F1246" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1246" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="A1247" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1247" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:40</t>
+        </is>
+      </c>
+      <c r="C1247" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1247" s="2">
+        <v>22.2</v>
+      </c>
+      <c r="E1247" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F1247" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1247" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1248" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:50</t>
+        </is>
+      </c>
+      <c r="C1248" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1248" s="2">
+        <v>22.6</v>
+      </c>
+      <c r="E1248" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F1248" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1248" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1249" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:00</t>
+        </is>
+      </c>
+      <c r="C1249" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1249" s="2">
+        <v>22.9</v>
+      </c>
+      <c r="E1249" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F1249" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1249" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1250" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:10</t>
+        </is>
+      </c>
+      <c r="C1250" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1250" s="2">
+        <v>23.2</v>
+      </c>
+      <c r="E1250" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F1250" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1250" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1251" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:20</t>
+        </is>
+      </c>
+      <c r="C1251" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1251" s="2">
+        <v>23.3</v>
+      </c>
+      <c r="E1251" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F1251" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1251" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1252">
+      <c r="A1252" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1252" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:30</t>
+        </is>
+      </c>
+      <c r="C1252" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1252" s="2">
+        <v>23.4</v>
+      </c>
+      <c r="E1252" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F1252" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1252" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1253" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:40</t>
+        </is>
+      </c>
+      <c r="C1253" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1253" s="2">
+        <v>23.8</v>
+      </c>
+      <c r="E1253" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F1253" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1253" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1254" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:50</t>
+        </is>
+      </c>
+      <c r="C1254" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1254" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="E1254" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F1254" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1254" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1255" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:00</t>
+        </is>
+      </c>
+      <c r="C1255" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1255" s="2">
+        <v>24.4</v>
+      </c>
+      <c r="E1255" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F1255" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1255" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1256" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:10</t>
+        </is>
+      </c>
+      <c r="C1256" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1256" s="2">
+        <v>24.6</v>
+      </c>
+      <c r="E1256" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F1256" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1256" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1257" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:20</t>
+        </is>
+      </c>
+      <c r="C1257" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1257" s="2">
+        <v>24.3</v>
+      </c>
+      <c r="E1257" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F1257" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1257" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1258">
+      <c r="A1258" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1258" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:30</t>
+        </is>
+      </c>
+      <c r="C1258" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1258" s="2">
+        <v>24.8</v>
+      </c>
+      <c r="E1258" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F1258" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1258" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1259" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:40</t>
+        </is>
+      </c>
+      <c r="C1259" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1259" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="E1259" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F1259" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1259" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1260" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:50</t>
+        </is>
+      </c>
+      <c r="C1260" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1260" s="2">
+        <v>25.2</v>
+      </c>
+      <c r="E1260" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F1260" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1260" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1261" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:00</t>
+        </is>
+      </c>
+      <c r="C1261" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1261" s="2">
+        <v>25.5</v>
+      </c>
+      <c r="E1261" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F1261" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1261" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1262">
+      <c r="A1262" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1262" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:10</t>
+        </is>
+      </c>
+      <c r="C1262" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1262" s="2">
+        <v>25.6</v>
+      </c>
+      <c r="E1262" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F1262" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1262" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1263" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:20</t>
+        </is>
+      </c>
+      <c r="C1263" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1263" s="2">
+        <v>26.1</v>
+      </c>
+      <c r="E1263" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F1263" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1263" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1264">
+      <c r="A1264" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1264" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:30</t>
+        </is>
+      </c>
+      <c r="C1264" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1264" s="2">
+        <v>26.3</v>
+      </c>
+      <c r="E1264" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F1264" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1264" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1265">
+      <c r="A1265" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1265" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:40</t>
+        </is>
+      </c>
+      <c r="C1265" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1265" s="2">
+        <v>27.2</v>
+      </c>
+      <c r="E1265" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F1265" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1265" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1266">
+      <c r="A1266" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1266" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:50</t>
+        </is>
+      </c>
+      <c r="C1266" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1266" s="2">
+        <v>27.5</v>
+      </c>
+      <c r="E1266" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F1266" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1266" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1267">
+      <c r="A1267" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1267" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:00</t>
+        </is>
+      </c>
+      <c r="C1267" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1267" s="2">
+        <v>27.2</v>
+      </c>
+      <c r="E1267" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F1267" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1267" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1268">
+      <c r="A1268" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1268" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:10</t>
+        </is>
+      </c>
+      <c r="C1268" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1268" s="2">
+        <v>27.2</v>
+      </c>
+      <c r="E1268" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F1268" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1268" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1269">
+      <c r="A1269" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1269" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:20</t>
+        </is>
+      </c>
+      <c r="C1269" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1269" s="2">
+        <v>26.8</v>
+      </c>
+      <c r="E1269" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F1269" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1269" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1270">
+      <c r="A1270" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1270" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:30</t>
+        </is>
+      </c>
+      <c r="C1270" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1270" s="2">
+        <v>26.5</v>
+      </c>
+      <c r="E1270" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F1270" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1270" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1271" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:40</t>
+        </is>
+      </c>
+      <c r="C1271" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1271" s="2">
+        <v>25.3</v>
+      </c>
+      <c r="E1271" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F1271" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1271" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1272" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:50</t>
+        </is>
+      </c>
+      <c r="C1272" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1272" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="E1272" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F1272" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1272" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1273" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:00</t>
+        </is>
+      </c>
+      <c r="C1273" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1273" s="2">
+        <v>25.1</v>
+      </c>
+      <c r="E1273" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F1273" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1273" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1274" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:10</t>
+        </is>
+      </c>
+      <c r="C1274" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1274" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="E1274" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F1274" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1274" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1275" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:20</t>
+        </is>
+      </c>
+      <c r="C1275" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1275" s="2">
+        <v>23.7</v>
+      </c>
+      <c r="E1275" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F1275" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1275" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1276" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:30</t>
+        </is>
+      </c>
+      <c r="C1276" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1276" s="2">
+        <v>23.7</v>
+      </c>
+      <c r="E1276" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F1276" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1276" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1277" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:40</t>
+        </is>
+      </c>
+      <c r="C1277" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1277" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="E1277" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F1277" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1277" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1278" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:50</t>
+        </is>
+      </c>
+      <c r="C1278" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1278" s="2">
+        <v>24.2</v>
+      </c>
+      <c r="E1278" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F1278" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1278" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1279" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:00</t>
+        </is>
+      </c>
+      <c r="C1279" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1279" s="2">
+        <v>24.7</v>
+      </c>
+      <c r="E1279" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F1279" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1279" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1280">
+      <c r="A1280" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1280" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:10</t>
+        </is>
+      </c>
+      <c r="C1280" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1280" s="2">
+        <v>24.7</v>
+      </c>
+      <c r="E1280" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F1280" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1280" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1281" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:20</t>
+        </is>
+      </c>
+      <c r="C1281" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1281" s="2">
+        <v>24.7</v>
+      </c>
+      <c r="E1281" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F1281" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1281" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1282" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:30</t>
+        </is>
+      </c>
+      <c r="C1282" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1282" s="2">
+        <v>24.7</v>
+      </c>
+      <c r="E1282" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F1282" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1282" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1283" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:40</t>
+        </is>
+      </c>
+      <c r="C1283" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1283" s="2">
+        <v>24.4</v>
+      </c>
+      <c r="E1283" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F1283" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1283" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1284" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:50</t>
+        </is>
+      </c>
+      <c r="C1284" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1284" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="E1284" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F1284" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1284" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1285" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:00</t>
+        </is>
+      </c>
+      <c r="C1285" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1285" s="2">
+        <v>23.4</v>
+      </c>
+      <c r="E1285" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F1285" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1285" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1286" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:10</t>
+        </is>
+      </c>
+      <c r="C1286" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1286" s="2">
+        <v>23.1</v>
+      </c>
+      <c r="E1286" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F1286" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1286" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1287" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:20</t>
+        </is>
+      </c>
+      <c r="C1287" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1287" s="2">
+        <v>22.7</v>
+      </c>
+      <c r="E1287" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F1287" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1287" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1288" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:30</t>
+        </is>
+      </c>
+      <c r="C1288" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1288" s="2">
+        <v>22.2</v>
+      </c>
+      <c r="E1288" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F1288" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1288" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1289" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:40</t>
+        </is>
+      </c>
+      <c r="C1289" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1289" s="2">
+        <v>22.4</v>
+      </c>
+      <c r="E1289" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F1289" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1289" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1290" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:50</t>
+        </is>
+      </c>
+      <c r="C1290" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1290" s="2">
+        <v>22.5</v>
+      </c>
+      <c r="E1290" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F1290" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1290" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1291" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:00</t>
+        </is>
+      </c>
+      <c r="C1291" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1291" s="2">
+        <v>22.2</v>
+      </c>
+      <c r="E1291" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F1291" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1291" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1292" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:10</t>
+        </is>
+      </c>
+      <c r="C1292" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1292" s="2">
+        <v>21.8</v>
+      </c>
+      <c r="E1292" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F1292" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1292" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1293" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:20</t>
+        </is>
+      </c>
+      <c r="C1293" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1293" s="2">
+        <v>21.2</v>
+      </c>
+      <c r="E1293" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F1293" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1293" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1294" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:30</t>
+        </is>
+      </c>
+      <c r="C1294" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1294" s="2">
+        <v>20.9</v>
+      </c>
+      <c r="E1294" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F1294" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1294" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1295" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:40</t>
+        </is>
+      </c>
+      <c r="C1295" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1295" s="2">
+        <v>20.7</v>
+      </c>
+      <c r="E1295" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F1295" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1295" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1296" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:50</t>
+        </is>
+      </c>
+      <c r="C1296" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1296" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="E1296" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F1296" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1296" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1297" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:00</t>
+        </is>
+      </c>
+      <c r="C1297" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1297" s="2">
+        <v>19.4</v>
+      </c>
+      <c r="E1297" s="2">
+        <v>74.0</v>
+      </c>
+      <c r="F1297" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="G1297" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1298" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:10</t>
+        </is>
+      </c>
+      <c r="C1298" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1298" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="E1298" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F1298" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1298" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1299" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:20</t>
+        </is>
+      </c>
+      <c r="C1299" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1299" s="2">
+        <v>18.6</v>
+      </c>
+      <c r="E1299" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F1299" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1299" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1300" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:30</t>
+        </is>
+      </c>
+      <c r="C1300" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1300" s="2">
+        <v>18.5</v>
+      </c>
+      <c r="E1300" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F1300" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1300" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1301" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:40</t>
+        </is>
+      </c>
+      <c r="C1301" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1301" s="2">
+        <v>18.4</v>
+      </c>
+      <c r="E1301" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F1301" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1301" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1302" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:50</t>
+        </is>
+      </c>
+      <c r="C1302" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1302" s="2">
+        <v>18.2</v>
+      </c>
+      <c r="E1302" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F1302" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1302" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1303" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:00</t>
+        </is>
+      </c>
+      <c r="C1303" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1303" s="2">
+        <v>18.2</v>
+      </c>
+      <c r="E1303" s="2">
+        <v>84.0</v>
+      </c>
+      <c r="F1303" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1303" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1304" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:10</t>
+        </is>
+      </c>
+      <c r="C1304" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1304" s="2">
+        <v>17.7</v>
+      </c>
+      <c r="E1304" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F1304" s="2">
+        <v>1.2</v>
+      </c>
+      <c r="G1304" s="2">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1305" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:20</t>
+        </is>
+      </c>
+      <c r="C1305" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1305" s="2">
+        <v>17.6</v>
+      </c>
+      <c r="E1305" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F1305" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1305" s="2">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="1306">
+      <c r="A1306" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1306" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:30</t>
+        </is>
+      </c>
+      <c r="C1306" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1306" s="2">
+        <v>17.4</v>
+      </c>
+      <c r="E1306" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F1306" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1306" s="2">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="1307">
+      <c r="A1307" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1307" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:40</t>
+        </is>
+      </c>
+      <c r="C1307" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1307" s="2">
+        <v>17.3</v>
+      </c>
+      <c r="E1307" s="2">
+        <v>90.0</v>
+      </c>
+      <c r="F1307" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1307" s="2">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="1308">
+      <c r="A1308" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1308" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:50</t>
+        </is>
+      </c>
+      <c r="C1308" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1308" s="2">
+        <v>17.2</v>
+      </c>
+      <c r="E1308" s="2">
+        <v>89.0</v>
+      </c>
+      <c r="F1308" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1308" s="2">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="1309">
+      <c r="A1309" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1309" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:00</t>
+        </is>
+      </c>
+      <c r="C1309" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1309" s="2">
+        <v>17.1</v>
+      </c>
+      <c r="E1309" s="2">
+        <v>90.0</v>
+      </c>
+      <c r="F1309" s="2">
+        <v>0.4</v>
+      </c>
+      <c r="G1309" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1310">
+      <c r="A1310" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1310" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:10</t>
+        </is>
+      </c>
+      <c r="C1310" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1310" s="2">
+        <v>16.8</v>
+      </c>
+      <c r="E1310" s="2">
+        <v>92.0</v>
+      </c>
+      <c r="F1310" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1310" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1311">
+      <c r="A1311" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1311" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:20</t>
+        </is>
+      </c>
+      <c r="C1311" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1311" s="2">
+        <v>16.6</v>
+      </c>
+      <c r="E1311" s="2">
+        <v>93.0</v>
+      </c>
+      <c r="F1311" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1311" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1312" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:30</t>
+        </is>
+      </c>
+      <c r="C1312" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1312" s="2">
+        <v>16.4</v>
+      </c>
+      <c r="E1312" s="2">
+        <v>93.0</v>
+      </c>
+      <c r="F1312" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1312" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1313" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:40</t>
+        </is>
+      </c>
+      <c r="C1313" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1313" s="2">
+        <v>16.3</v>
+      </c>
+      <c r="E1313" s="2">
+        <v>93.0</v>
+      </c>
+      <c r="F1313" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1313" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1314" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:50</t>
+        </is>
+      </c>
+      <c r="C1314" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1314" s="2">
+        <v>16.1</v>
+      </c>
+      <c r="E1314" s="2">
+        <v>93.0</v>
+      </c>
+      <c r="F1314" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1314" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1315">
+      <c r="A1315" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1315" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:00</t>
+        </is>
+      </c>
+      <c r="C1315" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1315" s="2">
+        <v>16.0</v>
+      </c>
+      <c r="E1315" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F1315" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1315" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1316">
+      <c r="A1316" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1316" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:10</t>
+        </is>
+      </c>
+      <c r="C1316" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1316" s="2">
+        <v>15.9</v>
+      </c>
+      <c r="E1316" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F1316" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1316" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1317">
+      <c r="A1317" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1317" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:20</t>
+        </is>
+      </c>
+      <c r="C1317" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1317" s="2">
+        <v>15.8</v>
+      </c>
+      <c r="E1317" s="2">
+        <v>95.0</v>
+      </c>
+      <c r="F1317" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1317" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1318">
+      <c r="A1318" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1318" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:30</t>
+        </is>
+      </c>
+      <c r="C1318" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1318" s="2">
+        <v>15.6</v>
+      </c>
+      <c r="E1318" s="2">
+        <v>94.0</v>
+      </c>
+      <c r="F1318" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1318" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1319">
+      <c r="A1319" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1319" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:40</t>
+        </is>
+      </c>
+      <c r="C1319" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1319" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="E1319" s="2">
+        <v>95.0</v>
+      </c>
+      <c r="F1319" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1319" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1320">
+      <c r="A1320" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1320" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:50</t>
+        </is>
+      </c>
+      <c r="C1320" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1320" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="E1320" s="2">
+        <v>95.0</v>
+      </c>
+      <c r="F1320" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1320" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1321">
+      <c r="A1321" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1321" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:00</t>
+        </is>
+      </c>
+      <c r="C1321" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1321" s="2">
+        <v>15.4</v>
+      </c>
+      <c r="E1321" s="2">
+        <v>95.0</v>
+      </c>
+      <c r="F1321" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1321" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1322">
+      <c r="A1322" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1322" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:10</t>
+        </is>
+      </c>
+      <c r="C1322" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1322" s="2">
+        <v>15.3</v>
+      </c>
+      <c r="E1322" s="2">
+        <v>95.0</v>
+      </c>
+      <c r="F1322" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1322" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="A1323" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1323" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:20</t>
+        </is>
+      </c>
+      <c r="C1323" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1323" s="2">
+        <v>15.2</v>
+      </c>
+      <c r="E1323" s="2">
+        <v>95.0</v>
+      </c>
+      <c r="F1323" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1323" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1324" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:30</t>
+        </is>
+      </c>
+      <c r="C1324" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1324" s="2">
+        <v>15.0</v>
+      </c>
+      <c r="E1324" s="2">
+        <v>96.0</v>
+      </c>
+      <c r="F1324" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1324" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1325">
+      <c r="A1325" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1325" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:40</t>
+        </is>
+      </c>
+      <c r="C1325" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1325" s="2">
+        <v>15.0</v>
+      </c>
+      <c r="E1325" s="2">
+        <v>96.0</v>
+      </c>
+      <c r="F1325" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1325" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1326">
+      <c r="A1326" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23.07.2026</t>
+        </is>
+      </c>
+      <c r="B1326" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:50</t>
+        </is>
+      </c>
+      <c r="C1326" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1326" s="2">
+        <v>14.9</v>
+      </c>
+      <c r="E1326" s="2">
+        <v>95.0</v>
+      </c>
+      <c r="F1326" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1326" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1327" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:00</t>
+        </is>
+      </c>
+      <c r="C1327" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1327" s="2">
+        <v>14.8</v>
+      </c>
+      <c r="E1327" s="2">
+        <v>96.0</v>
+      </c>
+      <c r="F1327" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1327" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1328">
+      <c r="A1328" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1328" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:10</t>
+        </is>
+      </c>
+      <c r="C1328" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1328" s="2">
+        <v>14.7</v>
+      </c>
+      <c r="E1328" s="2">
+        <v>95.0</v>
+      </c>
+      <c r="F1328" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1328" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1329">
+      <c r="A1329" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1329" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:20</t>
+        </is>
+      </c>
+      <c r="C1329" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1329" s="2">
+        <v>14.6</v>
+      </c>
+      <c r="E1329" s="2">
+        <v>96.0</v>
+      </c>
+      <c r="F1329" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1329" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G1186"/>
+  <autoFilter ref="A1:G1329"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ARSO Kranj zajem 2026-07-25 00:46 Europe/Ljubljana
</commit_message>
<xml_diff>
--- a/tabela_vremena/ARSO_Kranj.xlsx
+++ b/tabela_vremena/ARSO_Kranj.xlsx
@@ -38623,7 +38623,4212 @@
         <v>1.6</v>
       </c>
     </row>
+    <row r="1330">
+      <c r="A1330" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1330" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:30</t>
+        </is>
+      </c>
+      <c r="C1330" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1330" s="2">
+        <v>14.4</v>
+      </c>
+      <c r="E1330" s="2">
+        <v>95.0</v>
+      </c>
+      <c r="F1330" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1330" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1331">
+      <c r="A1331" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1331" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:40</t>
+        </is>
+      </c>
+      <c r="C1331" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1331" s="2">
+        <v>14.4</v>
+      </c>
+      <c r="E1331" s="2">
+        <v>96.0</v>
+      </c>
+      <c r="F1331" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1331" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1332">
+      <c r="A1332" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1332" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:50</t>
+        </is>
+      </c>
+      <c r="C1332" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1332" s="2">
+        <v>14.4</v>
+      </c>
+      <c r="E1332" s="2">
+        <v>96.0</v>
+      </c>
+      <c r="F1332" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1332" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="A1333" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1333" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:00</t>
+        </is>
+      </c>
+      <c r="C1333" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1333" s="2">
+        <v>14.4</v>
+      </c>
+      <c r="E1333" s="2">
+        <v>96.0</v>
+      </c>
+      <c r="F1333" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1333" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="A1334" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1334" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:10</t>
+        </is>
+      </c>
+      <c r="C1334" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1334" s="2">
+        <v>14.4</v>
+      </c>
+      <c r="E1334" s="2">
+        <v>96.0</v>
+      </c>
+      <c r="F1334" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1334" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1335">
+      <c r="A1335" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1335" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:20</t>
+        </is>
+      </c>
+      <c r="C1335" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1335" s="2">
+        <v>14.5</v>
+      </c>
+      <c r="E1335" s="2">
+        <v>96.0</v>
+      </c>
+      <c r="F1335" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1335" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="A1336" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1336" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:30</t>
+        </is>
+      </c>
+      <c r="C1336" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1336" s="2">
+        <v>14.4</v>
+      </c>
+      <c r="E1336" s="2">
+        <v>96.0</v>
+      </c>
+      <c r="F1336" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1336" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="A1337" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1337" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:40</t>
+        </is>
+      </c>
+      <c r="C1337" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1337" s="2">
+        <v>14.3</v>
+      </c>
+      <c r="E1337" s="2">
+        <v>96.0</v>
+      </c>
+      <c r="F1337" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1337" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1338">
+      <c r="A1338" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1338" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:50</t>
+        </is>
+      </c>
+      <c r="C1338" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1338" s="2">
+        <v>14.2</v>
+      </c>
+      <c r="E1338" s="2">
+        <v>95.0</v>
+      </c>
+      <c r="F1338" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1338" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="A1339" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1339" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:00</t>
+        </is>
+      </c>
+      <c r="C1339" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1339" s="2">
+        <v>14.0</v>
+      </c>
+      <c r="E1339" s="2">
+        <v>95.0</v>
+      </c>
+      <c r="F1339" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1339" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="A1340" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1340" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:10</t>
+        </is>
+      </c>
+      <c r="C1340" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1340" s="2">
+        <v>13.9</v>
+      </c>
+      <c r="E1340" s="2">
+        <v>95.0</v>
+      </c>
+      <c r="F1340" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1340" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="A1341" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1341" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:20</t>
+        </is>
+      </c>
+      <c r="C1341" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1341" s="2">
+        <v>13.9</v>
+      </c>
+      <c r="E1341" s="2">
+        <v>96.0</v>
+      </c>
+      <c r="F1341" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1341" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="A1342" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1342" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:30</t>
+        </is>
+      </c>
+      <c r="C1342" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1342" s="2">
+        <v>13.9</v>
+      </c>
+      <c r="E1342" s="2">
+        <v>96.0</v>
+      </c>
+      <c r="F1342" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1342" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1343" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:40</t>
+        </is>
+      </c>
+      <c r="C1343" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1343" s="2">
+        <v>13.8</v>
+      </c>
+      <c r="E1343" s="2">
+        <v>96.0</v>
+      </c>
+      <c r="F1343" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1343" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1344" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:50</t>
+        </is>
+      </c>
+      <c r="C1344" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1344" s="2">
+        <v>13.8</v>
+      </c>
+      <c r="E1344" s="2">
+        <v>96.0</v>
+      </c>
+      <c r="F1344" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1344" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1345" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:00</t>
+        </is>
+      </c>
+      <c r="C1345" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1345" s="2">
+        <v>13.8</v>
+      </c>
+      <c r="E1345" s="2">
+        <v>96.0</v>
+      </c>
+      <c r="F1345" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1345" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="A1346" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1346" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:10</t>
+        </is>
+      </c>
+      <c r="C1346" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1346" s="2">
+        <v>13.8</v>
+      </c>
+      <c r="E1346" s="2">
+        <v>96.0</v>
+      </c>
+      <c r="F1346" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1346" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1347">
+      <c r="A1347" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1347" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:20</t>
+        </is>
+      </c>
+      <c r="C1347" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1347" s="2">
+        <v>13.8</v>
+      </c>
+      <c r="E1347" s="2">
+        <v>96.0</v>
+      </c>
+      <c r="F1347" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1347" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1348">
+      <c r="A1348" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1348" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:30</t>
+        </is>
+      </c>
+      <c r="C1348" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1348" s="2">
+        <v>13.7</v>
+      </c>
+      <c r="E1348" s="2">
+        <v>96.0</v>
+      </c>
+      <c r="F1348" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1348" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1349">
+      <c r="A1349" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1349" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:40</t>
+        </is>
+      </c>
+      <c r="C1349" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1349" s="2">
+        <v>13.8</v>
+      </c>
+      <c r="E1349" s="2">
+        <v>97.0</v>
+      </c>
+      <c r="F1349" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1349" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1350">
+      <c r="A1350" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1350" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:50</t>
+        </is>
+      </c>
+      <c r="C1350" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1350" s="2">
+        <v>13.7</v>
+      </c>
+      <c r="E1350" s="2">
+        <v>97.0</v>
+      </c>
+      <c r="F1350" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1350" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1351">
+      <c r="A1351" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1351" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:00</t>
+        </is>
+      </c>
+      <c r="C1351" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1351" s="2">
+        <v>13.7</v>
+      </c>
+      <c r="E1351" s="2">
+        <v>97.0</v>
+      </c>
+      <c r="F1351" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1351" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="A1352" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1352" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:10</t>
+        </is>
+      </c>
+      <c r="C1352" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1352" s="2">
+        <v>13.6</v>
+      </c>
+      <c r="E1352" s="2">
+        <v>97.0</v>
+      </c>
+      <c r="F1352" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1352" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1353">
+      <c r="A1353" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1353" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:20</t>
+        </is>
+      </c>
+      <c r="C1353" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1353" s="2">
+        <v>13.6</v>
+      </c>
+      <c r="E1353" s="2">
+        <v>98.0</v>
+      </c>
+      <c r="F1353" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1353" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1354">
+      <c r="A1354" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1354" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:30</t>
+        </is>
+      </c>
+      <c r="C1354" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1354" s="2">
+        <v>13.5</v>
+      </c>
+      <c r="E1354" s="2">
+        <v>98.0</v>
+      </c>
+      <c r="F1354" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1354" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1355">
+      <c r="A1355" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1355" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:40</t>
+        </is>
+      </c>
+      <c r="C1355" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1355" s="2">
+        <v>13.5</v>
+      </c>
+      <c r="E1355" s="2">
+        <v>98.0</v>
+      </c>
+      <c r="F1355" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1355" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1356">
+      <c r="A1356" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1356" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:50</t>
+        </is>
+      </c>
+      <c r="C1356" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1356" s="2">
+        <v>13.4</v>
+      </c>
+      <c r="E1356" s="2">
+        <v>98.0</v>
+      </c>
+      <c r="F1356" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1356" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1357">
+      <c r="A1357" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1357" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:00</t>
+        </is>
+      </c>
+      <c r="C1357" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1357" s="2">
+        <v>13.3</v>
+      </c>
+      <c r="E1357" s="2">
+        <v>97.0</v>
+      </c>
+      <c r="F1357" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1357" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1358">
+      <c r="A1358" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1358" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:10</t>
+        </is>
+      </c>
+      <c r="C1358" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1358" s="2">
+        <v>13.3</v>
+      </c>
+      <c r="E1358" s="2">
+        <v>98.0</v>
+      </c>
+      <c r="F1358" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1358" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1359">
+      <c r="A1359" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1359" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:20</t>
+        </is>
+      </c>
+      <c r="C1359" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1359" s="2">
+        <v>13.3</v>
+      </c>
+      <c r="E1359" s="2">
+        <v>98.0</v>
+      </c>
+      <c r="F1359" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1359" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1360">
+      <c r="A1360" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1360" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:30</t>
+        </is>
+      </c>
+      <c r="C1360" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1360" s="2">
+        <v>13.3</v>
+      </c>
+      <c r="E1360" s="2">
+        <v>98.0</v>
+      </c>
+      <c r="F1360" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1360" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1361">
+      <c r="A1361" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1361" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:40</t>
+        </is>
+      </c>
+      <c r="C1361" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1361" s="2">
+        <v>13.3</v>
+      </c>
+      <c r="E1361" s="2">
+        <v>98.0</v>
+      </c>
+      <c r="F1361" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1361" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1362">
+      <c r="A1362" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1362" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:50</t>
+        </is>
+      </c>
+      <c r="C1362" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1362" s="2">
+        <v>13.3</v>
+      </c>
+      <c r="E1362" s="2">
+        <v>98.0</v>
+      </c>
+      <c r="F1362" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1362" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1363">
+      <c r="A1363" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1363" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:00</t>
+        </is>
+      </c>
+      <c r="C1363" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1363" s="2">
+        <v>13.4</v>
+      </c>
+      <c r="E1363" s="2">
+        <v>98.0</v>
+      </c>
+      <c r="F1363" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1363" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1364">
+      <c r="A1364" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1364" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:10</t>
+        </is>
+      </c>
+      <c r="C1364" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1364" s="2">
+        <v>13.4</v>
+      </c>
+      <c r="E1364" s="2">
+        <v>98.0</v>
+      </c>
+      <c r="F1364" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1364" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1365">
+      <c r="A1365" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1365" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:20</t>
+        </is>
+      </c>
+      <c r="C1365" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1365" s="2">
+        <v>13.4</v>
+      </c>
+      <c r="E1365" s="2">
+        <v>98.0</v>
+      </c>
+      <c r="F1365" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1365" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1366">
+      <c r="A1366" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1366" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:30</t>
+        </is>
+      </c>
+      <c r="C1366" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1366" s="2">
+        <v>13.3</v>
+      </c>
+      <c r="E1366" s="2">
+        <v>98.0</v>
+      </c>
+      <c r="F1366" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1366" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1367">
+      <c r="A1367" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1367" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:40</t>
+        </is>
+      </c>
+      <c r="C1367" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1367" s="2">
+        <v>13.1</v>
+      </c>
+      <c r="E1367" s="2">
+        <v>98.0</v>
+      </c>
+      <c r="F1367" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1367" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1368">
+      <c r="A1368" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1368" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:50</t>
+        </is>
+      </c>
+      <c r="C1368" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1368" s="2">
+        <v>13.1</v>
+      </c>
+      <c r="E1368" s="2">
+        <v>97.0</v>
+      </c>
+      <c r="F1368" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1368" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1369">
+      <c r="A1369" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1369" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:00</t>
+        </is>
+      </c>
+      <c r="C1369" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1369" s="2">
+        <v>13.3</v>
+      </c>
+      <c r="E1369" s="2">
+        <v>98.0</v>
+      </c>
+      <c r="F1369" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1369" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1370">
+      <c r="A1370" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1370" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:10</t>
+        </is>
+      </c>
+      <c r="C1370" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1370" s="2">
+        <v>13.4</v>
+      </c>
+      <c r="E1370" s="2">
+        <v>97.0</v>
+      </c>
+      <c r="F1370" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1370" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1371">
+      <c r="A1371" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1371" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:20</t>
+        </is>
+      </c>
+      <c r="C1371" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1371" s="2">
+        <v>13.7</v>
+      </c>
+      <c r="E1371" s="2">
+        <v>95.0</v>
+      </c>
+      <c r="F1371" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1371" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1372">
+      <c r="A1372" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1372" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:30</t>
+        </is>
+      </c>
+      <c r="C1372" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1372" s="2">
+        <v>13.9</v>
+      </c>
+      <c r="E1372" s="2">
+        <v>93.0</v>
+      </c>
+      <c r="F1372" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1372" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1373">
+      <c r="A1373" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1373" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:40</t>
+        </is>
+      </c>
+      <c r="C1373" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1373" s="2">
+        <v>14.1</v>
+      </c>
+      <c r="E1373" s="2">
+        <v>91.0</v>
+      </c>
+      <c r="F1373" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1373" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1374">
+      <c r="A1374" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1374" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:50</t>
+        </is>
+      </c>
+      <c r="C1374" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1374" s="2">
+        <v>14.5</v>
+      </c>
+      <c r="E1374" s="2">
+        <v>92.0</v>
+      </c>
+      <c r="F1374" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1374" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1375">
+      <c r="A1375" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1375" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:00</t>
+        </is>
+      </c>
+      <c r="C1375" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1375" s="2">
+        <v>15.0</v>
+      </c>
+      <c r="E1375" s="2">
+        <v>90.0</v>
+      </c>
+      <c r="F1375" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1375" s="2">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="1376">
+      <c r="A1376" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1376" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:10</t>
+        </is>
+      </c>
+      <c r="C1376" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1376" s="2">
+        <v>16.1</v>
+      </c>
+      <c r="E1376" s="2">
+        <v>84.0</v>
+      </c>
+      <c r="F1376" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1376" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1377">
+      <c r="A1377" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1377" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:20</t>
+        </is>
+      </c>
+      <c r="C1377" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1377" s="2">
+        <v>16.2</v>
+      </c>
+      <c r="E1377" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F1377" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1377" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1378">
+      <c r="A1378" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1378" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:30</t>
+        </is>
+      </c>
+      <c r="C1378" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1378" s="2">
+        <v>16.8</v>
+      </c>
+      <c r="E1378" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F1378" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1378" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1379">
+      <c r="A1379" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1379" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:40</t>
+        </is>
+      </c>
+      <c r="C1379" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1379" s="2">
+        <v>17.4</v>
+      </c>
+      <c r="E1379" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F1379" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1379" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1380">
+      <c r="A1380" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1380" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:50</t>
+        </is>
+      </c>
+      <c r="C1380" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1380" s="2">
+        <v>17.5</v>
+      </c>
+      <c r="E1380" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F1380" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1380" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1381">
+      <c r="A1381" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1381" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:00</t>
+        </is>
+      </c>
+      <c r="C1381" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1381" s="2">
+        <v>17.9</v>
+      </c>
+      <c r="E1381" s="2">
+        <v>74.0</v>
+      </c>
+      <c r="F1381" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1381" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1382">
+      <c r="A1382" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1382" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:10</t>
+        </is>
+      </c>
+      <c r="C1382" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1382" s="2">
+        <v>17.8</v>
+      </c>
+      <c r="E1382" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="F1382" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1382" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1383">
+      <c r="A1383" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1383" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:20</t>
+        </is>
+      </c>
+      <c r="C1383" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1383" s="2">
+        <v>18.3</v>
+      </c>
+      <c r="E1383" s="2">
+        <v>69.0</v>
+      </c>
+      <c r="F1383" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1383" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1384">
+      <c r="A1384" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1384" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:30</t>
+        </is>
+      </c>
+      <c r="C1384" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1384" s="2">
+        <v>19.2</v>
+      </c>
+      <c r="E1384" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F1384" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1384" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1385">
+      <c r="A1385" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1385" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:40</t>
+        </is>
+      </c>
+      <c r="C1385" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1385" s="2">
+        <v>19.4</v>
+      </c>
+      <c r="E1385" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F1385" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1385" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1386">
+      <c r="A1386" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1386" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:50</t>
+        </is>
+      </c>
+      <c r="C1386" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1386" s="2">
+        <v>18.8</v>
+      </c>
+      <c r="E1386" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F1386" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1386" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1387">
+      <c r="A1387" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1387" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:00</t>
+        </is>
+      </c>
+      <c r="C1387" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1387" s="2">
+        <v>18.9</v>
+      </c>
+      <c r="E1387" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F1387" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1387" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1388">
+      <c r="A1388" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1388" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:10</t>
+        </is>
+      </c>
+      <c r="C1388" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1388" s="2">
+        <v>19.5</v>
+      </c>
+      <c r="E1388" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F1388" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1388" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1389">
+      <c r="A1389" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1389" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:20</t>
+        </is>
+      </c>
+      <c r="C1389" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1389" s="2">
+        <v>19.8</v>
+      </c>
+      <c r="E1389" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F1389" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1389" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1390">
+      <c r="A1390" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1390" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:30</t>
+        </is>
+      </c>
+      <c r="C1390" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1390" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="E1390" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F1390" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1390" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1391">
+      <c r="A1391" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1391" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:40</t>
+        </is>
+      </c>
+      <c r="C1391" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1391" s="2">
+        <v>20.5</v>
+      </c>
+      <c r="E1391" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F1391" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1391" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1392">
+      <c r="A1392" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1392" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:50</t>
+        </is>
+      </c>
+      <c r="C1392" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1392" s="2">
+        <v>20.4</v>
+      </c>
+      <c r="E1392" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F1392" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1392" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1393">
+      <c r="A1393" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1393" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:00</t>
+        </is>
+      </c>
+      <c r="C1393" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1393" s="2">
+        <v>20.6</v>
+      </c>
+      <c r="E1393" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F1393" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1393" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1394">
+      <c r="A1394" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1394" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:10</t>
+        </is>
+      </c>
+      <c r="C1394" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1394" s="2">
+        <v>20.9</v>
+      </c>
+      <c r="E1394" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F1394" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1394" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1395">
+      <c r="A1395" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1395" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:20</t>
+        </is>
+      </c>
+      <c r="C1395" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1395" s="2">
+        <v>21.2</v>
+      </c>
+      <c r="E1395" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F1395" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1395" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1396">
+      <c r="A1396" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1396" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:30</t>
+        </is>
+      </c>
+      <c r="C1396" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1396" s="2">
+        <v>21.7</v>
+      </c>
+      <c r="E1396" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F1396" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1396" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1397">
+      <c r="A1397" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1397" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:40</t>
+        </is>
+      </c>
+      <c r="C1397" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1397" s="2">
+        <v>21.9</v>
+      </c>
+      <c r="E1397" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F1397" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1397" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1398">
+      <c r="A1398" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1398" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:50</t>
+        </is>
+      </c>
+      <c r="C1398" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1398" s="2">
+        <v>21.5</v>
+      </c>
+      <c r="E1398" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F1398" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1398" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1399">
+      <c r="A1399" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1399" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:00</t>
+        </is>
+      </c>
+      <c r="C1399" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1399" s="2">
+        <v>21.8</v>
+      </c>
+      <c r="E1399" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F1399" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1399" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1400">
+      <c r="A1400" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1400" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:10</t>
+        </is>
+      </c>
+      <c r="C1400" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1400" s="2">
+        <v>22.2</v>
+      </c>
+      <c r="E1400" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F1400" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1400" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1401">
+      <c r="A1401" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1401" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:20</t>
+        </is>
+      </c>
+      <c r="C1401" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1401" s="2">
+        <v>22.8</v>
+      </c>
+      <c r="E1401" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F1401" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1401" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1402">
+      <c r="A1402" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1402" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:30</t>
+        </is>
+      </c>
+      <c r="C1402" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1402" s="2">
+        <v>22.6</v>
+      </c>
+      <c r="E1402" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F1402" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1402" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1403">
+      <c r="A1403" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1403" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:40</t>
+        </is>
+      </c>
+      <c r="C1403" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1403" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="E1403" s="2">
+        <v>38.0</v>
+      </c>
+      <c r="F1403" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1403" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1404">
+      <c r="A1404" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1404" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:50</t>
+        </is>
+      </c>
+      <c r="C1404" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1404" s="2">
+        <v>23.5</v>
+      </c>
+      <c r="E1404" s="2">
+        <v>37.0</v>
+      </c>
+      <c r="F1404" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1404" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1405">
+      <c r="A1405" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1405" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:00</t>
+        </is>
+      </c>
+      <c r="C1405" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1405" s="2">
+        <v>23.7</v>
+      </c>
+      <c r="E1405" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F1405" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1405" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1406">
+      <c r="A1406" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1406" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:10</t>
+        </is>
+      </c>
+      <c r="C1406" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1406" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="E1406" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F1406" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1406" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1407">
+      <c r="A1407" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1407" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:20</t>
+        </is>
+      </c>
+      <c r="C1407" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1407" s="2">
+        <v>24.1</v>
+      </c>
+      <c r="E1407" s="2">
+        <v>37.0</v>
+      </c>
+      <c r="F1407" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1407" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1408">
+      <c r="A1408" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1408" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:30</t>
+        </is>
+      </c>
+      <c r="C1408" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1408" s="2">
+        <v>23.5</v>
+      </c>
+      <c r="E1408" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F1408" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1408" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1409">
+      <c r="A1409" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1409" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:40</t>
+        </is>
+      </c>
+      <c r="C1409" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1409" s="2">
+        <v>24.7</v>
+      </c>
+      <c r="E1409" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F1409" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1409" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1410">
+      <c r="A1410" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1410" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:50</t>
+        </is>
+      </c>
+      <c r="C1410" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1410" s="2">
+        <v>24.6</v>
+      </c>
+      <c r="E1410" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F1410" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1410" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1411">
+      <c r="A1411" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1411" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:00</t>
+        </is>
+      </c>
+      <c r="C1411" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1411" s="2">
+        <v>24.5</v>
+      </c>
+      <c r="E1411" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F1411" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1411" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1412">
+      <c r="A1412" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1412" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:10</t>
+        </is>
+      </c>
+      <c r="C1412" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1412" s="2">
+        <v>24.8</v>
+      </c>
+      <c r="E1412" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F1412" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1412" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1413">
+      <c r="A1413" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1413" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:20</t>
+        </is>
+      </c>
+      <c r="C1413" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1413" s="2">
+        <v>24.8</v>
+      </c>
+      <c r="E1413" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F1413" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1413" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1414">
+      <c r="A1414" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1414" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:30</t>
+        </is>
+      </c>
+      <c r="C1414" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1414" s="2">
+        <v>25.1</v>
+      </c>
+      <c r="E1414" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="F1414" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1414" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1415">
+      <c r="A1415" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1415" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:40</t>
+        </is>
+      </c>
+      <c r="C1415" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1415" s="2">
+        <v>25.2</v>
+      </c>
+      <c r="E1415" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F1415" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1415" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1416">
+      <c r="A1416" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1416" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:50</t>
+        </is>
+      </c>
+      <c r="C1416" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1416" s="2">
+        <v>25.4</v>
+      </c>
+      <c r="E1416" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="F1416" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1416" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1417">
+      <c r="A1417" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1417" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:00</t>
+        </is>
+      </c>
+      <c r="C1417" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1417" s="2">
+        <v>25.6</v>
+      </c>
+      <c r="E1417" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F1417" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1417" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1418">
+      <c r="A1418" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1418" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:10</t>
+        </is>
+      </c>
+      <c r="C1418" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1418" s="2">
+        <v>25.3</v>
+      </c>
+      <c r="E1418" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F1418" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1418" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1419">
+      <c r="A1419" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1419" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:20</t>
+        </is>
+      </c>
+      <c r="C1419" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1419" s="2">
+        <v>24.8</v>
+      </c>
+      <c r="E1419" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F1419" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1419" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1420">
+      <c r="A1420" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1420" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:30</t>
+        </is>
+      </c>
+      <c r="C1420" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1420" s="2">
+        <v>25.2</v>
+      </c>
+      <c r="E1420" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F1420" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1420" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1421">
+      <c r="A1421" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1421" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:40</t>
+        </is>
+      </c>
+      <c r="C1421" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1421" s="2">
+        <v>24.9</v>
+      </c>
+      <c r="E1421" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F1421" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1421" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1422">
+      <c r="A1422" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1422" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:50</t>
+        </is>
+      </c>
+      <c r="C1422" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1422" s="2">
+        <v>24.9</v>
+      </c>
+      <c r="E1422" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F1422" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1422" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1423">
+      <c r="A1423" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1423" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:00</t>
+        </is>
+      </c>
+      <c r="C1423" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1423" s="2">
+        <v>24.5</v>
+      </c>
+      <c r="E1423" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F1423" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1423" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1424">
+      <c r="A1424" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1424" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:10</t>
+        </is>
+      </c>
+      <c r="C1424" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1424" s="2">
+        <v>24.8</v>
+      </c>
+      <c r="E1424" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="F1424" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1424" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1425">
+      <c r="A1425" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1425" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:20</t>
+        </is>
+      </c>
+      <c r="C1425" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1425" s="2">
+        <v>24.6</v>
+      </c>
+      <c r="E1425" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F1425" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1425" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1426">
+      <c r="A1426" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1426" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:30</t>
+        </is>
+      </c>
+      <c r="C1426" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1426" s="2">
+        <v>24.6</v>
+      </c>
+      <c r="E1426" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F1426" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1426" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1427">
+      <c r="A1427" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1427" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:40</t>
+        </is>
+      </c>
+      <c r="C1427" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1427" s="2">
+        <v>24.6</v>
+      </c>
+      <c r="E1427" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F1427" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1427" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1428">
+      <c r="A1428" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1428" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:50</t>
+        </is>
+      </c>
+      <c r="C1428" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1428" s="2">
+        <v>24.6</v>
+      </c>
+      <c r="E1428" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="F1428" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1428" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1429">
+      <c r="A1429" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1429" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:00</t>
+        </is>
+      </c>
+      <c r="C1429" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1429" s="2">
+        <v>24.5</v>
+      </c>
+      <c r="E1429" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="F1429" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1429" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1430">
+      <c r="A1430" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1430" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:10</t>
+        </is>
+      </c>
+      <c r="C1430" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1430" s="2">
+        <v>24.3</v>
+      </c>
+      <c r="E1430" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="F1430" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1430" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1431">
+      <c r="A1431" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1431" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:20</t>
+        </is>
+      </c>
+      <c r="C1431" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1431" s="2">
+        <v>24.7</v>
+      </c>
+      <c r="E1431" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F1431" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1431" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1432">
+      <c r="A1432" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1432" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:30</t>
+        </is>
+      </c>
+      <c r="C1432" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1432" s="2">
+        <v>24.8</v>
+      </c>
+      <c r="E1432" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F1432" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1432" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1433">
+      <c r="A1433" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1433" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:40</t>
+        </is>
+      </c>
+      <c r="C1433" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1433" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="E1433" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F1433" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1433" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1434">
+      <c r="A1434" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1434" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:50</t>
+        </is>
+      </c>
+      <c r="C1434" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1434" s="2">
+        <v>24.8</v>
+      </c>
+      <c r="E1434" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F1434" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1434" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1435">
+      <c r="A1435" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1435" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:00</t>
+        </is>
+      </c>
+      <c r="C1435" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1435" s="2">
+        <v>25.4</v>
+      </c>
+      <c r="E1435" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F1435" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1435" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1436">
+      <c r="A1436" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1436" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:10</t>
+        </is>
+      </c>
+      <c r="C1436" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1436" s="2">
+        <v>25.4</v>
+      </c>
+      <c r="E1436" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F1436" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1436" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1437">
+      <c r="A1437" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1437" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:20</t>
+        </is>
+      </c>
+      <c r="C1437" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1437" s="2">
+        <v>25.2</v>
+      </c>
+      <c r="E1437" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F1437" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1437" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1438">
+      <c r="A1438" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1438" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:30</t>
+        </is>
+      </c>
+      <c r="C1438" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1438" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="E1438" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F1438" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1438" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1439">
+      <c r="A1439" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1439" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:40</t>
+        </is>
+      </c>
+      <c r="C1439" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1439" s="2">
+        <v>25.3</v>
+      </c>
+      <c r="E1439" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F1439" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1439" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1440">
+      <c r="A1440" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1440" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:50</t>
+        </is>
+      </c>
+      <c r="C1440" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1440" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="E1440" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F1440" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1440" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1441">
+      <c r="A1441" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1441" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:00</t>
+        </is>
+      </c>
+      <c r="C1441" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1441" s="2">
+        <v>24.7</v>
+      </c>
+      <c r="E1441" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F1441" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1441" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1442">
+      <c r="A1442" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1442" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:10</t>
+        </is>
+      </c>
+      <c r="C1442" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1442" s="2">
+        <v>24.2</v>
+      </c>
+      <c r="E1442" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F1442" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1442" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1443">
+      <c r="A1443" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1443" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:20</t>
+        </is>
+      </c>
+      <c r="C1443" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1443" s="2">
+        <v>23.4</v>
+      </c>
+      <c r="E1443" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="F1443" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1443" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1444">
+      <c r="A1444" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1444" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:30</t>
+        </is>
+      </c>
+      <c r="C1444" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1444" s="2">
+        <v>23.3</v>
+      </c>
+      <c r="E1444" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="F1444" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1444" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1445">
+      <c r="A1445" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1445" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:40</t>
+        </is>
+      </c>
+      <c r="C1445" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1445" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="E1445" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="F1445" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1445" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1446">
+      <c r="A1446" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1446" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:50</t>
+        </is>
+      </c>
+      <c r="C1446" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1446" s="2">
+        <v>22.8</v>
+      </c>
+      <c r="E1446" s="2">
+        <v>37.0</v>
+      </c>
+      <c r="F1446" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1446" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1447">
+      <c r="A1447" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1447" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:00</t>
+        </is>
+      </c>
+      <c r="C1447" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1447" s="2">
+        <v>22.6</v>
+      </c>
+      <c r="E1447" s="2">
+        <v>38.0</v>
+      </c>
+      <c r="F1447" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1447" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1448">
+      <c r="A1448" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1448" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:10</t>
+        </is>
+      </c>
+      <c r="C1448" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1448" s="2">
+        <v>22.1</v>
+      </c>
+      <c r="E1448" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F1448" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1448" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1449">
+      <c r="A1449" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1449" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:20</t>
+        </is>
+      </c>
+      <c r="C1449" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1449" s="2">
+        <v>21.8</v>
+      </c>
+      <c r="E1449" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F1449" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1449" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1450">
+      <c r="A1450" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1450" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:30</t>
+        </is>
+      </c>
+      <c r="C1450" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1450" s="2">
+        <v>21.6</v>
+      </c>
+      <c r="E1450" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F1450" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1450" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1451">
+      <c r="A1451" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1451" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:40</t>
+        </is>
+      </c>
+      <c r="C1451" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1451" s="2">
+        <v>21.3</v>
+      </c>
+      <c r="E1451" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F1451" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1451" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1452">
+      <c r="A1452" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1452" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:50</t>
+        </is>
+      </c>
+      <c r="C1452" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1452" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="E1452" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F1452" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1452" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1453">
+      <c r="A1453" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1453" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:00</t>
+        </is>
+      </c>
+      <c r="C1453" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1453" s="2">
+        <v>20.4</v>
+      </c>
+      <c r="E1453" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F1453" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1453" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1454">
+      <c r="A1454" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1454" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:10</t>
+        </is>
+      </c>
+      <c r="C1454" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1454" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="E1454" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F1454" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1454" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1455">
+      <c r="A1455" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1455" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:20</t>
+        </is>
+      </c>
+      <c r="C1455" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1455" s="2">
+        <v>19.5</v>
+      </c>
+      <c r="E1455" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F1455" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1455" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1456">
+      <c r="A1456" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1456" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:30</t>
+        </is>
+      </c>
+      <c r="C1456" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1456" s="2">
+        <v>19.2</v>
+      </c>
+      <c r="E1456" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F1456" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1456" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1457">
+      <c r="A1457" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1457" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:40</t>
+        </is>
+      </c>
+      <c r="C1457" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1457" s="2">
+        <v>18.7</v>
+      </c>
+      <c r="E1457" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F1457" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1457" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1458">
+      <c r="A1458" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1458" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:50</t>
+        </is>
+      </c>
+      <c r="C1458" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1458" s="2">
+        <v>18.2</v>
+      </c>
+      <c r="E1458" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F1458" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1458" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1459">
+      <c r="A1459" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1459" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:00</t>
+        </is>
+      </c>
+      <c r="C1459" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1459" s="2">
+        <v>17.7</v>
+      </c>
+      <c r="E1459" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F1459" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1459" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1460">
+      <c r="A1460" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1460" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:10</t>
+        </is>
+      </c>
+      <c r="C1460" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1460" s="2">
+        <v>17.2</v>
+      </c>
+      <c r="E1460" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F1460" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1460" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1461">
+      <c r="A1461" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1461" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:20</t>
+        </is>
+      </c>
+      <c r="C1461" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1461" s="2">
+        <v>16.8</v>
+      </c>
+      <c r="E1461" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F1461" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1461" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1462">
+      <c r="A1462" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1462" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:30</t>
+        </is>
+      </c>
+      <c r="C1462" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1462" s="2">
+        <v>16.6</v>
+      </c>
+      <c r="E1462" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F1462" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1462" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1463">
+      <c r="A1463" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1463" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:40</t>
+        </is>
+      </c>
+      <c r="C1463" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1463" s="2">
+        <v>16.3</v>
+      </c>
+      <c r="E1463" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F1463" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1463" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1464">
+      <c r="A1464" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1464" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:50</t>
+        </is>
+      </c>
+      <c r="C1464" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1464" s="2">
+        <v>16.1</v>
+      </c>
+      <c r="E1464" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F1464" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1464" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1465">
+      <c r="A1465" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1465" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:00</t>
+        </is>
+      </c>
+      <c r="C1465" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1465" s="2">
+        <v>15.8</v>
+      </c>
+      <c r="E1465" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F1465" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1465" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1466">
+      <c r="A1466" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1466" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:10</t>
+        </is>
+      </c>
+      <c r="C1466" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1466" s="2">
+        <v>15.7</v>
+      </c>
+      <c r="E1466" s="2">
+        <v>69.0</v>
+      </c>
+      <c r="F1466" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1466" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1467">
+      <c r="A1467" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1467" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:20</t>
+        </is>
+      </c>
+      <c r="C1467" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1467" s="2">
+        <v>15.7</v>
+      </c>
+      <c r="E1467" s="2">
+        <v>69.0</v>
+      </c>
+      <c r="F1467" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1467" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1468">
+      <c r="A1468" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1468" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:30</t>
+        </is>
+      </c>
+      <c r="C1468" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1468" s="2">
+        <v>15.6</v>
+      </c>
+      <c r="E1468" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F1468" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1468" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1469">
+      <c r="A1469" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1469" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:40</t>
+        </is>
+      </c>
+      <c r="C1469" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1469" s="2">
+        <v>15.3</v>
+      </c>
+      <c r="E1469" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F1469" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1469" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1470">
+      <c r="A1470" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">24.07.2026</t>
+        </is>
+      </c>
+      <c r="B1470" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:50</t>
+        </is>
+      </c>
+      <c r="C1470" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1470" s="2">
+        <v>15.1</v>
+      </c>
+      <c r="E1470" s="2">
+        <v>72.0</v>
+      </c>
+      <c r="F1470" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1470" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1471">
+      <c r="A1471" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1471" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:00</t>
+        </is>
+      </c>
+      <c r="C1471" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1471" s="2">
+        <v>15.0</v>
+      </c>
+      <c r="E1471" s="2">
+        <v>72.0</v>
+      </c>
+      <c r="F1471" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1471" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1472">
+      <c r="A1472" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1472" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:10</t>
+        </is>
+      </c>
+      <c r="C1472" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1472" s="2">
+        <v>15.0</v>
+      </c>
+      <c r="E1472" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F1472" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1472" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1473">
+      <c r="A1473" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1473" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:20</t>
+        </is>
+      </c>
+      <c r="C1473" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1473" s="2">
+        <v>14.8</v>
+      </c>
+      <c r="E1473" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="F1473" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1473" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1474">
+      <c r="A1474" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1474" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:30</t>
+        </is>
+      </c>
+      <c r="C1474" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1474" s="2">
+        <v>14.6</v>
+      </c>
+      <c r="E1474" s="2">
+        <v>74.0</v>
+      </c>
+      <c r="F1474" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1474" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G1329"/>
+  <autoFilter ref="A1:G1474"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ARSO Kranj zajem 2026-07-26 00:40 Europe/Ljubljana
</commit_message>
<xml_diff>
--- a/tabela_vremena/ARSO_Kranj.xlsx
+++ b/tabela_vremena/ARSO_Kranj.xlsx
@@ -42828,7 +42828,4154 @@
         <v>0.0</v>
       </c>
     </row>
+    <row r="1475">
+      <c r="A1475" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1475" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:40</t>
+        </is>
+      </c>
+      <c r="C1475" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1475" s="2">
+        <v>14.4</v>
+      </c>
+      <c r="E1475" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F1475" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1475" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1476">
+      <c r="A1476" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1476" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:50</t>
+        </is>
+      </c>
+      <c r="C1476" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1476" s="2">
+        <v>14.1</v>
+      </c>
+      <c r="E1476" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F1476" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1476" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1477">
+      <c r="A1477" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1477" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:00</t>
+        </is>
+      </c>
+      <c r="C1477" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1477" s="2">
+        <v>14.0</v>
+      </c>
+      <c r="E1477" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F1477" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1477" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1478">
+      <c r="A1478" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1478" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:10</t>
+        </is>
+      </c>
+      <c r="C1478" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1478" s="2">
+        <v>14.0</v>
+      </c>
+      <c r="E1478" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F1478" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1478" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1479">
+      <c r="A1479" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1479" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:20</t>
+        </is>
+      </c>
+      <c r="C1479" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1479" s="2">
+        <v>13.9</v>
+      </c>
+      <c r="E1479" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F1479" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1479" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1480">
+      <c r="A1480" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1480" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:30</t>
+        </is>
+      </c>
+      <c r="C1480" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1480" s="2">
+        <v>14.0</v>
+      </c>
+      <c r="E1480" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F1480" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1480" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1481">
+      <c r="A1481" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1481" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:40</t>
+        </is>
+      </c>
+      <c r="C1481" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1481" s="2">
+        <v>14.0</v>
+      </c>
+      <c r="E1481" s="2">
+        <v>74.0</v>
+      </c>
+      <c r="F1481" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1481" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1482">
+      <c r="A1482" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1482" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:50</t>
+        </is>
+      </c>
+      <c r="C1482" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1482" s="2">
+        <v>14.1</v>
+      </c>
+      <c r="E1482" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="F1482" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1482" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1483">
+      <c r="A1483" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1483" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:00</t>
+        </is>
+      </c>
+      <c r="C1483" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1483" s="2">
+        <v>14.0</v>
+      </c>
+      <c r="E1483" s="2">
+        <v>74.0</v>
+      </c>
+      <c r="F1483" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1483" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1484">
+      <c r="A1484" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1484" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:10</t>
+        </is>
+      </c>
+      <c r="C1484" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1484" s="2">
+        <v>13.8</v>
+      </c>
+      <c r="E1484" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F1484" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1484" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1485">
+      <c r="A1485" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1485" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:20</t>
+        </is>
+      </c>
+      <c r="C1485" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1485" s="2">
+        <v>13.7</v>
+      </c>
+      <c r="E1485" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F1485" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1485" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1486">
+      <c r="A1486" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1486" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:30</t>
+        </is>
+      </c>
+      <c r="C1486" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1486" s="2">
+        <v>13.5</v>
+      </c>
+      <c r="E1486" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F1486" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1486" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1487">
+      <c r="A1487" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1487" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:40</t>
+        </is>
+      </c>
+      <c r="C1487" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1487" s="2">
+        <v>13.3</v>
+      </c>
+      <c r="E1487" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F1487" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1487" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1488">
+      <c r="A1488" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1488" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:50</t>
+        </is>
+      </c>
+      <c r="C1488" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1488" s="2">
+        <v>13.1</v>
+      </c>
+      <c r="E1488" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F1488" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1488" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1489">
+      <c r="A1489" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1489" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:00</t>
+        </is>
+      </c>
+      <c r="C1489" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1489" s="2">
+        <v>12.9</v>
+      </c>
+      <c r="E1489" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F1489" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1489" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1490">
+      <c r="A1490" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1490" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:10</t>
+        </is>
+      </c>
+      <c r="C1490" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1490" s="2">
+        <v>12.8</v>
+      </c>
+      <c r="E1490" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F1490" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1490" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1491">
+      <c r="A1491" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1491" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:20</t>
+        </is>
+      </c>
+      <c r="C1491" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1491" s="2">
+        <v>12.7</v>
+      </c>
+      <c r="E1491" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F1491" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1491" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1492">
+      <c r="A1492" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1492" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:30</t>
+        </is>
+      </c>
+      <c r="C1492" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1492" s="2">
+        <v>12.6</v>
+      </c>
+      <c r="E1492" s="2">
+        <v>81.0</v>
+      </c>
+      <c r="F1492" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1492" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1493">
+      <c r="A1493" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1493" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:40</t>
+        </is>
+      </c>
+      <c r="C1493" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1493" s="2">
+        <v>12.6</v>
+      </c>
+      <c r="E1493" s="2">
+        <v>81.0</v>
+      </c>
+      <c r="F1493" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1493" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1494">
+      <c r="A1494" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1494" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:50</t>
+        </is>
+      </c>
+      <c r="C1494" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1494" s="2">
+        <v>12.4</v>
+      </c>
+      <c r="E1494" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F1494" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1494" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1495">
+      <c r="A1495" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1495" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:00</t>
+        </is>
+      </c>
+      <c r="C1495" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1495" s="2">
+        <v>12.1</v>
+      </c>
+      <c r="E1495" s="2">
+        <v>84.0</v>
+      </c>
+      <c r="F1495" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1495" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1496">
+      <c r="A1496" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1496" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:10</t>
+        </is>
+      </c>
+      <c r="C1496" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1496" s="2">
+        <v>11.9</v>
+      </c>
+      <c r="E1496" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F1496" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1496" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1497">
+      <c r="A1497" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1497" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:20</t>
+        </is>
+      </c>
+      <c r="C1497" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1497" s="2">
+        <v>11.8</v>
+      </c>
+      <c r="E1497" s="2">
+        <v>84.0</v>
+      </c>
+      <c r="F1497" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1497" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1498">
+      <c r="A1498" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1498" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:30</t>
+        </is>
+      </c>
+      <c r="C1498" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1498" s="2">
+        <v>11.7</v>
+      </c>
+      <c r="E1498" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F1498" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1498" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1499">
+      <c r="A1499" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1499" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:40</t>
+        </is>
+      </c>
+      <c r="C1499" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1499" s="2">
+        <v>11.7</v>
+      </c>
+      <c r="E1499" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F1499" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1499" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1500">
+      <c r="A1500" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1500" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:50</t>
+        </is>
+      </c>
+      <c r="C1500" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1500" s="2">
+        <v>11.7</v>
+      </c>
+      <c r="E1500" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F1500" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1500" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1501">
+      <c r="A1501" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1501" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:00</t>
+        </is>
+      </c>
+      <c r="C1501" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1501" s="2">
+        <v>11.5</v>
+      </c>
+      <c r="E1501" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F1501" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1501" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1502">
+      <c r="A1502" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1502" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:10</t>
+        </is>
+      </c>
+      <c r="C1502" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1502" s="2">
+        <v>11.3</v>
+      </c>
+      <c r="E1502" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F1502" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1502" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1503">
+      <c r="A1503" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1503" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:20</t>
+        </is>
+      </c>
+      <c r="C1503" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1503" s="2">
+        <v>11.2</v>
+      </c>
+      <c r="E1503" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F1503" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1503" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1504">
+      <c r="A1504" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1504" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:30</t>
+        </is>
+      </c>
+      <c r="C1504" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1504" s="2">
+        <v>11.2</v>
+      </c>
+      <c r="E1504" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F1504" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1504" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1505">
+      <c r="A1505" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1505" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:40</t>
+        </is>
+      </c>
+      <c r="C1505" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1505" s="2">
+        <v>11.3</v>
+      </c>
+      <c r="E1505" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F1505" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1505" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1506">
+      <c r="A1506" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1506" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:50</t>
+        </is>
+      </c>
+      <c r="C1506" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1506" s="2">
+        <v>11.3</v>
+      </c>
+      <c r="E1506" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F1506" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1506" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1507">
+      <c r="A1507" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1507" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:00</t>
+        </is>
+      </c>
+      <c r="C1507" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1507" s="2">
+        <v>11.3</v>
+      </c>
+      <c r="E1507" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F1507" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1507" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1508">
+      <c r="A1508" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1508" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:10</t>
+        </is>
+      </c>
+      <c r="C1508" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1508" s="2">
+        <v>11.4</v>
+      </c>
+      <c r="E1508" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F1508" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1508" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1509">
+      <c r="A1509" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1509" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:20</t>
+        </is>
+      </c>
+      <c r="C1509" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1509" s="2">
+        <v>11.4</v>
+      </c>
+      <c r="E1509" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F1509" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1509" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1510">
+      <c r="A1510" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1510" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:30</t>
+        </is>
+      </c>
+      <c r="C1510" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1510" s="2">
+        <v>11.8</v>
+      </c>
+      <c r="E1510" s="2">
+        <v>84.0</v>
+      </c>
+      <c r="F1510" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1510" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1511">
+      <c r="A1511" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1511" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:40</t>
+        </is>
+      </c>
+      <c r="C1511" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1511" s="2">
+        <v>12.0</v>
+      </c>
+      <c r="E1511" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F1511" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1511" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1512">
+      <c r="A1512" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1512" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:50</t>
+        </is>
+      </c>
+      <c r="C1512" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1512" s="2">
+        <v>12.1</v>
+      </c>
+      <c r="E1512" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F1512" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1512" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1513">
+      <c r="A1513" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1513" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:00</t>
+        </is>
+      </c>
+      <c r="C1513" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1513" s="2">
+        <v>12.2</v>
+      </c>
+      <c r="E1513" s="2">
+        <v>83.0</v>
+      </c>
+      <c r="F1513" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1513" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1514">
+      <c r="A1514" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1514" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:10</t>
+        </is>
+      </c>
+      <c r="C1514" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1514" s="2">
+        <v>12.4</v>
+      </c>
+      <c r="E1514" s="2">
+        <v>83.0</v>
+      </c>
+      <c r="F1514" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1514" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1515">
+      <c r="A1515" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1515" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:20</t>
+        </is>
+      </c>
+      <c r="C1515" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1515" s="2">
+        <v>12.7</v>
+      </c>
+      <c r="E1515" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F1515" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1515" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1516">
+      <c r="A1516" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1516" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:30</t>
+        </is>
+      </c>
+      <c r="C1516" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1516" s="2">
+        <v>13.0</v>
+      </c>
+      <c r="E1516" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F1516" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1516" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1517">
+      <c r="A1517" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1517" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:40</t>
+        </is>
+      </c>
+      <c r="C1517" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1517" s="2">
+        <v>13.3</v>
+      </c>
+      <c r="E1517" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F1517" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1517" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1518">
+      <c r="A1518" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1518" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:50</t>
+        </is>
+      </c>
+      <c r="C1518" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1518" s="2">
+        <v>13.8</v>
+      </c>
+      <c r="E1518" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F1518" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1518" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1519">
+      <c r="A1519" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1519" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:00</t>
+        </is>
+      </c>
+      <c r="C1519" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1519" s="2">
+        <v>14.0</v>
+      </c>
+      <c r="E1519" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F1519" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1519" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1520">
+      <c r="A1520" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1520" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:10</t>
+        </is>
+      </c>
+      <c r="C1520" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1520" s="2">
+        <v>14.5</v>
+      </c>
+      <c r="E1520" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="F1520" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1520" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1521">
+      <c r="A1521" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1521" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:20</t>
+        </is>
+      </c>
+      <c r="C1521" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1521" s="2">
+        <v>15.3</v>
+      </c>
+      <c r="E1521" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F1521" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1521" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1522">
+      <c r="A1522" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1522" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:30</t>
+        </is>
+      </c>
+      <c r="C1522" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1522" s="2">
+        <v>15.9</v>
+      </c>
+      <c r="E1522" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F1522" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1522" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1523">
+      <c r="A1523" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1523" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:40</t>
+        </is>
+      </c>
+      <c r="C1523" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1523" s="2">
+        <v>16.8</v>
+      </c>
+      <c r="E1523" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F1523" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1523" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1524">
+      <c r="A1524" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1524" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:50</t>
+        </is>
+      </c>
+      <c r="C1524" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1524" s="2">
+        <v>17.8</v>
+      </c>
+      <c r="E1524" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F1524" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1524" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1525">
+      <c r="A1525" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1525" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:00</t>
+        </is>
+      </c>
+      <c r="C1525" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1525" s="2">
+        <v>18.0</v>
+      </c>
+      <c r="E1525" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F1525" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1525" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1526">
+      <c r="A1526" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1526" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:10</t>
+        </is>
+      </c>
+      <c r="C1526" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1526" s="2">
+        <v>18.2</v>
+      </c>
+      <c r="E1526" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F1526" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1526" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1527">
+      <c r="A1527" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1527" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:20</t>
+        </is>
+      </c>
+      <c r="C1527" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1527" s="2">
+        <v>18.8</v>
+      </c>
+      <c r="E1527" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F1527" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1527" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1528">
+      <c r="A1528" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1528" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:30</t>
+        </is>
+      </c>
+      <c r="C1528" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1528" s="2">
+        <v>19.7</v>
+      </c>
+      <c r="E1528" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F1528" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1528" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1529">
+      <c r="A1529" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1529" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:40</t>
+        </is>
+      </c>
+      <c r="C1529" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1529" s="2">
+        <v>20.1</v>
+      </c>
+      <c r="E1529" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F1529" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1529" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1530">
+      <c r="A1530" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1530" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:50</t>
+        </is>
+      </c>
+      <c r="C1530" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1530" s="2">
+        <v>20.3</v>
+      </c>
+      <c r="E1530" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F1530" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1530" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1531">
+      <c r="A1531" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1531" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:00</t>
+        </is>
+      </c>
+      <c r="C1531" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1531" s="2">
+        <v>20.4</v>
+      </c>
+      <c r="E1531" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F1531" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1531" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1532">
+      <c r="A1532" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1532" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:10</t>
+        </is>
+      </c>
+      <c r="C1532" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1532" s="2">
+        <v>21.1</v>
+      </c>
+      <c r="E1532" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F1532" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1532" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1533">
+      <c r="A1533" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1533" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:20</t>
+        </is>
+      </c>
+      <c r="C1533" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1533" s="2">
+        <v>21.5</v>
+      </c>
+      <c r="E1533" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F1533" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1533" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1534">
+      <c r="A1534" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1534" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:30</t>
+        </is>
+      </c>
+      <c r="C1534" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1534" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="E1534" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F1534" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1534" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1535">
+      <c r="A1535" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1535" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:40</t>
+        </is>
+      </c>
+      <c r="C1535" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1535" s="2">
+        <v>22.7</v>
+      </c>
+      <c r="E1535" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F1535" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1535" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1536">
+      <c r="A1536" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1536" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:50</t>
+        </is>
+      </c>
+      <c r="C1536" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1536" s="2">
+        <v>23.2</v>
+      </c>
+      <c r="E1536" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F1536" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1536" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1537">
+      <c r="A1537" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1537" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:00</t>
+        </is>
+      </c>
+      <c r="C1537" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1537" s="2">
+        <v>23.6</v>
+      </c>
+      <c r="E1537" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F1537" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1537" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1538">
+      <c r="A1538" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1538" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:10</t>
+        </is>
+      </c>
+      <c r="C1538" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1538" s="2">
+        <v>24.2</v>
+      </c>
+      <c r="E1538" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F1538" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1538" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1539">
+      <c r="A1539" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1539" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:20</t>
+        </is>
+      </c>
+      <c r="C1539" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1539" s="2">
+        <v>24.7</v>
+      </c>
+      <c r="E1539" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F1539" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1539" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1540">
+      <c r="A1540" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1540" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:30</t>
+        </is>
+      </c>
+      <c r="C1540" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1540" s="2">
+        <v>24.3</v>
+      </c>
+      <c r="E1540" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F1540" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1540" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1541">
+      <c r="A1541" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1541" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:40</t>
+        </is>
+      </c>
+      <c r="C1541" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1541" s="2">
+        <v>24.7</v>
+      </c>
+      <c r="E1541" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F1541" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1541" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1542">
+      <c r="A1542" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1542" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:50</t>
+        </is>
+      </c>
+      <c r="C1542" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1542" s="2">
+        <v>25.3</v>
+      </c>
+      <c r="E1542" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F1542" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1542" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1543">
+      <c r="A1543" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1543" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:00</t>
+        </is>
+      </c>
+      <c r="C1543" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1543" s="2">
+        <v>25.9</v>
+      </c>
+      <c r="E1543" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F1543" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1543" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1544">
+      <c r="A1544" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1544" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:10</t>
+        </is>
+      </c>
+      <c r="C1544" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1544" s="2">
+        <v>25.7</v>
+      </c>
+      <c r="E1544" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F1544" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1544" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1545">
+      <c r="A1545" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1545" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:20</t>
+        </is>
+      </c>
+      <c r="C1545" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1545" s="2">
+        <v>25.6</v>
+      </c>
+      <c r="E1545" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F1545" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1545" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1546">
+      <c r="A1546" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1546" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:30</t>
+        </is>
+      </c>
+      <c r="C1546" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1546" s="2">
+        <v>25.9</v>
+      </c>
+      <c r="E1546" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F1546" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1546" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1547">
+      <c r="A1547" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1547" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:40</t>
+        </is>
+      </c>
+      <c r="C1547" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1547" s="2">
+        <v>26.5</v>
+      </c>
+      <c r="E1547" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F1547" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1547" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1548">
+      <c r="A1548" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1548" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:50</t>
+        </is>
+      </c>
+      <c r="C1548" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1548" s="2">
+        <v>26.5</v>
+      </c>
+      <c r="E1548" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F1548" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1548" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1549">
+      <c r="A1549" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1549" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:00</t>
+        </is>
+      </c>
+      <c r="C1549" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1549" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="E1549" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F1549" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1549" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1550">
+      <c r="A1550" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1550" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:10</t>
+        </is>
+      </c>
+      <c r="C1550" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1550" s="2">
+        <v>26.6</v>
+      </c>
+      <c r="E1550" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F1550" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1550" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1551">
+      <c r="A1551" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1551" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:20</t>
+        </is>
+      </c>
+      <c r="C1551" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1551" s="2">
+        <v>26.7</v>
+      </c>
+      <c r="E1551" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F1551" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1551" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1552">
+      <c r="A1552" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1552" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:30</t>
+        </is>
+      </c>
+      <c r="C1552" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1552" s="2">
+        <v>26.9</v>
+      </c>
+      <c r="E1552" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F1552" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1552" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1553">
+      <c r="A1553" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1553" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:40</t>
+        </is>
+      </c>
+      <c r="C1553" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1553" s="2">
+        <v>26.9</v>
+      </c>
+      <c r="E1553" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F1553" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1553" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1554">
+      <c r="A1554" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1554" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:50</t>
+        </is>
+      </c>
+      <c r="C1554" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1554" s="2">
+        <v>26.7</v>
+      </c>
+      <c r="E1554" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F1554" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1554" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1555">
+      <c r="A1555" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1555" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:00</t>
+        </is>
+      </c>
+      <c r="C1555" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1555" s="2">
+        <v>27.4</v>
+      </c>
+      <c r="E1555" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F1555" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1555" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1556">
+      <c r="A1556" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1556" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:10</t>
+        </is>
+      </c>
+      <c r="C1556" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1556" s="2">
+        <v>27.5</v>
+      </c>
+      <c r="E1556" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F1556" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1556" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1557">
+      <c r="A1557" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1557" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:20</t>
+        </is>
+      </c>
+      <c r="C1557" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1557" s="2">
+        <v>27.4</v>
+      </c>
+      <c r="E1557" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F1557" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1557" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1558">
+      <c r="A1558" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1558" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:30</t>
+        </is>
+      </c>
+      <c r="C1558" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1558" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="E1558" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F1558" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1558" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1559">
+      <c r="A1559" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1559" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:40</t>
+        </is>
+      </c>
+      <c r="C1559" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1559" s="2">
+        <v>27.9</v>
+      </c>
+      <c r="E1559" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F1559" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1559" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1560">
+      <c r="A1560" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1560" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:50</t>
+        </is>
+      </c>
+      <c r="C1560" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1560" s="2">
+        <v>27.5</v>
+      </c>
+      <c r="E1560" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F1560" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1560" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1561">
+      <c r="A1561" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1561" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:00</t>
+        </is>
+      </c>
+      <c r="C1561" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1561" s="2">
+        <v>27.4</v>
+      </c>
+      <c r="E1561" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F1561" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1561" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1562">
+      <c r="A1562" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1562" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:10</t>
+        </is>
+      </c>
+      <c r="C1562" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1562" s="2">
+        <v>27.4</v>
+      </c>
+      <c r="E1562" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F1562" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1562" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1563">
+      <c r="A1563" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1563" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:20</t>
+        </is>
+      </c>
+      <c r="C1563" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1563" s="2">
+        <v>27.1</v>
+      </c>
+      <c r="E1563" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F1563" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1563" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1564">
+      <c r="A1564" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1564" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:30</t>
+        </is>
+      </c>
+      <c r="C1564" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1564" s="2">
+        <v>27.1</v>
+      </c>
+      <c r="E1564" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F1564" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1564" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1565">
+      <c r="A1565" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1565" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:40</t>
+        </is>
+      </c>
+      <c r="C1565" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1565" s="2">
+        <v>26.7</v>
+      </c>
+      <c r="E1565" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F1565" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1565" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1566">
+      <c r="A1566" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1566" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:50</t>
+        </is>
+      </c>
+      <c r="C1566" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1566" s="2">
+        <v>26.8</v>
+      </c>
+      <c r="E1566" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F1566" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1566" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1567">
+      <c r="A1567" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1567" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:00</t>
+        </is>
+      </c>
+      <c r="C1567" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1567" s="2">
+        <v>26.9</v>
+      </c>
+      <c r="E1567" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F1567" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1567" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1568">
+      <c r="A1568" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1568" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:10</t>
+        </is>
+      </c>
+      <c r="C1568" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1568" s="2">
+        <v>26.6</v>
+      </c>
+      <c r="E1568" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F1568" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1568" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1569">
+      <c r="A1569" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1569" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:20</t>
+        </is>
+      </c>
+      <c r="C1569" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1569" s="2">
+        <v>26.7</v>
+      </c>
+      <c r="E1569" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F1569" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1569" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1570">
+      <c r="A1570" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1570" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:30</t>
+        </is>
+      </c>
+      <c r="C1570" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1570" s="2">
+        <v>26.8</v>
+      </c>
+      <c r="E1570" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F1570" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1570" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1571">
+      <c r="A1571" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1571" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:40</t>
+        </is>
+      </c>
+      <c r="C1571" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1571" s="2">
+        <v>26.5</v>
+      </c>
+      <c r="E1571" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F1571" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1571" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1572">
+      <c r="A1572" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1572" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:50</t>
+        </is>
+      </c>
+      <c r="C1572" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1572" s="2">
+        <v>26.5</v>
+      </c>
+      <c r="E1572" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F1572" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1572" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1573">
+      <c r="A1573" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1573" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:00</t>
+        </is>
+      </c>
+      <c r="C1573" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1573" s="2">
+        <v>26.7</v>
+      </c>
+      <c r="E1573" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F1573" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1573" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1574">
+      <c r="A1574" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1574" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:10</t>
+        </is>
+      </c>
+      <c r="C1574" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1574" s="2">
+        <v>26.9</v>
+      </c>
+      <c r="E1574" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F1574" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1574" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1575">
+      <c r="A1575" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1575" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:20</t>
+        </is>
+      </c>
+      <c r="C1575" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1575" s="2">
+        <v>26.8</v>
+      </c>
+      <c r="E1575" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F1575" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1575" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1576">
+      <c r="A1576" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1576" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:30</t>
+        </is>
+      </c>
+      <c r="C1576" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1576" s="2">
+        <v>26.6</v>
+      </c>
+      <c r="E1576" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F1576" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1576" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1577">
+      <c r="A1577" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1577" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:40</t>
+        </is>
+      </c>
+      <c r="C1577" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1577" s="2">
+        <v>26.5</v>
+      </c>
+      <c r="E1577" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F1577" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1577" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1578">
+      <c r="A1578" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1578" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:50</t>
+        </is>
+      </c>
+      <c r="C1578" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1578" s="2">
+        <v>26.5</v>
+      </c>
+      <c r="E1578" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F1578" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1578" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1579">
+      <c r="A1579" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1579" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:00</t>
+        </is>
+      </c>
+      <c r="C1579" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1579" s="2">
+        <v>26.4</v>
+      </c>
+      <c r="E1579" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F1579" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1579" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1580">
+      <c r="A1580" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1580" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:10</t>
+        </is>
+      </c>
+      <c r="C1580" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1580" s="2">
+        <v>26.9</v>
+      </c>
+      <c r="E1580" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F1580" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1580" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1581">
+      <c r="A1581" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1581" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:20</t>
+        </is>
+      </c>
+      <c r="C1581" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1581" s="2">
+        <v>26.7</v>
+      </c>
+      <c r="E1581" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F1581" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1581" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1582">
+      <c r="A1582" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1582" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:30</t>
+        </is>
+      </c>
+      <c r="C1582" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1582" s="2">
+        <v>26.6</v>
+      </c>
+      <c r="E1582" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F1582" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1582" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1583">
+      <c r="A1583" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1583" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:40</t>
+        </is>
+      </c>
+      <c r="C1583" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1583" s="2">
+        <v>26.1</v>
+      </c>
+      <c r="E1583" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F1583" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1583" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1584">
+      <c r="A1584" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1584" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:50</t>
+        </is>
+      </c>
+      <c r="C1584" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1584" s="2">
+        <v>25.7</v>
+      </c>
+      <c r="E1584" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F1584" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1584" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1585">
+      <c r="A1585" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1585" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:00</t>
+        </is>
+      </c>
+      <c r="C1585" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1585" s="2">
+        <v>25.5</v>
+      </c>
+      <c r="E1585" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F1585" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1585" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1586">
+      <c r="A1586" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1586" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:10</t>
+        </is>
+      </c>
+      <c r="C1586" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1586" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="E1586" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F1586" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1586" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1587">
+      <c r="A1587" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1587" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:20</t>
+        </is>
+      </c>
+      <c r="C1587" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1587" s="2">
+        <v>24.6</v>
+      </c>
+      <c r="E1587" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F1587" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1587" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1588">
+      <c r="A1588" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1588" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:30</t>
+        </is>
+      </c>
+      <c r="C1588" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1588" s="2">
+        <v>24.4</v>
+      </c>
+      <c r="E1588" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F1588" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1588" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1589">
+      <c r="A1589" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1589" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:40</t>
+        </is>
+      </c>
+      <c r="C1589" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1589" s="2">
+        <v>24.2</v>
+      </c>
+      <c r="E1589" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F1589" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1589" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1590">
+      <c r="A1590" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1590" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:50</t>
+        </is>
+      </c>
+      <c r="C1590" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1590" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="E1590" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F1590" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1590" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1591">
+      <c r="A1591" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1591" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:00</t>
+        </is>
+      </c>
+      <c r="C1591" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1591" s="2">
+        <v>23.8</v>
+      </c>
+      <c r="E1591" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F1591" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1591" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1592">
+      <c r="A1592" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1592" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:10</t>
+        </is>
+      </c>
+      <c r="C1592" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1592" s="2">
+        <v>23.6</v>
+      </c>
+      <c r="E1592" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F1592" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1592" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1593">
+      <c r="A1593" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1593" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:20</t>
+        </is>
+      </c>
+      <c r="C1593" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1593" s="2">
+        <v>23.3</v>
+      </c>
+      <c r="E1593" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F1593" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1593" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1594">
+      <c r="A1594" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1594" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:30</t>
+        </is>
+      </c>
+      <c r="C1594" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1594" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="E1594" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F1594" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1594" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1595">
+      <c r="A1595" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1595" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:40</t>
+        </is>
+      </c>
+      <c r="C1595" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1595" s="2">
+        <v>22.7</v>
+      </c>
+      <c r="E1595" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F1595" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1595" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1596">
+      <c r="A1596" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1596" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:50</t>
+        </is>
+      </c>
+      <c r="C1596" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1596" s="2">
+        <v>22.4</v>
+      </c>
+      <c r="E1596" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F1596" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1596" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1597">
+      <c r="A1597" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1597" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:00</t>
+        </is>
+      </c>
+      <c r="C1597" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1597" s="2">
+        <v>22.1</v>
+      </c>
+      <c r="E1597" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F1597" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1597" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1598">
+      <c r="A1598" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1598" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:10</t>
+        </is>
+      </c>
+      <c r="C1598" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1598" s="2">
+        <v>21.8</v>
+      </c>
+      <c r="E1598" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F1598" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1598" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1599">
+      <c r="A1599" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1599" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:20</t>
+        </is>
+      </c>
+      <c r="C1599" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1599" s="2">
+        <v>21.6</v>
+      </c>
+      <c r="E1599" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F1599" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1599" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1600">
+      <c r="A1600" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1600" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:30</t>
+        </is>
+      </c>
+      <c r="C1600" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1600" s="2">
+        <v>21.4</v>
+      </c>
+      <c r="E1600" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F1600" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1600" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1601">
+      <c r="A1601" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1601" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:40</t>
+        </is>
+      </c>
+      <c r="C1601" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1601" s="2">
+        <v>21.1</v>
+      </c>
+      <c r="E1601" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F1601" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1601" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1602">
+      <c r="A1602" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1602" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:50</t>
+        </is>
+      </c>
+      <c r="C1602" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1602" s="2">
+        <v>20.9</v>
+      </c>
+      <c r="E1602" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F1602" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1602" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1603">
+      <c r="A1603" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1603" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:00</t>
+        </is>
+      </c>
+      <c r="C1603" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1603" s="2">
+        <v>20.4</v>
+      </c>
+      <c r="E1603" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F1603" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1603" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1604">
+      <c r="A1604" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1604" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:10</t>
+        </is>
+      </c>
+      <c r="C1604" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1604" s="2">
+        <v>19.8</v>
+      </c>
+      <c r="E1604" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F1604" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1604" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1605">
+      <c r="A1605" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1605" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:20</t>
+        </is>
+      </c>
+      <c r="C1605" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1605" s="2">
+        <v>19.5</v>
+      </c>
+      <c r="E1605" s="2">
+        <v>72.0</v>
+      </c>
+      <c r="F1605" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1605" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1606">
+      <c r="A1606" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1606" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:30</t>
+        </is>
+      </c>
+      <c r="C1606" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1606" s="2">
+        <v>19.2</v>
+      </c>
+      <c r="E1606" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="F1606" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1606" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1607">
+      <c r="A1607" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1607" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:40</t>
+        </is>
+      </c>
+      <c r="C1607" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1607" s="2">
+        <v>18.9</v>
+      </c>
+      <c r="E1607" s="2">
+        <v>74.0</v>
+      </c>
+      <c r="F1607" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1607" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1608">
+      <c r="A1608" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1608" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:50</t>
+        </is>
+      </c>
+      <c r="C1608" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1608" s="2">
+        <v>18.5</v>
+      </c>
+      <c r="E1608" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F1608" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1608" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1609">
+      <c r="A1609" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1609" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:00</t>
+        </is>
+      </c>
+      <c r="C1609" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1609" s="2">
+        <v>18.3</v>
+      </c>
+      <c r="E1609" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F1609" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1609" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1610">
+      <c r="A1610" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1610" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:10</t>
+        </is>
+      </c>
+      <c r="C1610" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1610" s="2">
+        <v>18.1</v>
+      </c>
+      <c r="E1610" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F1610" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1610" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1611">
+      <c r="A1611" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1611" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:20</t>
+        </is>
+      </c>
+      <c r="C1611" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1611" s="2">
+        <v>17.9</v>
+      </c>
+      <c r="E1611" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F1611" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1611" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1612">
+      <c r="A1612" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1612" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:30</t>
+        </is>
+      </c>
+      <c r="C1612" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1612" s="2">
+        <v>17.6</v>
+      </c>
+      <c r="E1612" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F1612" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1612" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1613">
+      <c r="A1613" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1613" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:40</t>
+        </is>
+      </c>
+      <c r="C1613" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1613" s="2">
+        <v>17.4</v>
+      </c>
+      <c r="E1613" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F1613" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1613" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1614">
+      <c r="A1614" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">25.07.2026</t>
+        </is>
+      </c>
+      <c r="B1614" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:50</t>
+        </is>
+      </c>
+      <c r="C1614" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1614" s="2">
+        <v>17.3</v>
+      </c>
+      <c r="E1614" s="2">
+        <v>81.0</v>
+      </c>
+      <c r="F1614" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1614" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1615">
+      <c r="A1615" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1615" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:00</t>
+        </is>
+      </c>
+      <c r="C1615" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1615" s="2">
+        <v>17.2</v>
+      </c>
+      <c r="E1615" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F1615" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1615" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1616">
+      <c r="A1616" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1616" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:10</t>
+        </is>
+      </c>
+      <c r="C1616" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1616" s="2">
+        <v>17.1</v>
+      </c>
+      <c r="E1616" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F1616" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1616" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1617">
+      <c r="A1617" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1617" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:20</t>
+        </is>
+      </c>
+      <c r="C1617" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1617" s="2">
+        <v>16.9</v>
+      </c>
+      <c r="E1617" s="2">
+        <v>83.0</v>
+      </c>
+      <c r="F1617" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1617" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G1474"/>
+  <autoFilter ref="A1:G1617"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ARSO Kranj zajem 2026-07-27 00:44 Europe/Ljubljana
</commit_message>
<xml_diff>
--- a/tabela_vremena/ARSO_Kranj.xlsx
+++ b/tabela_vremena/ARSO_Kranj.xlsx
@@ -46975,7 +46975,4212 @@
         <v>0.0</v>
       </c>
     </row>
+    <row r="1618">
+      <c r="A1618" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1618" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:30</t>
+        </is>
+      </c>
+      <c r="C1618" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1618" s="2">
+        <v>16.8</v>
+      </c>
+      <c r="E1618" s="2">
+        <v>83.0</v>
+      </c>
+      <c r="F1618" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1618" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1619">
+      <c r="A1619" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1619" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:40</t>
+        </is>
+      </c>
+      <c r="C1619" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1619" s="2">
+        <v>16.7</v>
+      </c>
+      <c r="E1619" s="2">
+        <v>83.0</v>
+      </c>
+      <c r="F1619" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1619" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1620">
+      <c r="A1620" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1620" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:50</t>
+        </is>
+      </c>
+      <c r="C1620" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1620" s="2">
+        <v>16.7</v>
+      </c>
+      <c r="E1620" s="2">
+        <v>83.0</v>
+      </c>
+      <c r="F1620" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1620" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1621">
+      <c r="A1621" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1621" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:00</t>
+        </is>
+      </c>
+      <c r="C1621" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1621" s="2">
+        <v>16.7</v>
+      </c>
+      <c r="E1621" s="2">
+        <v>84.0</v>
+      </c>
+      <c r="F1621" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1621" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1622">
+      <c r="A1622" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1622" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:10</t>
+        </is>
+      </c>
+      <c r="C1622" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1622" s="2">
+        <v>16.7</v>
+      </c>
+      <c r="E1622" s="2">
+        <v>83.0</v>
+      </c>
+      <c r="F1622" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1622" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1623">
+      <c r="A1623" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1623" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:20</t>
+        </is>
+      </c>
+      <c r="C1623" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1623" s="2">
+        <v>16.7</v>
+      </c>
+      <c r="E1623" s="2">
+        <v>83.0</v>
+      </c>
+      <c r="F1623" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1623" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1624">
+      <c r="A1624" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1624" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:30</t>
+        </is>
+      </c>
+      <c r="C1624" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1624" s="2">
+        <v>16.4</v>
+      </c>
+      <c r="E1624" s="2">
+        <v>84.0</v>
+      </c>
+      <c r="F1624" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1624" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1625">
+      <c r="A1625" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1625" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:40</t>
+        </is>
+      </c>
+      <c r="C1625" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1625" s="2">
+        <v>16.1</v>
+      </c>
+      <c r="E1625" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F1625" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1625" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1626">
+      <c r="A1626" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1626" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:50</t>
+        </is>
+      </c>
+      <c r="C1626" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1626" s="2">
+        <v>16.0</v>
+      </c>
+      <c r="E1626" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F1626" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1626" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1627">
+      <c r="A1627" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1627" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:00</t>
+        </is>
+      </c>
+      <c r="C1627" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1627" s="2">
+        <v>15.9</v>
+      </c>
+      <c r="E1627" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F1627" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1627" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1628">
+      <c r="A1628" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1628" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:10</t>
+        </is>
+      </c>
+      <c r="C1628" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1628" s="2">
+        <v>15.8</v>
+      </c>
+      <c r="E1628" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F1628" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1628" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1629">
+      <c r="A1629" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1629" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:20</t>
+        </is>
+      </c>
+      <c r="C1629" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1629" s="2">
+        <v>15.9</v>
+      </c>
+      <c r="E1629" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F1629" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1629" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1630">
+      <c r="A1630" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1630" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:30</t>
+        </is>
+      </c>
+      <c r="C1630" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1630" s="2">
+        <v>15.8</v>
+      </c>
+      <c r="E1630" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F1630" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1630" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1631">
+      <c r="A1631" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1631" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:40</t>
+        </is>
+      </c>
+      <c r="C1631" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1631" s="2">
+        <v>15.7</v>
+      </c>
+      <c r="E1631" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F1631" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1631" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1632">
+      <c r="A1632" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1632" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:50</t>
+        </is>
+      </c>
+      <c r="C1632" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1632" s="2">
+        <v>15.6</v>
+      </c>
+      <c r="E1632" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F1632" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1632" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1633">
+      <c r="A1633" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1633" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:00</t>
+        </is>
+      </c>
+      <c r="C1633" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1633" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="E1633" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F1633" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1633" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1634">
+      <c r="A1634" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1634" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:10</t>
+        </is>
+      </c>
+      <c r="C1634" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1634" s="2">
+        <v>15.6</v>
+      </c>
+      <c r="E1634" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F1634" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1634" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1635">
+      <c r="A1635" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1635" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:20</t>
+        </is>
+      </c>
+      <c r="C1635" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1635" s="2">
+        <v>15.6</v>
+      </c>
+      <c r="E1635" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F1635" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1635" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1636">
+      <c r="A1636" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1636" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:30</t>
+        </is>
+      </c>
+      <c r="C1636" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1636" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="E1636" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F1636" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1636" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1637">
+      <c r="A1637" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1637" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:40</t>
+        </is>
+      </c>
+      <c r="C1637" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1637" s="2">
+        <v>15.4</v>
+      </c>
+      <c r="E1637" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F1637" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1637" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1638">
+      <c r="A1638" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1638" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:50</t>
+        </is>
+      </c>
+      <c r="C1638" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1638" s="2">
+        <v>15.3</v>
+      </c>
+      <c r="E1638" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F1638" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1638" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1639">
+      <c r="A1639" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1639" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:00</t>
+        </is>
+      </c>
+      <c r="C1639" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1639" s="2">
+        <v>15.4</v>
+      </c>
+      <c r="E1639" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F1639" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1639" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1640">
+      <c r="A1640" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1640" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:10</t>
+        </is>
+      </c>
+      <c r="C1640" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1640" s="2">
+        <v>15.4</v>
+      </c>
+      <c r="E1640" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F1640" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1640" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1641">
+      <c r="A1641" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1641" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:20</t>
+        </is>
+      </c>
+      <c r="C1641" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1641" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="E1641" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F1641" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1641" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1642">
+      <c r="A1642" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1642" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:30</t>
+        </is>
+      </c>
+      <c r="C1642" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1642" s="2">
+        <v>15.4</v>
+      </c>
+      <c r="E1642" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F1642" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1642" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1643">
+      <c r="A1643" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1643" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:40</t>
+        </is>
+      </c>
+      <c r="C1643" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1643" s="2">
+        <v>15.4</v>
+      </c>
+      <c r="E1643" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F1643" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1643" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1644">
+      <c r="A1644" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1644" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:50</t>
+        </is>
+      </c>
+      <c r="C1644" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1644" s="2">
+        <v>15.4</v>
+      </c>
+      <c r="E1644" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F1644" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1644" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1645">
+      <c r="A1645" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1645" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:00</t>
+        </is>
+      </c>
+      <c r="C1645" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1645" s="2">
+        <v>15.4</v>
+      </c>
+      <c r="E1645" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F1645" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1645" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1646">
+      <c r="A1646" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1646" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:10</t>
+        </is>
+      </c>
+      <c r="C1646" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1646" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="E1646" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F1646" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1646" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1647">
+      <c r="A1647" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1647" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:20</t>
+        </is>
+      </c>
+      <c r="C1647" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1647" s="2">
+        <v>15.6</v>
+      </c>
+      <c r="E1647" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F1647" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1647" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1648">
+      <c r="A1648" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1648" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:30</t>
+        </is>
+      </c>
+      <c r="C1648" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1648" s="2">
+        <v>15.6</v>
+      </c>
+      <c r="E1648" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F1648" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1648" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1649">
+      <c r="A1649" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1649" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:40</t>
+        </is>
+      </c>
+      <c r="C1649" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1649" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="E1649" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F1649" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1649" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1650">
+      <c r="A1650" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1650" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:50</t>
+        </is>
+      </c>
+      <c r="C1650" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1650" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="E1650" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F1650" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1650" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1651">
+      <c r="A1651" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1651" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:00</t>
+        </is>
+      </c>
+      <c r="C1651" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1651" s="2">
+        <v>15.9</v>
+      </c>
+      <c r="E1651" s="2">
+        <v>84.0</v>
+      </c>
+      <c r="F1651" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1651" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1652">
+      <c r="A1652" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1652" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:10</t>
+        </is>
+      </c>
+      <c r="C1652" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1652" s="2">
+        <v>16.1</v>
+      </c>
+      <c r="E1652" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F1652" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1652" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1653">
+      <c r="A1653" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1653" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:20</t>
+        </is>
+      </c>
+      <c r="C1653" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1653" s="2">
+        <v>16.3</v>
+      </c>
+      <c r="E1653" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F1653" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1653" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1654">
+      <c r="A1654" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1654" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:30</t>
+        </is>
+      </c>
+      <c r="C1654" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1654" s="2">
+        <v>16.5</v>
+      </c>
+      <c r="E1654" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F1654" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1654" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1655">
+      <c r="A1655" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1655" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:40</t>
+        </is>
+      </c>
+      <c r="C1655" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1655" s="2">
+        <v>16.7</v>
+      </c>
+      <c r="E1655" s="2">
+        <v>81.0</v>
+      </c>
+      <c r="F1655" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1655" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1656">
+      <c r="A1656" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1656" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:50</t>
+        </is>
+      </c>
+      <c r="C1656" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1656" s="2">
+        <v>16.8</v>
+      </c>
+      <c r="E1656" s="2">
+        <v>81.0</v>
+      </c>
+      <c r="F1656" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1656" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1657">
+      <c r="A1657" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1657" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:00</t>
+        </is>
+      </c>
+      <c r="C1657" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1657" s="2">
+        <v>16.6</v>
+      </c>
+      <c r="E1657" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F1657" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1657" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1658">
+      <c r="A1658" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1658" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:10</t>
+        </is>
+      </c>
+      <c r="C1658" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1658" s="2">
+        <v>16.6</v>
+      </c>
+      <c r="E1658" s="2">
+        <v>83.0</v>
+      </c>
+      <c r="F1658" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1658" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1659">
+      <c r="A1659" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1659" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:20</t>
+        </is>
+      </c>
+      <c r="C1659" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1659" s="2">
+        <v>16.7</v>
+      </c>
+      <c r="E1659" s="2">
+        <v>83.0</v>
+      </c>
+      <c r="F1659" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1659" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1660">
+      <c r="A1660" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1660" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:30</t>
+        </is>
+      </c>
+      <c r="C1660" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1660" s="2">
+        <v>16.9</v>
+      </c>
+      <c r="E1660" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F1660" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1660" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1661">
+      <c r="A1661" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1661" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:40</t>
+        </is>
+      </c>
+      <c r="C1661" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1661" s="2">
+        <v>17.1</v>
+      </c>
+      <c r="E1661" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F1661" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1661" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1662">
+      <c r="A1662" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1662" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:50</t>
+        </is>
+      </c>
+      <c r="C1662" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1662" s="2">
+        <v>17.2</v>
+      </c>
+      <c r="E1662" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F1662" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1662" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1663">
+      <c r="A1663" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1663" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:00</t>
+        </is>
+      </c>
+      <c r="C1663" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1663" s="2">
+        <v>17.4</v>
+      </c>
+      <c r="E1663" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F1663" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1663" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1664">
+      <c r="A1664" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1664" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:10</t>
+        </is>
+      </c>
+      <c r="C1664" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1664" s="2">
+        <v>17.5</v>
+      </c>
+      <c r="E1664" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F1664" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1664" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1665">
+      <c r="A1665" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1665" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:20</t>
+        </is>
+      </c>
+      <c r="C1665" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1665" s="2">
+        <v>17.8</v>
+      </c>
+      <c r="E1665" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F1665" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1665" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1666">
+      <c r="A1666" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1666" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:30</t>
+        </is>
+      </c>
+      <c r="C1666" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1666" s="2">
+        <v>18.5</v>
+      </c>
+      <c r="E1666" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F1666" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1666" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1667">
+      <c r="A1667" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1667" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:40</t>
+        </is>
+      </c>
+      <c r="C1667" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1667" s="2">
+        <v>18.9</v>
+      </c>
+      <c r="E1667" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="F1667" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1667" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1668">
+      <c r="A1668" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1668" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:50</t>
+        </is>
+      </c>
+      <c r="C1668" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1668" s="2">
+        <v>19.5</v>
+      </c>
+      <c r="E1668" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F1668" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1668" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1669">
+      <c r="A1669" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1669" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:00</t>
+        </is>
+      </c>
+      <c r="C1669" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1669" s="2">
+        <v>19.7</v>
+      </c>
+      <c r="E1669" s="2">
+        <v>69.0</v>
+      </c>
+      <c r="F1669" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1669" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1670">
+      <c r="A1670" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1670" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:10</t>
+        </is>
+      </c>
+      <c r="C1670" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1670" s="2">
+        <v>20.2</v>
+      </c>
+      <c r="E1670" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F1670" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1670" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1671">
+      <c r="A1671" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1671" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:20</t>
+        </is>
+      </c>
+      <c r="C1671" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1671" s="2">
+        <v>21.2</v>
+      </c>
+      <c r="E1671" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F1671" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1671" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1672">
+      <c r="A1672" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1672" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:30</t>
+        </is>
+      </c>
+      <c r="C1672" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1672" s="2">
+        <v>21.4</v>
+      </c>
+      <c r="E1672" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F1672" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1672" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1673">
+      <c r="A1673" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1673" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:40</t>
+        </is>
+      </c>
+      <c r="C1673" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1673" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="E1673" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F1673" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1673" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1674">
+      <c r="A1674" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1674" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:50</t>
+        </is>
+      </c>
+      <c r="C1674" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1674" s="2">
+        <v>22.3</v>
+      </c>
+      <c r="E1674" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F1674" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1674" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1675">
+      <c r="A1675" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1675" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:00</t>
+        </is>
+      </c>
+      <c r="C1675" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1675" s="2">
+        <v>22.8</v>
+      </c>
+      <c r="E1675" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F1675" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1675" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1676">
+      <c r="A1676" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1676" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:10</t>
+        </is>
+      </c>
+      <c r="C1676" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1676" s="2">
+        <v>23.3</v>
+      </c>
+      <c r="E1676" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F1676" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1676" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1677">
+      <c r="A1677" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1677" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:20</t>
+        </is>
+      </c>
+      <c r="C1677" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1677" s="2">
+        <v>23.6</v>
+      </c>
+      <c r="E1677" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F1677" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1677" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1678">
+      <c r="A1678" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1678" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:30</t>
+        </is>
+      </c>
+      <c r="C1678" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1678" s="2">
+        <v>24.3</v>
+      </c>
+      <c r="E1678" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F1678" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1678" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1679">
+      <c r="A1679" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1679" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:40</t>
+        </is>
+      </c>
+      <c r="C1679" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1679" s="2">
+        <v>24.9</v>
+      </c>
+      <c r="E1679" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F1679" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1679" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1680">
+      <c r="A1680" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1680" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:50</t>
+        </is>
+      </c>
+      <c r="C1680" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1680" s="2">
+        <v>24.5</v>
+      </c>
+      <c r="E1680" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F1680" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1680" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1681">
+      <c r="A1681" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1681" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:00</t>
+        </is>
+      </c>
+      <c r="C1681" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1681" s="2">
+        <v>24.5</v>
+      </c>
+      <c r="E1681" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F1681" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1681" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1682">
+      <c r="A1682" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1682" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:10</t>
+        </is>
+      </c>
+      <c r="C1682" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1682" s="2">
+        <v>24.3</v>
+      </c>
+      <c r="E1682" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F1682" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1682" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1683">
+      <c r="A1683" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1683" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:20</t>
+        </is>
+      </c>
+      <c r="C1683" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1683" s="2">
+        <v>24.5</v>
+      </c>
+      <c r="E1683" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F1683" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1683" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1684">
+      <c r="A1684" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1684" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:30</t>
+        </is>
+      </c>
+      <c r="C1684" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1684" s="2">
+        <v>24.7</v>
+      </c>
+      <c r="E1684" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F1684" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1684" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1685">
+      <c r="A1685" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1685" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:40</t>
+        </is>
+      </c>
+      <c r="C1685" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1685" s="2">
+        <v>24.7</v>
+      </c>
+      <c r="E1685" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F1685" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1685" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1686">
+      <c r="A1686" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1686" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:50</t>
+        </is>
+      </c>
+      <c r="C1686" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1686" s="2">
+        <v>25.1</v>
+      </c>
+      <c r="E1686" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F1686" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1686" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1687">
+      <c r="A1687" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1687" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:00</t>
+        </is>
+      </c>
+      <c r="C1687" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1687" s="2">
+        <v>25.2</v>
+      </c>
+      <c r="E1687" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F1687" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1687" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1688">
+      <c r="A1688" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1688" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:10</t>
+        </is>
+      </c>
+      <c r="C1688" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1688" s="2">
+        <v>25.4</v>
+      </c>
+      <c r="E1688" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F1688" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1688" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1689">
+      <c r="A1689" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1689" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:20</t>
+        </is>
+      </c>
+      <c r="C1689" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1689" s="2">
+        <v>25.5</v>
+      </c>
+      <c r="E1689" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F1689" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1689" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1690">
+      <c r="A1690" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1690" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:30</t>
+        </is>
+      </c>
+      <c r="C1690" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1690" s="2">
+        <v>25.6</v>
+      </c>
+      <c r="E1690" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F1690" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1690" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1691">
+      <c r="A1691" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1691" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:40</t>
+        </is>
+      </c>
+      <c r="C1691" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1691" s="2">
+        <v>25.8</v>
+      </c>
+      <c r="E1691" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F1691" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1691" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1692">
+      <c r="A1692" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1692" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:50</t>
+        </is>
+      </c>
+      <c r="C1692" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1692" s="2">
+        <v>25.4</v>
+      </c>
+      <c r="E1692" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F1692" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1692" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1693">
+      <c r="A1693" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1693" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:00</t>
+        </is>
+      </c>
+      <c r="C1693" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1693" s="2">
+        <v>25.2</v>
+      </c>
+      <c r="E1693" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F1693" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1693" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1694">
+      <c r="A1694" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1694" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:10</t>
+        </is>
+      </c>
+      <c r="C1694" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1694" s="2">
+        <v>25.3</v>
+      </c>
+      <c r="E1694" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F1694" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1694" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1695">
+      <c r="A1695" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1695" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:20</t>
+        </is>
+      </c>
+      <c r="C1695" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1695" s="2">
+        <v>25.3</v>
+      </c>
+      <c r="E1695" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F1695" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1695" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1696">
+      <c r="A1696" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1696" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:30</t>
+        </is>
+      </c>
+      <c r="C1696" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1696" s="2">
+        <v>25.3</v>
+      </c>
+      <c r="E1696" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F1696" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1696" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1697">
+      <c r="A1697" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1697" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:40</t>
+        </is>
+      </c>
+      <c r="C1697" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1697" s="2">
+        <v>25.5</v>
+      </c>
+      <c r="E1697" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F1697" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1697" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1698">
+      <c r="A1698" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1698" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:50</t>
+        </is>
+      </c>
+      <c r="C1698" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1698" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="E1698" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F1698" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1698" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1699">
+      <c r="A1699" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1699" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:00</t>
+        </is>
+      </c>
+      <c r="C1699" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1699" s="2">
+        <v>26.5</v>
+      </c>
+      <c r="E1699" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F1699" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1699" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1700">
+      <c r="A1700" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1700" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:10</t>
+        </is>
+      </c>
+      <c r="C1700" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1700" s="2">
+        <v>26.4</v>
+      </c>
+      <c r="E1700" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F1700" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1700" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1701">
+      <c r="A1701" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1701" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:20</t>
+        </is>
+      </c>
+      <c r="C1701" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1701" s="2">
+        <v>26.1</v>
+      </c>
+      <c r="E1701" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F1701" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1701" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1702">
+      <c r="A1702" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1702" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:30</t>
+        </is>
+      </c>
+      <c r="C1702" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1702" s="2">
+        <v>26.3</v>
+      </c>
+      <c r="E1702" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F1702" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1702" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1703">
+      <c r="A1703" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1703" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:40</t>
+        </is>
+      </c>
+      <c r="C1703" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1703" s="2">
+        <v>26.1</v>
+      </c>
+      <c r="E1703" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F1703" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1703" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1704">
+      <c r="A1704" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1704" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:50</t>
+        </is>
+      </c>
+      <c r="C1704" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1704" s="2">
+        <v>26.9</v>
+      </c>
+      <c r="E1704" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F1704" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1704" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1705">
+      <c r="A1705" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1705" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:00</t>
+        </is>
+      </c>
+      <c r="C1705" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1705" s="2">
+        <v>26.7</v>
+      </c>
+      <c r="E1705" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F1705" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1705" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1706">
+      <c r="A1706" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1706" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:10</t>
+        </is>
+      </c>
+      <c r="C1706" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1706" s="2">
+        <v>27.5</v>
+      </c>
+      <c r="E1706" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F1706" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1706" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1707">
+      <c r="A1707" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1707" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:20</t>
+        </is>
+      </c>
+      <c r="C1707" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1707" s="2">
+        <v>26.8</v>
+      </c>
+      <c r="E1707" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F1707" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1707" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1708">
+      <c r="A1708" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1708" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:30</t>
+        </is>
+      </c>
+      <c r="C1708" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1708" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="E1708" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F1708" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1708" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1709">
+      <c r="A1709" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1709" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:40</t>
+        </is>
+      </c>
+      <c r="C1709" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1709" s="2">
+        <v>27.2</v>
+      </c>
+      <c r="E1709" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F1709" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1709" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1710">
+      <c r="A1710" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1710" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:50</t>
+        </is>
+      </c>
+      <c r="C1710" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1710" s="2">
+        <v>26.6</v>
+      </c>
+      <c r="E1710" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F1710" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1710" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1711">
+      <c r="A1711" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1711" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:00</t>
+        </is>
+      </c>
+      <c r="C1711" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1711" s="2">
+        <v>26.3</v>
+      </c>
+      <c r="E1711" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F1711" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1711" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1712">
+      <c r="A1712" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1712" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:10</t>
+        </is>
+      </c>
+      <c r="C1712" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1712" s="2">
+        <v>26.6</v>
+      </c>
+      <c r="E1712" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F1712" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1712" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1713">
+      <c r="A1713" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1713" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:20</t>
+        </is>
+      </c>
+      <c r="C1713" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1713" s="2">
+        <v>26.4</v>
+      </c>
+      <c r="E1713" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F1713" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1713" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1714">
+      <c r="A1714" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1714" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:30</t>
+        </is>
+      </c>
+      <c r="C1714" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1714" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="E1714" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F1714" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1714" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1715">
+      <c r="A1715" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1715" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:40</t>
+        </is>
+      </c>
+      <c r="C1715" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1715" s="2">
+        <v>25.5</v>
+      </c>
+      <c r="E1715" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F1715" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1715" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1716">
+      <c r="A1716" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1716" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:50</t>
+        </is>
+      </c>
+      <c r="C1716" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1716" s="2">
+        <v>25.3</v>
+      </c>
+      <c r="E1716" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F1716" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1716" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1717">
+      <c r="A1717" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1717" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:00</t>
+        </is>
+      </c>
+      <c r="C1717" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1717" s="2">
+        <v>25.3</v>
+      </c>
+      <c r="E1717" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F1717" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1717" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1718">
+      <c r="A1718" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1718" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:10</t>
+        </is>
+      </c>
+      <c r="C1718" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1718" s="2">
+        <v>25.3</v>
+      </c>
+      <c r="E1718" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F1718" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1718" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1719">
+      <c r="A1719" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1719" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:20</t>
+        </is>
+      </c>
+      <c r="C1719" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1719" s="2">
+        <v>25.2</v>
+      </c>
+      <c r="E1719" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F1719" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1719" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1720">
+      <c r="A1720" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1720" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:30</t>
+        </is>
+      </c>
+      <c r="C1720" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1720" s="2">
+        <v>25.2</v>
+      </c>
+      <c r="E1720" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F1720" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1720" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1721">
+      <c r="A1721" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1721" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:40</t>
+        </is>
+      </c>
+      <c r="C1721" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1721" s="2">
+        <v>24.8</v>
+      </c>
+      <c r="E1721" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F1721" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1721" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1722">
+      <c r="A1722" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1722" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:50</t>
+        </is>
+      </c>
+      <c r="C1722" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1722" s="2">
+        <v>24.5</v>
+      </c>
+      <c r="E1722" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F1722" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1722" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1723">
+      <c r="A1723" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1723" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:00</t>
+        </is>
+      </c>
+      <c r="C1723" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1723" s="2">
+        <v>24.4</v>
+      </c>
+      <c r="E1723" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F1723" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1723" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1724">
+      <c r="A1724" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1724" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:10</t>
+        </is>
+      </c>
+      <c r="C1724" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1724" s="2">
+        <v>24.4</v>
+      </c>
+      <c r="E1724" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F1724" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1724" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1725">
+      <c r="A1725" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1725" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:20</t>
+        </is>
+      </c>
+      <c r="C1725" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1725" s="2">
+        <v>24.2</v>
+      </c>
+      <c r="E1725" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F1725" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1725" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1726">
+      <c r="A1726" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1726" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:30</t>
+        </is>
+      </c>
+      <c r="C1726" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1726" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="E1726" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F1726" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1726" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1727">
+      <c r="A1727" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1727" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:40</t>
+        </is>
+      </c>
+      <c r="C1727" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1727" s="2">
+        <v>23.9</v>
+      </c>
+      <c r="E1727" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F1727" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1727" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1728">
+      <c r="A1728" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1728" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:50</t>
+        </is>
+      </c>
+      <c r="C1728" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1728" s="2">
+        <v>23.6</v>
+      </c>
+      <c r="E1728" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F1728" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1728" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1729">
+      <c r="A1729" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1729" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:00</t>
+        </is>
+      </c>
+      <c r="C1729" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1729" s="2">
+        <v>23.4</v>
+      </c>
+      <c r="E1729" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F1729" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1729" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1730">
+      <c r="A1730" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1730" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:10</t>
+        </is>
+      </c>
+      <c r="C1730" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1730" s="2">
+        <v>23.2</v>
+      </c>
+      <c r="E1730" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F1730" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1730" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1731">
+      <c r="A1731" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1731" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:20</t>
+        </is>
+      </c>
+      <c r="C1731" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1731" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="E1731" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F1731" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1731" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1732">
+      <c r="A1732" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1732" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:30</t>
+        </is>
+      </c>
+      <c r="C1732" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1732" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="E1732" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F1732" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1732" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1733">
+      <c r="A1733" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1733" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:40</t>
+        </is>
+      </c>
+      <c r="C1733" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1733" s="2">
+        <v>22.8</v>
+      </c>
+      <c r="E1733" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F1733" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1733" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1734">
+      <c r="A1734" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1734" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:50</t>
+        </is>
+      </c>
+      <c r="C1734" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1734" s="2">
+        <v>22.6</v>
+      </c>
+      <c r="E1734" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F1734" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1734" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1735">
+      <c r="A1735" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1735" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:00</t>
+        </is>
+      </c>
+      <c r="C1735" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1735" s="2">
+        <v>22.4</v>
+      </c>
+      <c r="E1735" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F1735" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1735" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1736">
+      <c r="A1736" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1736" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:10</t>
+        </is>
+      </c>
+      <c r="C1736" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1736" s="2">
+        <v>22.2</v>
+      </c>
+      <c r="E1736" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F1736" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1736" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1737">
+      <c r="A1737" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1737" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:20</t>
+        </is>
+      </c>
+      <c r="C1737" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1737" s="2">
+        <v>22.1</v>
+      </c>
+      <c r="E1737" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F1737" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1737" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1738">
+      <c r="A1738" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1738" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:30</t>
+        </is>
+      </c>
+      <c r="C1738" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1738" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="E1738" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F1738" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1738" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1739">
+      <c r="A1739" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1739" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:40</t>
+        </is>
+      </c>
+      <c r="C1739" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1739" s="2">
+        <v>21.8</v>
+      </c>
+      <c r="E1739" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F1739" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1739" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1740">
+      <c r="A1740" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1740" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:50</t>
+        </is>
+      </c>
+      <c r="C1740" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1740" s="2">
+        <v>21.6</v>
+      </c>
+      <c r="E1740" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F1740" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1740" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1741">
+      <c r="A1741" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1741" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:00</t>
+        </is>
+      </c>
+      <c r="C1741" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1741" s="2">
+        <v>21.4</v>
+      </c>
+      <c r="E1741" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F1741" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1741" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1742">
+      <c r="A1742" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1742" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:10</t>
+        </is>
+      </c>
+      <c r="C1742" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1742" s="2">
+        <v>21.1</v>
+      </c>
+      <c r="E1742" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F1742" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1742" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1743">
+      <c r="A1743" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1743" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:20</t>
+        </is>
+      </c>
+      <c r="C1743" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1743" s="2">
+        <v>20.8</v>
+      </c>
+      <c r="E1743" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F1743" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1743" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1744">
+      <c r="A1744" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1744" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:30</t>
+        </is>
+      </c>
+      <c r="C1744" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1744" s="2">
+        <v>20.6</v>
+      </c>
+      <c r="E1744" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F1744" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1744" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1745">
+      <c r="A1745" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1745" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:40</t>
+        </is>
+      </c>
+      <c r="C1745" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1745" s="2">
+        <v>20.1</v>
+      </c>
+      <c r="E1745" s="2">
+        <v>74.0</v>
+      </c>
+      <c r="F1745" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1745" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1746">
+      <c r="A1746" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1746" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:50</t>
+        </is>
+      </c>
+      <c r="C1746" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1746" s="2">
+        <v>19.9</v>
+      </c>
+      <c r="E1746" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F1746" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1746" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1747">
+      <c r="A1747" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1747" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:00</t>
+        </is>
+      </c>
+      <c r="C1747" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1747" s="2">
+        <v>19.6</v>
+      </c>
+      <c r="E1747" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F1747" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1747" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1748">
+      <c r="A1748" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1748" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:10</t>
+        </is>
+      </c>
+      <c r="C1748" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1748" s="2">
+        <v>19.3</v>
+      </c>
+      <c r="E1748" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F1748" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1748" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1749">
+      <c r="A1749" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1749" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:20</t>
+        </is>
+      </c>
+      <c r="C1749" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1749" s="2">
+        <v>19.2</v>
+      </c>
+      <c r="E1749" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F1749" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1749" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1750">
+      <c r="A1750" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1750" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:30</t>
+        </is>
+      </c>
+      <c r="C1750" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1750" s="2">
+        <v>19.1</v>
+      </c>
+      <c r="E1750" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F1750" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1750" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1751">
+      <c r="A1751" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1751" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:40</t>
+        </is>
+      </c>
+      <c r="C1751" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1751" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="E1751" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F1751" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1751" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1752">
+      <c r="A1752" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1752" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:50</t>
+        </is>
+      </c>
+      <c r="C1752" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1752" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="E1752" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F1752" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1752" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1753">
+      <c r="A1753" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1753" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:00</t>
+        </is>
+      </c>
+      <c r="C1753" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1753" s="2">
+        <v>18.9</v>
+      </c>
+      <c r="E1753" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F1753" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1753" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1754">
+      <c r="A1754" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1754" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:10</t>
+        </is>
+      </c>
+      <c r="C1754" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1754" s="2">
+        <v>18.9</v>
+      </c>
+      <c r="E1754" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F1754" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1754" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1755">
+      <c r="A1755" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1755" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:20</t>
+        </is>
+      </c>
+      <c r="C1755" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1755" s="2">
+        <v>18.9</v>
+      </c>
+      <c r="E1755" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F1755" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1755" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1756">
+      <c r="A1756" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1756" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:30</t>
+        </is>
+      </c>
+      <c r="C1756" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1756" s="2">
+        <v>18.6</v>
+      </c>
+      <c r="E1756" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F1756" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1756" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1757">
+      <c r="A1757" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1757" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:40</t>
+        </is>
+      </c>
+      <c r="C1757" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1757" s="2">
+        <v>18.4</v>
+      </c>
+      <c r="E1757" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F1757" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1757" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1758">
+      <c r="A1758" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">26.07.2026</t>
+        </is>
+      </c>
+      <c r="B1758" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:50</t>
+        </is>
+      </c>
+      <c r="C1758" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1758" s="2">
+        <v>18.1</v>
+      </c>
+      <c r="E1758" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F1758" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1758" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1759">
+      <c r="A1759" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1759" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:00</t>
+        </is>
+      </c>
+      <c r="C1759" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1759" s="2">
+        <v>17.9</v>
+      </c>
+      <c r="E1759" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F1759" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1759" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1760">
+      <c r="A1760" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1760" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:10</t>
+        </is>
+      </c>
+      <c r="C1760" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1760" s="2">
+        <v>17.6</v>
+      </c>
+      <c r="E1760" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F1760" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1760" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1761">
+      <c r="A1761" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1761" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:20</t>
+        </is>
+      </c>
+      <c r="C1761" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1761" s="2">
+        <v>17.5</v>
+      </c>
+      <c r="E1761" s="2">
+        <v>81.0</v>
+      </c>
+      <c r="F1761" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1761" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1762">
+      <c r="A1762" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1762" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:30</t>
+        </is>
+      </c>
+      <c r="C1762" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1762" s="2">
+        <v>17.5</v>
+      </c>
+      <c r="E1762" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F1762" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1762" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G1617"/>
+  <autoFilter ref="A1:G1762"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ARSO Kranj zajem 2026-07-28 00:45 Europe/Ljubljana
</commit_message>
<xml_diff>
--- a/tabela_vremena/ARSO_Kranj.xlsx
+++ b/tabela_vremena/ARSO_Kranj.xlsx
@@ -51180,7 +51180,4183 @@
         <v>0.0</v>
       </c>
     </row>
+    <row r="1763">
+      <c r="A1763" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1763" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:40</t>
+        </is>
+      </c>
+      <c r="C1763" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1763" s="2">
+        <v>17.4</v>
+      </c>
+      <c r="E1763" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F1763" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1763" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1764">
+      <c r="A1764" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1764" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:50</t>
+        </is>
+      </c>
+      <c r="C1764" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1764" s="2">
+        <v>17.3</v>
+      </c>
+      <c r="E1764" s="2">
+        <v>81.0</v>
+      </c>
+      <c r="F1764" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1764" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1765">
+      <c r="A1765" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1765" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:00</t>
+        </is>
+      </c>
+      <c r="C1765" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1765" s="2">
+        <v>17.2</v>
+      </c>
+      <c r="E1765" s="2">
+        <v>81.0</v>
+      </c>
+      <c r="F1765" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1765" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1766">
+      <c r="A1766" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1766" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:10</t>
+        </is>
+      </c>
+      <c r="C1766" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1766" s="2">
+        <v>17.1</v>
+      </c>
+      <c r="E1766" s="2">
+        <v>81.0</v>
+      </c>
+      <c r="F1766" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1766" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1767">
+      <c r="A1767" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1767" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:20</t>
+        </is>
+      </c>
+      <c r="C1767" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1767" s="2">
+        <v>17.2</v>
+      </c>
+      <c r="E1767" s="2">
+        <v>81.0</v>
+      </c>
+      <c r="F1767" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1767" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1768">
+      <c r="A1768" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1768" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:30</t>
+        </is>
+      </c>
+      <c r="C1768" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1768" s="2">
+        <v>17.2</v>
+      </c>
+      <c r="E1768" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F1768" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1768" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1769">
+      <c r="A1769" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1769" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:40</t>
+        </is>
+      </c>
+      <c r="C1769" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1769" s="2">
+        <v>17.2</v>
+      </c>
+      <c r="E1769" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F1769" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1769" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1770">
+      <c r="A1770" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1770" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:50</t>
+        </is>
+      </c>
+      <c r="C1770" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1770" s="2">
+        <v>17.1</v>
+      </c>
+      <c r="E1770" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F1770" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1770" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1771">
+      <c r="A1771" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1771" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:00</t>
+        </is>
+      </c>
+      <c r="C1771" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1771" s="2">
+        <v>17.1</v>
+      </c>
+      <c r="E1771" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F1771" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1771" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1772">
+      <c r="A1772" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1772" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:10</t>
+        </is>
+      </c>
+      <c r="C1772" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1772" s="2">
+        <v>17.0</v>
+      </c>
+      <c r="E1772" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F1772" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1772" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1773">
+      <c r="A1773" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1773" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:20</t>
+        </is>
+      </c>
+      <c r="C1773" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1773" s="2">
+        <v>16.8</v>
+      </c>
+      <c r="E1773" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F1773" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1773" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1774">
+      <c r="A1774" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1774" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:30</t>
+        </is>
+      </c>
+      <c r="C1774" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1774" s="2">
+        <v>16.6</v>
+      </c>
+      <c r="E1774" s="2">
+        <v>81.0</v>
+      </c>
+      <c r="F1774" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1774" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1775">
+      <c r="A1775" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1775" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:40</t>
+        </is>
+      </c>
+      <c r="C1775" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1775" s="2">
+        <v>16.3</v>
+      </c>
+      <c r="E1775" s="2">
+        <v>83.0</v>
+      </c>
+      <c r="F1775" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1775" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1776">
+      <c r="A1776" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1776" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:50</t>
+        </is>
+      </c>
+      <c r="C1776" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1776" s="2">
+        <v>16.1</v>
+      </c>
+      <c r="E1776" s="2">
+        <v>84.0</v>
+      </c>
+      <c r="F1776" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1776" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1777">
+      <c r="A1777" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1777" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:00</t>
+        </is>
+      </c>
+      <c r="C1777" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1777" s="2">
+        <v>16.0</v>
+      </c>
+      <c r="E1777" s="2">
+        <v>84.0</v>
+      </c>
+      <c r="F1777" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1777" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1778">
+      <c r="A1778" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1778" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:10</t>
+        </is>
+      </c>
+      <c r="C1778" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1778" s="2">
+        <v>16.0</v>
+      </c>
+      <c r="E1778" s="2">
+        <v>84.0</v>
+      </c>
+      <c r="F1778" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1778" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1779">
+      <c r="A1779" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1779" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:20</t>
+        </is>
+      </c>
+      <c r="C1779" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1779" s="2">
+        <v>15.9</v>
+      </c>
+      <c r="E1779" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F1779" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1779" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1780">
+      <c r="A1780" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1780" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:30</t>
+        </is>
+      </c>
+      <c r="C1780" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1780" s="2">
+        <v>15.7</v>
+      </c>
+      <c r="E1780" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F1780" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1780" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1781">
+      <c r="A1781" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1781" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:40</t>
+        </is>
+      </c>
+      <c r="C1781" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1781" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="E1781" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F1781" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1781" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1782">
+      <c r="A1782" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1782" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:50</t>
+        </is>
+      </c>
+      <c r="C1782" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1782" s="2">
+        <v>15.3</v>
+      </c>
+      <c r="E1782" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F1782" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1782" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1783">
+      <c r="A1783" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1783" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:00</t>
+        </is>
+      </c>
+      <c r="C1783" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1783" s="2">
+        <v>15.1</v>
+      </c>
+      <c r="E1783" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F1783" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1783" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1784">
+      <c r="A1784" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1784" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:10</t>
+        </is>
+      </c>
+      <c r="C1784" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1784" s="2">
+        <v>14.9</v>
+      </c>
+      <c r="E1784" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F1784" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1784" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1785">
+      <c r="A1785" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1785" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:20</t>
+        </is>
+      </c>
+      <c r="C1785" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1785" s="2">
+        <v>14.8</v>
+      </c>
+      <c r="E1785" s="2">
+        <v>90.0</v>
+      </c>
+      <c r="F1785" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1785" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1786">
+      <c r="A1786" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1786" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:30</t>
+        </is>
+      </c>
+      <c r="C1786" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1786" s="2">
+        <v>14.8</v>
+      </c>
+      <c r="E1786" s="2">
+        <v>89.0</v>
+      </c>
+      <c r="F1786" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1786" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1787">
+      <c r="A1787" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1787" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:40</t>
+        </is>
+      </c>
+      <c r="C1787" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1787" s="2">
+        <v>14.6</v>
+      </c>
+      <c r="E1787" s="2">
+        <v>89.0</v>
+      </c>
+      <c r="F1787" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1787" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1788">
+      <c r="A1788" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1788" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:50</t>
+        </is>
+      </c>
+      <c r="C1788" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1788" s="2">
+        <v>14.7</v>
+      </c>
+      <c r="E1788" s="2">
+        <v>89.0</v>
+      </c>
+      <c r="F1788" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1788" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1789">
+      <c r="A1789" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1789" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:00</t>
+        </is>
+      </c>
+      <c r="C1789" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1789" s="2">
+        <v>14.8</v>
+      </c>
+      <c r="E1789" s="2">
+        <v>89.0</v>
+      </c>
+      <c r="F1789" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1789" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1790">
+      <c r="A1790" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1790" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:10</t>
+        </is>
+      </c>
+      <c r="C1790" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1790" s="2">
+        <v>15.1</v>
+      </c>
+      <c r="E1790" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F1790" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1790" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1791">
+      <c r="A1791" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1791" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:20</t>
+        </is>
+      </c>
+      <c r="C1791" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1791" s="2">
+        <v>15.4</v>
+      </c>
+      <c r="E1791" s="2">
+        <v>84.0</v>
+      </c>
+      <c r="F1791" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1791" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1792">
+      <c r="A1792" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1792" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:30</t>
+        </is>
+      </c>
+      <c r="C1792" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1792" s="2">
+        <v>15.2</v>
+      </c>
+      <c r="E1792" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F1792" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1792" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1793">
+      <c r="A1793" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1793" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:40</t>
+        </is>
+      </c>
+      <c r="C1793" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1793" s="2">
+        <v>14.9</v>
+      </c>
+      <c r="E1793" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F1793" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1793" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1794">
+      <c r="A1794" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1794" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:50</t>
+        </is>
+      </c>
+      <c r="C1794" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1794" s="2">
+        <v>14.8</v>
+      </c>
+      <c r="E1794" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F1794" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1794" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1795">
+      <c r="A1795" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1795" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:00</t>
+        </is>
+      </c>
+      <c r="C1795" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1795" s="2">
+        <v>14.6</v>
+      </c>
+      <c r="E1795" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F1795" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1795" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1796">
+      <c r="A1796" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1796" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:10</t>
+        </is>
+      </c>
+      <c r="C1796" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1796" s="2">
+        <v>14.4</v>
+      </c>
+      <c r="E1796" s="2">
+        <v>89.0</v>
+      </c>
+      <c r="F1796" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1796" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1797">
+      <c r="A1797" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1797" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:20</t>
+        </is>
+      </c>
+      <c r="C1797" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1797" s="2">
+        <v>14.3</v>
+      </c>
+      <c r="E1797" s="2">
+        <v>90.0</v>
+      </c>
+      <c r="F1797" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1797" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1798">
+      <c r="A1798" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1798" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:30</t>
+        </is>
+      </c>
+      <c r="C1798" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1798" s="2">
+        <v>14.2</v>
+      </c>
+      <c r="E1798" s="2">
+        <v>90.0</v>
+      </c>
+      <c r="F1798" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1798" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1799">
+      <c r="A1799" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1799" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:40</t>
+        </is>
+      </c>
+      <c r="C1799" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1799" s="2">
+        <v>14.3</v>
+      </c>
+      <c r="E1799" s="2">
+        <v>90.0</v>
+      </c>
+      <c r="F1799" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1799" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1800">
+      <c r="A1800" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1800" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:50</t>
+        </is>
+      </c>
+      <c r="C1800" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1800" s="2">
+        <v>14.9</v>
+      </c>
+      <c r="E1800" s="2">
+        <v>88.0</v>
+      </c>
+      <c r="F1800" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1800" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1801">
+      <c r="A1801" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1801" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:00</t>
+        </is>
+      </c>
+      <c r="C1801" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1801" s="2">
+        <v>15.1</v>
+      </c>
+      <c r="E1801" s="2">
+        <v>87.0</v>
+      </c>
+      <c r="F1801" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1801" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1802">
+      <c r="A1802" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1802" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:10</t>
+        </is>
+      </c>
+      <c r="C1802" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1802" s="2">
+        <v>15.4</v>
+      </c>
+      <c r="E1802" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F1802" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1802" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1803">
+      <c r="A1803" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1803" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:20</t>
+        </is>
+      </c>
+      <c r="C1803" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1803" s="2">
+        <v>15.9</v>
+      </c>
+      <c r="E1803" s="2">
+        <v>83.0</v>
+      </c>
+      <c r="F1803" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1803" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1804">
+      <c r="A1804" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1804" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:30</t>
+        </is>
+      </c>
+      <c r="C1804" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1804" s="2">
+        <v>16.4</v>
+      </c>
+      <c r="E1804" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F1804" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1804" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1805">
+      <c r="A1805" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1805" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:40</t>
+        </is>
+      </c>
+      <c r="C1805" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1805" s="2">
+        <v>16.7</v>
+      </c>
+      <c r="E1805" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F1805" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1805" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1806">
+      <c r="A1806" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1806" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:50</t>
+        </is>
+      </c>
+      <c r="C1806" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1806" s="2">
+        <v>17.0</v>
+      </c>
+      <c r="E1806" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F1806" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1806" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1807">
+      <c r="A1807" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1807" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:00</t>
+        </is>
+      </c>
+      <c r="C1807" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1807" s="2">
+        <v>17.6</v>
+      </c>
+      <c r="E1807" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F1807" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1807" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1808">
+      <c r="A1808" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1808" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:10</t>
+        </is>
+      </c>
+      <c r="C1808" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1808" s="2">
+        <v>18.4</v>
+      </c>
+      <c r="E1808" s="2">
+        <v>72.0</v>
+      </c>
+      <c r="F1808" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1808" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1809">
+      <c r="A1809" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1809" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:20</t>
+        </is>
+      </c>
+      <c r="C1809" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1809" s="2">
+        <v>18.6</v>
+      </c>
+      <c r="E1809" s="2">
+        <v>69.0</v>
+      </c>
+      <c r="F1809" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1809" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1810">
+      <c r="A1810" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1810" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:30</t>
+        </is>
+      </c>
+      <c r="C1810" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1810" s="2">
+        <v>19.2</v>
+      </c>
+      <c r="E1810" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F1810" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1810" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1811">
+      <c r="A1811" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1811" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:40</t>
+        </is>
+      </c>
+      <c r="C1811" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1811" s="2">
+        <v>19.7</v>
+      </c>
+      <c r="E1811" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F1811" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1811" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1812">
+      <c r="A1812" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1812" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:50</t>
+        </is>
+      </c>
+      <c r="C1812" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1812" s="2">
+        <v>19.9</v>
+      </c>
+      <c r="E1812" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F1812" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1812" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1813">
+      <c r="A1813" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1813" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:00</t>
+        </is>
+      </c>
+      <c r="C1813" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1813" s="2">
+        <v>20.5</v>
+      </c>
+      <c r="E1813" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F1813" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1813" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1814">
+      <c r="A1814" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1814" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:10</t>
+        </is>
+      </c>
+      <c r="C1814" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1814" s="2">
+        <v>21.2</v>
+      </c>
+      <c r="E1814" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F1814" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1814" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1815">
+      <c r="A1815" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1815" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:20</t>
+        </is>
+      </c>
+      <c r="C1815" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1815" s="2">
+        <v>21.3</v>
+      </c>
+      <c r="E1815" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F1815" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1815" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1816">
+      <c r="A1816" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1816" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:30</t>
+        </is>
+      </c>
+      <c r="C1816" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1816" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="E1816" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F1816" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1816" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1817">
+      <c r="A1817" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1817" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:40</t>
+        </is>
+      </c>
+      <c r="C1817" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1817" s="2">
+        <v>22.4</v>
+      </c>
+      <c r="E1817" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F1817" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1817" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1818">
+      <c r="A1818" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1818" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:50</t>
+        </is>
+      </c>
+      <c r="C1818" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1818" s="2">
+        <v>23.1</v>
+      </c>
+      <c r="E1818" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F1818" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1818" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1819">
+      <c r="A1819" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1819" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:00</t>
+        </is>
+      </c>
+      <c r="C1819" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1819" s="2">
+        <v>23.6</v>
+      </c>
+      <c r="E1819" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F1819" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1819" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1820">
+      <c r="A1820" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1820" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:10</t>
+        </is>
+      </c>
+      <c r="C1820" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1820" s="2">
+        <v>23.7</v>
+      </c>
+      <c r="E1820" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F1820" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1820" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1821">
+      <c r="A1821" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1821" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:20</t>
+        </is>
+      </c>
+      <c r="C1821" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1821" s="2">
+        <v>24.1</v>
+      </c>
+      <c r="E1821" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F1821" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1821" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1822">
+      <c r="A1822" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1822" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:30</t>
+        </is>
+      </c>
+      <c r="C1822" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1822" s="2">
+        <v>24.9</v>
+      </c>
+      <c r="E1822" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F1822" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1822" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1823">
+      <c r="A1823" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1823" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:40</t>
+        </is>
+      </c>
+      <c r="C1823" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1823" s="2">
+        <v>25.2</v>
+      </c>
+      <c r="E1823" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F1823" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1823" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1824">
+      <c r="A1824" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1824" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:50</t>
+        </is>
+      </c>
+      <c r="C1824" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1824" s="2">
+        <v>25.8</v>
+      </c>
+      <c r="E1824" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F1824" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1824" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1825">
+      <c r="A1825" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1825" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:00</t>
+        </is>
+      </c>
+      <c r="C1825" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1825" s="2">
+        <v>25.3</v>
+      </c>
+      <c r="E1825" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F1825" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1825" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1826">
+      <c r="A1826" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1826" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:10</t>
+        </is>
+      </c>
+      <c r="C1826" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1826" s="2">
+        <v>25.8</v>
+      </c>
+      <c r="E1826" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F1826" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1826" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1827">
+      <c r="A1827" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1827" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:20</t>
+        </is>
+      </c>
+      <c r="C1827" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1827" s="2">
+        <v>26.1</v>
+      </c>
+      <c r="E1827" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F1827" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1827" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1828">
+      <c r="A1828" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1828" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:30</t>
+        </is>
+      </c>
+      <c r="C1828" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1828" s="2">
+        <v>26.4</v>
+      </c>
+      <c r="E1828" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F1828" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1828" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1829">
+      <c r="A1829" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1829" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:40</t>
+        </is>
+      </c>
+      <c r="C1829" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1829" s="2">
+        <v>27.2</v>
+      </c>
+      <c r="E1829" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F1829" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1829" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1830">
+      <c r="A1830" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1830" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:50</t>
+        </is>
+      </c>
+      <c r="C1830" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1830" s="2">
+        <v>27.2</v>
+      </c>
+      <c r="E1830" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F1830" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1830" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1831">
+      <c r="A1831" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1831" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:00</t>
+        </is>
+      </c>
+      <c r="C1831" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1831" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="E1831" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F1831" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1831" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1832">
+      <c r="A1832" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1832" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:10</t>
+        </is>
+      </c>
+      <c r="C1832" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1832" s="2">
+        <v>28.5</v>
+      </c>
+      <c r="E1832" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F1832" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1832" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1833">
+      <c r="A1833" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1833" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:20</t>
+        </is>
+      </c>
+      <c r="C1833" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1833" s="2">
+        <v>29.3</v>
+      </c>
+      <c r="E1833" s="2">
+        <v>38.0</v>
+      </c>
+      <c r="F1833" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1833" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1834">
+      <c r="A1834" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1834" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:30</t>
+        </is>
+      </c>
+      <c r="C1834" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1834" s="2">
+        <v>29.8</v>
+      </c>
+      <c r="E1834" s="2">
+        <v>37.0</v>
+      </c>
+      <c r="F1834" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1834" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1835">
+      <c r="A1835" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1835" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:40</t>
+        </is>
+      </c>
+      <c r="C1835" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1835" s="2">
+        <v>29.4</v>
+      </c>
+      <c r="E1835" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F1835" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1835" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1836">
+      <c r="A1836" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1836" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:50</t>
+        </is>
+      </c>
+      <c r="C1836" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1836" s="2">
+        <v>29.7</v>
+      </c>
+      <c r="E1836" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F1836" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1836" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1837">
+      <c r="A1837" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1837" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:00</t>
+        </is>
+      </c>
+      <c r="C1837" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1837" s="2">
+        <v>29.9</v>
+      </c>
+      <c r="E1837" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F1837" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1837" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1838">
+      <c r="A1838" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1838" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:10</t>
+        </is>
+      </c>
+      <c r="C1838" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1838" s="2">
+        <v>29.5</v>
+      </c>
+      <c r="E1838" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="F1838" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1838" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1839">
+      <c r="A1839" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1839" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:20</t>
+        </is>
+      </c>
+      <c r="C1839" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1839" s="2">
+        <v>29.2</v>
+      </c>
+      <c r="E1839" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F1839" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1839" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1840">
+      <c r="A1840" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1840" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:30</t>
+        </is>
+      </c>
+      <c r="C1840" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1840" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="E1840" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="F1840" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1840" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1841">
+      <c r="A1841" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1841" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:40</t>
+        </is>
+      </c>
+      <c r="C1841" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1841" s="2">
+        <v>29.4</v>
+      </c>
+      <c r="E1841" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="F1841" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1841" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1842">
+      <c r="A1842" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1842" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:50</t>
+        </is>
+      </c>
+      <c r="C1842" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1842" s="2">
+        <v>29.8</v>
+      </c>
+      <c r="E1842" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F1842" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1842" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1843">
+      <c r="A1843" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1843" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:00</t>
+        </is>
+      </c>
+      <c r="C1843" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1843" s="2">
+        <v>29.5</v>
+      </c>
+      <c r="E1843" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F1843" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1843" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1844">
+      <c r="A1844" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1844" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:10</t>
+        </is>
+      </c>
+      <c r="C1844" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1844" s="2">
+        <v>29.7</v>
+      </c>
+      <c r="E1844" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="F1844" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1844" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1845">
+      <c r="A1845" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1845" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:20</t>
+        </is>
+      </c>
+      <c r="C1845" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1845" s="2">
+        <v>29.4</v>
+      </c>
+      <c r="E1845" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F1845" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1845" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1846">
+      <c r="A1846" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1846" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:30</t>
+        </is>
+      </c>
+      <c r="C1846" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1846" s="2">
+        <v>29.1</v>
+      </c>
+      <c r="E1846" s="2">
+        <v>37.0</v>
+      </c>
+      <c r="F1846" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1846" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1847">
+      <c r="A1847" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1847" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:40</t>
+        </is>
+      </c>
+      <c r="C1847" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1847" s="2">
+        <v>28.8</v>
+      </c>
+      <c r="E1847" s="2">
+        <v>37.0</v>
+      </c>
+      <c r="F1847" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1847" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1848">
+      <c r="A1848" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1848" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:50</t>
+        </is>
+      </c>
+      <c r="C1848" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1848" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="E1848" s="2">
+        <v>37.0</v>
+      </c>
+      <c r="F1848" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1848" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1849">
+      <c r="A1849" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1849" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:00</t>
+        </is>
+      </c>
+      <c r="C1849" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1849" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="E1849" s="2">
+        <v>37.0</v>
+      </c>
+      <c r="F1849" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1849" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1850">
+      <c r="A1850" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1850" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:10</t>
+        </is>
+      </c>
+      <c r="C1850" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1850" s="2">
+        <v>29.2</v>
+      </c>
+      <c r="E1850" s="2">
+        <v>37.0</v>
+      </c>
+      <c r="F1850" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1850" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1851">
+      <c r="A1851" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1851" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:20</t>
+        </is>
+      </c>
+      <c r="C1851" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1851" s="2">
+        <v>29.6</v>
+      </c>
+      <c r="E1851" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="F1851" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1851" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1852">
+      <c r="A1852" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1852" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:30</t>
+        </is>
+      </c>
+      <c r="C1852" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1852" s="2">
+        <v>30.2</v>
+      </c>
+      <c r="E1852" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F1852" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1852" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1853">
+      <c r="A1853" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1853" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:40</t>
+        </is>
+      </c>
+      <c r="C1853" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1853" s="2">
+        <v>30.1</v>
+      </c>
+      <c r="E1853" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F1853" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1853" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1854">
+      <c r="A1854" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1854" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:50</t>
+        </is>
+      </c>
+      <c r="C1854" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1854" s="2">
+        <v>29.8</v>
+      </c>
+      <c r="E1854" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F1854" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1854" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1855">
+      <c r="A1855" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1855" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:00</t>
+        </is>
+      </c>
+      <c r="C1855" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1855" s="2">
+        <v>29.5</v>
+      </c>
+      <c r="E1855" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F1855" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1855" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1856">
+      <c r="A1856" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1856" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:10</t>
+        </is>
+      </c>
+      <c r="C1856" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1856" s="2">
+        <v>29.8</v>
+      </c>
+      <c r="E1856" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F1856" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1856" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1857">
+      <c r="A1857" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1857" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:20</t>
+        </is>
+      </c>
+      <c r="C1857" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1857" s="2">
+        <v>30.2</v>
+      </c>
+      <c r="E1857" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="F1857" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1857" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1858">
+      <c r="A1858" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1858" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:30</t>
+        </is>
+      </c>
+      <c r="C1858" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1858" s="2">
+        <v>30.3</v>
+      </c>
+      <c r="E1858" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F1858" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1858" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1859">
+      <c r="A1859" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1859" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:40</t>
+        </is>
+      </c>
+      <c r="C1859" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1859" s="2">
+        <v>30.3</v>
+      </c>
+      <c r="E1859" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F1859" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1859" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1860">
+      <c r="A1860" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1860" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:50</t>
+        </is>
+      </c>
+      <c r="C1860" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1860" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="E1860" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F1860" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1860" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1861">
+      <c r="A1861" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1861" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:00</t>
+        </is>
+      </c>
+      <c r="C1861" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1861" s="2">
+        <v>30.4</v>
+      </c>
+      <c r="E1861" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F1861" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1861" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1862">
+      <c r="A1862" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1862" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:10</t>
+        </is>
+      </c>
+      <c r="C1862" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1862" s="2">
+        <v>30.3</v>
+      </c>
+      <c r="E1862" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="F1862" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1862" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1863">
+      <c r="A1863" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1863" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:20</t>
+        </is>
+      </c>
+      <c r="C1863" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1863" s="2">
+        <v>30.4</v>
+      </c>
+      <c r="E1863" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F1863" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1863" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1864">
+      <c r="A1864" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1864" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:30</t>
+        </is>
+      </c>
+      <c r="C1864" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1864" s="2">
+        <v>30.2</v>
+      </c>
+      <c r="E1864" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F1864" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1864" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1865">
+      <c r="A1865" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1865" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:40</t>
+        </is>
+      </c>
+      <c r="C1865" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1865" s="2">
+        <v>30.3</v>
+      </c>
+      <c r="E1865" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F1865" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1865" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1866">
+      <c r="A1866" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1866" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:50</t>
+        </is>
+      </c>
+      <c r="C1866" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1866" s="2">
+        <v>30.8</v>
+      </c>
+      <c r="E1866" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F1866" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1866" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1867">
+      <c r="A1867" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1867" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:00</t>
+        </is>
+      </c>
+      <c r="C1867" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1867" s="2">
+        <v>30.8</v>
+      </c>
+      <c r="E1867" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F1867" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1867" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1868">
+      <c r="A1868" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1868" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:10</t>
+        </is>
+      </c>
+      <c r="C1868" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1868" s="2">
+        <v>30.6</v>
+      </c>
+      <c r="E1868" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F1868" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1868" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1869">
+      <c r="A1869" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1869" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:20</t>
+        </is>
+      </c>
+      <c r="C1869" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1869" s="2">
+        <v>30.2</v>
+      </c>
+      <c r="E1869" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="F1869" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1869" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1870">
+      <c r="A1870" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1870" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:30</t>
+        </is>
+      </c>
+      <c r="C1870" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1870" s="2">
+        <v>30.1</v>
+      </c>
+      <c r="E1870" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="F1870" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1870" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1871">
+      <c r="A1871" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1871" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:40</t>
+        </is>
+      </c>
+      <c r="C1871" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1871" s="2">
+        <v>29.9</v>
+      </c>
+      <c r="E1871" s="2">
+        <v>38.0</v>
+      </c>
+      <c r="F1871" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1871" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1872">
+      <c r="A1872" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1872" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:50</t>
+        </is>
+      </c>
+      <c r="C1872" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1872" s="2">
+        <v>29.6</v>
+      </c>
+      <c r="E1872" s="2">
+        <v>38.0</v>
+      </c>
+      <c r="F1872" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1872" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1873">
+      <c r="A1873" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1873" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:00</t>
+        </is>
+      </c>
+      <c r="C1873" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1873" s="2">
+        <v>29.4</v>
+      </c>
+      <c r="E1873" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F1873" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1873" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1874">
+      <c r="A1874" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1874" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:10</t>
+        </is>
+      </c>
+      <c r="C1874" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1874" s="2">
+        <v>28.9</v>
+      </c>
+      <c r="E1874" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F1874" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1874" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1875">
+      <c r="A1875" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1875" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:20</t>
+        </is>
+      </c>
+      <c r="C1875" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1875" s="2">
+        <v>28.7</v>
+      </c>
+      <c r="E1875" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F1875" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1875" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1876">
+      <c r="A1876" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1876" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:30</t>
+        </is>
+      </c>
+      <c r="C1876" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1876" s="2">
+        <v>28.4</v>
+      </c>
+      <c r="E1876" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F1876" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1876" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1877">
+      <c r="A1877" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1877" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:40</t>
+        </is>
+      </c>
+      <c r="C1877" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1877" s="2">
+        <v>28.2</v>
+      </c>
+      <c r="E1877" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F1877" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1877" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1878">
+      <c r="A1878" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1878" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:50</t>
+        </is>
+      </c>
+      <c r="C1878" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1878" s="2">
+        <v>27.9</v>
+      </c>
+      <c r="E1878" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F1878" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1878" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1879">
+      <c r="A1879" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1879" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:00</t>
+        </is>
+      </c>
+      <c r="C1879" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1879" s="2">
+        <v>27.7</v>
+      </c>
+      <c r="E1879" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F1879" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1879" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1880">
+      <c r="A1880" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1880" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:10</t>
+        </is>
+      </c>
+      <c r="C1880" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1880" s="2">
+        <v>27.3</v>
+      </c>
+      <c r="E1880" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F1880" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1880" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1881">
+      <c r="A1881" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1881" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:20</t>
+        </is>
+      </c>
+      <c r="C1881" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1881" s="2">
+        <v>27.2</v>
+      </c>
+      <c r="E1881" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F1881" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1881" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1882">
+      <c r="A1882" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1882" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:30</t>
+        </is>
+      </c>
+      <c r="C1882" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1882" s="2">
+        <v>26.9</v>
+      </c>
+      <c r="E1882" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F1882" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1882" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1883">
+      <c r="A1883" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1883" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:40</t>
+        </is>
+      </c>
+      <c r="C1883" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1883" s="2">
+        <v>26.7</v>
+      </c>
+      <c r="E1883" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F1883" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1883" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1884">
+      <c r="A1884" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1884" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:50</t>
+        </is>
+      </c>
+      <c r="C1884" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1884" s="2">
+        <v>26.4</v>
+      </c>
+      <c r="E1884" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F1884" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1884" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1885">
+      <c r="A1885" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1885" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:00</t>
+        </is>
+      </c>
+      <c r="C1885" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1885" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="E1885" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F1885" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1885" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1886">
+      <c r="A1886" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1886" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:10</t>
+        </is>
+      </c>
+      <c r="C1886" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1886" s="2">
+        <v>25.6</v>
+      </c>
+      <c r="E1886" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F1886" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1886" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1887">
+      <c r="A1887" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1887" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:20</t>
+        </is>
+      </c>
+      <c r="C1887" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1887" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="E1887" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F1887" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1887" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1888">
+      <c r="A1888" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1888" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:30</t>
+        </is>
+      </c>
+      <c r="C1888" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1888" s="2">
+        <v>24.8</v>
+      </c>
+      <c r="E1888" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F1888" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1888" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1889">
+      <c r="A1889" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1889" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:40</t>
+        </is>
+      </c>
+      <c r="C1889" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1889" s="2">
+        <v>24.8</v>
+      </c>
+      <c r="E1889" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F1889" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1889" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1890">
+      <c r="A1890" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1890" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:50</t>
+        </is>
+      </c>
+      <c r="C1890" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1890" s="2">
+        <v>24.7</v>
+      </c>
+      <c r="E1890" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F1890" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1890" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1891">
+      <c r="A1891" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1891" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:00</t>
+        </is>
+      </c>
+      <c r="C1891" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1891" s="2">
+        <v>24.5</v>
+      </c>
+      <c r="E1891" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F1891" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1891" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1892">
+      <c r="A1892" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1892" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:10</t>
+        </is>
+      </c>
+      <c r="C1892" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1892" s="2">
+        <v>24.2</v>
+      </c>
+      <c r="E1892" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F1892" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1892" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1893">
+      <c r="A1893" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1893" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:20</t>
+        </is>
+      </c>
+      <c r="C1893" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1893" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="E1893" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F1893" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1893" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1894">
+      <c r="A1894" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1894" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:30</t>
+        </is>
+      </c>
+      <c r="C1894" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1894" s="2">
+        <v>23.7</v>
+      </c>
+      <c r="E1894" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F1894" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1894" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1895">
+      <c r="A1895" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1895" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:40</t>
+        </is>
+      </c>
+      <c r="C1895" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1895" s="2">
+        <v>23.5</v>
+      </c>
+      <c r="E1895" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F1895" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1895" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1896">
+      <c r="A1896" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1896" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:50</t>
+        </is>
+      </c>
+      <c r="C1896" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1896" s="2">
+        <v>23.4</v>
+      </c>
+      <c r="E1896" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F1896" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1896" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1897">
+      <c r="A1897" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1897" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:00</t>
+        </is>
+      </c>
+      <c r="C1897" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1897" s="2">
+        <v>23.2</v>
+      </c>
+      <c r="E1897" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F1897" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1897" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1898">
+      <c r="A1898" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1898" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:10</t>
+        </is>
+      </c>
+      <c r="C1898" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1898" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="E1898" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F1898" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1898" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1899">
+      <c r="A1899" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1899" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:20</t>
+        </is>
+      </c>
+      <c r="C1899" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1899" s="2">
+        <v>22.7</v>
+      </c>
+      <c r="E1899" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F1899" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1899" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1900">
+      <c r="A1900" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1900" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:30</t>
+        </is>
+      </c>
+      <c r="C1900" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1900" s="2">
+        <v>22.6</v>
+      </c>
+      <c r="E1900" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F1900" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1900" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1901">
+      <c r="A1901" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1901" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:40</t>
+        </is>
+      </c>
+      <c r="C1901" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1901" s="2">
+        <v>22.4</v>
+      </c>
+      <c r="E1901" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F1901" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1901" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1902">
+      <c r="A1902" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">27.07.2026</t>
+        </is>
+      </c>
+      <c r="B1902" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:50</t>
+        </is>
+      </c>
+      <c r="C1902" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1902" s="2">
+        <v>22.5</v>
+      </c>
+      <c r="E1902" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F1902" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1902" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1903">
+      <c r="A1903" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1903" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:00</t>
+        </is>
+      </c>
+      <c r="C1903" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1903" s="2">
+        <v>22.5</v>
+      </c>
+      <c r="E1903" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F1903" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1903" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1904">
+      <c r="A1904" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1904" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:10</t>
+        </is>
+      </c>
+      <c r="C1904" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1904" s="2">
+        <v>22.3</v>
+      </c>
+      <c r="E1904" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F1904" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1904" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1905">
+      <c r="A1905" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1905" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:20</t>
+        </is>
+      </c>
+      <c r="C1905" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1905" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="E1905" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F1905" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1905" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1906">
+      <c r="A1906" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1906" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:30</t>
+        </is>
+      </c>
+      <c r="C1906" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1906" s="2">
+        <v>21.8</v>
+      </c>
+      <c r="E1906" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F1906" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1906" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G1762"/>
+  <autoFilter ref="A1:G1906"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ARSO Kranj zajem 2026-07-29 00:44 Europe/Ljubljana
</commit_message>
<xml_diff>
--- a/tabela_vremena/ARSO_Kranj.xlsx
+++ b/tabela_vremena/ARSO_Kranj.xlsx
@@ -55356,7 +55356,4183 @@
         <v>0.0</v>
       </c>
     </row>
+    <row r="1907">
+      <c r="A1907" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1907" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:40</t>
+        </is>
+      </c>
+      <c r="C1907" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1907" s="2">
+        <v>21.5</v>
+      </c>
+      <c r="E1907" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F1907" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1907" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1908">
+      <c r="A1908" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1908" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:50</t>
+        </is>
+      </c>
+      <c r="C1908" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1908" s="2">
+        <v>21.1</v>
+      </c>
+      <c r="E1908" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F1908" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1908" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1909">
+      <c r="A1909" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1909" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:00</t>
+        </is>
+      </c>
+      <c r="C1909" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1909" s="2">
+        <v>20.7</v>
+      </c>
+      <c r="E1909" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F1909" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1909" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1910">
+      <c r="A1910" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1910" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:10</t>
+        </is>
+      </c>
+      <c r="C1910" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1910" s="2">
+        <v>20.4</v>
+      </c>
+      <c r="E1910" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F1910" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1910" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1911">
+      <c r="A1911" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1911" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:20</t>
+        </is>
+      </c>
+      <c r="C1911" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1911" s="2">
+        <v>20.1</v>
+      </c>
+      <c r="E1911" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="F1911" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1911" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1912">
+      <c r="A1912" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1912" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:30</t>
+        </is>
+      </c>
+      <c r="C1912" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1912" s="2">
+        <v>19.8</v>
+      </c>
+      <c r="E1912" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F1912" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1912" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1913">
+      <c r="A1913" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1913" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:40</t>
+        </is>
+      </c>
+      <c r="C1913" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1913" s="2">
+        <v>19.5</v>
+      </c>
+      <c r="E1913" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F1913" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1913" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1914">
+      <c r="A1914" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1914" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:50</t>
+        </is>
+      </c>
+      <c r="C1914" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1914" s="2">
+        <v>19.3</v>
+      </c>
+      <c r="E1914" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F1914" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1914" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1915">
+      <c r="A1915" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1915" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:00</t>
+        </is>
+      </c>
+      <c r="C1915" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1915" s="2">
+        <v>19.1</v>
+      </c>
+      <c r="E1915" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F1915" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1915" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1916">
+      <c r="A1916" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1916" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:10</t>
+        </is>
+      </c>
+      <c r="C1916" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1916" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="E1916" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F1916" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1916" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1917">
+      <c r="A1917" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1917" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:20</t>
+        </is>
+      </c>
+      <c r="C1917" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1917" s="2">
+        <v>18.8</v>
+      </c>
+      <c r="E1917" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F1917" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1917" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1918">
+      <c r="A1918" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1918" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:30</t>
+        </is>
+      </c>
+      <c r="C1918" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1918" s="2">
+        <v>18.6</v>
+      </c>
+      <c r="E1918" s="2">
+        <v>81.0</v>
+      </c>
+      <c r="F1918" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1918" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1919">
+      <c r="A1919" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1919" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:40</t>
+        </is>
+      </c>
+      <c r="C1919" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1919" s="2">
+        <v>18.7</v>
+      </c>
+      <c r="E1919" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F1919" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1919" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1920">
+      <c r="A1920" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1920" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:50</t>
+        </is>
+      </c>
+      <c r="C1920" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1920" s="2">
+        <v>18.9</v>
+      </c>
+      <c r="E1920" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F1920" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1920" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1921">
+      <c r="A1921" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1921" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:00</t>
+        </is>
+      </c>
+      <c r="C1921" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1921" s="2">
+        <v>19.1</v>
+      </c>
+      <c r="E1921" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F1921" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1921" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1922">
+      <c r="A1922" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1922" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:10</t>
+        </is>
+      </c>
+      <c r="C1922" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1922" s="2">
+        <v>19.2</v>
+      </c>
+      <c r="E1922" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F1922" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1922" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1923">
+      <c r="A1923" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1923" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:20</t>
+        </is>
+      </c>
+      <c r="C1923" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1923" s="2">
+        <v>19.2</v>
+      </c>
+      <c r="E1923" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F1923" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1923" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1924">
+      <c r="A1924" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1924" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:30</t>
+        </is>
+      </c>
+      <c r="C1924" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1924" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="E1924" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F1924" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1924" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1925">
+      <c r="A1925" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1925" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:40</t>
+        </is>
+      </c>
+      <c r="C1925" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1925" s="2">
+        <v>18.8</v>
+      </c>
+      <c r="E1925" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F1925" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1925" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1926">
+      <c r="A1926" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1926" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:50</t>
+        </is>
+      </c>
+      <c r="C1926" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1926" s="2">
+        <v>18.5</v>
+      </c>
+      <c r="E1926" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F1926" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1926" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1927">
+      <c r="A1927" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1927" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:00</t>
+        </is>
+      </c>
+      <c r="C1927" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1927" s="2">
+        <v>18.4</v>
+      </c>
+      <c r="E1927" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F1927" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1927" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1928">
+      <c r="A1928" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1928" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:10</t>
+        </is>
+      </c>
+      <c r="C1928" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1928" s="2">
+        <v>18.3</v>
+      </c>
+      <c r="E1928" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F1928" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1928" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1929">
+      <c r="A1929" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1929" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:20</t>
+        </is>
+      </c>
+      <c r="C1929" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1929" s="2">
+        <v>18.3</v>
+      </c>
+      <c r="E1929" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F1929" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1929" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1930">
+      <c r="A1930" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1930" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:30</t>
+        </is>
+      </c>
+      <c r="C1930" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1930" s="2">
+        <v>18.1</v>
+      </c>
+      <c r="E1930" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F1930" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1930" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1931">
+      <c r="A1931" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1931" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:40</t>
+        </is>
+      </c>
+      <c r="C1931" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1931" s="2">
+        <v>17.8</v>
+      </c>
+      <c r="E1931" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F1931" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1931" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1932">
+      <c r="A1932" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1932" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:50</t>
+        </is>
+      </c>
+      <c r="C1932" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1932" s="2">
+        <v>17.6</v>
+      </c>
+      <c r="E1932" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F1932" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1932" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1933">
+      <c r="A1933" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1933" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:00</t>
+        </is>
+      </c>
+      <c r="C1933" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1933" s="2">
+        <v>17.4</v>
+      </c>
+      <c r="E1933" s="2">
+        <v>83.0</v>
+      </c>
+      <c r="F1933" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1933" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1934">
+      <c r="A1934" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1934" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:10</t>
+        </is>
+      </c>
+      <c r="C1934" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1934" s="2">
+        <v>17.5</v>
+      </c>
+      <c r="E1934" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F1934" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1934" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1935">
+      <c r="A1935" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1935" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:20</t>
+        </is>
+      </c>
+      <c r="C1935" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1935" s="2">
+        <v>17.3</v>
+      </c>
+      <c r="E1935" s="2">
+        <v>84.0</v>
+      </c>
+      <c r="F1935" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1935" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1936">
+      <c r="A1936" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1936" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:30</t>
+        </is>
+      </c>
+      <c r="C1936" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1936" s="2">
+        <v>17.2</v>
+      </c>
+      <c r="E1936" s="2">
+        <v>84.0</v>
+      </c>
+      <c r="F1936" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1936" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1937">
+      <c r="A1937" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1937" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:40</t>
+        </is>
+      </c>
+      <c r="C1937" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1937" s="2">
+        <v>17.2</v>
+      </c>
+      <c r="E1937" s="2">
+        <v>84.0</v>
+      </c>
+      <c r="F1937" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1937" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1938">
+      <c r="A1938" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1938" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:50</t>
+        </is>
+      </c>
+      <c r="C1938" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1938" s="2">
+        <v>17.3</v>
+      </c>
+      <c r="E1938" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F1938" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1938" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1939">
+      <c r="A1939" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1939" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:00</t>
+        </is>
+      </c>
+      <c r="C1939" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1939" s="2">
+        <v>17.3</v>
+      </c>
+      <c r="E1939" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F1939" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1939" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1940">
+      <c r="A1940" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1940" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:10</t>
+        </is>
+      </c>
+      <c r="C1940" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1940" s="2">
+        <v>17.2</v>
+      </c>
+      <c r="E1940" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F1940" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1940" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1941">
+      <c r="A1941" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1941" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:20</t>
+        </is>
+      </c>
+      <c r="C1941" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1941" s="2">
+        <v>17.1</v>
+      </c>
+      <c r="E1941" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F1941" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1941" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1942">
+      <c r="A1942" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1942" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:30</t>
+        </is>
+      </c>
+      <c r="C1942" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1942" s="2">
+        <v>17.1</v>
+      </c>
+      <c r="E1942" s="2">
+        <v>86.0</v>
+      </c>
+      <c r="F1942" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1942" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1943">
+      <c r="A1943" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1943" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:40</t>
+        </is>
+      </c>
+      <c r="C1943" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1943" s="2">
+        <v>17.4</v>
+      </c>
+      <c r="E1943" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F1943" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1943" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1944">
+      <c r="A1944" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1944" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:50</t>
+        </is>
+      </c>
+      <c r="C1944" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1944" s="2">
+        <v>17.6</v>
+      </c>
+      <c r="E1944" s="2">
+        <v>84.0</v>
+      </c>
+      <c r="F1944" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1944" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1945">
+      <c r="A1945" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1945" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:00</t>
+        </is>
+      </c>
+      <c r="C1945" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1945" s="2">
+        <v>17.8</v>
+      </c>
+      <c r="E1945" s="2">
+        <v>84.0</v>
+      </c>
+      <c r="F1945" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1945" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1946">
+      <c r="A1946" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1946" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:10</t>
+        </is>
+      </c>
+      <c r="C1946" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1946" s="2">
+        <v>18.1</v>
+      </c>
+      <c r="E1946" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F1946" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1946" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1947">
+      <c r="A1947" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1947" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:20</t>
+        </is>
+      </c>
+      <c r="C1947" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1947" s="2">
+        <v>18.8</v>
+      </c>
+      <c r="E1947" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F1947" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1947" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1948">
+      <c r="A1948" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1948" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:30</t>
+        </is>
+      </c>
+      <c r="C1948" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1948" s="2">
+        <v>19.4</v>
+      </c>
+      <c r="E1948" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F1948" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1948" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1949">
+      <c r="A1949" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1949" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:40</t>
+        </is>
+      </c>
+      <c r="C1949" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1949" s="2">
+        <v>20.7</v>
+      </c>
+      <c r="E1949" s="2">
+        <v>72.0</v>
+      </c>
+      <c r="F1949" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1949" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1950">
+      <c r="A1950" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1950" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:50</t>
+        </is>
+      </c>
+      <c r="C1950" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1950" s="2">
+        <v>20.7</v>
+      </c>
+      <c r="E1950" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F1950" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1950" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1951">
+      <c r="A1951" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1951" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:00</t>
+        </is>
+      </c>
+      <c r="C1951" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1951" s="2">
+        <v>21.2</v>
+      </c>
+      <c r="E1951" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F1951" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1951" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1952">
+      <c r="A1952" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1952" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:10</t>
+        </is>
+      </c>
+      <c r="C1952" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1952" s="2">
+        <v>21.4</v>
+      </c>
+      <c r="E1952" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F1952" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1952" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1953">
+      <c r="A1953" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1953" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:20</t>
+        </is>
+      </c>
+      <c r="C1953" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1953" s="2">
+        <v>21.9</v>
+      </c>
+      <c r="E1953" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F1953" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1953" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1954">
+      <c r="A1954" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1954" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:30</t>
+        </is>
+      </c>
+      <c r="C1954" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1954" s="2">
+        <v>22.5</v>
+      </c>
+      <c r="E1954" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F1954" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1954" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1955">
+      <c r="A1955" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1955" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:40</t>
+        </is>
+      </c>
+      <c r="C1955" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1955" s="2">
+        <v>22.7</v>
+      </c>
+      <c r="E1955" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F1955" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1955" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1956">
+      <c r="A1956" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1956" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:50</t>
+        </is>
+      </c>
+      <c r="C1956" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1956" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="E1956" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F1956" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1956" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1957">
+      <c r="A1957" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1957" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:00</t>
+        </is>
+      </c>
+      <c r="C1957" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1957" s="2">
+        <v>23.9</v>
+      </c>
+      <c r="E1957" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F1957" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1957" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1958">
+      <c r="A1958" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1958" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:10</t>
+        </is>
+      </c>
+      <c r="C1958" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1958" s="2">
+        <v>23.8</v>
+      </c>
+      <c r="E1958" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F1958" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1958" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1959">
+      <c r="A1959" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1959" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:20</t>
+        </is>
+      </c>
+      <c r="C1959" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1959" s="2">
+        <v>24.1</v>
+      </c>
+      <c r="E1959" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F1959" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1959" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1960">
+      <c r="A1960" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1960" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:30</t>
+        </is>
+      </c>
+      <c r="C1960" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1960" s="2">
+        <v>24.6</v>
+      </c>
+      <c r="E1960" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F1960" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1960" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1961">
+      <c r="A1961" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1961" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:40</t>
+        </is>
+      </c>
+      <c r="C1961" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1961" s="2">
+        <v>24.8</v>
+      </c>
+      <c r="E1961" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F1961" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1961" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1962">
+      <c r="A1962" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1962" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:50</t>
+        </is>
+      </c>
+      <c r="C1962" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1962" s="2">
+        <v>24.7</v>
+      </c>
+      <c r="E1962" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F1962" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1962" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1963">
+      <c r="A1963" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1963" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:00</t>
+        </is>
+      </c>
+      <c r="C1963" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1963" s="2">
+        <v>25.6</v>
+      </c>
+      <c r="E1963" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F1963" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1963" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1964">
+      <c r="A1964" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1964" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:10</t>
+        </is>
+      </c>
+      <c r="C1964" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1964" s="2">
+        <v>25.2</v>
+      </c>
+      <c r="E1964" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F1964" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1964" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1965">
+      <c r="A1965" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1965" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:20</t>
+        </is>
+      </c>
+      <c r="C1965" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1965" s="2">
+        <v>25.3</v>
+      </c>
+      <c r="E1965" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F1965" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1965" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1966">
+      <c r="A1966" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1966" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:30</t>
+        </is>
+      </c>
+      <c r="C1966" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1966" s="2">
+        <v>25.5</v>
+      </c>
+      <c r="E1966" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F1966" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1966" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1967">
+      <c r="A1967" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1967" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:40</t>
+        </is>
+      </c>
+      <c r="C1967" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1967" s="2">
+        <v>26.1</v>
+      </c>
+      <c r="E1967" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F1967" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1967" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1968">
+      <c r="A1968" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1968" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:50</t>
+        </is>
+      </c>
+      <c r="C1968" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1968" s="2">
+        <v>26.3</v>
+      </c>
+      <c r="E1968" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F1968" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1968" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1969">
+      <c r="A1969" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1969" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:00</t>
+        </is>
+      </c>
+      <c r="C1969" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1969" s="2">
+        <v>26.6</v>
+      </c>
+      <c r="E1969" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F1969" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1969" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1970">
+      <c r="A1970" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1970" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:10</t>
+        </is>
+      </c>
+      <c r="C1970" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1970" s="2">
+        <v>26.9</v>
+      </c>
+      <c r="E1970" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F1970" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1970" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1971">
+      <c r="A1971" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1971" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:20</t>
+        </is>
+      </c>
+      <c r="C1971" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1971" s="2">
+        <v>27.1</v>
+      </c>
+      <c r="E1971" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F1971" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1971" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1972">
+      <c r="A1972" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1972" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:30</t>
+        </is>
+      </c>
+      <c r="C1972" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1972" s="2">
+        <v>27.3</v>
+      </c>
+      <c r="E1972" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F1972" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1972" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1973">
+      <c r="A1973" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1973" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:40</t>
+        </is>
+      </c>
+      <c r="C1973" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1973" s="2">
+        <v>27.6</v>
+      </c>
+      <c r="E1973" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F1973" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1973" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1974">
+      <c r="A1974" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1974" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:50</t>
+        </is>
+      </c>
+      <c r="C1974" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1974" s="2">
+        <v>27.6</v>
+      </c>
+      <c r="E1974" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F1974" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1974" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1975">
+      <c r="A1975" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1975" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:00</t>
+        </is>
+      </c>
+      <c r="C1975" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1975" s="2">
+        <v>27.3</v>
+      </c>
+      <c r="E1975" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F1975" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1975" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1976">
+      <c r="A1976" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1976" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:10</t>
+        </is>
+      </c>
+      <c r="C1976" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1976" s="2">
+        <v>27.5</v>
+      </c>
+      <c r="E1976" s="2">
+        <v>37.0</v>
+      </c>
+      <c r="F1976" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1976" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1977">
+      <c r="A1977" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1977" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:20</t>
+        </is>
+      </c>
+      <c r="C1977" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1977" s="2">
+        <v>27.6</v>
+      </c>
+      <c r="E1977" s="2">
+        <v>37.0</v>
+      </c>
+      <c r="F1977" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1977" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1978">
+      <c r="A1978" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1978" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:30</t>
+        </is>
+      </c>
+      <c r="C1978" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1978" s="2">
+        <v>28.5</v>
+      </c>
+      <c r="E1978" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="F1978" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1978" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1979">
+      <c r="A1979" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1979" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:40</t>
+        </is>
+      </c>
+      <c r="C1979" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1979" s="2">
+        <v>28.3</v>
+      </c>
+      <c r="E1979" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F1979" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1979" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1980">
+      <c r="A1980" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1980" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:50</t>
+        </is>
+      </c>
+      <c r="C1980" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1980" s="2">
+        <v>28.7</v>
+      </c>
+      <c r="E1980" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F1980" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1980" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1981">
+      <c r="A1981" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1981" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:00</t>
+        </is>
+      </c>
+      <c r="C1981" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1981" s="2">
+        <v>28.8</v>
+      </c>
+      <c r="E1981" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F1981" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1981" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1982">
+      <c r="A1982" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1982" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:10</t>
+        </is>
+      </c>
+      <c r="C1982" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1982" s="2">
+        <v>28.8</v>
+      </c>
+      <c r="E1982" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F1982" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1982" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1983">
+      <c r="A1983" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1983" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:20</t>
+        </is>
+      </c>
+      <c r="C1983" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1983" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="E1983" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F1983" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1983" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1984">
+      <c r="A1984" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1984" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:30</t>
+        </is>
+      </c>
+      <c r="C1984" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1984" s="2">
+        <v>29.3</v>
+      </c>
+      <c r="E1984" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F1984" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1984" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1985">
+      <c r="A1985" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1985" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:40</t>
+        </is>
+      </c>
+      <c r="C1985" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1985" s="2">
+        <v>29.1</v>
+      </c>
+      <c r="E1985" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F1985" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1985" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1986">
+      <c r="A1986" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1986" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:50</t>
+        </is>
+      </c>
+      <c r="C1986" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1986" s="2">
+        <v>29.8</v>
+      </c>
+      <c r="E1986" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="F1986" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1986" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1987">
+      <c r="A1987" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1987" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:00</t>
+        </is>
+      </c>
+      <c r="C1987" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1987" s="2">
+        <v>29.2</v>
+      </c>
+      <c r="E1987" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F1987" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1987" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1988">
+      <c r="A1988" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1988" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:10</t>
+        </is>
+      </c>
+      <c r="C1988" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1988" s="2">
+        <v>29.3</v>
+      </c>
+      <c r="E1988" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F1988" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1988" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1989">
+      <c r="A1989" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1989" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:20</t>
+        </is>
+      </c>
+      <c r="C1989" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1989" s="2">
+        <v>29.9</v>
+      </c>
+      <c r="E1989" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F1989" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1989" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1990">
+      <c r="A1990" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1990" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:30</t>
+        </is>
+      </c>
+      <c r="C1990" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1990" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="E1990" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F1990" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1990" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1991">
+      <c r="A1991" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1991" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:40</t>
+        </is>
+      </c>
+      <c r="C1991" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1991" s="2">
+        <v>30.2</v>
+      </c>
+      <c r="E1991" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F1991" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1991" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1992">
+      <c r="A1992" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1992" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:50</t>
+        </is>
+      </c>
+      <c r="C1992" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1992" s="2">
+        <v>30.7</v>
+      </c>
+      <c r="E1992" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="F1992" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1992" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1993">
+      <c r="A1993" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1993" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:00</t>
+        </is>
+      </c>
+      <c r="C1993" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1993" s="2">
+        <v>30.2</v>
+      </c>
+      <c r="E1993" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F1993" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1993" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1994">
+      <c r="A1994" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1994" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:10</t>
+        </is>
+      </c>
+      <c r="C1994" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1994" s="2">
+        <v>29.8</v>
+      </c>
+      <c r="E1994" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F1994" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1994" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1995">
+      <c r="A1995" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1995" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:20</t>
+        </is>
+      </c>
+      <c r="C1995" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1995" s="2">
+        <v>30.2</v>
+      </c>
+      <c r="E1995" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F1995" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1995" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1996">
+      <c r="A1996" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1996" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:30</t>
+        </is>
+      </c>
+      <c r="C1996" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1996" s="2">
+        <v>30.3</v>
+      </c>
+      <c r="E1996" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F1996" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1996" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1997">
+      <c r="A1997" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1997" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:40</t>
+        </is>
+      </c>
+      <c r="C1997" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1997" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="E1997" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F1997" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1997" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1998">
+      <c r="A1998" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1998" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:50</t>
+        </is>
+      </c>
+      <c r="C1998" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1998" s="2">
+        <v>29.8</v>
+      </c>
+      <c r="E1998" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F1998" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1998" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="1999">
+      <c r="A1999" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B1999" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:00</t>
+        </is>
+      </c>
+      <c r="C1999" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D1999" s="2">
+        <v>29.7</v>
+      </c>
+      <c r="E1999" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F1999" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G1999" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2000">
+      <c r="A2000" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2000" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:10</t>
+        </is>
+      </c>
+      <c r="C2000" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2000" s="2">
+        <v>29.5</v>
+      </c>
+      <c r="E2000" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F2000" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2000" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2001">
+      <c r="A2001" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2001" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:20</t>
+        </is>
+      </c>
+      <c r="C2001" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2001" s="2">
+        <v>29.7</v>
+      </c>
+      <c r="E2001" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F2001" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2001" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2002">
+      <c r="A2002" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2002" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:30</t>
+        </is>
+      </c>
+      <c r="C2002" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2002" s="2">
+        <v>29.7</v>
+      </c>
+      <c r="E2002" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F2002" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2002" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2003">
+      <c r="A2003" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2003" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:40</t>
+        </is>
+      </c>
+      <c r="C2003" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2003" s="2">
+        <v>29.8</v>
+      </c>
+      <c r="E2003" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F2003" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2003" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2004">
+      <c r="A2004" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2004" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:50</t>
+        </is>
+      </c>
+      <c r="C2004" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2004" s="2">
+        <v>29.9</v>
+      </c>
+      <c r="E2004" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F2004" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2004" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2005">
+      <c r="A2005" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2005" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:00</t>
+        </is>
+      </c>
+      <c r="C2005" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2005" s="2">
+        <v>30.2</v>
+      </c>
+      <c r="E2005" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F2005" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2005" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2006">
+      <c r="A2006" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2006" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:10</t>
+        </is>
+      </c>
+      <c r="C2006" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2006" s="2">
+        <v>30.1</v>
+      </c>
+      <c r="E2006" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F2006" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2006" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2007">
+      <c r="A2007" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2007" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:20</t>
+        </is>
+      </c>
+      <c r="C2007" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2007" s="2">
+        <v>29.9</v>
+      </c>
+      <c r="E2007" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F2007" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2007" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2008">
+      <c r="A2008" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2008" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:30</t>
+        </is>
+      </c>
+      <c r="C2008" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2008" s="2">
+        <v>30.1</v>
+      </c>
+      <c r="E2008" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F2008" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2008" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2009">
+      <c r="A2009" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2009" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:40</t>
+        </is>
+      </c>
+      <c r="C2009" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2009" s="2">
+        <v>30.8</v>
+      </c>
+      <c r="E2009" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F2009" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2009" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2010">
+      <c r="A2010" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2010" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:50</t>
+        </is>
+      </c>
+      <c r="C2010" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2010" s="2">
+        <v>30.8</v>
+      </c>
+      <c r="E2010" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F2010" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2010" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2011">
+      <c r="A2011" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2011" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:00</t>
+        </is>
+      </c>
+      <c r="C2011" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2011" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="E2011" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F2011" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2011" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2012">
+      <c r="A2012" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2012" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:10</t>
+        </is>
+      </c>
+      <c r="C2012" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2012" s="2">
+        <v>31.5</v>
+      </c>
+      <c r="E2012" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F2012" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2012" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2013">
+      <c r="A2013" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2013" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:20</t>
+        </is>
+      </c>
+      <c r="C2013" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2013" s="2">
+        <v>31.2</v>
+      </c>
+      <c r="E2013" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F2013" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2013" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2014">
+      <c r="A2014" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2014" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:30</t>
+        </is>
+      </c>
+      <c r="C2014" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2014" s="2">
+        <v>31.3</v>
+      </c>
+      <c r="E2014" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F2014" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2014" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2015">
+      <c r="A2015" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2015" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:40</t>
+        </is>
+      </c>
+      <c r="C2015" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2015" s="2">
+        <v>31.2</v>
+      </c>
+      <c r="E2015" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F2015" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2015" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2016">
+      <c r="A2016" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2016" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:50</t>
+        </is>
+      </c>
+      <c r="C2016" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2016" s="2">
+        <v>31.4</v>
+      </c>
+      <c r="E2016" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F2016" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2016" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2017">
+      <c r="A2017" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2017" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:00</t>
+        </is>
+      </c>
+      <c r="C2017" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2017" s="2">
+        <v>31.1</v>
+      </c>
+      <c r="E2017" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F2017" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2017" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2018">
+      <c r="A2018" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2018" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:10</t>
+        </is>
+      </c>
+      <c r="C2018" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2018" s="2">
+        <v>30.5</v>
+      </c>
+      <c r="E2018" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F2018" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2018" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2019">
+      <c r="A2019" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2019" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:20</t>
+        </is>
+      </c>
+      <c r="C2019" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2019" s="2">
+        <v>30.1</v>
+      </c>
+      <c r="E2019" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F2019" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2019" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2020">
+      <c r="A2020" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2020" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:30</t>
+        </is>
+      </c>
+      <c r="C2020" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2020" s="2">
+        <v>29.9</v>
+      </c>
+      <c r="E2020" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F2020" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2020" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2021">
+      <c r="A2021" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2021" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:40</t>
+        </is>
+      </c>
+      <c r="C2021" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2021" s="2">
+        <v>29.7</v>
+      </c>
+      <c r="E2021" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="F2021" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2021" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2022">
+      <c r="A2022" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2022" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:50</t>
+        </is>
+      </c>
+      <c r="C2022" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2022" s="2">
+        <v>29.5</v>
+      </c>
+      <c r="E2022" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="F2022" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2022" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2023">
+      <c r="A2023" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2023" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:00</t>
+        </is>
+      </c>
+      <c r="C2023" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2023" s="2">
+        <v>29.3</v>
+      </c>
+      <c r="E2023" s="2">
+        <v>37.0</v>
+      </c>
+      <c r="F2023" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2023" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2024">
+      <c r="A2024" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2024" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:10</t>
+        </is>
+      </c>
+      <c r="C2024" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2024" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="E2024" s="2">
+        <v>38.0</v>
+      </c>
+      <c r="F2024" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2024" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2025">
+      <c r="A2025" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2025" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:20</t>
+        </is>
+      </c>
+      <c r="C2025" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2025" s="2">
+        <v>28.8</v>
+      </c>
+      <c r="E2025" s="2">
+        <v>38.0</v>
+      </c>
+      <c r="F2025" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2025" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2026">
+      <c r="A2026" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2026" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:30</t>
+        </is>
+      </c>
+      <c r="C2026" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2026" s="2">
+        <v>28.3</v>
+      </c>
+      <c r="E2026" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F2026" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2026" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2027">
+      <c r="A2027" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2027" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:40</t>
+        </is>
+      </c>
+      <c r="C2027" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2027" s="2">
+        <v>27.6</v>
+      </c>
+      <c r="E2027" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F2027" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2027" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2028">
+      <c r="A2028" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2028" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:50</t>
+        </is>
+      </c>
+      <c r="C2028" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2028" s="2">
+        <v>27.3</v>
+      </c>
+      <c r="E2028" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F2028" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2028" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2029">
+      <c r="A2029" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2029" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:00</t>
+        </is>
+      </c>
+      <c r="C2029" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2029" s="2">
+        <v>26.9</v>
+      </c>
+      <c r="E2029" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F2029" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2029" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2030">
+      <c r="A2030" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2030" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:10</t>
+        </is>
+      </c>
+      <c r="C2030" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2030" s="2">
+        <v>26.5</v>
+      </c>
+      <c r="E2030" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F2030" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2030" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2031">
+      <c r="A2031" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2031" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:20</t>
+        </is>
+      </c>
+      <c r="C2031" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2031" s="2">
+        <v>26.1</v>
+      </c>
+      <c r="E2031" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F2031" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2031" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2032">
+      <c r="A2032" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2032" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:30</t>
+        </is>
+      </c>
+      <c r="C2032" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2032" s="2">
+        <v>25.6</v>
+      </c>
+      <c r="E2032" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F2032" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2032" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2033">
+      <c r="A2033" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2033" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:40</t>
+        </is>
+      </c>
+      <c r="C2033" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2033" s="2">
+        <v>24.9</v>
+      </c>
+      <c r="E2033" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F2033" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2033" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2034">
+      <c r="A2034" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2034" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:50</t>
+        </is>
+      </c>
+      <c r="C2034" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2034" s="2">
+        <v>24.2</v>
+      </c>
+      <c r="E2034" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F2034" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2034" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2035">
+      <c r="A2035" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2035" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:00</t>
+        </is>
+      </c>
+      <c r="C2035" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2035" s="2">
+        <v>23.8</v>
+      </c>
+      <c r="E2035" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F2035" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2035" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2036">
+      <c r="A2036" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2036" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:10</t>
+        </is>
+      </c>
+      <c r="C2036" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2036" s="2">
+        <v>23.5</v>
+      </c>
+      <c r="E2036" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F2036" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2036" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2037">
+      <c r="A2037" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2037" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:20</t>
+        </is>
+      </c>
+      <c r="C2037" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2037" s="2">
+        <v>23.1</v>
+      </c>
+      <c r="E2037" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F2037" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2037" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2038">
+      <c r="A2038" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2038" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:30</t>
+        </is>
+      </c>
+      <c r="C2038" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2038" s="2">
+        <v>22.7</v>
+      </c>
+      <c r="E2038" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2038" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2038" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2039">
+      <c r="A2039" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2039" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:40</t>
+        </is>
+      </c>
+      <c r="C2039" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2039" s="2">
+        <v>22.3</v>
+      </c>
+      <c r="E2039" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2039" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2039" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2040">
+      <c r="A2040" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2040" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:50</t>
+        </is>
+      </c>
+      <c r="C2040" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2040" s="2">
+        <v>21.9</v>
+      </c>
+      <c r="E2040" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F2040" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2040" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2041">
+      <c r="A2041" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2041" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:00</t>
+        </is>
+      </c>
+      <c r="C2041" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2041" s="2">
+        <v>21.6</v>
+      </c>
+      <c r="E2041" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F2041" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2041" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2042">
+      <c r="A2042" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2042" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:10</t>
+        </is>
+      </c>
+      <c r="C2042" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2042" s="2">
+        <v>21.4</v>
+      </c>
+      <c r="E2042" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F2042" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2042" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2043">
+      <c r="A2043" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2043" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:20</t>
+        </is>
+      </c>
+      <c r="C2043" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2043" s="2">
+        <v>21.1</v>
+      </c>
+      <c r="E2043" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F2043" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2043" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2044">
+      <c r="A2044" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2044" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:30</t>
+        </is>
+      </c>
+      <c r="C2044" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2044" s="2">
+        <v>20.8</v>
+      </c>
+      <c r="E2044" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F2044" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2044" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2045">
+      <c r="A2045" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2045" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:40</t>
+        </is>
+      </c>
+      <c r="C2045" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2045" s="2">
+        <v>20.6</v>
+      </c>
+      <c r="E2045" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F2045" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2045" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2046">
+      <c r="A2046" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">28.07.2026</t>
+        </is>
+      </c>
+      <c r="B2046" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:50</t>
+        </is>
+      </c>
+      <c r="C2046" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2046" s="2">
+        <v>20.5</v>
+      </c>
+      <c r="E2046" s="2">
+        <v>72.0</v>
+      </c>
+      <c r="F2046" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2046" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2047">
+      <c r="A2047" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2047" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:00</t>
+        </is>
+      </c>
+      <c r="C2047" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2047" s="2">
+        <v>20.3</v>
+      </c>
+      <c r="E2047" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="F2047" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2047" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2048">
+      <c r="A2048" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2048" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:10</t>
+        </is>
+      </c>
+      <c r="C2048" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2048" s="2">
+        <v>20.2</v>
+      </c>
+      <c r="E2048" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="F2048" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2048" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2049">
+      <c r="A2049" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2049" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:20</t>
+        </is>
+      </c>
+      <c r="C2049" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2049" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="E2049" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="F2049" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2049" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2050">
+      <c r="A2050" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2050" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:30</t>
+        </is>
+      </c>
+      <c r="C2050" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2050" s="2">
+        <v>19.8</v>
+      </c>
+      <c r="E2050" s="2">
+        <v>74.0</v>
+      </c>
+      <c r="F2050" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2050" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G1906"/>
+  <autoFilter ref="A1:G2050"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ARSO Kranj zajem 2026-07-30 00:43 Europe/Ljubljana
</commit_message>
<xml_diff>
--- a/tabela_vremena/ARSO_Kranj.xlsx
+++ b/tabela_vremena/ARSO_Kranj.xlsx
@@ -59532,7 +59532,4183 @@
         <v>0.0</v>
       </c>
     </row>
+    <row r="2051">
+      <c r="A2051" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2051" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:40</t>
+        </is>
+      </c>
+      <c r="C2051" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2051" s="2">
+        <v>19.6</v>
+      </c>
+      <c r="E2051" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F2051" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2051" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2052">
+      <c r="A2052" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2052" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:50</t>
+        </is>
+      </c>
+      <c r="C2052" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2052" s="2">
+        <v>19.5</v>
+      </c>
+      <c r="E2052" s="2">
+        <v>74.0</v>
+      </c>
+      <c r="F2052" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2052" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2053">
+      <c r="A2053" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2053" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:00</t>
+        </is>
+      </c>
+      <c r="C2053" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2053" s="2">
+        <v>19.5</v>
+      </c>
+      <c r="E2053" s="2">
+        <v>74.0</v>
+      </c>
+      <c r="F2053" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2053" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2054">
+      <c r="A2054" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2054" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:10</t>
+        </is>
+      </c>
+      <c r="C2054" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2054" s="2">
+        <v>19.5</v>
+      </c>
+      <c r="E2054" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="F2054" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2054" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2055">
+      <c r="A2055" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2055" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:20</t>
+        </is>
+      </c>
+      <c r="C2055" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2055" s="2">
+        <v>19.4</v>
+      </c>
+      <c r="E2055" s="2">
+        <v>74.0</v>
+      </c>
+      <c r="F2055" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2055" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2056">
+      <c r="A2056" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2056" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:30</t>
+        </is>
+      </c>
+      <c r="C2056" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2056" s="2">
+        <v>19.3</v>
+      </c>
+      <c r="E2056" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F2056" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2056" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2057">
+      <c r="A2057" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2057" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:40</t>
+        </is>
+      </c>
+      <c r="C2057" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2057" s="2">
+        <v>19.1</v>
+      </c>
+      <c r="E2057" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F2057" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2057" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2058">
+      <c r="A2058" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2058" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:50</t>
+        </is>
+      </c>
+      <c r="C2058" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2058" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="E2058" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F2058" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2058" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2059">
+      <c r="A2059" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2059" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:00</t>
+        </is>
+      </c>
+      <c r="C2059" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2059" s="2">
+        <v>18.9</v>
+      </c>
+      <c r="E2059" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F2059" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2059" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2060">
+      <c r="A2060" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2060" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:10</t>
+        </is>
+      </c>
+      <c r="C2060" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2060" s="2">
+        <v>18.8</v>
+      </c>
+      <c r="E2060" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F2060" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2060" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2061">
+      <c r="A2061" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2061" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:20</t>
+        </is>
+      </c>
+      <c r="C2061" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2061" s="2">
+        <v>18.7</v>
+      </c>
+      <c r="E2061" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F2061" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2061" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2062">
+      <c r="A2062" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2062" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:30</t>
+        </is>
+      </c>
+      <c r="C2062" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2062" s="2">
+        <v>18.6</v>
+      </c>
+      <c r="E2062" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F2062" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2062" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2063">
+      <c r="A2063" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2063" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:40</t>
+        </is>
+      </c>
+      <c r="C2063" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2063" s="2">
+        <v>18.4</v>
+      </c>
+      <c r="E2063" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F2063" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2063" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2064">
+      <c r="A2064" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2064" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:50</t>
+        </is>
+      </c>
+      <c r="C2064" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2064" s="2">
+        <v>18.2</v>
+      </c>
+      <c r="E2064" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F2064" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2064" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2065">
+      <c r="A2065" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2065" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:00</t>
+        </is>
+      </c>
+      <c r="C2065" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2065" s="2">
+        <v>18.1</v>
+      </c>
+      <c r="E2065" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F2065" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2065" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2066">
+      <c r="A2066" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2066" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:10</t>
+        </is>
+      </c>
+      <c r="C2066" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2066" s="2">
+        <v>18.1</v>
+      </c>
+      <c r="E2066" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F2066" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2066" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2067">
+      <c r="A2067" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2067" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:20</t>
+        </is>
+      </c>
+      <c r="C2067" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2067" s="2">
+        <v>18.2</v>
+      </c>
+      <c r="E2067" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F2067" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2067" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2068">
+      <c r="A2068" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2068" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:30</t>
+        </is>
+      </c>
+      <c r="C2068" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2068" s="2">
+        <v>18.2</v>
+      </c>
+      <c r="E2068" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F2068" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2068" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2069">
+      <c r="A2069" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2069" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:40</t>
+        </is>
+      </c>
+      <c r="C2069" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2069" s="2">
+        <v>18.1</v>
+      </c>
+      <c r="E2069" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F2069" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2069" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2070">
+      <c r="A2070" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2070" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:50</t>
+        </is>
+      </c>
+      <c r="C2070" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2070" s="2">
+        <v>18.0</v>
+      </c>
+      <c r="E2070" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F2070" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2070" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2071">
+      <c r="A2071" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2071" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:00</t>
+        </is>
+      </c>
+      <c r="C2071" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2071" s="2">
+        <v>17.9</v>
+      </c>
+      <c r="E2071" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F2071" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2071" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2072">
+      <c r="A2072" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2072" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:10</t>
+        </is>
+      </c>
+      <c r="C2072" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2072" s="2">
+        <v>17.9</v>
+      </c>
+      <c r="E2072" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F2072" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2072" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2073">
+      <c r="A2073" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2073" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:20</t>
+        </is>
+      </c>
+      <c r="C2073" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2073" s="2">
+        <v>18.1</v>
+      </c>
+      <c r="E2073" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F2073" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2073" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2074">
+      <c r="A2074" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2074" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:30</t>
+        </is>
+      </c>
+      <c r="C2074" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2074" s="2">
+        <v>18.1</v>
+      </c>
+      <c r="E2074" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F2074" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2074" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2075">
+      <c r="A2075" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2075" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:40</t>
+        </is>
+      </c>
+      <c r="C2075" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2075" s="2">
+        <v>17.9</v>
+      </c>
+      <c r="E2075" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F2075" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2075" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2076">
+      <c r="A2076" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2076" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:50</t>
+        </is>
+      </c>
+      <c r="C2076" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2076" s="2">
+        <v>17.4</v>
+      </c>
+      <c r="E2076" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F2076" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2076" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2077">
+      <c r="A2077" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2077" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:00</t>
+        </is>
+      </c>
+      <c r="C2077" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2077" s="2">
+        <v>17.1</v>
+      </c>
+      <c r="E2077" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F2077" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2077" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2078">
+      <c r="A2078" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2078" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:10</t>
+        </is>
+      </c>
+      <c r="C2078" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2078" s="2">
+        <v>16.6</v>
+      </c>
+      <c r="E2078" s="2">
+        <v>84.0</v>
+      </c>
+      <c r="F2078" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2078" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2079">
+      <c r="A2079" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2079" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:20</t>
+        </is>
+      </c>
+      <c r="C2079" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2079" s="2">
+        <v>16.5</v>
+      </c>
+      <c r="E2079" s="2">
+        <v>84.0</v>
+      </c>
+      <c r="F2079" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2079" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2080">
+      <c r="A2080" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2080" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:30</t>
+        </is>
+      </c>
+      <c r="C2080" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2080" s="2">
+        <v>16.6</v>
+      </c>
+      <c r="E2080" s="2">
+        <v>84.0</v>
+      </c>
+      <c r="F2080" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2080" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2081">
+      <c r="A2081" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2081" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:40</t>
+        </is>
+      </c>
+      <c r="C2081" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2081" s="2">
+        <v>16.3</v>
+      </c>
+      <c r="E2081" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F2081" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2081" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2082">
+      <c r="A2082" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2082" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:50</t>
+        </is>
+      </c>
+      <c r="C2082" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2082" s="2">
+        <v>16.3</v>
+      </c>
+      <c r="E2082" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F2082" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2082" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2083">
+      <c r="A2083" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2083" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:00</t>
+        </is>
+      </c>
+      <c r="C2083" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2083" s="2">
+        <v>16.4</v>
+      </c>
+      <c r="E2083" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F2083" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2083" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2084">
+      <c r="A2084" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2084" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:10</t>
+        </is>
+      </c>
+      <c r="C2084" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2084" s="2">
+        <v>16.3</v>
+      </c>
+      <c r="E2084" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F2084" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2084" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2085">
+      <c r="A2085" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2085" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:20</t>
+        </is>
+      </c>
+      <c r="C2085" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2085" s="2">
+        <v>16.4</v>
+      </c>
+      <c r="E2085" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F2085" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2085" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2086">
+      <c r="A2086" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2086" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:30</t>
+        </is>
+      </c>
+      <c r="C2086" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2086" s="2">
+        <v>16.4</v>
+      </c>
+      <c r="E2086" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F2086" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2086" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2087">
+      <c r="A2087" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2087" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:40</t>
+        </is>
+      </c>
+      <c r="C2087" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2087" s="2">
+        <v>16.6</v>
+      </c>
+      <c r="E2087" s="2">
+        <v>85.0</v>
+      </c>
+      <c r="F2087" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2087" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2088">
+      <c r="A2088" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2088" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:50</t>
+        </is>
+      </c>
+      <c r="C2088" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2088" s="2">
+        <v>17.0</v>
+      </c>
+      <c r="E2088" s="2">
+        <v>83.0</v>
+      </c>
+      <c r="F2088" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2088" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2089">
+      <c r="A2089" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2089" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:00</t>
+        </is>
+      </c>
+      <c r="C2089" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2089" s="2">
+        <v>17.7</v>
+      </c>
+      <c r="E2089" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F2089" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2089" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2090">
+      <c r="A2090" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2090" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:10</t>
+        </is>
+      </c>
+      <c r="C2090" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2090" s="2">
+        <v>18.2</v>
+      </c>
+      <c r="E2090" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F2090" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2090" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2091">
+      <c r="A2091" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2091" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:20</t>
+        </is>
+      </c>
+      <c r="C2091" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2091" s="2">
+        <v>19.4</v>
+      </c>
+      <c r="E2091" s="2">
+        <v>74.0</v>
+      </c>
+      <c r="F2091" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2091" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2092">
+      <c r="A2092" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2092" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:30</t>
+        </is>
+      </c>
+      <c r="C2092" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2092" s="2">
+        <v>19.3</v>
+      </c>
+      <c r="E2092" s="2">
+        <v>74.0</v>
+      </c>
+      <c r="F2092" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2092" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2093">
+      <c r="A2093" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2093" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:40</t>
+        </is>
+      </c>
+      <c r="C2093" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2093" s="2">
+        <v>19.6</v>
+      </c>
+      <c r="E2093" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="F2093" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2093" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2094">
+      <c r="A2094" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2094" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:50</t>
+        </is>
+      </c>
+      <c r="C2094" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2094" s="2">
+        <v>20.2</v>
+      </c>
+      <c r="E2094" s="2">
+        <v>69.0</v>
+      </c>
+      <c r="F2094" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2094" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2095">
+      <c r="A2095" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2095" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:00</t>
+        </is>
+      </c>
+      <c r="C2095" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2095" s="2">
+        <v>20.5</v>
+      </c>
+      <c r="E2095" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F2095" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2095" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2096">
+      <c r="A2096" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2096" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:10</t>
+        </is>
+      </c>
+      <c r="C2096" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2096" s="2">
+        <v>20.7</v>
+      </c>
+      <c r="E2096" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F2096" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2096" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2097">
+      <c r="A2097" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2097" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:20</t>
+        </is>
+      </c>
+      <c r="C2097" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2097" s="2">
+        <v>21.4</v>
+      </c>
+      <c r="E2097" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2097" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2097" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2098">
+      <c r="A2098" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2098" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:30</t>
+        </is>
+      </c>
+      <c r="C2098" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2098" s="2">
+        <v>21.7</v>
+      </c>
+      <c r="E2098" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2098" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2098" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2099">
+      <c r="A2099" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2099" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:40</t>
+        </is>
+      </c>
+      <c r="C2099" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2099" s="2">
+        <v>22.2</v>
+      </c>
+      <c r="E2099" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F2099" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2099" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2100">
+      <c r="A2100" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2100" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:50</t>
+        </is>
+      </c>
+      <c r="C2100" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2100" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="E2100" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F2100" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2100" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2101">
+      <c r="A2101" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2101" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:00</t>
+        </is>
+      </c>
+      <c r="C2101" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2101" s="2">
+        <v>23.1</v>
+      </c>
+      <c r="E2101" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2101" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2101" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2102">
+      <c r="A2102" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2102" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:10</t>
+        </is>
+      </c>
+      <c r="C2102" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2102" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="E2102" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F2102" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2102" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2103">
+      <c r="A2103" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2103" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:20</t>
+        </is>
+      </c>
+      <c r="C2103" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2103" s="2">
+        <v>24.6</v>
+      </c>
+      <c r="E2103" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F2103" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2103" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2104">
+      <c r="A2104" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2104" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:30</t>
+        </is>
+      </c>
+      <c r="C2104" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2104" s="2">
+        <v>24.9</v>
+      </c>
+      <c r="E2104" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F2104" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2104" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2105">
+      <c r="A2105" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2105" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:40</t>
+        </is>
+      </c>
+      <c r="C2105" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2105" s="2">
+        <v>25.3</v>
+      </c>
+      <c r="E2105" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F2105" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2105" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2106">
+      <c r="A2106" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2106" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:50</t>
+        </is>
+      </c>
+      <c r="C2106" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2106" s="2">
+        <v>25.6</v>
+      </c>
+      <c r="E2106" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F2106" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2106" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2107">
+      <c r="A2107" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2107" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:00</t>
+        </is>
+      </c>
+      <c r="C2107" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2107" s="2">
+        <v>26.2</v>
+      </c>
+      <c r="E2107" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F2107" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2107" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2108">
+      <c r="A2108" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2108" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:10</t>
+        </is>
+      </c>
+      <c r="C2108" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2108" s="2">
+        <v>26.7</v>
+      </c>
+      <c r="E2108" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F2108" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2108" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2109">
+      <c r="A2109" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2109" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:20</t>
+        </is>
+      </c>
+      <c r="C2109" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2109" s="2">
+        <v>27.4</v>
+      </c>
+      <c r="E2109" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F2109" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2109" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2110">
+      <c r="A2110" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2110" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:30</t>
+        </is>
+      </c>
+      <c r="C2110" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2110" s="2">
+        <v>27.3</v>
+      </c>
+      <c r="E2110" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F2110" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2110" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2111">
+      <c r="A2111" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2111" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:40</t>
+        </is>
+      </c>
+      <c r="C2111" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2111" s="2">
+        <v>27.8</v>
+      </c>
+      <c r="E2111" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F2111" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2111" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2112">
+      <c r="A2112" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2112" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:50</t>
+        </is>
+      </c>
+      <c r="C2112" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2112" s="2">
+        <v>28.7</v>
+      </c>
+      <c r="E2112" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F2112" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2112" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2113">
+      <c r="A2113" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2113" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:00</t>
+        </is>
+      </c>
+      <c r="C2113" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2113" s="2">
+        <v>28.7</v>
+      </c>
+      <c r="E2113" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F2113" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2113" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2114">
+      <c r="A2114" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2114" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:10</t>
+        </is>
+      </c>
+      <c r="C2114" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2114" s="2">
+        <v>29.4</v>
+      </c>
+      <c r="E2114" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F2114" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2114" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2115">
+      <c r="A2115" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2115" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:20</t>
+        </is>
+      </c>
+      <c r="C2115" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2115" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="E2115" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F2115" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2115" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2116">
+      <c r="A2116" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2116" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:30</t>
+        </is>
+      </c>
+      <c r="C2116" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2116" s="2">
+        <v>30.4</v>
+      </c>
+      <c r="E2116" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F2116" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2116" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2117">
+      <c r="A2117" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2117" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:40</t>
+        </is>
+      </c>
+      <c r="C2117" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2117" s="2">
+        <v>29.8</v>
+      </c>
+      <c r="E2117" s="2">
+        <v>38.0</v>
+      </c>
+      <c r="F2117" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2117" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2118">
+      <c r="A2118" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2118" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:50</t>
+        </is>
+      </c>
+      <c r="C2118" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2118" s="2">
+        <v>30.6</v>
+      </c>
+      <c r="E2118" s="2">
+        <v>38.0</v>
+      </c>
+      <c r="F2118" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2118" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2119">
+      <c r="A2119" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2119" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:00</t>
+        </is>
+      </c>
+      <c r="C2119" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2119" s="2">
+        <v>30.6</v>
+      </c>
+      <c r="E2119" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F2119" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2119" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2120">
+      <c r="A2120" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2120" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:10</t>
+        </is>
+      </c>
+      <c r="C2120" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2120" s="2">
+        <v>30.8</v>
+      </c>
+      <c r="E2120" s="2">
+        <v>37.0</v>
+      </c>
+      <c r="F2120" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2120" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2121">
+      <c r="A2121" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2121" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:20</t>
+        </is>
+      </c>
+      <c r="C2121" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2121" s="2">
+        <v>31.4</v>
+      </c>
+      <c r="E2121" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F2121" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2121" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2122">
+      <c r="A2122" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2122" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:30</t>
+        </is>
+      </c>
+      <c r="C2122" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2122" s="2">
+        <v>32.1</v>
+      </c>
+      <c r="E2122" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F2122" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2122" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2123">
+      <c r="A2123" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2123" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:40</t>
+        </is>
+      </c>
+      <c r="C2123" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2123" s="2">
+        <v>31.9</v>
+      </c>
+      <c r="E2123" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F2123" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2123" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2124">
+      <c r="A2124" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2124" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:50</t>
+        </is>
+      </c>
+      <c r="C2124" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2124" s="2">
+        <v>32.2</v>
+      </c>
+      <c r="E2124" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F2124" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2124" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2125">
+      <c r="A2125" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2125" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:00</t>
+        </is>
+      </c>
+      <c r="C2125" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2125" s="2">
+        <v>32.4</v>
+      </c>
+      <c r="E2125" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F2125" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2125" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2126">
+      <c r="A2126" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2126" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:10</t>
+        </is>
+      </c>
+      <c r="C2126" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2126" s="2">
+        <v>33.2</v>
+      </c>
+      <c r="E2126" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F2126" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2126" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2127">
+      <c r="A2127" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2127" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:20</t>
+        </is>
+      </c>
+      <c r="C2127" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2127" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="E2127" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2127" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2127" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2128">
+      <c r="A2128" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2128" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:30</t>
+        </is>
+      </c>
+      <c r="C2128" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2128" s="2">
+        <v>33.3</v>
+      </c>
+      <c r="E2128" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2128" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2128" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2129">
+      <c r="A2129" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2129" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:40</t>
+        </is>
+      </c>
+      <c r="C2129" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2129" s="2">
+        <v>33.2</v>
+      </c>
+      <c r="E2129" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2129" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2129" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2130">
+      <c r="A2130" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2130" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:50</t>
+        </is>
+      </c>
+      <c r="C2130" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2130" s="2">
+        <v>33.3</v>
+      </c>
+      <c r="E2130" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F2130" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2130" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2131">
+      <c r="A2131" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2131" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:00</t>
+        </is>
+      </c>
+      <c r="C2131" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2131" s="2">
+        <v>33.5</v>
+      </c>
+      <c r="E2131" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F2131" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2131" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2132">
+      <c r="A2132" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2132" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:10</t>
+        </is>
+      </c>
+      <c r="C2132" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2132" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="E2132" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2132" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2132" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2133">
+      <c r="A2133" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2133" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:20</t>
+        </is>
+      </c>
+      <c r="C2133" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2133" s="2">
+        <v>34.2</v>
+      </c>
+      <c r="E2133" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2133" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2133" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2134">
+      <c r="A2134" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2134" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:30</t>
+        </is>
+      </c>
+      <c r="C2134" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2134" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="E2134" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F2134" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2134" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2135">
+      <c r="A2135" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2135" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:40</t>
+        </is>
+      </c>
+      <c r="C2135" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2135" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="E2135" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F2135" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2135" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2136">
+      <c r="A2136" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2136" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:50</t>
+        </is>
+      </c>
+      <c r="C2136" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2136" s="2">
+        <v>33.9</v>
+      </c>
+      <c r="E2136" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2136" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2136" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2137">
+      <c r="A2137" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2137" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:00</t>
+        </is>
+      </c>
+      <c r="C2137" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2137" s="2">
+        <v>34.5</v>
+      </c>
+      <c r="E2137" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2137" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2137" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2138">
+      <c r="A2138" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2138" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:10</t>
+        </is>
+      </c>
+      <c r="C2138" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2138" s="2">
+        <v>34.8</v>
+      </c>
+      <c r="E2138" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2138" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2138" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2139">
+      <c r="A2139" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2139" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:20</t>
+        </is>
+      </c>
+      <c r="C2139" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2139" s="2">
+        <v>34.3</v>
+      </c>
+      <c r="E2139" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2139" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2139" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2140">
+      <c r="A2140" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2140" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:30</t>
+        </is>
+      </c>
+      <c r="C2140" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2140" s="2">
+        <v>34.7</v>
+      </c>
+      <c r="E2140" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2140" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2140" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2141">
+      <c r="A2141" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2141" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:40</t>
+        </is>
+      </c>
+      <c r="C2141" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2141" s="2">
+        <v>33.8</v>
+      </c>
+      <c r="E2141" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2141" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2141" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2142">
+      <c r="A2142" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2142" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:50</t>
+        </is>
+      </c>
+      <c r="C2142" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2142" s="2">
+        <v>33.6</v>
+      </c>
+      <c r="E2142" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2142" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2142" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2143">
+      <c r="A2143" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2143" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:00</t>
+        </is>
+      </c>
+      <c r="C2143" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2143" s="2">
+        <v>33.8</v>
+      </c>
+      <c r="E2143" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2143" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2143" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2144">
+      <c r="A2144" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2144" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:10</t>
+        </is>
+      </c>
+      <c r="C2144" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2144" s="2">
+        <v>34.1</v>
+      </c>
+      <c r="E2144" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2144" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2144" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2145">
+      <c r="A2145" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2145" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:20</t>
+        </is>
+      </c>
+      <c r="C2145" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2145" s="2">
+        <v>33.7</v>
+      </c>
+      <c r="E2145" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2145" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2145" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2146">
+      <c r="A2146" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2146" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:30</t>
+        </is>
+      </c>
+      <c r="C2146" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2146" s="2">
+        <v>33.6</v>
+      </c>
+      <c r="E2146" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2146" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2146" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2147">
+      <c r="A2147" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2147" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:40</t>
+        </is>
+      </c>
+      <c r="C2147" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2147" s="2">
+        <v>33.7</v>
+      </c>
+      <c r="E2147" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2147" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2147" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2148">
+      <c r="A2148" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2148" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:50</t>
+        </is>
+      </c>
+      <c r="C2148" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2148" s="2">
+        <v>33.9</v>
+      </c>
+      <c r="E2148" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2148" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2148" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2149">
+      <c r="A2149" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2149" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:00</t>
+        </is>
+      </c>
+      <c r="C2149" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2149" s="2">
+        <v>33.7</v>
+      </c>
+      <c r="E2149" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2149" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2149" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2150">
+      <c r="A2150" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2150" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:10</t>
+        </is>
+      </c>
+      <c r="C2150" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2150" s="2">
+        <v>34.1</v>
+      </c>
+      <c r="E2150" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2150" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2150" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2151">
+      <c r="A2151" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2151" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:20</t>
+        </is>
+      </c>
+      <c r="C2151" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2151" s="2">
+        <v>34.1</v>
+      </c>
+      <c r="E2151" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2151" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2151" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2152">
+      <c r="A2152" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2152" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:30</t>
+        </is>
+      </c>
+      <c r="C2152" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2152" s="2">
+        <v>34.2</v>
+      </c>
+      <c r="E2152" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2152" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2152" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2153">
+      <c r="A2153" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2153" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:40</t>
+        </is>
+      </c>
+      <c r="C2153" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2153" s="2">
+        <v>34.3</v>
+      </c>
+      <c r="E2153" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2153" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2153" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2154">
+      <c r="A2154" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2154" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:50</t>
+        </is>
+      </c>
+      <c r="C2154" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2154" s="2">
+        <v>34.8</v>
+      </c>
+      <c r="E2154" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2154" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2154" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2155">
+      <c r="A2155" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2155" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:00</t>
+        </is>
+      </c>
+      <c r="C2155" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2155" s="2">
+        <v>34.8</v>
+      </c>
+      <c r="E2155" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2155" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2155" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2156">
+      <c r="A2156" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2156" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:10</t>
+        </is>
+      </c>
+      <c r="C2156" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2156" s="2">
+        <v>35.2</v>
+      </c>
+      <c r="E2156" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2156" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2156" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2157">
+      <c r="A2157" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2157" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:20</t>
+        </is>
+      </c>
+      <c r="C2157" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2157" s="2">
+        <v>34.6</v>
+      </c>
+      <c r="E2157" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2157" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2157" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2158">
+      <c r="A2158" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2158" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:30</t>
+        </is>
+      </c>
+      <c r="C2158" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2158" s="2">
+        <v>34.3</v>
+      </c>
+      <c r="E2158" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2158" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2158" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2159">
+      <c r="A2159" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2159" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:40</t>
+        </is>
+      </c>
+      <c r="C2159" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2159" s="2">
+        <v>34.5</v>
+      </c>
+      <c r="E2159" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2159" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2159" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2160">
+      <c r="A2160" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2160" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:50</t>
+        </is>
+      </c>
+      <c r="C2160" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2160" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="E2160" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2160" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2160" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2161">
+      <c r="A2161" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2161" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:00</t>
+        </is>
+      </c>
+      <c r="C2161" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2161" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="E2161" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2161" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2161" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2162">
+      <c r="A2162" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2162" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:10</t>
+        </is>
+      </c>
+      <c r="C2162" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2162" s="2">
+        <v>33.2</v>
+      </c>
+      <c r="E2162" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2162" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2162" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2163">
+      <c r="A2163" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2163" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:20</t>
+        </is>
+      </c>
+      <c r="C2163" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2163" s="2">
+        <v>32.8</v>
+      </c>
+      <c r="E2163" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F2163" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2163" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2164">
+      <c r="A2164" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2164" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:30</t>
+        </is>
+      </c>
+      <c r="C2164" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2164" s="2">
+        <v>32.4</v>
+      </c>
+      <c r="E2164" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="F2164" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2164" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2165">
+      <c r="A2165" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2165" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:40</t>
+        </is>
+      </c>
+      <c r="C2165" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2165" s="2">
+        <v>31.8</v>
+      </c>
+      <c r="E2165" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="F2165" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2165" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2166">
+      <c r="A2166" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2166" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:50</t>
+        </is>
+      </c>
+      <c r="C2166" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2166" s="2">
+        <v>31.3</v>
+      </c>
+      <c r="E2166" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F2166" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2166" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2167">
+      <c r="A2167" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2167" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:00</t>
+        </is>
+      </c>
+      <c r="C2167" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2167" s="2">
+        <v>30.8</v>
+      </c>
+      <c r="E2167" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F2167" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2167" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2168">
+      <c r="A2168" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2168" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:10</t>
+        </is>
+      </c>
+      <c r="C2168" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2168" s="2">
+        <v>30.5</v>
+      </c>
+      <c r="E2168" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F2168" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2168" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2169">
+      <c r="A2169" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2169" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:20</t>
+        </is>
+      </c>
+      <c r="C2169" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2169" s="2">
+        <v>29.9</v>
+      </c>
+      <c r="E2169" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="F2169" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2169" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2170">
+      <c r="A2170" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2170" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:30</t>
+        </is>
+      </c>
+      <c r="C2170" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2170" s="2">
+        <v>29.3</v>
+      </c>
+      <c r="E2170" s="2">
+        <v>38.0</v>
+      </c>
+      <c r="F2170" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2170" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2171">
+      <c r="A2171" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2171" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:40</t>
+        </is>
+      </c>
+      <c r="C2171" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2171" s="2">
+        <v>28.8</v>
+      </c>
+      <c r="E2171" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F2171" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2171" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2172">
+      <c r="A2172" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2172" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:50</t>
+        </is>
+      </c>
+      <c r="C2172" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2172" s="2">
+        <v>28.5</v>
+      </c>
+      <c r="E2172" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F2172" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2172" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2173">
+      <c r="A2173" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2173" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:00</t>
+        </is>
+      </c>
+      <c r="C2173" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2173" s="2">
+        <v>27.8</v>
+      </c>
+      <c r="E2173" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F2173" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2173" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2174">
+      <c r="A2174" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2174" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:10</t>
+        </is>
+      </c>
+      <c r="C2174" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2174" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="E2174" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F2174" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2174" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2175">
+      <c r="A2175" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2175" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:20</t>
+        </is>
+      </c>
+      <c r="C2175" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2175" s="2">
+        <v>26.6</v>
+      </c>
+      <c r="E2175" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F2175" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2175" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2176">
+      <c r="A2176" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2176" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:30</t>
+        </is>
+      </c>
+      <c r="C2176" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2176" s="2">
+        <v>26.2</v>
+      </c>
+      <c r="E2176" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F2176" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2176" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2177">
+      <c r="A2177" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2177" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:40</t>
+        </is>
+      </c>
+      <c r="C2177" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2177" s="2">
+        <v>25.9</v>
+      </c>
+      <c r="E2177" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F2177" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2177" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2178">
+      <c r="A2178" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2178" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:50</t>
+        </is>
+      </c>
+      <c r="C2178" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2178" s="2">
+        <v>25.4</v>
+      </c>
+      <c r="E2178" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F2178" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2178" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2179">
+      <c r="A2179" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2179" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:00</t>
+        </is>
+      </c>
+      <c r="C2179" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2179" s="2">
+        <v>24.9</v>
+      </c>
+      <c r="E2179" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F2179" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2179" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2180">
+      <c r="A2180" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2180" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:10</t>
+        </is>
+      </c>
+      <c r="C2180" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2180" s="2">
+        <v>24.5</v>
+      </c>
+      <c r="E2180" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F2180" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2180" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2181">
+      <c r="A2181" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2181" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:20</t>
+        </is>
+      </c>
+      <c r="C2181" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2181" s="2">
+        <v>24.4</v>
+      </c>
+      <c r="E2181" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F2181" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2181" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2182">
+      <c r="A2182" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2182" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:30</t>
+        </is>
+      </c>
+      <c r="C2182" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2182" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="E2182" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F2182" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2182" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2183">
+      <c r="A2183" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2183" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:40</t>
+        </is>
+      </c>
+      <c r="C2183" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2183" s="2">
+        <v>23.7</v>
+      </c>
+      <c r="E2183" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F2183" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2183" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2184">
+      <c r="A2184" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2184" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:50</t>
+        </is>
+      </c>
+      <c r="C2184" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2184" s="2">
+        <v>23.5</v>
+      </c>
+      <c r="E2184" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F2184" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2184" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2185">
+      <c r="A2185" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2185" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:00</t>
+        </is>
+      </c>
+      <c r="C2185" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2185" s="2">
+        <v>23.2</v>
+      </c>
+      <c r="E2185" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2185" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2185" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2186">
+      <c r="A2186" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2186" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:10</t>
+        </is>
+      </c>
+      <c r="C2186" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2186" s="2">
+        <v>23.2</v>
+      </c>
+      <c r="E2186" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2186" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2186" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2187">
+      <c r="A2187" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2187" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:20</t>
+        </is>
+      </c>
+      <c r="C2187" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2187" s="2">
+        <v>22.9</v>
+      </c>
+      <c r="E2187" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2187" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2187" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2188">
+      <c r="A2188" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2188" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:30</t>
+        </is>
+      </c>
+      <c r="C2188" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2188" s="2">
+        <v>22.6</v>
+      </c>
+      <c r="E2188" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2188" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2188" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2189">
+      <c r="A2189" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2189" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:40</t>
+        </is>
+      </c>
+      <c r="C2189" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2189" s="2">
+        <v>22.4</v>
+      </c>
+      <c r="E2189" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F2189" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2189" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2190">
+      <c r="A2190" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">29.07.2026</t>
+        </is>
+      </c>
+      <c r="B2190" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:50</t>
+        </is>
+      </c>
+      <c r="C2190" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2190" s="2">
+        <v>22.2</v>
+      </c>
+      <c r="E2190" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F2190" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2190" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2191">
+      <c r="A2191" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2191" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:00</t>
+        </is>
+      </c>
+      <c r="C2191" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2191" s="2">
+        <v>21.9</v>
+      </c>
+      <c r="E2191" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F2191" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2191" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2192">
+      <c r="A2192" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2192" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:10</t>
+        </is>
+      </c>
+      <c r="C2192" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2192" s="2">
+        <v>21.7</v>
+      </c>
+      <c r="E2192" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F2192" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2192" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2193">
+      <c r="A2193" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2193" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:20</t>
+        </is>
+      </c>
+      <c r="C2193" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2193" s="2">
+        <v>21.5</v>
+      </c>
+      <c r="E2193" s="2">
+        <v>69.0</v>
+      </c>
+      <c r="F2193" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2193" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2194">
+      <c r="A2194" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2194" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:30</t>
+        </is>
+      </c>
+      <c r="C2194" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2194" s="2">
+        <v>21.5</v>
+      </c>
+      <c r="E2194" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F2194" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2194" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G2050"/>
+  <autoFilter ref="A1:G2194"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ARSO Kranj zajem 2026-07-31 00:49 Europe/Ljubljana
</commit_message>
<xml_diff>
--- a/tabela_vremena/ARSO_Kranj.xlsx
+++ b/tabela_vremena/ARSO_Kranj.xlsx
@@ -63708,7 +63708,4154 @@
         <v>0.0</v>
       </c>
     </row>
+    <row r="2195">
+      <c r="A2195" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2195" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:40</t>
+        </is>
+      </c>
+      <c r="C2195" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2195" s="2">
+        <v>21.2</v>
+      </c>
+      <c r="E2195" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F2195" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2195" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2196">
+      <c r="A2196" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2196" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:50</t>
+        </is>
+      </c>
+      <c r="C2196" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2196" s="2">
+        <v>21.1</v>
+      </c>
+      <c r="E2196" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F2196" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2196" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2197">
+      <c r="A2197" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2197" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:00</t>
+        </is>
+      </c>
+      <c r="C2197" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2197" s="2">
+        <v>20.9</v>
+      </c>
+      <c r="E2197" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F2197" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2197" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2198">
+      <c r="A2198" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2198" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:10</t>
+        </is>
+      </c>
+      <c r="C2198" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2198" s="2">
+        <v>20.9</v>
+      </c>
+      <c r="E2198" s="2">
+        <v>69.0</v>
+      </c>
+      <c r="F2198" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2198" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2199">
+      <c r="A2199" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2199" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:20</t>
+        </is>
+      </c>
+      <c r="C2199" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2199" s="2">
+        <v>20.7</v>
+      </c>
+      <c r="E2199" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F2199" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2199" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2200">
+      <c r="A2200" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2200" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:30</t>
+        </is>
+      </c>
+      <c r="C2200" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2200" s="2">
+        <v>20.5</v>
+      </c>
+      <c r="E2200" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F2200" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2200" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2201">
+      <c r="A2201" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2201" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:40</t>
+        </is>
+      </c>
+      <c r="C2201" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2201" s="2">
+        <v>20.3</v>
+      </c>
+      <c r="E2201" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F2201" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2201" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2202">
+      <c r="A2202" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2202" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:50</t>
+        </is>
+      </c>
+      <c r="C2202" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2202" s="2">
+        <v>20.2</v>
+      </c>
+      <c r="E2202" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F2202" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2202" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2203">
+      <c r="A2203" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2203" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:00</t>
+        </is>
+      </c>
+      <c r="C2203" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2203" s="2">
+        <v>20.1</v>
+      </c>
+      <c r="E2203" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="F2203" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2203" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2204">
+      <c r="A2204" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2204" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:10</t>
+        </is>
+      </c>
+      <c r="C2204" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2204" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="E2204" s="2">
+        <v>72.0</v>
+      </c>
+      <c r="F2204" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2204" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2205">
+      <c r="A2205" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2205" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:20</t>
+        </is>
+      </c>
+      <c r="C2205" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2205" s="2">
+        <v>20.2</v>
+      </c>
+      <c r="E2205" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F2205" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2205" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2206">
+      <c r="A2206" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2206" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:30</t>
+        </is>
+      </c>
+      <c r="C2206" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2206" s="2">
+        <v>20.3</v>
+      </c>
+      <c r="E2206" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F2206" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2206" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2207">
+      <c r="A2207" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2207" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:40</t>
+        </is>
+      </c>
+      <c r="C2207" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2207" s="2">
+        <v>20.3</v>
+      </c>
+      <c r="E2207" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F2207" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2207" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2208">
+      <c r="A2208" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2208" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:50</t>
+        </is>
+      </c>
+      <c r="C2208" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2208" s="2">
+        <v>20.2</v>
+      </c>
+      <c r="E2208" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F2208" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2208" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2209">
+      <c r="A2209" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2209" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:00</t>
+        </is>
+      </c>
+      <c r="C2209" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2209" s="2">
+        <v>20.2</v>
+      </c>
+      <c r="E2209" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F2209" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2209" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2210">
+      <c r="A2210" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2210" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:10</t>
+        </is>
+      </c>
+      <c r="C2210" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2210" s="2">
+        <v>20.2</v>
+      </c>
+      <c r="E2210" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F2210" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2210" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2211">
+      <c r="A2211" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2211" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:20</t>
+        </is>
+      </c>
+      <c r="C2211" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2211" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="E2211" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F2211" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2211" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2212">
+      <c r="A2212" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2212" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:30</t>
+        </is>
+      </c>
+      <c r="C2212" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2212" s="2">
+        <v>20.1</v>
+      </c>
+      <c r="E2212" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F2212" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2212" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2213">
+      <c r="A2213" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2213" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:40</t>
+        </is>
+      </c>
+      <c r="C2213" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2213" s="2">
+        <v>20.2</v>
+      </c>
+      <c r="E2213" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2213" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2213" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2214">
+      <c r="A2214" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2214" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:50</t>
+        </is>
+      </c>
+      <c r="C2214" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2214" s="2">
+        <v>20.4</v>
+      </c>
+      <c r="E2214" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2214" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2214" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2215">
+      <c r="A2215" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2215" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:00</t>
+        </is>
+      </c>
+      <c r="C2215" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2215" s="2">
+        <v>20.2</v>
+      </c>
+      <c r="E2215" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F2215" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2215" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2216">
+      <c r="A2216" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2216" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:10</t>
+        </is>
+      </c>
+      <c r="C2216" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2216" s="2">
+        <v>19.8</v>
+      </c>
+      <c r="E2216" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F2216" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2216" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2217">
+      <c r="A2217" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2217" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:20</t>
+        </is>
+      </c>
+      <c r="C2217" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2217" s="2">
+        <v>19.5</v>
+      </c>
+      <c r="E2217" s="2">
+        <v>69.0</v>
+      </c>
+      <c r="F2217" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2217" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2218">
+      <c r="A2218" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2218" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:30</t>
+        </is>
+      </c>
+      <c r="C2218" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2218" s="2">
+        <v>19.3</v>
+      </c>
+      <c r="E2218" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F2218" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2218" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2219">
+      <c r="A2219" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2219" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:40</t>
+        </is>
+      </c>
+      <c r="C2219" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2219" s="2">
+        <v>19.2</v>
+      </c>
+      <c r="E2219" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F2219" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2219" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2220">
+      <c r="A2220" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2220" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:50</t>
+        </is>
+      </c>
+      <c r="C2220" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2220" s="2">
+        <v>19.1</v>
+      </c>
+      <c r="E2220" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F2220" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2220" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2221">
+      <c r="A2221" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2221" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:00</t>
+        </is>
+      </c>
+      <c r="C2221" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2221" s="2">
+        <v>18.9</v>
+      </c>
+      <c r="E2221" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F2221" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2221" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2222">
+      <c r="A2222" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2222" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:10</t>
+        </is>
+      </c>
+      <c r="C2222" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2222" s="2">
+        <v>18.8</v>
+      </c>
+      <c r="E2222" s="2">
+        <v>72.0</v>
+      </c>
+      <c r="F2222" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2222" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2223">
+      <c r="A2223" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2223" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:20</t>
+        </is>
+      </c>
+      <c r="C2223" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2223" s="2">
+        <v>18.9</v>
+      </c>
+      <c r="E2223" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F2223" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2223" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2224">
+      <c r="A2224" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2224" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:30</t>
+        </is>
+      </c>
+      <c r="C2224" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2224" s="2">
+        <v>18.8</v>
+      </c>
+      <c r="E2224" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F2224" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2224" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2225">
+      <c r="A2225" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2225" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:40</t>
+        </is>
+      </c>
+      <c r="C2225" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2225" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="E2225" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F2225" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2225" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2226">
+      <c r="A2226" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2226" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:50</t>
+        </is>
+      </c>
+      <c r="C2226" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2226" s="2">
+        <v>18.9</v>
+      </c>
+      <c r="E2226" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F2226" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2226" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2227">
+      <c r="A2227" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2227" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:00</t>
+        </is>
+      </c>
+      <c r="C2227" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2227" s="2">
+        <v>18.7</v>
+      </c>
+      <c r="E2227" s="2">
+        <v>72.0</v>
+      </c>
+      <c r="F2227" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2227" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2228">
+      <c r="A2228" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2228" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:10</t>
+        </is>
+      </c>
+      <c r="C2228" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2228" s="2">
+        <v>18.5</v>
+      </c>
+      <c r="E2228" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="F2228" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2228" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2229">
+      <c r="A2229" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2229" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:20</t>
+        </is>
+      </c>
+      <c r="C2229" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2229" s="2">
+        <v>18.4</v>
+      </c>
+      <c r="E2229" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="F2229" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2229" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2230">
+      <c r="A2230" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2230" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:30</t>
+        </is>
+      </c>
+      <c r="C2230" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2230" s="2">
+        <v>18.3</v>
+      </c>
+      <c r="E2230" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F2230" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2230" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2231">
+      <c r="A2231" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2231" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:40</t>
+        </is>
+      </c>
+      <c r="C2231" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2231" s="2">
+        <v>18.5</v>
+      </c>
+      <c r="E2231" s="2">
+        <v>74.0</v>
+      </c>
+      <c r="F2231" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2231" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2232">
+      <c r="A2232" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2232" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:50</t>
+        </is>
+      </c>
+      <c r="C2232" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2232" s="2">
+        <v>19.1</v>
+      </c>
+      <c r="E2232" s="2">
+        <v>72.0</v>
+      </c>
+      <c r="F2232" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2232" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2233">
+      <c r="A2233" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2233" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:00</t>
+        </is>
+      </c>
+      <c r="C2233" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2233" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="E2233" s="2">
+        <v>69.0</v>
+      </c>
+      <c r="F2233" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2233" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2234">
+      <c r="A2234" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2234" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:10</t>
+        </is>
+      </c>
+      <c r="C2234" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2234" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="E2234" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F2234" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2234" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2235">
+      <c r="A2235" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2235" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:20</t>
+        </is>
+      </c>
+      <c r="C2235" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2235" s="2">
+        <v>20.2</v>
+      </c>
+      <c r="E2235" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F2235" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2235" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2236">
+      <c r="A2236" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2236" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:30</t>
+        </is>
+      </c>
+      <c r="C2236" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2236" s="2">
+        <v>20.6</v>
+      </c>
+      <c r="E2236" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F2236" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2236" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2237">
+      <c r="A2237" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2237" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:40</t>
+        </is>
+      </c>
+      <c r="C2237" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2237" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="E2237" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F2237" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2237" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2238">
+      <c r="A2238" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2238" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:50</t>
+        </is>
+      </c>
+      <c r="C2238" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2238" s="2">
+        <v>21.3</v>
+      </c>
+      <c r="E2238" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2238" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2238" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2239">
+      <c r="A2239" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2239" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:00</t>
+        </is>
+      </c>
+      <c r="C2239" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2239" s="2">
+        <v>21.8</v>
+      </c>
+      <c r="E2239" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F2239" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2239" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2240">
+      <c r="A2240" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2240" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:10</t>
+        </is>
+      </c>
+      <c r="C2240" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2240" s="2">
+        <v>22.1</v>
+      </c>
+      <c r="E2240" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F2240" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2240" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2241">
+      <c r="A2241" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2241" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:20</t>
+        </is>
+      </c>
+      <c r="C2241" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2241" s="2">
+        <v>22.7</v>
+      </c>
+      <c r="E2241" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F2241" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2241" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2242">
+      <c r="A2242" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2242" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:30</t>
+        </is>
+      </c>
+      <c r="C2242" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2242" s="2">
+        <v>23.1</v>
+      </c>
+      <c r="E2242" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F2242" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2242" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2243">
+      <c r="A2243" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2243" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:40</t>
+        </is>
+      </c>
+      <c r="C2243" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2243" s="2">
+        <v>23.1</v>
+      </c>
+      <c r="E2243" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F2243" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2243" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2244">
+      <c r="A2244" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2244" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:50</t>
+        </is>
+      </c>
+      <c r="C2244" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2244" s="2">
+        <v>23.8</v>
+      </c>
+      <c r="E2244" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F2244" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2244" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2245">
+      <c r="A2245" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2245" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:00</t>
+        </is>
+      </c>
+      <c r="C2245" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2245" s="2">
+        <v>24.2</v>
+      </c>
+      <c r="E2245" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F2245" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2245" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2246">
+      <c r="A2246" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2246" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:10</t>
+        </is>
+      </c>
+      <c r="C2246" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2246" s="2">
+        <v>25.1</v>
+      </c>
+      <c r="E2246" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F2246" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2246" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2247">
+      <c r="A2247" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2247" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:20</t>
+        </is>
+      </c>
+      <c r="C2247" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2247" s="2">
+        <v>25.6</v>
+      </c>
+      <c r="E2247" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F2247" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2247" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2248">
+      <c r="A2248" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2248" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:30</t>
+        </is>
+      </c>
+      <c r="C2248" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2248" s="2">
+        <v>26.2</v>
+      </c>
+      <c r="E2248" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F2248" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2248" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2249">
+      <c r="A2249" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2249" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:40</t>
+        </is>
+      </c>
+      <c r="C2249" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2249" s="2">
+        <v>26.7</v>
+      </c>
+      <c r="E2249" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F2249" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2249" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2250">
+      <c r="A2250" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2250" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:50</t>
+        </is>
+      </c>
+      <c r="C2250" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2250" s="2">
+        <v>27.2</v>
+      </c>
+      <c r="E2250" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F2250" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2250" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2251">
+      <c r="A2251" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2251" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:00</t>
+        </is>
+      </c>
+      <c r="C2251" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2251" s="2">
+        <v>27.5</v>
+      </c>
+      <c r="E2251" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F2251" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2251" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2252">
+      <c r="A2252" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2252" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:10</t>
+        </is>
+      </c>
+      <c r="C2252" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2252" s="2">
+        <v>28.3</v>
+      </c>
+      <c r="E2252" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F2252" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2252" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2253">
+      <c r="A2253" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2253" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:20</t>
+        </is>
+      </c>
+      <c r="C2253" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2253" s="2">
+        <v>28.4</v>
+      </c>
+      <c r="E2253" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F2253" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2253" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2254">
+      <c r="A2254" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2254" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:30</t>
+        </is>
+      </c>
+      <c r="C2254" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2254" s="2">
+        <v>29.2</v>
+      </c>
+      <c r="E2254" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F2254" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2254" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2255">
+      <c r="A2255" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2255" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:40</t>
+        </is>
+      </c>
+      <c r="C2255" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2255" s="2">
+        <v>30.1</v>
+      </c>
+      <c r="E2255" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F2255" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2255" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2256">
+      <c r="A2256" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2256" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:50</t>
+        </is>
+      </c>
+      <c r="C2256" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2256" s="2">
+        <v>30.2</v>
+      </c>
+      <c r="E2256" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="F2256" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2256" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2257">
+      <c r="A2257" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2257" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:00</t>
+        </is>
+      </c>
+      <c r="C2257" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2257" s="2">
+        <v>30.2</v>
+      </c>
+      <c r="E2257" s="2">
+        <v>37.0</v>
+      </c>
+      <c r="F2257" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2257" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2258">
+      <c r="A2258" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2258" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:10</t>
+        </is>
+      </c>
+      <c r="C2258" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2258" s="2">
+        <v>31.1</v>
+      </c>
+      <c r="E2258" s="2">
+        <v>37.0</v>
+      </c>
+      <c r="F2258" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2258" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2259">
+      <c r="A2259" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2259" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:20</t>
+        </is>
+      </c>
+      <c r="C2259" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2259" s="2">
+        <v>30.9</v>
+      </c>
+      <c r="E2259" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="F2259" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2259" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2260">
+      <c r="A2260" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2260" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:30</t>
+        </is>
+      </c>
+      <c r="C2260" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2260" s="2">
+        <v>31.1</v>
+      </c>
+      <c r="E2260" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="F2260" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2260" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2261">
+      <c r="A2261" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2261" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:40</t>
+        </is>
+      </c>
+      <c r="C2261" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2261" s="2">
+        <v>31.6</v>
+      </c>
+      <c r="E2261" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F2261" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2261" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2262">
+      <c r="A2262" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2262" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:50</t>
+        </is>
+      </c>
+      <c r="C2262" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2262" s="2">
+        <v>31.8</v>
+      </c>
+      <c r="E2262" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F2262" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2262" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2263">
+      <c r="A2263" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2263" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:00</t>
+        </is>
+      </c>
+      <c r="C2263" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2263" s="2">
+        <v>31.6</v>
+      </c>
+      <c r="E2263" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F2263" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2263" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2264">
+      <c r="A2264" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2264" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:10</t>
+        </is>
+      </c>
+      <c r="C2264" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2264" s="2">
+        <v>32.5</v>
+      </c>
+      <c r="E2264" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F2264" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2264" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2265">
+      <c r="A2265" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2265" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:20</t>
+        </is>
+      </c>
+      <c r="C2265" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2265" s="2">
+        <v>32.5</v>
+      </c>
+      <c r="E2265" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F2265" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2265" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2266">
+      <c r="A2266" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2266" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:30</t>
+        </is>
+      </c>
+      <c r="C2266" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2266" s="2">
+        <v>32.7</v>
+      </c>
+      <c r="E2266" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F2266" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2266" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2267">
+      <c r="A2267" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2267" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:40</t>
+        </is>
+      </c>
+      <c r="C2267" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2267" s="2">
+        <v>32.9</v>
+      </c>
+      <c r="E2267" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F2267" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2267" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2268">
+      <c r="A2268" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2268" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:50</t>
+        </is>
+      </c>
+      <c r="C2268" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2268" s="2">
+        <v>33.6</v>
+      </c>
+      <c r="E2268" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F2268" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2268" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2269">
+      <c r="A2269" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2269" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:00</t>
+        </is>
+      </c>
+      <c r="C2269" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2269" s="2">
+        <v>33.6</v>
+      </c>
+      <c r="E2269" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="F2269" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2269" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2270">
+      <c r="A2270" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2270" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:10</t>
+        </is>
+      </c>
+      <c r="C2270" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2270" s="2">
+        <v>33.7</v>
+      </c>
+      <c r="E2270" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F2270" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2270" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2271">
+      <c r="A2271" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2271" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:20</t>
+        </is>
+      </c>
+      <c r="C2271" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2271" s="2">
+        <v>34.3</v>
+      </c>
+      <c r="E2271" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F2271" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2271" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2272">
+      <c r="A2272" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2272" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:30</t>
+        </is>
+      </c>
+      <c r="C2272" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2272" s="2">
+        <v>33.9</v>
+      </c>
+      <c r="E2272" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F2272" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2272" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2273">
+      <c r="A2273" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2273" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:40</t>
+        </is>
+      </c>
+      <c r="C2273" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2273" s="2">
+        <v>34.6</v>
+      </c>
+      <c r="E2273" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F2273" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2273" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2274">
+      <c r="A2274" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2274" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:50</t>
+        </is>
+      </c>
+      <c r="C2274" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2274" s="2">
+        <v>34.3</v>
+      </c>
+      <c r="E2274" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F2274" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2274" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2275">
+      <c r="A2275" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2275" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:00</t>
+        </is>
+      </c>
+      <c r="C2275" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2275" s="2">
+        <v>35.2</v>
+      </c>
+      <c r="E2275" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2275" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2275" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2276">
+      <c r="A2276" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2276" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:10</t>
+        </is>
+      </c>
+      <c r="C2276" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2276" s="2">
+        <v>34.6</v>
+      </c>
+      <c r="E2276" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2276" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2276" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2277">
+      <c r="A2277" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2277" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:20</t>
+        </is>
+      </c>
+      <c r="C2277" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2277" s="2">
+        <v>35.3</v>
+      </c>
+      <c r="E2277" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F2277" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2277" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2278">
+      <c r="A2278" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2278" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:30</t>
+        </is>
+      </c>
+      <c r="C2278" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2278" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="E2278" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F2278" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2278" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2279">
+      <c r="A2279" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2279" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:40</t>
+        </is>
+      </c>
+      <c r="C2279" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2279" s="2">
+        <v>35.3</v>
+      </c>
+      <c r="E2279" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2279" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2279" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2280">
+      <c r="A2280" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2280" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:50</t>
+        </is>
+      </c>
+      <c r="C2280" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2280" s="2">
+        <v>35.2</v>
+      </c>
+      <c r="E2280" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2280" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2280" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2281">
+      <c r="A2281" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2281" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:00</t>
+        </is>
+      </c>
+      <c r="C2281" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2281" s="2">
+        <v>35.3</v>
+      </c>
+      <c r="E2281" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2281" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2281" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2282">
+      <c r="A2282" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2282" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:10</t>
+        </is>
+      </c>
+      <c r="C2282" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2282" s="2">
+        <v>35.2</v>
+      </c>
+      <c r="E2282" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2282" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2282" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2283">
+      <c r="A2283" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2283" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:20</t>
+        </is>
+      </c>
+      <c r="C2283" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2283" s="2">
+        <v>35.5</v>
+      </c>
+      <c r="E2283" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2283" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2283" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2284">
+      <c r="A2284" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2284" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:30</t>
+        </is>
+      </c>
+      <c r="C2284" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2284" s="2">
+        <v>35.6</v>
+      </c>
+      <c r="E2284" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2284" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2284" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2285">
+      <c r="A2285" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2285" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:40</t>
+        </is>
+      </c>
+      <c r="C2285" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2285" s="2">
+        <v>35.2</v>
+      </c>
+      <c r="E2285" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2285" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2285" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2286">
+      <c r="A2286" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2286" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:50</t>
+        </is>
+      </c>
+      <c r="C2286" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2286" s="2">
+        <v>35.2</v>
+      </c>
+      <c r="E2286" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2286" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2286" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2287">
+      <c r="A2287" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2287" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:00</t>
+        </is>
+      </c>
+      <c r="C2287" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2287" s="2">
+        <v>34.7</v>
+      </c>
+      <c r="E2287" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2287" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2287" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2288">
+      <c r="A2288" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2288" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:10</t>
+        </is>
+      </c>
+      <c r="C2288" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2288" s="2">
+        <v>34.4</v>
+      </c>
+      <c r="E2288" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2288" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2288" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2289">
+      <c r="A2289" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2289" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:20</t>
+        </is>
+      </c>
+      <c r="C2289" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2289" s="2">
+        <v>34.7</v>
+      </c>
+      <c r="E2289" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2289" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2289" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2290">
+      <c r="A2290" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2290" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:30</t>
+        </is>
+      </c>
+      <c r="C2290" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2290" s="2">
+        <v>34.6</v>
+      </c>
+      <c r="E2290" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2290" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2290" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2291">
+      <c r="A2291" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2291" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:40</t>
+        </is>
+      </c>
+      <c r="C2291" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2291" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="E2291" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2291" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2291" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2292">
+      <c r="A2292" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2292" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:50</t>
+        </is>
+      </c>
+      <c r="C2292" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2292" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="E2292" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2292" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2292" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2293">
+      <c r="A2293" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2293" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:00</t>
+        </is>
+      </c>
+      <c r="C2293" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2293" s="2">
+        <v>35.2</v>
+      </c>
+      <c r="E2293" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="F2293" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2293" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2294">
+      <c r="A2294" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2294" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:10</t>
+        </is>
+      </c>
+      <c r="C2294" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2294" s="2">
+        <v>35.2</v>
+      </c>
+      <c r="E2294" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2294" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2294" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2295">
+      <c r="A2295" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2295" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:20</t>
+        </is>
+      </c>
+      <c r="C2295" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2295" s="2">
+        <v>35.1</v>
+      </c>
+      <c r="E2295" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2295" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2295" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2296">
+      <c r="A2296" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2296" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:30</t>
+        </is>
+      </c>
+      <c r="C2296" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2296" s="2">
+        <v>34.9</v>
+      </c>
+      <c r="E2296" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2296" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2296" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2297">
+      <c r="A2297" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2297" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:40</t>
+        </is>
+      </c>
+      <c r="C2297" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2297" s="2">
+        <v>35.2</v>
+      </c>
+      <c r="E2297" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2297" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2297" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2298">
+      <c r="A2298" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2298" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:50</t>
+        </is>
+      </c>
+      <c r="C2298" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2298" s="2">
+        <v>35.6</v>
+      </c>
+      <c r="E2298" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2298" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2298" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2299">
+      <c r="A2299" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2299" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:00</t>
+        </is>
+      </c>
+      <c r="C2299" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2299" s="2">
+        <v>35.5</v>
+      </c>
+      <c r="E2299" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2299" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2299" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2300">
+      <c r="A2300" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2300" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:10</t>
+        </is>
+      </c>
+      <c r="C2300" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2300" s="2">
+        <v>35.5</v>
+      </c>
+      <c r="E2300" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2300" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2300" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2301">
+      <c r="A2301" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2301" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:20</t>
+        </is>
+      </c>
+      <c r="C2301" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2301" s="2">
+        <v>35.6</v>
+      </c>
+      <c r="E2301" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2301" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2301" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2302">
+      <c r="A2302" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2302" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:30</t>
+        </is>
+      </c>
+      <c r="C2302" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2302" s="2">
+        <v>35.4</v>
+      </c>
+      <c r="E2302" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2302" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2302" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2303">
+      <c r="A2303" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2303" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:40</t>
+        </is>
+      </c>
+      <c r="C2303" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2303" s="2">
+        <v>35.4</v>
+      </c>
+      <c r="E2303" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2303" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2303" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2304">
+      <c r="A2304" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2304" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:50</t>
+        </is>
+      </c>
+      <c r="C2304" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2304" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="E2304" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2304" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2304" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2305">
+      <c r="A2305" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2305" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:00</t>
+        </is>
+      </c>
+      <c r="C2305" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2305" s="2">
+        <v>34.9</v>
+      </c>
+      <c r="E2305" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2305" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2305" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2306">
+      <c r="A2306" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2306" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:10</t>
+        </is>
+      </c>
+      <c r="C2306" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2306" s="2">
+        <v>34.3</v>
+      </c>
+      <c r="E2306" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2306" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2306" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2307">
+      <c r="A2307" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2307" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:20</t>
+        </is>
+      </c>
+      <c r="C2307" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2307" s="2">
+        <v>33.9</v>
+      </c>
+      <c r="E2307" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2307" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2307" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2308">
+      <c r="A2308" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2308" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:30</t>
+        </is>
+      </c>
+      <c r="C2308" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2308" s="2">
+        <v>33.6</v>
+      </c>
+      <c r="E2308" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F2308" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2308" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2309">
+      <c r="A2309" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2309" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:40</t>
+        </is>
+      </c>
+      <c r="C2309" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2309" s="2">
+        <v>33.3</v>
+      </c>
+      <c r="E2309" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="F2309" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2309" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2310">
+      <c r="A2310" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2310" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:50</t>
+        </is>
+      </c>
+      <c r="C2310" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2310" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="E2310" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="F2310" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2310" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2311">
+      <c r="A2311" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2311" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:00</t>
+        </is>
+      </c>
+      <c r="C2311" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2311" s="2">
+        <v>32.7</v>
+      </c>
+      <c r="E2311" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F2311" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2311" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2312">
+      <c r="A2312" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2312" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:10</t>
+        </is>
+      </c>
+      <c r="C2312" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2312" s="2">
+        <v>32.4</v>
+      </c>
+      <c r="E2312" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F2312" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2312" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2313">
+      <c r="A2313" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2313" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:20</t>
+        </is>
+      </c>
+      <c r="C2313" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2313" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="E2313" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F2313" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2313" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2314">
+      <c r="A2314" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2314" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:30</t>
+        </is>
+      </c>
+      <c r="C2314" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2314" s="2">
+        <v>31.7</v>
+      </c>
+      <c r="E2314" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F2314" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2314" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2315">
+      <c r="A2315" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2315" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:40</t>
+        </is>
+      </c>
+      <c r="C2315" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2315" s="2">
+        <v>31.1</v>
+      </c>
+      <c r="E2315" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="F2315" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2315" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2316">
+      <c r="A2316" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2316" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:50</t>
+        </is>
+      </c>
+      <c r="C2316" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2316" s="2">
+        <v>30.7</v>
+      </c>
+      <c r="E2316" s="2">
+        <v>37.0</v>
+      </c>
+      <c r="F2316" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2316" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2317">
+      <c r="A2317" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2317" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:00</t>
+        </is>
+      </c>
+      <c r="C2317" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2317" s="2">
+        <v>30.1</v>
+      </c>
+      <c r="E2317" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F2317" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2317" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2318">
+      <c r="A2318" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2318" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:20</t>
+        </is>
+      </c>
+      <c r="C2318" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2318" s="2">
+        <v>28.7</v>
+      </c>
+      <c r="E2318" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F2318" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2318" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2319">
+      <c r="A2319" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2319" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:30</t>
+        </is>
+      </c>
+      <c r="C2319" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2319" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="E2319" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F2319" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2319" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2320">
+      <c r="A2320" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2320" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:40</t>
+        </is>
+      </c>
+      <c r="C2320" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2320" s="2">
+        <v>27.4</v>
+      </c>
+      <c r="E2320" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F2320" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2320" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2321">
+      <c r="A2321" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2321" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:50</t>
+        </is>
+      </c>
+      <c r="C2321" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2321" s="2">
+        <v>26.9</v>
+      </c>
+      <c r="E2321" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F2321" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2321" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2322">
+      <c r="A2322" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2322" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:00</t>
+        </is>
+      </c>
+      <c r="C2322" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2322" s="2">
+        <v>26.4</v>
+      </c>
+      <c r="E2322" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F2322" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2322" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2323">
+      <c r="A2323" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2323" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:10</t>
+        </is>
+      </c>
+      <c r="C2323" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2323" s="2">
+        <v>26.1</v>
+      </c>
+      <c r="E2323" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F2323" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2323" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2324">
+      <c r="A2324" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2324" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:20</t>
+        </is>
+      </c>
+      <c r="C2324" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2324" s="2">
+        <v>25.6</v>
+      </c>
+      <c r="E2324" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2324" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2324" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2325">
+      <c r="A2325" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2325" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:30</t>
+        </is>
+      </c>
+      <c r="C2325" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2325" s="2">
+        <v>25.2</v>
+      </c>
+      <c r="E2325" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F2325" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2325" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2326">
+      <c r="A2326" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2326" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:40</t>
+        </is>
+      </c>
+      <c r="C2326" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2326" s="2">
+        <v>24.8</v>
+      </c>
+      <c r="E2326" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F2326" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2326" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2327">
+      <c r="A2327" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2327" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:50</t>
+        </is>
+      </c>
+      <c r="C2327" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2327" s="2">
+        <v>24.5</v>
+      </c>
+      <c r="E2327" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F2327" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2327" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2328">
+      <c r="A2328" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2328" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:00</t>
+        </is>
+      </c>
+      <c r="C2328" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2328" s="2">
+        <v>24.2</v>
+      </c>
+      <c r="E2328" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F2328" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2328" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2329">
+      <c r="A2329" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2329" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:10</t>
+        </is>
+      </c>
+      <c r="C2329" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2329" s="2">
+        <v>24.1</v>
+      </c>
+      <c r="E2329" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F2329" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2329" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2330">
+      <c r="A2330" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2330" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:20</t>
+        </is>
+      </c>
+      <c r="C2330" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2330" s="2">
+        <v>23.8</v>
+      </c>
+      <c r="E2330" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F2330" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2330" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2331">
+      <c r="A2331" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2331" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:30</t>
+        </is>
+      </c>
+      <c r="C2331" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2331" s="2">
+        <v>23.8</v>
+      </c>
+      <c r="E2331" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F2331" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2331" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2332">
+      <c r="A2332" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2332" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:40</t>
+        </is>
+      </c>
+      <c r="C2332" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2332" s="2">
+        <v>23.6</v>
+      </c>
+      <c r="E2332" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F2332" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2332" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2333">
+      <c r="A2333" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">30.07.2026</t>
+        </is>
+      </c>
+      <c r="B2333" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:50</t>
+        </is>
+      </c>
+      <c r="C2333" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2333" s="2">
+        <v>23.5</v>
+      </c>
+      <c r="E2333" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F2333" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2333" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2334">
+      <c r="A2334" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2334" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:00</t>
+        </is>
+      </c>
+      <c r="C2334" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2334" s="2">
+        <v>23.5</v>
+      </c>
+      <c r="E2334" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F2334" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2334" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2335">
+      <c r="A2335" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2335" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:10</t>
+        </is>
+      </c>
+      <c r="C2335" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2335" s="2">
+        <v>23.5</v>
+      </c>
+      <c r="E2335" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F2335" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2335" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2336">
+      <c r="A2336" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2336" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:20</t>
+        </is>
+      </c>
+      <c r="C2336" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2336" s="2">
+        <v>23.4</v>
+      </c>
+      <c r="E2336" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F2336" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2336" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2337">
+      <c r="A2337" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2337" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:30</t>
+        </is>
+      </c>
+      <c r="C2337" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2337" s="2">
+        <v>23.3</v>
+      </c>
+      <c r="E2337" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F2337" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2337" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G2194"/>
+  <autoFilter ref="A1:G2337"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ARSO Kranj zajem 2026-08-01 00:45 Europe/Ljubljana
</commit_message>
<xml_diff>
--- a/tabela_vremena/ARSO_Kranj.xlsx
+++ b/tabela_vremena/ARSO_Kranj.xlsx
@@ -67283,7 +67283,7 @@
       </c>
       <c r="B2318" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">21:20</t>
+          <t xml:space="preserve">21:10</t>
         </is>
       </c>
       <c r="C2318" t="inlineStr" s="0">
@@ -67292,10 +67292,10 @@
         </is>
       </c>
       <c r="D2318" s="2">
-        <v>28.7</v>
+        <v>29.5</v>
       </c>
       <c r="E2318" s="2">
-        <v>43.0</v>
+        <v>41.0</v>
       </c>
       <c r="F2318" s="2">
         <v>0.0</v>
@@ -67312,7 +67312,7 @@
       </c>
       <c r="B2319" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">21:30</t>
+          <t xml:space="preserve">21:20</t>
         </is>
       </c>
       <c r="C2319" t="inlineStr" s="0">
@@ -67321,10 +67321,10 @@
         </is>
       </c>
       <c r="D2319" s="2">
-        <v>28.0</v>
+        <v>28.7</v>
       </c>
       <c r="E2319" s="2">
-        <v>49.0</v>
+        <v>43.0</v>
       </c>
       <c r="F2319" s="2">
         <v>0.0</v>
@@ -67341,7 +67341,7 @@
       </c>
       <c r="B2320" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">21:40</t>
+          <t xml:space="preserve">21:30</t>
         </is>
       </c>
       <c r="C2320" t="inlineStr" s="0">
@@ -67350,10 +67350,10 @@
         </is>
       </c>
       <c r="D2320" s="2">
-        <v>27.4</v>
+        <v>28.0</v>
       </c>
       <c r="E2320" s="2">
-        <v>52.0</v>
+        <v>49.0</v>
       </c>
       <c r="F2320" s="2">
         <v>0.0</v>
@@ -67370,7 +67370,7 @@
       </c>
       <c r="B2321" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">21:50</t>
+          <t xml:space="preserve">21:40</t>
         </is>
       </c>
       <c r="C2321" t="inlineStr" s="0">
@@ -67379,10 +67379,10 @@
         </is>
       </c>
       <c r="D2321" s="2">
-        <v>26.9</v>
+        <v>27.4</v>
       </c>
       <c r="E2321" s="2">
-        <v>54.0</v>
+        <v>52.0</v>
       </c>
       <c r="F2321" s="2">
         <v>0.0</v>
@@ -67399,7 +67399,7 @@
       </c>
       <c r="B2322" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">22:00</t>
+          <t xml:space="preserve">21:50</t>
         </is>
       </c>
       <c r="C2322" t="inlineStr" s="0">
@@ -67408,10 +67408,10 @@
         </is>
       </c>
       <c r="D2322" s="2">
-        <v>26.4</v>
+        <v>26.9</v>
       </c>
       <c r="E2322" s="2">
-        <v>55.0</v>
+        <v>54.0</v>
       </c>
       <c r="F2322" s="2">
         <v>0.0</v>
@@ -67428,7 +67428,7 @@
       </c>
       <c r="B2323" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">22:10</t>
+          <t xml:space="preserve">22:00</t>
         </is>
       </c>
       <c r="C2323" t="inlineStr" s="0">
@@ -67437,10 +67437,10 @@
         </is>
       </c>
       <c r="D2323" s="2">
-        <v>26.1</v>
+        <v>26.4</v>
       </c>
       <c r="E2323" s="2">
-        <v>56.0</v>
+        <v>55.0</v>
       </c>
       <c r="F2323" s="2">
         <v>0.0</v>
@@ -67457,7 +67457,7 @@
       </c>
       <c r="B2324" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">22:20</t>
+          <t xml:space="preserve">22:10</t>
         </is>
       </c>
       <c r="C2324" t="inlineStr" s="0">
@@ -67466,10 +67466,10 @@
         </is>
       </c>
       <c r="D2324" s="2">
-        <v>25.6</v>
+        <v>26.1</v>
       </c>
       <c r="E2324" s="2">
-        <v>58.0</v>
+        <v>56.0</v>
       </c>
       <c r="F2324" s="2">
         <v>0.0</v>
@@ -67486,7 +67486,7 @@
       </c>
       <c r="B2325" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">22:30</t>
+          <t xml:space="preserve">22:20</t>
         </is>
       </c>
       <c r="C2325" t="inlineStr" s="0">
@@ -67495,10 +67495,10 @@
         </is>
       </c>
       <c r="D2325" s="2">
-        <v>25.2</v>
+        <v>25.6</v>
       </c>
       <c r="E2325" s="2">
-        <v>59.0</v>
+        <v>58.0</v>
       </c>
       <c r="F2325" s="2">
         <v>0.0</v>
@@ -67515,7 +67515,7 @@
       </c>
       <c r="B2326" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">22:40</t>
+          <t xml:space="preserve">22:30</t>
         </is>
       </c>
       <c r="C2326" t="inlineStr" s="0">
@@ -67524,10 +67524,10 @@
         </is>
       </c>
       <c r="D2326" s="2">
-        <v>24.8</v>
+        <v>25.2</v>
       </c>
       <c r="E2326" s="2">
-        <v>61.0</v>
+        <v>59.0</v>
       </c>
       <c r="F2326" s="2">
         <v>0.0</v>
@@ -67544,7 +67544,7 @@
       </c>
       <c r="B2327" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">22:50</t>
+          <t xml:space="preserve">22:40</t>
         </is>
       </c>
       <c r="C2327" t="inlineStr" s="0">
@@ -67553,10 +67553,10 @@
         </is>
       </c>
       <c r="D2327" s="2">
-        <v>24.5</v>
+        <v>24.8</v>
       </c>
       <c r="E2327" s="2">
-        <v>62.0</v>
+        <v>61.0</v>
       </c>
       <c r="F2327" s="2">
         <v>0.0</v>
@@ -67573,7 +67573,7 @@
       </c>
       <c r="B2328" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">23:00</t>
+          <t xml:space="preserve">22:50</t>
         </is>
       </c>
       <c r="C2328" t="inlineStr" s="0">
@@ -67582,10 +67582,10 @@
         </is>
       </c>
       <c r="D2328" s="2">
-        <v>24.2</v>
+        <v>24.5</v>
       </c>
       <c r="E2328" s="2">
-        <v>63.0</v>
+        <v>62.0</v>
       </c>
       <c r="F2328" s="2">
         <v>0.0</v>
@@ -67602,7 +67602,7 @@
       </c>
       <c r="B2329" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">23:10</t>
+          <t xml:space="preserve">23:00</t>
         </is>
       </c>
       <c r="C2329" t="inlineStr" s="0">
@@ -67611,7 +67611,7 @@
         </is>
       </c>
       <c r="D2329" s="2">
-        <v>24.1</v>
+        <v>24.2</v>
       </c>
       <c r="E2329" s="2">
         <v>63.0</v>
@@ -67631,7 +67631,7 @@
       </c>
       <c r="B2330" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">23:20</t>
+          <t xml:space="preserve">23:10</t>
         </is>
       </c>
       <c r="C2330" t="inlineStr" s="0">
@@ -67640,10 +67640,10 @@
         </is>
       </c>
       <c r="D2330" s="2">
-        <v>23.8</v>
+        <v>24.1</v>
       </c>
       <c r="E2330" s="2">
-        <v>62.0</v>
+        <v>63.0</v>
       </c>
       <c r="F2330" s="2">
         <v>0.0</v>
@@ -67660,7 +67660,7 @@
       </c>
       <c r="B2331" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">23:30</t>
+          <t xml:space="preserve">23:20</t>
         </is>
       </c>
       <c r="C2331" t="inlineStr" s="0">
@@ -67672,7 +67672,7 @@
         <v>23.8</v>
       </c>
       <c r="E2331" s="2">
-        <v>63.0</v>
+        <v>62.0</v>
       </c>
       <c r="F2331" s="2">
         <v>0.0</v>
@@ -67689,7 +67689,7 @@
       </c>
       <c r="B2332" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">23:40</t>
+          <t xml:space="preserve">23:30</t>
         </is>
       </c>
       <c r="C2332" t="inlineStr" s="0">
@@ -67698,7 +67698,7 @@
         </is>
       </c>
       <c r="D2332" s="2">
-        <v>23.6</v>
+        <v>23.8</v>
       </c>
       <c r="E2332" s="2">
         <v>63.0</v>
@@ -67718,7 +67718,7 @@
       </c>
       <c r="B2333" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">23:50</t>
+          <t xml:space="preserve">23:40</t>
         </is>
       </c>
       <c r="C2333" t="inlineStr" s="0">
@@ -67727,7 +67727,7 @@
         </is>
       </c>
       <c r="D2333" s="2">
-        <v>23.5</v>
+        <v>23.6</v>
       </c>
       <c r="E2333" s="2">
         <v>63.0</v>
@@ -67742,12 +67742,12 @@
     <row r="2334">
       <c r="A2334" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">31.07.2026</t>
+          <t xml:space="preserve">30.07.2026</t>
         </is>
       </c>
       <c r="B2334" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">00:00</t>
+          <t xml:space="preserve">23:50</t>
         </is>
       </c>
       <c r="C2334" t="inlineStr" s="0">
@@ -67759,7 +67759,7 @@
         <v>23.5</v>
       </c>
       <c r="E2334" s="2">
-        <v>61.0</v>
+        <v>63.0</v>
       </c>
       <c r="F2334" s="2">
         <v>0.0</v>
@@ -67776,7 +67776,7 @@
       </c>
       <c r="B2335" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">00:10</t>
+          <t xml:space="preserve">00:00</t>
         </is>
       </c>
       <c r="C2335" t="inlineStr" s="0">
@@ -67805,7 +67805,7 @@
       </c>
       <c r="B2336" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">00:20</t>
+          <t xml:space="preserve">00:10</t>
         </is>
       </c>
       <c r="C2336" t="inlineStr" s="0">
@@ -67814,7 +67814,7 @@
         </is>
       </c>
       <c r="D2336" s="2">
-        <v>23.4</v>
+        <v>23.5</v>
       </c>
       <c r="E2336" s="2">
         <v>61.0</v>
@@ -67834,28 +67834,4233 @@
       </c>
       <c r="B2337" t="inlineStr" s="0">
         <is>
+          <t xml:space="preserve">00:20</t>
+        </is>
+      </c>
+      <c r="C2337" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2337" s="2">
+        <v>23.4</v>
+      </c>
+      <c r="E2337" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F2337" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2337" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2338">
+      <c r="A2338" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2338" t="inlineStr" s="0">
+        <is>
           <t xml:space="preserve">00:30</t>
         </is>
       </c>
-      <c r="C2337" t="inlineStr" s="0">
-        <is>
-          <t xml:space="preserve">Kranj</t>
-        </is>
-      </c>
-      <c r="D2337" s="2">
+      <c r="C2338" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2338" s="2">
         <v>23.3</v>
       </c>
-      <c r="E2337" s="2">
+      <c r="E2338" s="2">
         <v>60.0</v>
       </c>
-      <c r="F2337" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="G2337" s="2">
+      <c r="F2338" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2338" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2339">
+      <c r="A2339" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2339" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:40</t>
+        </is>
+      </c>
+      <c r="C2339" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2339" s="2">
+        <v>23.1</v>
+      </c>
+      <c r="E2339" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F2339" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2339" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2340">
+      <c r="A2340" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2340" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:50</t>
+        </is>
+      </c>
+      <c r="C2340" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2340" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="E2340" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F2340" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2340" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2341">
+      <c r="A2341" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2341" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:00</t>
+        </is>
+      </c>
+      <c r="C2341" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2341" s="2">
+        <v>22.8</v>
+      </c>
+      <c r="E2341" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F2341" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2341" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2342">
+      <c r="A2342" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2342" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:10</t>
+        </is>
+      </c>
+      <c r="C2342" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2342" s="2">
+        <v>22.7</v>
+      </c>
+      <c r="E2342" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F2342" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2342" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2343">
+      <c r="A2343" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2343" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:20</t>
+        </is>
+      </c>
+      <c r="C2343" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2343" s="2">
+        <v>22.5</v>
+      </c>
+      <c r="E2343" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2343" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2343" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2344">
+      <c r="A2344" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2344" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:30</t>
+        </is>
+      </c>
+      <c r="C2344" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2344" s="2">
+        <v>22.2</v>
+      </c>
+      <c r="E2344" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F2344" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2344" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2345">
+      <c r="A2345" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2345" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:40</t>
+        </is>
+      </c>
+      <c r="C2345" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2345" s="2">
+        <v>22.1</v>
+      </c>
+      <c r="E2345" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2345" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2345" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2346">
+      <c r="A2346" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2346" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:50</t>
+        </is>
+      </c>
+      <c r="C2346" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2346" s="2">
+        <v>22.1</v>
+      </c>
+      <c r="E2346" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2346" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2346" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2347">
+      <c r="A2347" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2347" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:00</t>
+        </is>
+      </c>
+      <c r="C2347" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2347" s="2">
+        <v>22.1</v>
+      </c>
+      <c r="E2347" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2347" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2347" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2348">
+      <c r="A2348" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2348" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:10</t>
+        </is>
+      </c>
+      <c r="C2348" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2348" s="2">
+        <v>22.1</v>
+      </c>
+      <c r="E2348" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2348" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2348" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2349">
+      <c r="A2349" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2349" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:20</t>
+        </is>
+      </c>
+      <c r="C2349" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2349" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="E2349" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2349" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2349" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2350">
+      <c r="A2350" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2350" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:30</t>
+        </is>
+      </c>
+      <c r="C2350" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2350" s="2">
+        <v>21.8</v>
+      </c>
+      <c r="E2350" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2350" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2350" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2351">
+      <c r="A2351" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2351" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:40</t>
+        </is>
+      </c>
+      <c r="C2351" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2351" s="2">
+        <v>21.8</v>
+      </c>
+      <c r="E2351" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F2351" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2351" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2352">
+      <c r="A2352" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2352" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:50</t>
+        </is>
+      </c>
+      <c r="C2352" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2352" s="2">
+        <v>21.9</v>
+      </c>
+      <c r="E2352" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2352" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2352" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2353">
+      <c r="A2353" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2353" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:00</t>
+        </is>
+      </c>
+      <c r="C2353" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2353" s="2">
+        <v>21.9</v>
+      </c>
+      <c r="E2353" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2353" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2353" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2354">
+      <c r="A2354" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2354" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:10</t>
+        </is>
+      </c>
+      <c r="C2354" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2354" s="2">
+        <v>21.6</v>
+      </c>
+      <c r="E2354" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2354" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2354" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2355">
+      <c r="A2355" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2355" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:20</t>
+        </is>
+      </c>
+      <c r="C2355" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2355" s="2">
+        <v>21.5</v>
+      </c>
+      <c r="E2355" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2355" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2355" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2356">
+      <c r="A2356" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2356" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:30</t>
+        </is>
+      </c>
+      <c r="C2356" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2356" s="2">
+        <v>21.5</v>
+      </c>
+      <c r="E2356" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2356" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2356" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2357">
+      <c r="A2357" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2357" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:40</t>
+        </is>
+      </c>
+      <c r="C2357" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2357" s="2">
+        <v>21.4</v>
+      </c>
+      <c r="E2357" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F2357" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2357" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2358">
+      <c r="A2358" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2358" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:50</t>
+        </is>
+      </c>
+      <c r="C2358" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2358" s="2">
+        <v>21.4</v>
+      </c>
+      <c r="E2358" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F2358" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2358" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2359">
+      <c r="A2359" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2359" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:00</t>
+        </is>
+      </c>
+      <c r="C2359" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2359" s="2">
+        <v>21.4</v>
+      </c>
+      <c r="E2359" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2359" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2359" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2360">
+      <c r="A2360" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2360" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:10</t>
+        </is>
+      </c>
+      <c r="C2360" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2360" s="2">
+        <v>21.5</v>
+      </c>
+      <c r="E2360" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2360" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2360" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2361">
+      <c r="A2361" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2361" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:20</t>
+        </is>
+      </c>
+      <c r="C2361" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2361" s="2">
+        <v>21.4</v>
+      </c>
+      <c r="E2361" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2361" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2361" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2362">
+      <c r="A2362" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2362" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:30</t>
+        </is>
+      </c>
+      <c r="C2362" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2362" s="2">
+        <v>21.2</v>
+      </c>
+      <c r="E2362" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F2362" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2362" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2363">
+      <c r="A2363" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2363" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:40</t>
+        </is>
+      </c>
+      <c r="C2363" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2363" s="2">
+        <v>21.1</v>
+      </c>
+      <c r="E2363" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F2363" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2363" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2364">
+      <c r="A2364" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2364" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:50</t>
+        </is>
+      </c>
+      <c r="C2364" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2364" s="2">
+        <v>21.1</v>
+      </c>
+      <c r="E2364" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F2364" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2364" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2365">
+      <c r="A2365" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2365" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:00</t>
+        </is>
+      </c>
+      <c r="C2365" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2365" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="E2365" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F2365" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2365" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2366">
+      <c r="A2366" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2366" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:10</t>
+        </is>
+      </c>
+      <c r="C2366" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2366" s="2">
+        <v>20.8</v>
+      </c>
+      <c r="E2366" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F2366" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2366" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2367">
+      <c r="A2367" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2367" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:20</t>
+        </is>
+      </c>
+      <c r="C2367" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2367" s="2">
+        <v>20.6</v>
+      </c>
+      <c r="E2367" s="2">
+        <v>69.0</v>
+      </c>
+      <c r="F2367" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2367" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2368">
+      <c r="A2368" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2368" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:30</t>
+        </is>
+      </c>
+      <c r="C2368" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2368" s="2">
+        <v>20.4</v>
+      </c>
+      <c r="E2368" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F2368" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2368" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2369">
+      <c r="A2369" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2369" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:40</t>
+        </is>
+      </c>
+      <c r="C2369" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2369" s="2">
+        <v>20.2</v>
+      </c>
+      <c r="E2369" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F2369" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2369" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2370">
+      <c r="A2370" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2370" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:50</t>
+        </is>
+      </c>
+      <c r="C2370" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2370" s="2">
+        <v>19.8</v>
+      </c>
+      <c r="E2370" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F2370" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2370" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2371">
+      <c r="A2371" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2371" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:00</t>
+        </is>
+      </c>
+      <c r="C2371" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2371" s="2">
+        <v>19.6</v>
+      </c>
+      <c r="E2371" s="2">
+        <v>74.0</v>
+      </c>
+      <c r="F2371" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2371" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2372">
+      <c r="A2372" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2372" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:10</t>
+        </is>
+      </c>
+      <c r="C2372" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2372" s="2">
+        <v>19.4</v>
+      </c>
+      <c r="E2372" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F2372" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2372" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2373">
+      <c r="A2373" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2373" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:20</t>
+        </is>
+      </c>
+      <c r="C2373" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2373" s="2">
+        <v>19.1</v>
+      </c>
+      <c r="E2373" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F2373" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2373" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2374">
+      <c r="A2374" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2374" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:30</t>
+        </is>
+      </c>
+      <c r="C2374" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2374" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="E2374" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F2374" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2374" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2375">
+      <c r="A2375" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2375" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:40</t>
+        </is>
+      </c>
+      <c r="C2375" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2375" s="2">
+        <v>19.1</v>
+      </c>
+      <c r="E2375" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F2375" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2375" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2376">
+      <c r="A2376" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2376" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:50</t>
+        </is>
+      </c>
+      <c r="C2376" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2376" s="2">
+        <v>19.6</v>
+      </c>
+      <c r="E2376" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="F2376" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2376" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2377">
+      <c r="A2377" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2377" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:00</t>
+        </is>
+      </c>
+      <c r="C2377" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2377" s="2">
+        <v>19.9</v>
+      </c>
+      <c r="E2377" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="F2377" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2377" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2378">
+      <c r="A2378" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2378" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:10</t>
+        </is>
+      </c>
+      <c r="C2378" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2378" s="2">
+        <v>20.7</v>
+      </c>
+      <c r="E2378" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F2378" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2378" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2379">
+      <c r="A2379" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2379" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:20</t>
+        </is>
+      </c>
+      <c r="C2379" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2379" s="2">
+        <v>20.6</v>
+      </c>
+      <c r="E2379" s="2">
+        <v>72.0</v>
+      </c>
+      <c r="F2379" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2379" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2380">
+      <c r="A2380" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2380" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:30</t>
+        </is>
+      </c>
+      <c r="C2380" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2380" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="E2380" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F2380" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2380" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2381">
+      <c r="A2381" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2381" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:40</t>
+        </is>
+      </c>
+      <c r="C2381" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2381" s="2">
+        <v>21.9</v>
+      </c>
+      <c r="E2381" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F2381" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2381" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2382">
+      <c r="A2382" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2382" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:50</t>
+        </is>
+      </c>
+      <c r="C2382" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2382" s="2">
+        <v>22.4</v>
+      </c>
+      <c r="E2382" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F2382" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2382" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2383">
+      <c r="A2383" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2383" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:00</t>
+        </is>
+      </c>
+      <c r="C2383" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2383" s="2">
+        <v>22.7</v>
+      </c>
+      <c r="E2383" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2383" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2383" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2384">
+      <c r="A2384" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2384" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:10</t>
+        </is>
+      </c>
+      <c r="C2384" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2384" s="2">
+        <v>22.7</v>
+      </c>
+      <c r="E2384" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2384" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2384" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2385">
+      <c r="A2385" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2385" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:20</t>
+        </is>
+      </c>
+      <c r="C2385" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2385" s="2">
+        <v>23.8</v>
+      </c>
+      <c r="E2385" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F2385" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2385" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2386">
+      <c r="A2386" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2386" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:30</t>
+        </is>
+      </c>
+      <c r="C2386" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2386" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="E2386" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F2386" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2386" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2387">
+      <c r="A2387" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2387" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:40</t>
+        </is>
+      </c>
+      <c r="C2387" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2387" s="2">
+        <v>24.2</v>
+      </c>
+      <c r="E2387" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2387" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2387" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2388">
+      <c r="A2388" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2388" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:50</t>
+        </is>
+      </c>
+      <c r="C2388" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2388" s="2">
+        <v>24.6</v>
+      </c>
+      <c r="E2388" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F2388" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2388" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2389">
+      <c r="A2389" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2389" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:00</t>
+        </is>
+      </c>
+      <c r="C2389" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2389" s="2">
+        <v>25.3</v>
+      </c>
+      <c r="E2389" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F2389" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2389" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2390">
+      <c r="A2390" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2390" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:10</t>
+        </is>
+      </c>
+      <c r="C2390" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2390" s="2">
+        <v>25.5</v>
+      </c>
+      <c r="E2390" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F2390" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2390" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2391">
+      <c r="A2391" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2391" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:20</t>
+        </is>
+      </c>
+      <c r="C2391" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2391" s="2">
+        <v>26.3</v>
+      </c>
+      <c r="E2391" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F2391" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2391" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2392">
+      <c r="A2392" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2392" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:30</t>
+        </is>
+      </c>
+      <c r="C2392" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2392" s="2">
+        <v>27.5</v>
+      </c>
+      <c r="E2392" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F2392" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2392" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2393">
+      <c r="A2393" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2393" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:40</t>
+        </is>
+      </c>
+      <c r="C2393" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2393" s="2">
+        <v>27.3</v>
+      </c>
+      <c r="E2393" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F2393" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2393" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2394">
+      <c r="A2394" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2394" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:50</t>
+        </is>
+      </c>
+      <c r="C2394" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2394" s="2">
+        <v>28.1</v>
+      </c>
+      <c r="E2394" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F2394" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2394" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2395">
+      <c r="A2395" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2395" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:00</t>
+        </is>
+      </c>
+      <c r="C2395" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2395" s="2">
+        <v>28.3</v>
+      </c>
+      <c r="E2395" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F2395" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2395" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2396">
+      <c r="A2396" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2396" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:10</t>
+        </is>
+      </c>
+      <c r="C2396" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2396" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="E2396" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F2396" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2396" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2397">
+      <c r="A2397" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2397" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:20</t>
+        </is>
+      </c>
+      <c r="C2397" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2397" s="2">
+        <v>29.4</v>
+      </c>
+      <c r="E2397" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F2397" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2397" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2398">
+      <c r="A2398" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2398" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:30</t>
+        </is>
+      </c>
+      <c r="C2398" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2398" s="2">
+        <v>29.7</v>
+      </c>
+      <c r="E2398" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F2398" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2398" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2399">
+      <c r="A2399" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2399" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:40</t>
+        </is>
+      </c>
+      <c r="C2399" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2399" s="2">
+        <v>30.2</v>
+      </c>
+      <c r="E2399" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F2399" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2399" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2400">
+      <c r="A2400" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2400" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:50</t>
+        </is>
+      </c>
+      <c r="C2400" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2400" s="2">
+        <v>30.7</v>
+      </c>
+      <c r="E2400" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F2400" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2400" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2401">
+      <c r="A2401" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2401" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:00</t>
+        </is>
+      </c>
+      <c r="C2401" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2401" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="E2401" s="2">
+        <v>38.0</v>
+      </c>
+      <c r="F2401" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2401" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2402">
+      <c r="A2402" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2402" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:10</t>
+        </is>
+      </c>
+      <c r="C2402" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2402" s="2">
+        <v>31.6</v>
+      </c>
+      <c r="E2402" s="2">
+        <v>37.0</v>
+      </c>
+      <c r="F2402" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2402" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2403">
+      <c r="A2403" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2403" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:20</t>
+        </is>
+      </c>
+      <c r="C2403" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2403" s="2">
+        <v>31.8</v>
+      </c>
+      <c r="E2403" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="F2403" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2403" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2404">
+      <c r="A2404" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2404" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:30</t>
+        </is>
+      </c>
+      <c r="C2404" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2404" s="2">
+        <v>32.3</v>
+      </c>
+      <c r="E2404" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F2404" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2404" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2405">
+      <c r="A2405" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2405" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:40</t>
+        </is>
+      </c>
+      <c r="C2405" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2405" s="2">
+        <v>32.9</v>
+      </c>
+      <c r="E2405" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F2405" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2405" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2406">
+      <c r="A2406" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2406" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:50</t>
+        </is>
+      </c>
+      <c r="C2406" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2406" s="2">
+        <v>32.5</v>
+      </c>
+      <c r="E2406" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F2406" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2406" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2407">
+      <c r="A2407" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2407" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:00</t>
+        </is>
+      </c>
+      <c r="C2407" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2407" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="E2407" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F2407" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2407" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2408">
+      <c r="A2408" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2408" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:10</t>
+        </is>
+      </c>
+      <c r="C2408" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2408" s="2">
+        <v>33.6</v>
+      </c>
+      <c r="E2408" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="F2408" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2408" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2409">
+      <c r="A2409" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2409" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:20</t>
+        </is>
+      </c>
+      <c r="C2409" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2409" s="2">
+        <v>33.9</v>
+      </c>
+      <c r="E2409" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F2409" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2409" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2410">
+      <c r="A2410" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2410" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:30</t>
+        </is>
+      </c>
+      <c r="C2410" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2410" s="2">
+        <v>34.1</v>
+      </c>
+      <c r="E2410" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F2410" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2410" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2411">
+      <c r="A2411" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2411" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:40</t>
+        </is>
+      </c>
+      <c r="C2411" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2411" s="2">
+        <v>34.1</v>
+      </c>
+      <c r="E2411" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F2411" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2411" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2412">
+      <c r="A2412" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2412" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:50</t>
+        </is>
+      </c>
+      <c r="C2412" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2412" s="2">
+        <v>34.3</v>
+      </c>
+      <c r="E2412" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F2412" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2412" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2413">
+      <c r="A2413" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2413" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:00</t>
+        </is>
+      </c>
+      <c r="C2413" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2413" s="2">
+        <v>34.6</v>
+      </c>
+      <c r="E2413" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F2413" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2413" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2414">
+      <c r="A2414" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2414" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:10</t>
+        </is>
+      </c>
+      <c r="C2414" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2414" s="2">
+        <v>34.5</v>
+      </c>
+      <c r="E2414" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F2414" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2414" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2415">
+      <c r="A2415" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2415" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:20</t>
+        </is>
+      </c>
+      <c r="C2415" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2415" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="E2415" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F2415" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2415" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2416">
+      <c r="A2416" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2416" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:30</t>
+        </is>
+      </c>
+      <c r="C2416" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2416" s="2">
+        <v>34.9</v>
+      </c>
+      <c r="E2416" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F2416" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2416" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2417">
+      <c r="A2417" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2417" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:40</t>
+        </is>
+      </c>
+      <c r="C2417" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2417" s="2">
+        <v>35.2</v>
+      </c>
+      <c r="E2417" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2417" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2417" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2418">
+      <c r="A2418" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2418" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:50</t>
+        </is>
+      </c>
+      <c r="C2418" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2418" s="2">
+        <v>35.7</v>
+      </c>
+      <c r="E2418" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2418" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2418" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2419">
+      <c r="A2419" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2419" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:00</t>
+        </is>
+      </c>
+      <c r="C2419" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2419" s="2">
+        <v>35.5</v>
+      </c>
+      <c r="E2419" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2419" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2419" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2420">
+      <c r="A2420" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2420" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:10</t>
+        </is>
+      </c>
+      <c r="C2420" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2420" s="2">
+        <v>35.5</v>
+      </c>
+      <c r="E2420" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2420" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2420" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2421">
+      <c r="A2421" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2421" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:20</t>
+        </is>
+      </c>
+      <c r="C2421" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2421" s="2">
+        <v>35.7</v>
+      </c>
+      <c r="E2421" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2421" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2421" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2422">
+      <c r="A2422" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2422" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:30</t>
+        </is>
+      </c>
+      <c r="C2422" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2422" s="2">
+        <v>35.6</v>
+      </c>
+      <c r="E2422" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2422" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2422" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2423">
+      <c r="A2423" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2423" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:40</t>
+        </is>
+      </c>
+      <c r="C2423" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2423" s="2">
+        <v>36.2</v>
+      </c>
+      <c r="E2423" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2423" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2423" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2424">
+      <c r="A2424" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2424" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:50</t>
+        </is>
+      </c>
+      <c r="C2424" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2424" s="2">
+        <v>36.4</v>
+      </c>
+      <c r="E2424" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2424" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2424" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2425">
+      <c r="A2425" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2425" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:00</t>
+        </is>
+      </c>
+      <c r="C2425" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2425" s="2">
+        <v>36.3</v>
+      </c>
+      <c r="E2425" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2425" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2425" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2426">
+      <c r="A2426" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2426" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:10</t>
+        </is>
+      </c>
+      <c r="C2426" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2426" s="2">
+        <v>36.4</v>
+      </c>
+      <c r="E2426" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2426" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2426" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2427">
+      <c r="A2427" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2427" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:20</t>
+        </is>
+      </c>
+      <c r="C2427" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2427" s="2">
+        <v>36.2</v>
+      </c>
+      <c r="E2427" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2427" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2427" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2428">
+      <c r="A2428" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2428" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:30</t>
+        </is>
+      </c>
+      <c r="C2428" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2428" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="E2428" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2428" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2428" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2429">
+      <c r="A2429" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2429" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:40</t>
+        </is>
+      </c>
+      <c r="C2429" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2429" s="2">
+        <v>35.9</v>
+      </c>
+      <c r="E2429" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2429" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2429" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2430">
+      <c r="A2430" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2430" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:50</t>
+        </is>
+      </c>
+      <c r="C2430" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2430" s="2">
+        <v>35.2</v>
+      </c>
+      <c r="E2430" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2430" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2430" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2431">
+      <c r="A2431" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2431" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:00</t>
+        </is>
+      </c>
+      <c r="C2431" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2431" s="2">
+        <v>35.8</v>
+      </c>
+      <c r="E2431" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2431" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2431" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2432">
+      <c r="A2432" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2432" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:10</t>
+        </is>
+      </c>
+      <c r="C2432" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2432" s="2">
+        <v>35.9</v>
+      </c>
+      <c r="E2432" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2432" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2432" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2433">
+      <c r="A2433" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2433" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:20</t>
+        </is>
+      </c>
+      <c r="C2433" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2433" s="2">
+        <v>36.2</v>
+      </c>
+      <c r="E2433" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="F2433" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2433" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2434">
+      <c r="A2434" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2434" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:30</t>
+        </is>
+      </c>
+      <c r="C2434" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2434" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="E2434" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2434" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2434" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2435">
+      <c r="A2435" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2435" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:40</t>
+        </is>
+      </c>
+      <c r="C2435" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2435" s="2">
+        <v>36.3</v>
+      </c>
+      <c r="E2435" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="F2435" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2435" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2436">
+      <c r="A2436" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2436" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:50</t>
+        </is>
+      </c>
+      <c r="C2436" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2436" s="2">
+        <v>36.1</v>
+      </c>
+      <c r="E2436" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="F2436" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2436" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2437">
+      <c r="A2437" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2437" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:00</t>
+        </is>
+      </c>
+      <c r="C2437" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2437" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="E2437" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="F2437" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2437" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2438">
+      <c r="A2438" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2438" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:10</t>
+        </is>
+      </c>
+      <c r="C2438" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2438" s="2">
+        <v>36.2</v>
+      </c>
+      <c r="E2438" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="F2438" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2438" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2439">
+      <c r="A2439" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2439" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:20</t>
+        </is>
+      </c>
+      <c r="C2439" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2439" s="2">
+        <v>35.5</v>
+      </c>
+      <c r="E2439" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="F2439" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2439" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2440">
+      <c r="A2440" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2440" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:30</t>
+        </is>
+      </c>
+      <c r="C2440" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2440" s="2">
+        <v>35.5</v>
+      </c>
+      <c r="E2440" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2440" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2440" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2441">
+      <c r="A2441" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2441" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:40</t>
+        </is>
+      </c>
+      <c r="C2441" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2441" s="2">
+        <v>31.2</v>
+      </c>
+      <c r="E2441" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F2441" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2441" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2442">
+      <c r="A2442" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2442" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:50</t>
+        </is>
+      </c>
+      <c r="C2442" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2442" s="2">
+        <v>29.6</v>
+      </c>
+      <c r="E2442" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F2442" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2442" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2443">
+      <c r="A2443" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2443" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:00</t>
+        </is>
+      </c>
+      <c r="C2443" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2443" s="2">
+        <v>29.2</v>
+      </c>
+      <c r="E2443" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F2443" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2443" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2444">
+      <c r="A2444" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2444" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:10</t>
+        </is>
+      </c>
+      <c r="C2444" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2444" s="2">
+        <v>29.2</v>
+      </c>
+      <c r="E2444" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F2444" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2444" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2445">
+      <c r="A2445" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2445" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:20</t>
+        </is>
+      </c>
+      <c r="C2445" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2445" s="2">
+        <v>29.2</v>
+      </c>
+      <c r="E2445" s="2">
+        <v>38.0</v>
+      </c>
+      <c r="F2445" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2445" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2446">
+      <c r="A2446" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2446" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:30</t>
+        </is>
+      </c>
+      <c r="C2446" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2446" s="2">
+        <v>29.1</v>
+      </c>
+      <c r="E2446" s="2">
+        <v>38.0</v>
+      </c>
+      <c r="F2446" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2446" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2447">
+      <c r="A2447" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2447" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:40</t>
+        </is>
+      </c>
+      <c r="C2447" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2447" s="2">
+        <v>29.2</v>
+      </c>
+      <c r="E2447" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F2447" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2447" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2448">
+      <c r="A2448" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2448" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:50</t>
+        </is>
+      </c>
+      <c r="C2448" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2448" s="2">
+        <v>29.3</v>
+      </c>
+      <c r="E2448" s="2">
+        <v>38.0</v>
+      </c>
+      <c r="F2448" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2448" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2449">
+      <c r="A2449" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2449" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:00</t>
+        </is>
+      </c>
+      <c r="C2449" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2449" s="2">
+        <v>29.3</v>
+      </c>
+      <c r="E2449" s="2">
+        <v>38.0</v>
+      </c>
+      <c r="F2449" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2449" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2450">
+      <c r="A2450" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2450" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:10</t>
+        </is>
+      </c>
+      <c r="C2450" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2450" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="E2450" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F2450" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2450" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2451">
+      <c r="A2451" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2451" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:20</t>
+        </is>
+      </c>
+      <c r="C2451" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2451" s="2">
+        <v>28.9</v>
+      </c>
+      <c r="E2451" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F2451" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2451" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2452">
+      <c r="A2452" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2452" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:30</t>
+        </is>
+      </c>
+      <c r="C2452" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2452" s="2">
+        <v>28.9</v>
+      </c>
+      <c r="E2452" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F2452" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2452" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2453">
+      <c r="A2453" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2453" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:40</t>
+        </is>
+      </c>
+      <c r="C2453" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2453" s="2">
+        <v>28.7</v>
+      </c>
+      <c r="E2453" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F2453" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2453" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2454">
+      <c r="A2454" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2454" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:50</t>
+        </is>
+      </c>
+      <c r="C2454" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2454" s="2">
+        <v>28.3</v>
+      </c>
+      <c r="E2454" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F2454" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2454" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2455">
+      <c r="A2455" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2455" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:00</t>
+        </is>
+      </c>
+      <c r="C2455" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2455" s="2">
+        <v>27.7</v>
+      </c>
+      <c r="E2455" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F2455" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2455" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2456">
+      <c r="A2456" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2456" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:10</t>
+        </is>
+      </c>
+      <c r="C2456" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2456" s="2">
+        <v>27.4</v>
+      </c>
+      <c r="E2456" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F2456" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2456" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2457">
+      <c r="A2457" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2457" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:20</t>
+        </is>
+      </c>
+      <c r="C2457" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2457" s="2">
+        <v>27.2</v>
+      </c>
+      <c r="E2457" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F2457" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2457" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2458">
+      <c r="A2458" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2458" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:30</t>
+        </is>
+      </c>
+      <c r="C2458" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2458" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="E2458" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F2458" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2458" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2459">
+      <c r="A2459" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2459" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:40</t>
+        </is>
+      </c>
+      <c r="C2459" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2459" s="2">
+        <v>26.7</v>
+      </c>
+      <c r="E2459" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F2459" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2459" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2460">
+      <c r="A2460" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2460" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:50</t>
+        </is>
+      </c>
+      <c r="C2460" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2460" s="2">
+        <v>26.4</v>
+      </c>
+      <c r="E2460" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F2460" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2460" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2461">
+      <c r="A2461" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2461" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:00</t>
+        </is>
+      </c>
+      <c r="C2461" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2461" s="2">
+        <v>26.2</v>
+      </c>
+      <c r="E2461" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F2461" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2461" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2462">
+      <c r="A2462" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2462" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:10</t>
+        </is>
+      </c>
+      <c r="C2462" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2462" s="2">
+        <v>25.7</v>
+      </c>
+      <c r="E2462" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F2462" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2462" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2463">
+      <c r="A2463" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2463" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:20</t>
+        </is>
+      </c>
+      <c r="C2463" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2463" s="2">
+        <v>25.4</v>
+      </c>
+      <c r="E2463" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F2463" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2463" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2464">
+      <c r="A2464" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2464" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:30</t>
+        </is>
+      </c>
+      <c r="C2464" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2464" s="2">
+        <v>25.1</v>
+      </c>
+      <c r="E2464" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F2464" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2464" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2465">
+      <c r="A2465" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2465" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:40</t>
+        </is>
+      </c>
+      <c r="C2465" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2465" s="2">
+        <v>24.9</v>
+      </c>
+      <c r="E2465" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F2465" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2465" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2466">
+      <c r="A2466" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2466" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:50</t>
+        </is>
+      </c>
+      <c r="C2466" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2466" s="2">
+        <v>24.8</v>
+      </c>
+      <c r="E2466" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F2466" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2466" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2467">
+      <c r="A2467" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2467" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:00</t>
+        </is>
+      </c>
+      <c r="C2467" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2467" s="2">
+        <v>24.7</v>
+      </c>
+      <c r="E2467" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F2467" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2467" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2468">
+      <c r="A2468" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2468" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:10</t>
+        </is>
+      </c>
+      <c r="C2468" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2468" s="2">
+        <v>24.5</v>
+      </c>
+      <c r="E2468" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F2468" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2468" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2469">
+      <c r="A2469" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2469" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:20</t>
+        </is>
+      </c>
+      <c r="C2469" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2469" s="2">
+        <v>24.4</v>
+      </c>
+      <c r="E2469" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F2469" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2469" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2470">
+      <c r="A2470" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2470" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:30</t>
+        </is>
+      </c>
+      <c r="C2470" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2470" s="2">
+        <v>24.3</v>
+      </c>
+      <c r="E2470" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F2470" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2470" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2471">
+      <c r="A2471" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2471" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:40</t>
+        </is>
+      </c>
+      <c r="C2471" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2471" s="2">
+        <v>24.1</v>
+      </c>
+      <c r="E2471" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2471" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2471" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2472">
+      <c r="A2472" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2472" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:50</t>
+        </is>
+      </c>
+      <c r="C2472" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2472" s="2">
+        <v>23.9</v>
+      </c>
+      <c r="E2472" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2472" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2472" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2473">
+      <c r="A2473" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2473" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:00</t>
+        </is>
+      </c>
+      <c r="C2473" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2473" s="2">
+        <v>23.9</v>
+      </c>
+      <c r="E2473" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2473" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2473" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2474">
+      <c r="A2474" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2474" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:10</t>
+        </is>
+      </c>
+      <c r="C2474" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2474" s="2">
+        <v>23.7</v>
+      </c>
+      <c r="E2474" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F2474" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2474" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2475">
+      <c r="A2475" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2475" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:20</t>
+        </is>
+      </c>
+      <c r="C2475" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2475" s="2">
+        <v>23.6</v>
+      </c>
+      <c r="E2475" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F2475" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2475" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2476">
+      <c r="A2476" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2476" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:30</t>
+        </is>
+      </c>
+      <c r="C2476" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2476" s="2">
+        <v>23.6</v>
+      </c>
+      <c r="E2476" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F2476" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2476" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2477">
+      <c r="A2477" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2477" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:40</t>
+        </is>
+      </c>
+      <c r="C2477" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2477" s="2">
+        <v>23.5</v>
+      </c>
+      <c r="E2477" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F2477" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2477" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2478">
+      <c r="A2478" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">31.07.2026</t>
+        </is>
+      </c>
+      <c r="B2478" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:50</t>
+        </is>
+      </c>
+      <c r="C2478" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2478" s="2">
+        <v>23.4</v>
+      </c>
+      <c r="E2478" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F2478" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2478" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2479">
+      <c r="A2479" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2479" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:00</t>
+        </is>
+      </c>
+      <c r="C2479" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2479" s="2">
+        <v>23.4</v>
+      </c>
+      <c r="E2479" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2479" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2479" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2480">
+      <c r="A2480" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2480" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:10</t>
+        </is>
+      </c>
+      <c r="C2480" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2480" s="2">
+        <v>23.4</v>
+      </c>
+      <c r="E2480" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2480" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2480" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2481">
+      <c r="A2481" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2481" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:20</t>
+        </is>
+      </c>
+      <c r="C2481" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2481" s="2">
+        <v>23.4</v>
+      </c>
+      <c r="E2481" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2481" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2481" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2482">
+      <c r="A2482" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2482" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:30</t>
+        </is>
+      </c>
+      <c r="C2482" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2482" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="E2482" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F2482" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2482" s="2">
         <v>0.0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G2337"/>
+  <autoFilter ref="A1:G2482"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ARSO Kranj zajem 2026-08-02 00:40 Europe/Ljubljana
</commit_message>
<xml_diff>
--- a/tabela_vremena/ARSO_Kranj.xlsx
+++ b/tabela_vremena/ARSO_Kranj.xlsx
@@ -72060,7 +72060,4154 @@
         <v>0.0</v>
       </c>
     </row>
+    <row r="2483">
+      <c r="A2483" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2483" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:40</t>
+        </is>
+      </c>
+      <c r="C2483" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2483" s="2">
+        <v>22.8</v>
+      </c>
+      <c r="E2483" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F2483" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2483" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2484">
+      <c r="A2484" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2484" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:50</t>
+        </is>
+      </c>
+      <c r="C2484" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2484" s="2">
+        <v>22.9</v>
+      </c>
+      <c r="E2484" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F2484" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2484" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2485">
+      <c r="A2485" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2485" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:00</t>
+        </is>
+      </c>
+      <c r="C2485" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2485" s="2">
+        <v>22.8</v>
+      </c>
+      <c r="E2485" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F2485" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2485" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2486">
+      <c r="A2486" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2486" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:10</t>
+        </is>
+      </c>
+      <c r="C2486" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2486" s="2">
+        <v>22.7</v>
+      </c>
+      <c r="E2486" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F2486" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2486" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2487">
+      <c r="A2487" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2487" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:20</t>
+        </is>
+      </c>
+      <c r="C2487" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2487" s="2">
+        <v>22.5</v>
+      </c>
+      <c r="E2487" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F2487" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2487" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2488">
+      <c r="A2488" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2488" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:30</t>
+        </is>
+      </c>
+      <c r="C2488" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2488" s="2">
+        <v>22.5</v>
+      </c>
+      <c r="E2488" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F2488" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2488" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2489">
+      <c r="A2489" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2489" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:40</t>
+        </is>
+      </c>
+      <c r="C2489" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2489" s="2">
+        <v>22.2</v>
+      </c>
+      <c r="E2489" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F2489" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2489" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2490">
+      <c r="A2490" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2490" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:50</t>
+        </is>
+      </c>
+      <c r="C2490" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2490" s="2">
+        <v>22.2</v>
+      </c>
+      <c r="E2490" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F2490" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2490" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2491">
+      <c r="A2491" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2491" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:00</t>
+        </is>
+      </c>
+      <c r="C2491" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2491" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="E2491" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F2491" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2491" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2492">
+      <c r="A2492" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2492" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:10</t>
+        </is>
+      </c>
+      <c r="C2492" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2492" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="E2492" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F2492" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2492" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2493">
+      <c r="A2493" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2493" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:20</t>
+        </is>
+      </c>
+      <c r="C2493" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2493" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="E2493" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F2493" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2493" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2494">
+      <c r="A2494" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2494" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:30</t>
+        </is>
+      </c>
+      <c r="C2494" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2494" s="2">
+        <v>21.9</v>
+      </c>
+      <c r="E2494" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F2494" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2494" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2495">
+      <c r="A2495" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2495" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:40</t>
+        </is>
+      </c>
+      <c r="C2495" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2495" s="2">
+        <v>21.8</v>
+      </c>
+      <c r="E2495" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F2495" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2495" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2496">
+      <c r="A2496" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2496" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:50</t>
+        </is>
+      </c>
+      <c r="C2496" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2496" s="2">
+        <v>21.8</v>
+      </c>
+      <c r="E2496" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F2496" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2496" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2497">
+      <c r="A2497" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2497" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:00</t>
+        </is>
+      </c>
+      <c r="C2497" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2497" s="2">
+        <v>21.8</v>
+      </c>
+      <c r="E2497" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F2497" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2497" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2498">
+      <c r="A2498" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2498" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:10</t>
+        </is>
+      </c>
+      <c r="C2498" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2498" s="2">
+        <v>21.5</v>
+      </c>
+      <c r="E2498" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F2498" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2498" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2499">
+      <c r="A2499" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2499" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:20</t>
+        </is>
+      </c>
+      <c r="C2499" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2499" s="2">
+        <v>21.3</v>
+      </c>
+      <c r="E2499" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2499" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2499" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2500">
+      <c r="A2500" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2500" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:30</t>
+        </is>
+      </c>
+      <c r="C2500" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2500" s="2">
+        <v>21.1</v>
+      </c>
+      <c r="E2500" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2500" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2500" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2501">
+      <c r="A2501" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2501" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:40</t>
+        </is>
+      </c>
+      <c r="C2501" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2501" s="2">
+        <v>21.1</v>
+      </c>
+      <c r="E2501" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2501" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2501" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2502">
+      <c r="A2502" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2502" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:50</t>
+        </is>
+      </c>
+      <c r="C2502" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2502" s="2">
+        <v>21.2</v>
+      </c>
+      <c r="E2502" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F2502" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2502" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2503">
+      <c r="A2503" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2503" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:00</t>
+        </is>
+      </c>
+      <c r="C2503" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2503" s="2">
+        <v>21.1</v>
+      </c>
+      <c r="E2503" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2503" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2503" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2504">
+      <c r="A2504" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2504" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:10</t>
+        </is>
+      </c>
+      <c r="C2504" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2504" s="2">
+        <v>20.8</v>
+      </c>
+      <c r="E2504" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2504" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2504" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2505">
+      <c r="A2505" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2505" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:20</t>
+        </is>
+      </c>
+      <c r="C2505" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2505" s="2">
+        <v>20.5</v>
+      </c>
+      <c r="E2505" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F2505" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2505" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2506">
+      <c r="A2506" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2506" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:30</t>
+        </is>
+      </c>
+      <c r="C2506" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2506" s="2">
+        <v>20.5</v>
+      </c>
+      <c r="E2506" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F2506" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2506" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2507">
+      <c r="A2507" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2507" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:40</t>
+        </is>
+      </c>
+      <c r="C2507" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2507" s="2">
+        <v>20.6</v>
+      </c>
+      <c r="E2507" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F2507" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2507" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2508">
+      <c r="A2508" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2508" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:50</t>
+        </is>
+      </c>
+      <c r="C2508" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2508" s="2">
+        <v>20.4</v>
+      </c>
+      <c r="E2508" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F2508" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2508" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2509">
+      <c r="A2509" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2509" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:00</t>
+        </is>
+      </c>
+      <c r="C2509" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2509" s="2">
+        <v>20.3</v>
+      </c>
+      <c r="E2509" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F2509" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2509" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2510">
+      <c r="A2510" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2510" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:10</t>
+        </is>
+      </c>
+      <c r="C2510" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2510" s="2">
+        <v>20.3</v>
+      </c>
+      <c r="E2510" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F2510" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2510" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2511">
+      <c r="A2511" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2511" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:20</t>
+        </is>
+      </c>
+      <c r="C2511" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2511" s="2">
+        <v>20.1</v>
+      </c>
+      <c r="E2511" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F2511" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2511" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2512">
+      <c r="A2512" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2512" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:30</t>
+        </is>
+      </c>
+      <c r="C2512" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2512" s="2">
+        <v>20.1</v>
+      </c>
+      <c r="E2512" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F2512" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2512" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2513">
+      <c r="A2513" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2513" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:40</t>
+        </is>
+      </c>
+      <c r="C2513" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2513" s="2">
+        <v>20.2</v>
+      </c>
+      <c r="E2513" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F2513" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2513" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2514">
+      <c r="A2514" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2514" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:50</t>
+        </is>
+      </c>
+      <c r="C2514" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2514" s="2">
+        <v>20.2</v>
+      </c>
+      <c r="E2514" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F2514" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2514" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2515">
+      <c r="A2515" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2515" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:00</t>
+        </is>
+      </c>
+      <c r="C2515" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2515" s="2">
+        <v>20.1</v>
+      </c>
+      <c r="E2515" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F2515" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2515" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2516">
+      <c r="A2516" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2516" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:10</t>
+        </is>
+      </c>
+      <c r="C2516" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2516" s="2">
+        <v>19.9</v>
+      </c>
+      <c r="E2516" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F2516" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2516" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2517">
+      <c r="A2517" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2517" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:20</t>
+        </is>
+      </c>
+      <c r="C2517" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2517" s="2">
+        <v>19.9</v>
+      </c>
+      <c r="E2517" s="2">
+        <v>69.0</v>
+      </c>
+      <c r="F2517" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2517" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2518">
+      <c r="A2518" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2518" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:30</t>
+        </is>
+      </c>
+      <c r="C2518" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2518" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="E2518" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F2518" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2518" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2519">
+      <c r="A2519" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2519" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:40</t>
+        </is>
+      </c>
+      <c r="C2519" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2519" s="2">
+        <v>20.1</v>
+      </c>
+      <c r="E2519" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F2519" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2519" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2520">
+      <c r="A2520" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2520" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:50</t>
+        </is>
+      </c>
+      <c r="C2520" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2520" s="2">
+        <v>20.3</v>
+      </c>
+      <c r="E2520" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F2520" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2520" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2521">
+      <c r="A2521" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2521" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:00</t>
+        </is>
+      </c>
+      <c r="C2521" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2521" s="2">
+        <v>20.5</v>
+      </c>
+      <c r="E2521" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F2521" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2521" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2522">
+      <c r="A2522" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2522" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:10</t>
+        </is>
+      </c>
+      <c r="C2522" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2522" s="2">
+        <v>20.8</v>
+      </c>
+      <c r="E2522" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2522" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2522" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2523">
+      <c r="A2523" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2523" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:20</t>
+        </is>
+      </c>
+      <c r="C2523" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2523" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="E2523" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2523" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2523" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2524">
+      <c r="A2524" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2524" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:30</t>
+        </is>
+      </c>
+      <c r="C2524" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2524" s="2">
+        <v>21.4</v>
+      </c>
+      <c r="E2524" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F2524" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2524" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2525">
+      <c r="A2525" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2525" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:40</t>
+        </is>
+      </c>
+      <c r="C2525" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2525" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="E2525" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F2525" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2525" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2526">
+      <c r="A2526" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2526" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:50</t>
+        </is>
+      </c>
+      <c r="C2526" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2526" s="2">
+        <v>22.6</v>
+      </c>
+      <c r="E2526" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F2526" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2526" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2527">
+      <c r="A2527" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2527" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:00</t>
+        </is>
+      </c>
+      <c r="C2527" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2527" s="2">
+        <v>23.1</v>
+      </c>
+      <c r="E2527" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2527" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2527" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2528">
+      <c r="A2528" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2528" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:10</t>
+        </is>
+      </c>
+      <c r="C2528" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2528" s="2">
+        <v>23.9</v>
+      </c>
+      <c r="E2528" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F2528" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2528" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2529">
+      <c r="A2529" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2529" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:20</t>
+        </is>
+      </c>
+      <c r="C2529" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2529" s="2">
+        <v>24.3</v>
+      </c>
+      <c r="E2529" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F2529" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2529" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2530">
+      <c r="A2530" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2530" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:30</t>
+        </is>
+      </c>
+      <c r="C2530" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2530" s="2">
+        <v>25.2</v>
+      </c>
+      <c r="E2530" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F2530" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2530" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2531">
+      <c r="A2531" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2531" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:40</t>
+        </is>
+      </c>
+      <c r="C2531" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2531" s="2">
+        <v>25.9</v>
+      </c>
+      <c r="E2531" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F2531" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2531" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2532">
+      <c r="A2532" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2532" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:50</t>
+        </is>
+      </c>
+      <c r="C2532" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2532" s="2">
+        <v>26.7</v>
+      </c>
+      <c r="E2532" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F2532" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2532" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2533">
+      <c r="A2533" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2533" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:00</t>
+        </is>
+      </c>
+      <c r="C2533" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2533" s="2">
+        <v>27.2</v>
+      </c>
+      <c r="E2533" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F2533" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2533" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2534">
+      <c r="A2534" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2534" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:10</t>
+        </is>
+      </c>
+      <c r="C2534" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2534" s="2">
+        <v>27.7</v>
+      </c>
+      <c r="E2534" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F2534" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2534" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2535">
+      <c r="A2535" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2535" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:20</t>
+        </is>
+      </c>
+      <c r="C2535" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2535" s="2">
+        <v>27.9</v>
+      </c>
+      <c r="E2535" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F2535" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2535" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2536">
+      <c r="A2536" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2536" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:30</t>
+        </is>
+      </c>
+      <c r="C2536" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2536" s="2">
+        <v>27.8</v>
+      </c>
+      <c r="E2536" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F2536" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2536" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2537">
+      <c r="A2537" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2537" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:40</t>
+        </is>
+      </c>
+      <c r="C2537" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2537" s="2">
+        <v>28.2</v>
+      </c>
+      <c r="E2537" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F2537" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2537" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2538">
+      <c r="A2538" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2538" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:50</t>
+        </is>
+      </c>
+      <c r="C2538" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2538" s="2">
+        <v>27.9</v>
+      </c>
+      <c r="E2538" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F2538" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2538" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2539">
+      <c r="A2539" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2539" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:00</t>
+        </is>
+      </c>
+      <c r="C2539" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2539" s="2">
+        <v>27.3</v>
+      </c>
+      <c r="E2539" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F2539" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2539" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2540">
+      <c r="A2540" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2540" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:10</t>
+        </is>
+      </c>
+      <c r="C2540" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2540" s="2">
+        <v>27.5</v>
+      </c>
+      <c r="E2540" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F2540" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2540" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2541">
+      <c r="A2541" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2541" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:20</t>
+        </is>
+      </c>
+      <c r="C2541" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2541" s="2">
+        <v>28.3</v>
+      </c>
+      <c r="E2541" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F2541" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2541" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2542">
+      <c r="A2542" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2542" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:30</t>
+        </is>
+      </c>
+      <c r="C2542" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2542" s="2">
+        <v>28.7</v>
+      </c>
+      <c r="E2542" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F2542" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2542" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2543">
+      <c r="A2543" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2543" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:40</t>
+        </is>
+      </c>
+      <c r="C2543" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2543" s="2">
+        <v>29.4</v>
+      </c>
+      <c r="E2543" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F2543" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2543" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2544">
+      <c r="A2544" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2544" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:50</t>
+        </is>
+      </c>
+      <c r="C2544" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2544" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="E2544" s="2">
+        <v>38.0</v>
+      </c>
+      <c r="F2544" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2544" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2545">
+      <c r="A2545" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2545" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:00</t>
+        </is>
+      </c>
+      <c r="C2545" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2545" s="2">
+        <v>30.3</v>
+      </c>
+      <c r="E2545" s="2">
+        <v>37.0</v>
+      </c>
+      <c r="F2545" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2545" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2546">
+      <c r="A2546" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2546" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:10</t>
+        </is>
+      </c>
+      <c r="C2546" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2546" s="2">
+        <v>31.1</v>
+      </c>
+      <c r="E2546" s="2">
+        <v>37.0</v>
+      </c>
+      <c r="F2546" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2546" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2547">
+      <c r="A2547" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2547" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:20</t>
+        </is>
+      </c>
+      <c r="C2547" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2547" s="2">
+        <v>31.4</v>
+      </c>
+      <c r="E2547" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="F2547" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2547" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2548">
+      <c r="A2548" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2548" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:30</t>
+        </is>
+      </c>
+      <c r="C2548" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2548" s="2">
+        <v>32.1</v>
+      </c>
+      <c r="E2548" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F2548" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2548" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2549">
+      <c r="A2549" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2549" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:40</t>
+        </is>
+      </c>
+      <c r="C2549" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2549" s="2">
+        <v>32.5</v>
+      </c>
+      <c r="E2549" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F2549" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2549" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2550">
+      <c r="A2550" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2550" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:50</t>
+        </is>
+      </c>
+      <c r="C2550" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2550" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="E2550" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="F2550" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2550" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2551">
+      <c r="A2551" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2551" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:00</t>
+        </is>
+      </c>
+      <c r="C2551" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2551" s="2">
+        <v>33.2</v>
+      </c>
+      <c r="E2551" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F2551" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2551" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2552">
+      <c r="A2552" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2552" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:10</t>
+        </is>
+      </c>
+      <c r="C2552" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2552" s="2">
+        <v>33.9</v>
+      </c>
+      <c r="E2552" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2552" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2552" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2553">
+      <c r="A2553" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2553" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:20</t>
+        </is>
+      </c>
+      <c r="C2553" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2553" s="2">
+        <v>34.6</v>
+      </c>
+      <c r="E2553" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2553" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2553" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2554">
+      <c r="A2554" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2554" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:30</t>
+        </is>
+      </c>
+      <c r="C2554" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2554" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="E2554" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2554" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2554" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2555">
+      <c r="A2555" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2555" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:40</t>
+        </is>
+      </c>
+      <c r="C2555" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2555" s="2">
+        <v>34.3</v>
+      </c>
+      <c r="E2555" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2555" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2555" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2556">
+      <c r="A2556" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2556" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:50</t>
+        </is>
+      </c>
+      <c r="C2556" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2556" s="2">
+        <v>33.7</v>
+      </c>
+      <c r="E2556" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2556" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2556" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2557">
+      <c r="A2557" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2557" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:00</t>
+        </is>
+      </c>
+      <c r="C2557" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2557" s="2">
+        <v>34.5</v>
+      </c>
+      <c r="E2557" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2557" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2557" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2558">
+      <c r="A2558" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2558" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:10</t>
+        </is>
+      </c>
+      <c r="C2558" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2558" s="2">
+        <v>34.8</v>
+      </c>
+      <c r="E2558" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2558" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2558" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2559">
+      <c r="A2559" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2559" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:20</t>
+        </is>
+      </c>
+      <c r="C2559" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2559" s="2">
+        <v>35.2</v>
+      </c>
+      <c r="E2559" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2559" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2559" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2560">
+      <c r="A2560" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2560" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:30</t>
+        </is>
+      </c>
+      <c r="C2560" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2560" s="2">
+        <v>35.3</v>
+      </c>
+      <c r="E2560" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2560" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2560" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2561">
+      <c r="A2561" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2561" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:40</t>
+        </is>
+      </c>
+      <c r="C2561" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2561" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="E2561" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2561" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2561" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2562">
+      <c r="A2562" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2562" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:50</t>
+        </is>
+      </c>
+      <c r="C2562" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2562" s="2">
+        <v>35.7</v>
+      </c>
+      <c r="E2562" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2562" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2562" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2563">
+      <c r="A2563" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2563" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:00</t>
+        </is>
+      </c>
+      <c r="C2563" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2563" s="2">
+        <v>35.8</v>
+      </c>
+      <c r="E2563" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2563" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2563" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2564">
+      <c r="A2564" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2564" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:10</t>
+        </is>
+      </c>
+      <c r="C2564" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2564" s="2">
+        <v>35.3</v>
+      </c>
+      <c r="E2564" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2564" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2564" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2565">
+      <c r="A2565" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2565" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:20</t>
+        </is>
+      </c>
+      <c r="C2565" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2565" s="2">
+        <v>35.7</v>
+      </c>
+      <c r="E2565" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="F2565" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2565" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2566">
+      <c r="A2566" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2566" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:30</t>
+        </is>
+      </c>
+      <c r="C2566" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2566" s="2">
+        <v>36.2</v>
+      </c>
+      <c r="E2566" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="F2566" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2566" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2567">
+      <c r="A2567" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2567" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:40</t>
+        </is>
+      </c>
+      <c r="C2567" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2567" s="2">
+        <v>36.2</v>
+      </c>
+      <c r="E2567" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="F2567" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2567" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2568">
+      <c r="A2568" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2568" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:50</t>
+        </is>
+      </c>
+      <c r="C2568" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2568" s="2">
+        <v>35.7</v>
+      </c>
+      <c r="E2568" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="F2568" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2568" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2569">
+      <c r="A2569" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2569" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:00</t>
+        </is>
+      </c>
+      <c r="C2569" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2569" s="2">
+        <v>36.8</v>
+      </c>
+      <c r="E2569" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="F2569" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2569" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2570">
+      <c r="A2570" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2570" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:10</t>
+        </is>
+      </c>
+      <c r="C2570" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2570" s="2">
+        <v>36.6</v>
+      </c>
+      <c r="E2570" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="F2570" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2570" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2571">
+      <c r="A2571" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2571" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:20</t>
+        </is>
+      </c>
+      <c r="C2571" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2571" s="2">
+        <v>36.3</v>
+      </c>
+      <c r="E2571" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="F2571" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2571" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2572">
+      <c r="A2572" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2572" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:30</t>
+        </is>
+      </c>
+      <c r="C2572" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2572" s="2">
+        <v>35.9</v>
+      </c>
+      <c r="E2572" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="F2572" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2572" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2573">
+      <c r="A2573" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2573" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:40</t>
+        </is>
+      </c>
+      <c r="C2573" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2573" s="2">
+        <v>35.9</v>
+      </c>
+      <c r="E2573" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="F2573" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2573" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2574">
+      <c r="A2574" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2574" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:50</t>
+        </is>
+      </c>
+      <c r="C2574" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2574" s="2">
+        <v>36.3</v>
+      </c>
+      <c r="E2574" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2574" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2574" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2575">
+      <c r="A2575" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2575" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:00</t>
+        </is>
+      </c>
+      <c r="C2575" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2575" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="E2575" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2575" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2575" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2576">
+      <c r="A2576" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2576" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:10</t>
+        </is>
+      </c>
+      <c r="C2576" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2576" s="2">
+        <v>36.1</v>
+      </c>
+      <c r="E2576" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2576" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2576" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2577">
+      <c r="A2577" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2577" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:20</t>
+        </is>
+      </c>
+      <c r="C2577" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2577" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="E2577" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2577" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2577" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2578">
+      <c r="A2578" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2578" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:30</t>
+        </is>
+      </c>
+      <c r="C2578" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2578" s="2">
+        <v>36.3</v>
+      </c>
+      <c r="E2578" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2578" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2578" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2579">
+      <c r="A2579" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2579" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:40</t>
+        </is>
+      </c>
+      <c r="C2579" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2579" s="2">
+        <v>35.8</v>
+      </c>
+      <c r="E2579" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2579" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2579" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2580">
+      <c r="A2580" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2580" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:50</t>
+        </is>
+      </c>
+      <c r="C2580" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2580" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="E2580" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2580" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2580" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2581">
+      <c r="A2581" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2581" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:00</t>
+        </is>
+      </c>
+      <c r="C2581" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2581" s="2">
+        <v>36.1</v>
+      </c>
+      <c r="E2581" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2581" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2581" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2582">
+      <c r="A2582" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2582" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:10</t>
+        </is>
+      </c>
+      <c r="C2582" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2582" s="2">
+        <v>35.5</v>
+      </c>
+      <c r="E2582" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2582" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2582" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2583">
+      <c r="A2583" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2583" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:20</t>
+        </is>
+      </c>
+      <c r="C2583" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2583" s="2">
+        <v>35.5</v>
+      </c>
+      <c r="E2583" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2583" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2583" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2584">
+      <c r="A2584" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2584" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:30</t>
+        </is>
+      </c>
+      <c r="C2584" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2584" s="2">
+        <v>35.8</v>
+      </c>
+      <c r="E2584" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2584" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2584" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2585">
+      <c r="A2585" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2585" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:40</t>
+        </is>
+      </c>
+      <c r="C2585" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2585" s="2">
+        <v>36.4</v>
+      </c>
+      <c r="E2585" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2585" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2585" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2586">
+      <c r="A2586" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2586" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:50</t>
+        </is>
+      </c>
+      <c r="C2586" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2586" s="2">
+        <v>36.4</v>
+      </c>
+      <c r="E2586" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2586" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2586" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2587">
+      <c r="A2587" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2587" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:00</t>
+        </is>
+      </c>
+      <c r="C2587" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2587" s="2">
+        <v>35.9</v>
+      </c>
+      <c r="E2587" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2587" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2587" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2588">
+      <c r="A2588" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2588" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:10</t>
+        </is>
+      </c>
+      <c r="C2588" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2588" s="2">
+        <v>35.3</v>
+      </c>
+      <c r="E2588" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2588" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2588" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2589">
+      <c r="A2589" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2589" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:20</t>
+        </is>
+      </c>
+      <c r="C2589" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2589" s="2">
+        <v>35.1</v>
+      </c>
+      <c r="E2589" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2589" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2589" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2590">
+      <c r="A2590" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2590" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:30</t>
+        </is>
+      </c>
+      <c r="C2590" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2590" s="2">
+        <v>34.7</v>
+      </c>
+      <c r="E2590" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2590" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2590" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2591">
+      <c r="A2591" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2591" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:40</t>
+        </is>
+      </c>
+      <c r="C2591" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2591" s="2">
+        <v>34.3</v>
+      </c>
+      <c r="E2591" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2591" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2591" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2592">
+      <c r="A2592" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2592" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:50</t>
+        </is>
+      </c>
+      <c r="C2592" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2592" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="E2592" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2592" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2592" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2593">
+      <c r="A2593" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2593" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:00</t>
+        </is>
+      </c>
+      <c r="C2593" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2593" s="2">
+        <v>33.8</v>
+      </c>
+      <c r="E2593" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2593" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2593" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2594">
+      <c r="A2594" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2594" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:10</t>
+        </is>
+      </c>
+      <c r="C2594" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2594" s="2">
+        <v>32.3</v>
+      </c>
+      <c r="E2594" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F2594" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2594" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2595">
+      <c r="A2595" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2595" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:20</t>
+        </is>
+      </c>
+      <c r="C2595" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2595" s="2">
+        <v>29.7</v>
+      </c>
+      <c r="E2595" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F2595" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2595" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2596">
+      <c r="A2596" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2596" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:30</t>
+        </is>
+      </c>
+      <c r="C2596" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2596" s="2">
+        <v>27.8</v>
+      </c>
+      <c r="E2596" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F2596" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2596" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2597">
+      <c r="A2597" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2597" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:40</t>
+        </is>
+      </c>
+      <c r="C2597" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2597" s="2">
+        <v>25.9</v>
+      </c>
+      <c r="E2597" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F2597" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2597" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2598">
+      <c r="A2598" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2598" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:50</t>
+        </is>
+      </c>
+      <c r="C2598" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2598" s="2">
+        <v>25.2</v>
+      </c>
+      <c r="E2598" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F2598" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2598" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2599">
+      <c r="A2599" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2599" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:00</t>
+        </is>
+      </c>
+      <c r="C2599" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2599" s="2">
+        <v>24.6</v>
+      </c>
+      <c r="E2599" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F2599" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2599" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2600">
+      <c r="A2600" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2600" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:10</t>
+        </is>
+      </c>
+      <c r="C2600" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2600" s="2">
+        <v>24.2</v>
+      </c>
+      <c r="E2600" s="2">
+        <v>69.0</v>
+      </c>
+      <c r="F2600" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2600" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2601">
+      <c r="A2601" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2601" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:20</t>
+        </is>
+      </c>
+      <c r="C2601" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2601" s="2">
+        <v>24.2</v>
+      </c>
+      <c r="E2601" s="2">
+        <v>69.0</v>
+      </c>
+      <c r="F2601" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2601" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2602">
+      <c r="A2602" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2602" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:30</t>
+        </is>
+      </c>
+      <c r="C2602" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2602" s="2">
+        <v>24.1</v>
+      </c>
+      <c r="E2602" s="2">
+        <v>69.0</v>
+      </c>
+      <c r="F2602" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2602" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2603">
+      <c r="A2603" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2603" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:40</t>
+        </is>
+      </c>
+      <c r="C2603" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2603" s="2">
+        <v>23.9</v>
+      </c>
+      <c r="E2603" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F2603" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2603" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2604">
+      <c r="A2604" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2604" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:50</t>
+        </is>
+      </c>
+      <c r="C2604" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2604" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="E2604" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F2604" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2604" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2605">
+      <c r="A2605" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2605" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:00</t>
+        </is>
+      </c>
+      <c r="C2605" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2605" s="2">
+        <v>24.3</v>
+      </c>
+      <c r="E2605" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F2605" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2605" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2606">
+      <c r="A2606" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2606" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:10</t>
+        </is>
+      </c>
+      <c r="C2606" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2606" s="2">
+        <v>24.5</v>
+      </c>
+      <c r="E2606" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2606" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2606" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2607">
+      <c r="A2607" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2607" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:20</t>
+        </is>
+      </c>
+      <c r="C2607" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2607" s="2">
+        <v>24.6</v>
+      </c>
+      <c r="E2607" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F2607" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2607" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2608">
+      <c r="A2608" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2608" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:30</t>
+        </is>
+      </c>
+      <c r="C2608" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2608" s="2">
+        <v>24.3</v>
+      </c>
+      <c r="E2608" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2608" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2608" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2609">
+      <c r="A2609" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2609" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:40</t>
+        </is>
+      </c>
+      <c r="C2609" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2609" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="E2609" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F2609" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2609" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2610">
+      <c r="A2610" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2610" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:50</t>
+        </is>
+      </c>
+      <c r="C2610" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2610" s="2">
+        <v>23.7</v>
+      </c>
+      <c r="E2610" s="2">
+        <v>69.0</v>
+      </c>
+      <c r="F2610" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2610" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2611">
+      <c r="A2611" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2611" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:00</t>
+        </is>
+      </c>
+      <c r="C2611" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2611" s="2">
+        <v>23.6</v>
+      </c>
+      <c r="E2611" s="2">
+        <v>69.0</v>
+      </c>
+      <c r="F2611" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2611" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2612">
+      <c r="A2612" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2612" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:10</t>
+        </is>
+      </c>
+      <c r="C2612" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2612" s="2">
+        <v>23.8</v>
+      </c>
+      <c r="E2612" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F2612" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2612" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2613">
+      <c r="A2613" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2613" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:20</t>
+        </is>
+      </c>
+      <c r="C2613" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2613" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="E2613" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F2613" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2613" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2614">
+      <c r="A2614" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2614" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:30</t>
+        </is>
+      </c>
+      <c r="C2614" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2614" s="2">
+        <v>24.2</v>
+      </c>
+      <c r="E2614" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2614" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2614" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2615">
+      <c r="A2615" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2615" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:40</t>
+        </is>
+      </c>
+      <c r="C2615" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2615" s="2">
+        <v>24.3</v>
+      </c>
+      <c r="E2615" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2615" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2615" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2616">
+      <c r="A2616" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2616" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:50</t>
+        </is>
+      </c>
+      <c r="C2616" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2616" s="2">
+        <v>24.3</v>
+      </c>
+      <c r="E2616" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2616" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2616" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2617">
+      <c r="A2617" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2617" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:00</t>
+        </is>
+      </c>
+      <c r="C2617" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2617" s="2">
+        <v>24.5</v>
+      </c>
+      <c r="E2617" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F2617" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2617" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2618">
+      <c r="A2618" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2618" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:10</t>
+        </is>
+      </c>
+      <c r="C2618" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2618" s="2">
+        <v>24.2</v>
+      </c>
+      <c r="E2618" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2618" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2618" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2619">
+      <c r="A2619" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2619" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:20</t>
+        </is>
+      </c>
+      <c r="C2619" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2619" s="2">
+        <v>24.1</v>
+      </c>
+      <c r="E2619" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2619" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2619" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2620">
+      <c r="A2620" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2620" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:30</t>
+        </is>
+      </c>
+      <c r="C2620" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2620" s="2">
+        <v>24.2</v>
+      </c>
+      <c r="E2620" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2620" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2620" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2621">
+      <c r="A2621" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2621" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:40</t>
+        </is>
+      </c>
+      <c r="C2621" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2621" s="2">
+        <v>24.2</v>
+      </c>
+      <c r="E2621" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F2621" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2621" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2622">
+      <c r="A2622" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01.08.2026</t>
+        </is>
+      </c>
+      <c r="B2622" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:50</t>
+        </is>
+      </c>
+      <c r="C2622" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2622" s="2">
+        <v>24.1</v>
+      </c>
+      <c r="E2622" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F2622" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2622" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2623">
+      <c r="A2623" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2623" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:00</t>
+        </is>
+      </c>
+      <c r="C2623" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2623" s="2">
+        <v>24.1</v>
+      </c>
+      <c r="E2623" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F2623" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2623" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2624">
+      <c r="A2624" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2624" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:10</t>
+        </is>
+      </c>
+      <c r="C2624" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2624" s="2">
+        <v>24.2</v>
+      </c>
+      <c r="E2624" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F2624" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2624" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2625">
+      <c r="A2625" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2625" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:20</t>
+        </is>
+      </c>
+      <c r="C2625" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2625" s="2">
+        <v>24.1</v>
+      </c>
+      <c r="E2625" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F2625" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2625" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G2482"/>
+  <autoFilter ref="A1:G2625"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ARSO Kranj zajem 2026-08-03 00:41 Europe/Ljubljana
</commit_message>
<xml_diff>
--- a/tabela_vremena/ARSO_Kranj.xlsx
+++ b/tabela_vremena/ARSO_Kranj.xlsx
@@ -76207,7 +76207,4212 @@
         <v>0.0</v>
       </c>
     </row>
+    <row r="2626">
+      <c r="A2626" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2626" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:30</t>
+        </is>
+      </c>
+      <c r="C2626" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2626" s="2">
+        <v>24.2</v>
+      </c>
+      <c r="E2626" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F2626" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2626" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2627">
+      <c r="A2627" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2627" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:40</t>
+        </is>
+      </c>
+      <c r="C2627" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2627" s="2">
+        <v>24.1</v>
+      </c>
+      <c r="E2627" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F2627" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2627" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2628">
+      <c r="A2628" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2628" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:50</t>
+        </is>
+      </c>
+      <c r="C2628" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2628" s="2">
+        <v>24.1</v>
+      </c>
+      <c r="E2628" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F2628" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2628" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2629">
+      <c r="A2629" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2629" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:00</t>
+        </is>
+      </c>
+      <c r="C2629" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2629" s="2">
+        <v>23.9</v>
+      </c>
+      <c r="E2629" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F2629" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2629" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2630">
+      <c r="A2630" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2630" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:10</t>
+        </is>
+      </c>
+      <c r="C2630" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2630" s="2">
+        <v>24.1</v>
+      </c>
+      <c r="E2630" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F2630" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2630" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2631">
+      <c r="A2631" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2631" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:20</t>
+        </is>
+      </c>
+      <c r="C2631" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2631" s="2">
+        <v>23.9</v>
+      </c>
+      <c r="E2631" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F2631" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2631" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2632">
+      <c r="A2632" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2632" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:30</t>
+        </is>
+      </c>
+      <c r="C2632" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2632" s="2">
+        <v>23.8</v>
+      </c>
+      <c r="E2632" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F2632" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2632" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2633">
+      <c r="A2633" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2633" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:40</t>
+        </is>
+      </c>
+      <c r="C2633" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2633" s="2">
+        <v>23.7</v>
+      </c>
+      <c r="E2633" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F2633" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2633" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2634">
+      <c r="A2634" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2634" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:50</t>
+        </is>
+      </c>
+      <c r="C2634" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2634" s="2">
+        <v>23.5</v>
+      </c>
+      <c r="E2634" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F2634" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2634" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2635">
+      <c r="A2635" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2635" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:00</t>
+        </is>
+      </c>
+      <c r="C2635" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2635" s="2">
+        <v>23.1</v>
+      </c>
+      <c r="E2635" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F2635" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2635" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2636">
+      <c r="A2636" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2636" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:10</t>
+        </is>
+      </c>
+      <c r="C2636" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2636" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="E2636" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F2636" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2636" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2637">
+      <c r="A2637" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2637" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:20</t>
+        </is>
+      </c>
+      <c r="C2637" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2637" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="E2637" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F2637" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2637" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2638">
+      <c r="A2638" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2638" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:30</t>
+        </is>
+      </c>
+      <c r="C2638" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2638" s="2">
+        <v>22.9</v>
+      </c>
+      <c r="E2638" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F2638" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2638" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2639">
+      <c r="A2639" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2639" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:40</t>
+        </is>
+      </c>
+      <c r="C2639" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2639" s="2">
+        <v>22.6</v>
+      </c>
+      <c r="E2639" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2639" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2639" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2640">
+      <c r="A2640" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2640" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:50</t>
+        </is>
+      </c>
+      <c r="C2640" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2640" s="2">
+        <v>22.4</v>
+      </c>
+      <c r="E2640" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F2640" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2640" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2641">
+      <c r="A2641" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2641" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:00</t>
+        </is>
+      </c>
+      <c r="C2641" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2641" s="2">
+        <v>22.2</v>
+      </c>
+      <c r="E2641" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F2641" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2641" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2642">
+      <c r="A2642" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2642" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:10</t>
+        </is>
+      </c>
+      <c r="C2642" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2642" s="2">
+        <v>21.7</v>
+      </c>
+      <c r="E2642" s="2">
+        <v>72.0</v>
+      </c>
+      <c r="F2642" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2642" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2643">
+      <c r="A2643" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2643" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:20</t>
+        </is>
+      </c>
+      <c r="C2643" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2643" s="2">
+        <v>21.5</v>
+      </c>
+      <c r="E2643" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="F2643" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2643" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2644">
+      <c r="A2644" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2644" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:30</t>
+        </is>
+      </c>
+      <c r="C2644" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2644" s="2">
+        <v>21.1</v>
+      </c>
+      <c r="E2644" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F2644" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2644" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2645">
+      <c r="A2645" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2645" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:40</t>
+        </is>
+      </c>
+      <c r="C2645" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2645" s="2">
+        <v>21.2</v>
+      </c>
+      <c r="E2645" s="2">
+        <v>73.0</v>
+      </c>
+      <c r="F2645" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2645" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2646">
+      <c r="A2646" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2646" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:50</t>
+        </is>
+      </c>
+      <c r="C2646" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2646" s="2">
+        <v>20.7</v>
+      </c>
+      <c r="E2646" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F2646" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2646" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2647">
+      <c r="A2647" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2647" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:00</t>
+        </is>
+      </c>
+      <c r="C2647" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2647" s="2">
+        <v>20.4</v>
+      </c>
+      <c r="E2647" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F2647" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2647" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2648">
+      <c r="A2648" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2648" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:10</t>
+        </is>
+      </c>
+      <c r="C2648" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2648" s="2">
+        <v>20.2</v>
+      </c>
+      <c r="E2648" s="2">
+        <v>79.0</v>
+      </c>
+      <c r="F2648" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2648" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2649">
+      <c r="A2649" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2649" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:20</t>
+        </is>
+      </c>
+      <c r="C2649" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2649" s="2">
+        <v>19.9</v>
+      </c>
+      <c r="E2649" s="2">
+        <v>81.0</v>
+      </c>
+      <c r="F2649" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2649" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2650">
+      <c r="A2650" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2650" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:30</t>
+        </is>
+      </c>
+      <c r="C2650" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2650" s="2">
+        <v>19.7</v>
+      </c>
+      <c r="E2650" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F2650" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2650" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2651">
+      <c r="A2651" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2651" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:40</t>
+        </is>
+      </c>
+      <c r="C2651" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2651" s="2">
+        <v>19.5</v>
+      </c>
+      <c r="E2651" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F2651" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2651" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2652">
+      <c r="A2652" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2652" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:50</t>
+        </is>
+      </c>
+      <c r="C2652" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2652" s="2">
+        <v>19.5</v>
+      </c>
+      <c r="E2652" s="2">
+        <v>83.0</v>
+      </c>
+      <c r="F2652" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2652" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2653">
+      <c r="A2653" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2653" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:00</t>
+        </is>
+      </c>
+      <c r="C2653" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2653" s="2">
+        <v>19.5</v>
+      </c>
+      <c r="E2653" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F2653" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2653" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2654">
+      <c r="A2654" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2654" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:10</t>
+        </is>
+      </c>
+      <c r="C2654" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2654" s="2">
+        <v>19.5</v>
+      </c>
+      <c r="E2654" s="2">
+        <v>81.0</v>
+      </c>
+      <c r="F2654" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2654" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2655">
+      <c r="A2655" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2655" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:20</t>
+        </is>
+      </c>
+      <c r="C2655" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2655" s="2">
+        <v>19.4</v>
+      </c>
+      <c r="E2655" s="2">
+        <v>82.0</v>
+      </c>
+      <c r="F2655" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2655" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2656">
+      <c r="A2656" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2656" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:30</t>
+        </is>
+      </c>
+      <c r="C2656" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2656" s="2">
+        <v>19.5</v>
+      </c>
+      <c r="E2656" s="2">
+        <v>80.0</v>
+      </c>
+      <c r="F2656" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2656" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2657">
+      <c r="A2657" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2657" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:40</t>
+        </is>
+      </c>
+      <c r="C2657" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2657" s="2">
+        <v>19.7</v>
+      </c>
+      <c r="E2657" s="2">
+        <v>78.0</v>
+      </c>
+      <c r="F2657" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2657" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2658">
+      <c r="A2658" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2658" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:50</t>
+        </is>
+      </c>
+      <c r="C2658" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2658" s="2">
+        <v>19.8</v>
+      </c>
+      <c r="E2658" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F2658" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2658" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2659">
+      <c r="A2659" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2659" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:00</t>
+        </is>
+      </c>
+      <c r="C2659" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2659" s="2">
+        <v>19.8</v>
+      </c>
+      <c r="E2659" s="2">
+        <v>77.0</v>
+      </c>
+      <c r="F2659" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2659" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2660">
+      <c r="A2660" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2660" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:10</t>
+        </is>
+      </c>
+      <c r="C2660" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2660" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="E2660" s="2">
+        <v>76.0</v>
+      </c>
+      <c r="F2660" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2660" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2661">
+      <c r="A2661" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2661" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:20</t>
+        </is>
+      </c>
+      <c r="C2661" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2661" s="2">
+        <v>20.2</v>
+      </c>
+      <c r="E2661" s="2">
+        <v>74.0</v>
+      </c>
+      <c r="F2661" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2661" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2662">
+      <c r="A2662" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2662" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:30</t>
+        </is>
+      </c>
+      <c r="C2662" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2662" s="2">
+        <v>20.6</v>
+      </c>
+      <c r="E2662" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F2662" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2662" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2663">
+      <c r="A2663" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2663" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:40</t>
+        </is>
+      </c>
+      <c r="C2663" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2663" s="2">
+        <v>20.7</v>
+      </c>
+      <c r="E2663" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F2663" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2663" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2664">
+      <c r="A2664" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2664" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:50</t>
+        </is>
+      </c>
+      <c r="C2664" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2664" s="2">
+        <v>20.9</v>
+      </c>
+      <c r="E2664" s="2">
+        <v>71.0</v>
+      </c>
+      <c r="F2664" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2664" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2665">
+      <c r="A2665" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2665" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:00</t>
+        </is>
+      </c>
+      <c r="C2665" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2665" s="2">
+        <v>21.1</v>
+      </c>
+      <c r="E2665" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F2665" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2665" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2666">
+      <c r="A2666" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2666" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:10</t>
+        </is>
+      </c>
+      <c r="C2666" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2666" s="2">
+        <v>21.6</v>
+      </c>
+      <c r="E2666" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F2666" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2666" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2667">
+      <c r="A2667" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2667" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:20</t>
+        </is>
+      </c>
+      <c r="C2667" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2667" s="2">
+        <v>22.1</v>
+      </c>
+      <c r="E2667" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F2667" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2667" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2668">
+      <c r="A2668" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2668" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:30</t>
+        </is>
+      </c>
+      <c r="C2668" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2668" s="2">
+        <v>22.6</v>
+      </c>
+      <c r="E2668" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2668" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2668" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2669">
+      <c r="A2669" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2669" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:40</t>
+        </is>
+      </c>
+      <c r="C2669" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2669" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="E2669" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F2669" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2669" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2670">
+      <c r="A2670" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2670" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:50</t>
+        </is>
+      </c>
+      <c r="C2670" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2670" s="2">
+        <v>23.4</v>
+      </c>
+      <c r="E2670" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F2670" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2670" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2671">
+      <c r="A2671" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2671" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:00</t>
+        </is>
+      </c>
+      <c r="C2671" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2671" s="2">
+        <v>23.6</v>
+      </c>
+      <c r="E2671" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F2671" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2671" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2672">
+      <c r="A2672" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2672" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:10</t>
+        </is>
+      </c>
+      <c r="C2672" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2672" s="2">
+        <v>24.1</v>
+      </c>
+      <c r="E2672" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2672" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2672" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2673">
+      <c r="A2673" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2673" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:20</t>
+        </is>
+      </c>
+      <c r="C2673" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2673" s="2">
+        <v>24.6</v>
+      </c>
+      <c r="E2673" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F2673" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2673" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2674">
+      <c r="A2674" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2674" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:30</t>
+        </is>
+      </c>
+      <c r="C2674" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2674" s="2">
+        <v>25.2</v>
+      </c>
+      <c r="E2674" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F2674" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2674" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2675">
+      <c r="A2675" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2675" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:40</t>
+        </is>
+      </c>
+      <c r="C2675" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2675" s="2">
+        <v>25.5</v>
+      </c>
+      <c r="E2675" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F2675" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2675" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2676">
+      <c r="A2676" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2676" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:50</t>
+        </is>
+      </c>
+      <c r="C2676" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2676" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="E2676" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F2676" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2676" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2677">
+      <c r="A2677" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2677" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:00</t>
+        </is>
+      </c>
+      <c r="C2677" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2677" s="2">
+        <v>26.7</v>
+      </c>
+      <c r="E2677" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F2677" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2677" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2678">
+      <c r="A2678" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2678" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:10</t>
+        </is>
+      </c>
+      <c r="C2678" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2678" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="E2678" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F2678" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2678" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2679">
+      <c r="A2679" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2679" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:20</t>
+        </is>
+      </c>
+      <c r="C2679" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2679" s="2">
+        <v>27.8</v>
+      </c>
+      <c r="E2679" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F2679" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2679" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2680">
+      <c r="A2680" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2680" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:30</t>
+        </is>
+      </c>
+      <c r="C2680" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2680" s="2">
+        <v>28.2</v>
+      </c>
+      <c r="E2680" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F2680" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2680" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2681">
+      <c r="A2681" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2681" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:40</t>
+        </is>
+      </c>
+      <c r="C2681" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2681" s="2">
+        <v>28.7</v>
+      </c>
+      <c r="E2681" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F2681" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2681" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2682">
+      <c r="A2682" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2682" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:50</t>
+        </is>
+      </c>
+      <c r="C2682" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2682" s="2">
+        <v>28.7</v>
+      </c>
+      <c r="E2682" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F2682" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2682" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2683">
+      <c r="A2683" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2683" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:00</t>
+        </is>
+      </c>
+      <c r="C2683" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2683" s="2">
+        <v>28.2</v>
+      </c>
+      <c r="E2683" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F2683" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2683" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2684">
+      <c r="A2684" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2684" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:10</t>
+        </is>
+      </c>
+      <c r="C2684" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2684" s="2">
+        <v>29.1</v>
+      </c>
+      <c r="E2684" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F2684" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2684" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2685">
+      <c r="A2685" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2685" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:20</t>
+        </is>
+      </c>
+      <c r="C2685" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2685" s="2">
+        <v>28.8</v>
+      </c>
+      <c r="E2685" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F2685" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2685" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2686">
+      <c r="A2686" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2686" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:30</t>
+        </is>
+      </c>
+      <c r="C2686" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2686" s="2">
+        <v>29.7</v>
+      </c>
+      <c r="E2686" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F2686" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2686" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2687">
+      <c r="A2687" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2687" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:40</t>
+        </is>
+      </c>
+      <c r="C2687" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2687" s="2">
+        <v>30.2</v>
+      </c>
+      <c r="E2687" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F2687" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2687" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2688">
+      <c r="A2688" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2688" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:50</t>
+        </is>
+      </c>
+      <c r="C2688" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2688" s="2">
+        <v>30.4</v>
+      </c>
+      <c r="E2688" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F2688" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2688" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2689">
+      <c r="A2689" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2689" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:00</t>
+        </is>
+      </c>
+      <c r="C2689" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2689" s="2">
+        <v>30.7</v>
+      </c>
+      <c r="E2689" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F2689" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2689" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2690">
+      <c r="A2690" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2690" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:10</t>
+        </is>
+      </c>
+      <c r="C2690" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2690" s="2">
+        <v>31.2</v>
+      </c>
+      <c r="E2690" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F2690" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2690" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2691">
+      <c r="A2691" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2691" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:20</t>
+        </is>
+      </c>
+      <c r="C2691" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2691" s="2">
+        <v>31.5</v>
+      </c>
+      <c r="E2691" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F2691" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2691" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2692">
+      <c r="A2692" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2692" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:30</t>
+        </is>
+      </c>
+      <c r="C2692" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2692" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="E2692" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="F2692" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2692" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2693">
+      <c r="A2693" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2693" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:40</t>
+        </is>
+      </c>
+      <c r="C2693" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2693" s="2">
+        <v>32.1</v>
+      </c>
+      <c r="E2693" s="2">
+        <v>37.0</v>
+      </c>
+      <c r="F2693" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2693" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2694">
+      <c r="A2694" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2694" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:50</t>
+        </is>
+      </c>
+      <c r="C2694" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2694" s="2">
+        <v>32.3</v>
+      </c>
+      <c r="E2694" s="2">
+        <v>37.0</v>
+      </c>
+      <c r="F2694" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2694" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2695">
+      <c r="A2695" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2695" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:00</t>
+        </is>
+      </c>
+      <c r="C2695" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2695" s="2">
+        <v>32.8</v>
+      </c>
+      <c r="E2695" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="F2695" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2695" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2696">
+      <c r="A2696" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2696" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:10</t>
+        </is>
+      </c>
+      <c r="C2696" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2696" s="2">
+        <v>32.9</v>
+      </c>
+      <c r="E2696" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F2696" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2696" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2697">
+      <c r="A2697" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2697" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:20</t>
+        </is>
+      </c>
+      <c r="C2697" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2697" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="E2697" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F2697" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2697" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2698">
+      <c r="A2698" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2698" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:30</t>
+        </is>
+      </c>
+      <c r="C2698" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2698" s="2">
+        <v>33.2</v>
+      </c>
+      <c r="E2698" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F2698" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2698" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2699">
+      <c r="A2699" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2699" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:40</t>
+        </is>
+      </c>
+      <c r="C2699" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2699" s="2">
+        <v>33.5</v>
+      </c>
+      <c r="E2699" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="F2699" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2699" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2700">
+      <c r="A2700" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2700" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:50</t>
+        </is>
+      </c>
+      <c r="C2700" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2700" s="2">
+        <v>33.5</v>
+      </c>
+      <c r="E2700" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F2700" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2700" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2701">
+      <c r="A2701" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2701" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:00</t>
+        </is>
+      </c>
+      <c r="C2701" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2701" s="2">
+        <v>33.8</v>
+      </c>
+      <c r="E2701" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="F2701" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2701" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2702">
+      <c r="A2702" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2702" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:10</t>
+        </is>
+      </c>
+      <c r="C2702" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2702" s="2">
+        <v>34.2</v>
+      </c>
+      <c r="E2702" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2702" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2702" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2703">
+      <c r="A2703" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2703" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:20</t>
+        </is>
+      </c>
+      <c r="C2703" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2703" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="E2703" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F2703" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2703" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2704">
+      <c r="A2704" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2704" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:30</t>
+        </is>
+      </c>
+      <c r="C2704" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2704" s="2">
+        <v>34.3</v>
+      </c>
+      <c r="E2704" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F2704" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2704" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2705">
+      <c r="A2705" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2705" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:40</t>
+        </is>
+      </c>
+      <c r="C2705" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2705" s="2">
+        <v>34.3</v>
+      </c>
+      <c r="E2705" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2705" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2705" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2706">
+      <c r="A2706" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2706" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:50</t>
+        </is>
+      </c>
+      <c r="C2706" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2706" s="2">
+        <v>34.8</v>
+      </c>
+      <c r="E2706" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2706" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2706" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2707">
+      <c r="A2707" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2707" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:00</t>
+        </is>
+      </c>
+      <c r="C2707" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2707" s="2">
+        <v>34.8</v>
+      </c>
+      <c r="E2707" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2707" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2707" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2708">
+      <c r="A2708" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2708" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:10</t>
+        </is>
+      </c>
+      <c r="C2708" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2708" s="2">
+        <v>35.3</v>
+      </c>
+      <c r="E2708" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2708" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2708" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2709">
+      <c r="A2709" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2709" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:20</t>
+        </is>
+      </c>
+      <c r="C2709" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2709" s="2">
+        <v>35.3</v>
+      </c>
+      <c r="E2709" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2709" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2709" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2710">
+      <c r="A2710" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2710" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:30</t>
+        </is>
+      </c>
+      <c r="C2710" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2710" s="2">
+        <v>35.4</v>
+      </c>
+      <c r="E2710" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2710" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2710" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2711">
+      <c r="A2711" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2711" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:40</t>
+        </is>
+      </c>
+      <c r="C2711" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2711" s="2">
+        <v>35.1</v>
+      </c>
+      <c r="E2711" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2711" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2711" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2712">
+      <c r="A2712" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2712" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:50</t>
+        </is>
+      </c>
+      <c r="C2712" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2712" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="E2712" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2712" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2712" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2713">
+      <c r="A2713" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2713" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:00</t>
+        </is>
+      </c>
+      <c r="C2713" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2713" s="2">
+        <v>35.4</v>
+      </c>
+      <c r="E2713" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2713" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2713" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2714">
+      <c r="A2714" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2714" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:10</t>
+        </is>
+      </c>
+      <c r="C2714" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2714" s="2">
+        <v>34.8</v>
+      </c>
+      <c r="E2714" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2714" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2714" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2715">
+      <c r="A2715" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2715" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:20</t>
+        </is>
+      </c>
+      <c r="C2715" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2715" s="2">
+        <v>35.2</v>
+      </c>
+      <c r="E2715" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2715" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2715" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2716">
+      <c r="A2716" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2716" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:30</t>
+        </is>
+      </c>
+      <c r="C2716" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2716" s="2">
+        <v>35.1</v>
+      </c>
+      <c r="E2716" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2716" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2716" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2717">
+      <c r="A2717" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2717" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:40</t>
+        </is>
+      </c>
+      <c r="C2717" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2717" s="2">
+        <v>35.1</v>
+      </c>
+      <c r="E2717" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2717" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2717" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2718">
+      <c r="A2718" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2718" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:50</t>
+        </is>
+      </c>
+      <c r="C2718" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2718" s="2">
+        <v>34.8</v>
+      </c>
+      <c r="E2718" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2718" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2718" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2719">
+      <c r="A2719" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2719" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:00</t>
+        </is>
+      </c>
+      <c r="C2719" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2719" s="2">
+        <v>34.5</v>
+      </c>
+      <c r="E2719" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2719" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2719" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2720">
+      <c r="A2720" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2720" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:10</t>
+        </is>
+      </c>
+      <c r="C2720" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2720" s="2">
+        <v>34.5</v>
+      </c>
+      <c r="E2720" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2720" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2720" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2721">
+      <c r="A2721" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2721" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:20</t>
+        </is>
+      </c>
+      <c r="C2721" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2721" s="2">
+        <v>34.8</v>
+      </c>
+      <c r="E2721" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2721" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2721" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2722">
+      <c r="A2722" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2722" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:30</t>
+        </is>
+      </c>
+      <c r="C2722" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2722" s="2">
+        <v>34.9</v>
+      </c>
+      <c r="E2722" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="F2722" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2722" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2723">
+      <c r="A2723" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2723" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:40</t>
+        </is>
+      </c>
+      <c r="C2723" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2723" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="E2723" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="F2723" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2723" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2724">
+      <c r="A2724" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2724" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:50</t>
+        </is>
+      </c>
+      <c r="C2724" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2724" s="2">
+        <v>34.9</v>
+      </c>
+      <c r="E2724" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="F2724" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2724" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2725">
+      <c r="A2725" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2725" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:00</t>
+        </is>
+      </c>
+      <c r="C2725" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2725" s="2">
+        <v>35.2</v>
+      </c>
+      <c r="E2725" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="F2725" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2725" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2726">
+      <c r="A2726" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2726" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:10</t>
+        </is>
+      </c>
+      <c r="C2726" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2726" s="2">
+        <v>35.2</v>
+      </c>
+      <c r="E2726" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="F2726" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2726" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2727">
+      <c r="A2727" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2727" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:20</t>
+        </is>
+      </c>
+      <c r="C2727" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2727" s="2">
+        <v>34.8</v>
+      </c>
+      <c r="E2727" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="F2727" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2727" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2728">
+      <c r="A2728" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2728" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:30</t>
+        </is>
+      </c>
+      <c r="C2728" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2728" s="2">
+        <v>34.9</v>
+      </c>
+      <c r="E2728" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="F2728" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2728" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2729">
+      <c r="A2729" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2729" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:40</t>
+        </is>
+      </c>
+      <c r="C2729" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2729" s="2">
+        <v>35.1</v>
+      </c>
+      <c r="E2729" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="F2729" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2729" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2730">
+      <c r="A2730" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2730" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:50</t>
+        </is>
+      </c>
+      <c r="C2730" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2730" s="2">
+        <v>35.3</v>
+      </c>
+      <c r="E2730" s="2">
+        <v>17.0</v>
+      </c>
+      <c r="F2730" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2730" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2731">
+      <c r="A2731" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2731" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:00</t>
+        </is>
+      </c>
+      <c r="C2731" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2731" s="2">
+        <v>35.3</v>
+      </c>
+      <c r="E2731" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="F2731" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2731" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2732">
+      <c r="A2732" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2732" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:10</t>
+        </is>
+      </c>
+      <c r="C2732" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2732" s="2">
+        <v>35.1</v>
+      </c>
+      <c r="E2732" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="F2732" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2732" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2733">
+      <c r="A2733" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2733" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:20</t>
+        </is>
+      </c>
+      <c r="C2733" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2733" s="2">
+        <v>35.1</v>
+      </c>
+      <c r="E2733" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="F2733" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2733" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2734">
+      <c r="A2734" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2734" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:30</t>
+        </is>
+      </c>
+      <c r="C2734" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2734" s="2">
+        <v>34.7</v>
+      </c>
+      <c r="E2734" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="F2734" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2734" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2735">
+      <c r="A2735" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2735" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:40</t>
+        </is>
+      </c>
+      <c r="C2735" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2735" s="2">
+        <v>34.6</v>
+      </c>
+      <c r="E2735" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="F2735" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2735" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2736">
+      <c r="A2736" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2736" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:50</t>
+        </is>
+      </c>
+      <c r="C2736" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2736" s="2">
+        <v>34.3</v>
+      </c>
+      <c r="E2736" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="F2736" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2736" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2737">
+      <c r="A2737" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2737" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:00</t>
+        </is>
+      </c>
+      <c r="C2737" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2737" s="2">
+        <v>33.9</v>
+      </c>
+      <c r="E2737" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2737" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2737" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2738">
+      <c r="A2738" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2738" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:10</t>
+        </is>
+      </c>
+      <c r="C2738" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2738" s="2">
+        <v>33.5</v>
+      </c>
+      <c r="E2738" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2738" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2738" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2739">
+      <c r="A2739" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2739" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:20</t>
+        </is>
+      </c>
+      <c r="C2739" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2739" s="2">
+        <v>33.2</v>
+      </c>
+      <c r="E2739" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2739" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2739" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2740">
+      <c r="A2740" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2740" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:30</t>
+        </is>
+      </c>
+      <c r="C2740" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2740" s="2">
+        <v>32.9</v>
+      </c>
+      <c r="E2740" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2740" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2740" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2741">
+      <c r="A2741" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2741" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:40</t>
+        </is>
+      </c>
+      <c r="C2741" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2741" s="2">
+        <v>32.6</v>
+      </c>
+      <c r="E2741" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2741" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2741" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2742">
+      <c r="A2742" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2742" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:50</t>
+        </is>
+      </c>
+      <c r="C2742" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2742" s="2">
+        <v>32.4</v>
+      </c>
+      <c r="E2742" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2742" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2742" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2743">
+      <c r="A2743" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2743" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:00</t>
+        </is>
+      </c>
+      <c r="C2743" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2743" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="E2743" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F2743" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2743" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2744">
+      <c r="A2744" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2744" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:10</t>
+        </is>
+      </c>
+      <c r="C2744" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2744" s="2">
+        <v>31.7</v>
+      </c>
+      <c r="E2744" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F2744" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2744" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2745">
+      <c r="A2745" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2745" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:20</t>
+        </is>
+      </c>
+      <c r="C2745" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2745" s="2">
+        <v>31.3</v>
+      </c>
+      <c r="E2745" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="F2745" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2745" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2746">
+      <c r="A2746" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2746" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:30</t>
+        </is>
+      </c>
+      <c r="C2746" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2746" s="2">
+        <v>30.9</v>
+      </c>
+      <c r="E2746" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F2746" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2746" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2747">
+      <c r="A2747" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2747" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:40</t>
+        </is>
+      </c>
+      <c r="C2747" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2747" s="2">
+        <v>30.4</v>
+      </c>
+      <c r="E2747" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F2747" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2747" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2748">
+      <c r="A2748" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2748" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:50</t>
+        </is>
+      </c>
+      <c r="C2748" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2748" s="2">
+        <v>29.8</v>
+      </c>
+      <c r="E2748" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F2748" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2748" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2749">
+      <c r="A2749" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2749" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:00</t>
+        </is>
+      </c>
+      <c r="C2749" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2749" s="2">
+        <v>29.2</v>
+      </c>
+      <c r="E2749" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="F2749" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2749" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2750">
+      <c r="A2750" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2750" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:10</t>
+        </is>
+      </c>
+      <c r="C2750" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2750" s="2">
+        <v>28.6</v>
+      </c>
+      <c r="E2750" s="2">
+        <v>38.0</v>
+      </c>
+      <c r="F2750" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2750" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2751">
+      <c r="A2751" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2751" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:20</t>
+        </is>
+      </c>
+      <c r="C2751" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2751" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="E2751" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F2751" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2751" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2752">
+      <c r="A2752" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2752" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:30</t>
+        </is>
+      </c>
+      <c r="C2752" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2752" s="2">
+        <v>27.3</v>
+      </c>
+      <c r="E2752" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F2752" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2752" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2753">
+      <c r="A2753" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2753" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:40</t>
+        </is>
+      </c>
+      <c r="C2753" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2753" s="2">
+        <v>26.7</v>
+      </c>
+      <c r="E2753" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F2753" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2753" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2754">
+      <c r="A2754" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2754" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:50</t>
+        </is>
+      </c>
+      <c r="C2754" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2754" s="2">
+        <v>26.2</v>
+      </c>
+      <c r="E2754" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F2754" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2754" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2755">
+      <c r="A2755" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2755" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:00</t>
+        </is>
+      </c>
+      <c r="C2755" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2755" s="2">
+        <v>25.6</v>
+      </c>
+      <c r="E2755" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F2755" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2755" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2756">
+      <c r="A2756" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2756" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:10</t>
+        </is>
+      </c>
+      <c r="C2756" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2756" s="2">
+        <v>25.2</v>
+      </c>
+      <c r="E2756" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F2756" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2756" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2757">
+      <c r="A2757" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2757" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:20</t>
+        </is>
+      </c>
+      <c r="C2757" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2757" s="2">
+        <v>24.9</v>
+      </c>
+      <c r="E2757" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F2757" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2757" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2758">
+      <c r="A2758" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2758" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:30</t>
+        </is>
+      </c>
+      <c r="C2758" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2758" s="2">
+        <v>24.8</v>
+      </c>
+      <c r="E2758" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F2758" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2758" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2759">
+      <c r="A2759" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2759" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:40</t>
+        </is>
+      </c>
+      <c r="C2759" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2759" s="2">
+        <v>24.5</v>
+      </c>
+      <c r="E2759" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F2759" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2759" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2760">
+      <c r="A2760" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2760" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:50</t>
+        </is>
+      </c>
+      <c r="C2760" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2760" s="2">
+        <v>24.3</v>
+      </c>
+      <c r="E2760" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F2760" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2760" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2761">
+      <c r="A2761" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2761" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:00</t>
+        </is>
+      </c>
+      <c r="C2761" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2761" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="E2761" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F2761" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2761" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2762">
+      <c r="A2762" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2762" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:10</t>
+        </is>
+      </c>
+      <c r="C2762" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2762" s="2">
+        <v>23.9</v>
+      </c>
+      <c r="E2762" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F2762" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2762" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2763">
+      <c r="A2763" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2763" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:20</t>
+        </is>
+      </c>
+      <c r="C2763" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2763" s="2">
+        <v>23.6</v>
+      </c>
+      <c r="E2763" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2763" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2763" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2764">
+      <c r="A2764" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2764" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:30</t>
+        </is>
+      </c>
+      <c r="C2764" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2764" s="2">
+        <v>23.4</v>
+      </c>
+      <c r="E2764" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2764" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2764" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2765">
+      <c r="A2765" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2765" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:40</t>
+        </is>
+      </c>
+      <c r="C2765" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2765" s="2">
+        <v>23.2</v>
+      </c>
+      <c r="E2765" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F2765" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2765" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2766">
+      <c r="A2766" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02.08.2026</t>
+        </is>
+      </c>
+      <c r="B2766" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:50</t>
+        </is>
+      </c>
+      <c r="C2766" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2766" s="2">
+        <v>23.2</v>
+      </c>
+      <c r="E2766" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2766" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2766" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2767">
+      <c r="A2767" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2767" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:00</t>
+        </is>
+      </c>
+      <c r="C2767" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2767" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="E2767" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2767" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2767" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2768">
+      <c r="A2768" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2768" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:10</t>
+        </is>
+      </c>
+      <c r="C2768" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2768" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="E2768" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2768" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2768" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2769">
+      <c r="A2769" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2769" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:20</t>
+        </is>
+      </c>
+      <c r="C2769" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2769" s="2">
+        <v>22.9</v>
+      </c>
+      <c r="E2769" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F2769" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2769" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2770">
+      <c r="A2770" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2770" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:30</t>
+        </is>
+      </c>
+      <c r="C2770" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2770" s="2">
+        <v>22.8</v>
+      </c>
+      <c r="E2770" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2770" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2770" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G2625"/>
+  <autoFilter ref="A1:G2770"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ARSO Kranj zajem 2026-08-04 00:43 Europe/Ljubljana
</commit_message>
<xml_diff>
--- a/tabela_vremena/ARSO_Kranj.xlsx
+++ b/tabela_vremena/ARSO_Kranj.xlsx
@@ -80412,7 +80412,4183 @@
         <v>0.0</v>
       </c>
     </row>
+    <row r="2771">
+      <c r="A2771" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2771" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:40</t>
+        </is>
+      </c>
+      <c r="C2771" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2771" s="2">
+        <v>22.7</v>
+      </c>
+      <c r="E2771" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F2771" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2771" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2772">
+      <c r="A2772" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2772" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:50</t>
+        </is>
+      </c>
+      <c r="C2772" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2772" s="2">
+        <v>22.5</v>
+      </c>
+      <c r="E2772" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F2772" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2772" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2773">
+      <c r="A2773" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2773" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:00</t>
+        </is>
+      </c>
+      <c r="C2773" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2773" s="2">
+        <v>22.5</v>
+      </c>
+      <c r="E2773" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F2773" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2773" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2774">
+      <c r="A2774" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2774" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:10</t>
+        </is>
+      </c>
+      <c r="C2774" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2774" s="2">
+        <v>22.5</v>
+      </c>
+      <c r="E2774" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F2774" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2774" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2775">
+      <c r="A2775" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2775" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:20</t>
+        </is>
+      </c>
+      <c r="C2775" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2775" s="2">
+        <v>22.3</v>
+      </c>
+      <c r="E2775" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2775" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2775" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2776">
+      <c r="A2776" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2776" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:30</t>
+        </is>
+      </c>
+      <c r="C2776" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2776" s="2">
+        <v>22.3</v>
+      </c>
+      <c r="E2776" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F2776" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2776" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2777">
+      <c r="A2777" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2777" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:40</t>
+        </is>
+      </c>
+      <c r="C2777" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2777" s="2">
+        <v>22.2</v>
+      </c>
+      <c r="E2777" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F2777" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2777" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2778">
+      <c r="A2778" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2778" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:50</t>
+        </is>
+      </c>
+      <c r="C2778" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2778" s="2">
+        <v>22.1</v>
+      </c>
+      <c r="E2778" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2778" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2778" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2779">
+      <c r="A2779" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2779" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:00</t>
+        </is>
+      </c>
+      <c r="C2779" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2779" s="2">
+        <v>22.1</v>
+      </c>
+      <c r="E2779" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2779" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2779" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2780">
+      <c r="A2780" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2780" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:10</t>
+        </is>
+      </c>
+      <c r="C2780" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2780" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="E2780" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2780" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2780" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2781">
+      <c r="A2781" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2781" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:20</t>
+        </is>
+      </c>
+      <c r="C2781" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2781" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="E2781" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2781" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2781" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2782">
+      <c r="A2782" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2782" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:30</t>
+        </is>
+      </c>
+      <c r="C2782" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2782" s="2">
+        <v>22.3</v>
+      </c>
+      <c r="E2782" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F2782" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2782" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2783">
+      <c r="A2783" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2783" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:40</t>
+        </is>
+      </c>
+      <c r="C2783" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2783" s="2">
+        <v>22.5</v>
+      </c>
+      <c r="E2783" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F2783" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2783" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2784">
+      <c r="A2784" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2784" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:50</t>
+        </is>
+      </c>
+      <c r="C2784" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2784" s="2">
+        <v>22.5</v>
+      </c>
+      <c r="E2784" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F2784" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2784" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2785">
+      <c r="A2785" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2785" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:00</t>
+        </is>
+      </c>
+      <c r="C2785" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2785" s="2">
+        <v>22.5</v>
+      </c>
+      <c r="E2785" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F2785" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2785" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2786">
+      <c r="A2786" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2786" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:10</t>
+        </is>
+      </c>
+      <c r="C2786" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2786" s="2">
+        <v>22.3</v>
+      </c>
+      <c r="E2786" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F2786" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2786" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2787">
+      <c r="A2787" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2787" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:20</t>
+        </is>
+      </c>
+      <c r="C2787" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2787" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="E2787" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2787" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2787" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2788">
+      <c r="A2788" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2788" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:30</t>
+        </is>
+      </c>
+      <c r="C2788" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2788" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="E2788" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2788" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2788" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2789">
+      <c r="A2789" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2789" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:40</t>
+        </is>
+      </c>
+      <c r="C2789" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2789" s="2">
+        <v>21.8</v>
+      </c>
+      <c r="E2789" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F2789" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2789" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2790">
+      <c r="A2790" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2790" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:50</t>
+        </is>
+      </c>
+      <c r="C2790" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2790" s="2">
+        <v>21.8</v>
+      </c>
+      <c r="E2790" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F2790" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2790" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2791">
+      <c r="A2791" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2791" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:00</t>
+        </is>
+      </c>
+      <c r="C2791" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2791" s="2">
+        <v>21.8</v>
+      </c>
+      <c r="E2791" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F2791" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2791" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2792">
+      <c r="A2792" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2792" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:10</t>
+        </is>
+      </c>
+      <c r="C2792" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2792" s="2">
+        <v>21.7</v>
+      </c>
+      <c r="E2792" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F2792" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2792" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2793">
+      <c r="A2793" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2793" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:20</t>
+        </is>
+      </c>
+      <c r="C2793" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2793" s="2">
+        <v>21.3</v>
+      </c>
+      <c r="E2793" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F2793" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2793" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2794">
+      <c r="A2794" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2794" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:30</t>
+        </is>
+      </c>
+      <c r="C2794" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2794" s="2">
+        <v>21.1</v>
+      </c>
+      <c r="E2794" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F2794" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2794" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2795">
+      <c r="A2795" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2795" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:40</t>
+        </is>
+      </c>
+      <c r="C2795" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2795" s="2">
+        <v>21.3</v>
+      </c>
+      <c r="E2795" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F2795" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2795" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2796">
+      <c r="A2796" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2796" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:50</t>
+        </is>
+      </c>
+      <c r="C2796" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2796" s="2">
+        <v>21.3</v>
+      </c>
+      <c r="E2796" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F2796" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2796" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2797">
+      <c r="A2797" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2797" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:00</t>
+        </is>
+      </c>
+      <c r="C2797" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2797" s="2">
+        <v>21.3</v>
+      </c>
+      <c r="E2797" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F2797" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2797" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2798">
+      <c r="A2798" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2798" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:10</t>
+        </is>
+      </c>
+      <c r="C2798" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2798" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="E2798" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F2798" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2798" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2799">
+      <c r="A2799" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2799" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:20</t>
+        </is>
+      </c>
+      <c r="C2799" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2799" s="2">
+        <v>20.8</v>
+      </c>
+      <c r="E2799" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F2799" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2799" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2800">
+      <c r="A2800" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2800" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:30</t>
+        </is>
+      </c>
+      <c r="C2800" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2800" s="2">
+        <v>20.6</v>
+      </c>
+      <c r="E2800" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2800" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2800" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2801">
+      <c r="A2801" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2801" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:40</t>
+        </is>
+      </c>
+      <c r="C2801" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2801" s="2">
+        <v>20.5</v>
+      </c>
+      <c r="E2801" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2801" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2801" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2802">
+      <c r="A2802" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2802" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:50</t>
+        </is>
+      </c>
+      <c r="C2802" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2802" s="2">
+        <v>20.4</v>
+      </c>
+      <c r="E2802" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2802" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2802" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2803">
+      <c r="A2803" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2803" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:00</t>
+        </is>
+      </c>
+      <c r="C2803" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2803" s="2">
+        <v>20.5</v>
+      </c>
+      <c r="E2803" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2803" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2803" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2804">
+      <c r="A2804" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2804" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:10</t>
+        </is>
+      </c>
+      <c r="C2804" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2804" s="2">
+        <v>20.6</v>
+      </c>
+      <c r="E2804" s="2">
+        <v>63.0</v>
+      </c>
+      <c r="F2804" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2804" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2805">
+      <c r="A2805" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2805" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:20</t>
+        </is>
+      </c>
+      <c r="C2805" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2805" s="2">
+        <v>20.5</v>
+      </c>
+      <c r="E2805" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2805" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2805" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2806">
+      <c r="A2806" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2806" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:30</t>
+        </is>
+      </c>
+      <c r="C2806" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2806" s="2">
+        <v>20.4</v>
+      </c>
+      <c r="E2806" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2806" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2806" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2807">
+      <c r="A2807" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2807" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:40</t>
+        </is>
+      </c>
+      <c r="C2807" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2807" s="2">
+        <v>20.4</v>
+      </c>
+      <c r="E2807" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2807" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2807" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2808">
+      <c r="A2808" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2808" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:50</t>
+        </is>
+      </c>
+      <c r="C2808" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2808" s="2">
+        <v>20.6</v>
+      </c>
+      <c r="E2808" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2808" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2808" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2809">
+      <c r="A2809" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2809" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:00</t>
+        </is>
+      </c>
+      <c r="C2809" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2809" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="E2809" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F2809" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2809" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2810">
+      <c r="A2810" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2810" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:10</t>
+        </is>
+      </c>
+      <c r="C2810" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2810" s="2">
+        <v>21.5</v>
+      </c>
+      <c r="E2810" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F2810" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2810" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2811">
+      <c r="A2811" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2811" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:20</t>
+        </is>
+      </c>
+      <c r="C2811" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2811" s="2">
+        <v>22.2</v>
+      </c>
+      <c r="E2811" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2811" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2811" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2812">
+      <c r="A2812" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2812" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:30</t>
+        </is>
+      </c>
+      <c r="C2812" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2812" s="2">
+        <v>22.6</v>
+      </c>
+      <c r="E2812" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F2812" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2812" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2813">
+      <c r="A2813" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2813" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:40</t>
+        </is>
+      </c>
+      <c r="C2813" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2813" s="2">
+        <v>22.8</v>
+      </c>
+      <c r="E2813" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F2813" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2813" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2814">
+      <c r="A2814" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2814" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:50</t>
+        </is>
+      </c>
+      <c r="C2814" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2814" s="2">
+        <v>23.3</v>
+      </c>
+      <c r="E2814" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F2814" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2814" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2815">
+      <c r="A2815" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2815" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:00</t>
+        </is>
+      </c>
+      <c r="C2815" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2815" s="2">
+        <v>23.8</v>
+      </c>
+      <c r="E2815" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F2815" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2815" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2816">
+      <c r="A2816" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2816" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:10</t>
+        </is>
+      </c>
+      <c r="C2816" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2816" s="2">
+        <v>24.2</v>
+      </c>
+      <c r="E2816" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F2816" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2816" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2817">
+      <c r="A2817" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2817" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:20</t>
+        </is>
+      </c>
+      <c r="C2817" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2817" s="2">
+        <v>24.5</v>
+      </c>
+      <c r="E2817" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F2817" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2817" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2818">
+      <c r="A2818" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2818" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:30</t>
+        </is>
+      </c>
+      <c r="C2818" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2818" s="2">
+        <v>25.2</v>
+      </c>
+      <c r="E2818" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F2818" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2818" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2819">
+      <c r="A2819" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2819" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:40</t>
+        </is>
+      </c>
+      <c r="C2819" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2819" s="2">
+        <v>25.8</v>
+      </c>
+      <c r="E2819" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F2819" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2819" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2820">
+      <c r="A2820" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2820" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:50</t>
+        </is>
+      </c>
+      <c r="C2820" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2820" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="E2820" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F2820" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2820" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2821">
+      <c r="A2821" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2821" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:00</t>
+        </is>
+      </c>
+      <c r="C2821" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2821" s="2">
+        <v>26.1</v>
+      </c>
+      <c r="E2821" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F2821" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2821" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2822">
+      <c r="A2822" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2822" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:10</t>
+        </is>
+      </c>
+      <c r="C2822" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2822" s="2">
+        <v>26.7</v>
+      </c>
+      <c r="E2822" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F2822" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2822" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2823">
+      <c r="A2823" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2823" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:20</t>
+        </is>
+      </c>
+      <c r="C2823" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2823" s="2">
+        <v>26.9</v>
+      </c>
+      <c r="E2823" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F2823" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2823" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2824">
+      <c r="A2824" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2824" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:30</t>
+        </is>
+      </c>
+      <c r="C2824" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2824" s="2">
+        <v>27.4</v>
+      </c>
+      <c r="E2824" s="2">
+        <v>44.0</v>
+      </c>
+      <c r="F2824" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2824" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2825">
+      <c r="A2825" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2825" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:40</t>
+        </is>
+      </c>
+      <c r="C2825" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2825" s="2">
+        <v>27.9</v>
+      </c>
+      <c r="E2825" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F2825" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2825" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2826">
+      <c r="A2826" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2826" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:50</t>
+        </is>
+      </c>
+      <c r="C2826" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2826" s="2">
+        <v>28.5</v>
+      </c>
+      <c r="E2826" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F2826" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2826" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2827">
+      <c r="A2827" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2827" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:00</t>
+        </is>
+      </c>
+      <c r="C2827" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2827" s="2">
+        <v>28.9</v>
+      </c>
+      <c r="E2827" s="2">
+        <v>41.0</v>
+      </c>
+      <c r="F2827" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2827" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2828">
+      <c r="A2828" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2828" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:10</t>
+        </is>
+      </c>
+      <c r="C2828" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2828" s="2">
+        <v>29.7</v>
+      </c>
+      <c r="E2828" s="2">
+        <v>38.0</v>
+      </c>
+      <c r="F2828" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2828" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2829">
+      <c r="A2829" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2829" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:20</t>
+        </is>
+      </c>
+      <c r="C2829" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2829" s="2">
+        <v>30.5</v>
+      </c>
+      <c r="E2829" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F2829" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2829" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2830">
+      <c r="A2830" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2830" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:30</t>
+        </is>
+      </c>
+      <c r="C2830" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2830" s="2">
+        <v>30.9</v>
+      </c>
+      <c r="E2830" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F2830" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2830" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2831">
+      <c r="A2831" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2831" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:40</t>
+        </is>
+      </c>
+      <c r="C2831" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2831" s="2">
+        <v>31.3</v>
+      </c>
+      <c r="E2831" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F2831" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2831" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2832">
+      <c r="A2832" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2832" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:50</t>
+        </is>
+      </c>
+      <c r="C2832" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2832" s="2">
+        <v>31.8</v>
+      </c>
+      <c r="E2832" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="F2832" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2832" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2833">
+      <c r="A2833" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2833" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:00</t>
+        </is>
+      </c>
+      <c r="C2833" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2833" s="2">
+        <v>32.5</v>
+      </c>
+      <c r="E2833" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F2833" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2833" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2834">
+      <c r="A2834" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2834" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:10</t>
+        </is>
+      </c>
+      <c r="C2834" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2834" s="2">
+        <v>32.9</v>
+      </c>
+      <c r="E2834" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F2834" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2834" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2835">
+      <c r="A2835" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2835" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:20</t>
+        </is>
+      </c>
+      <c r="C2835" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2835" s="2">
+        <v>32.9</v>
+      </c>
+      <c r="E2835" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2835" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2835" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2836">
+      <c r="A2836" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2836" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:30</t>
+        </is>
+      </c>
+      <c r="C2836" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2836" s="2">
+        <v>33.3</v>
+      </c>
+      <c r="E2836" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2836" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2836" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2837">
+      <c r="A2837" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2837" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:40</t>
+        </is>
+      </c>
+      <c r="C2837" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2837" s="2">
+        <v>34.1</v>
+      </c>
+      <c r="E2837" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2837" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2837" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2838">
+      <c r="A2838" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2838" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:50</t>
+        </is>
+      </c>
+      <c r="C2838" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2838" s="2">
+        <v>34.6</v>
+      </c>
+      <c r="E2838" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="F2838" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2838" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2839">
+      <c r="A2839" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2839" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:00</t>
+        </is>
+      </c>
+      <c r="C2839" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2839" s="2">
+        <v>34.2</v>
+      </c>
+      <c r="E2839" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2839" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2839" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2840">
+      <c r="A2840" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2840" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:10</t>
+        </is>
+      </c>
+      <c r="C2840" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2840" s="2">
+        <v>34.4</v>
+      </c>
+      <c r="E2840" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="F2840" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2840" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2841">
+      <c r="A2841" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2841" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:20</t>
+        </is>
+      </c>
+      <c r="C2841" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2841" s="2">
+        <v>34.5</v>
+      </c>
+      <c r="E2841" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2841" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2841" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2842">
+      <c r="A2842" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2842" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:30</t>
+        </is>
+      </c>
+      <c r="C2842" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2842" s="2">
+        <v>35.2</v>
+      </c>
+      <c r="E2842" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="F2842" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2842" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2843">
+      <c r="A2843" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2843" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:40</t>
+        </is>
+      </c>
+      <c r="C2843" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2843" s="2">
+        <v>34.6</v>
+      </c>
+      <c r="E2843" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="F2843" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2843" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2844">
+      <c r="A2844" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2844" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:50</t>
+        </is>
+      </c>
+      <c r="C2844" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2844" s="2">
+        <v>35.4</v>
+      </c>
+      <c r="E2844" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="F2844" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2844" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2845">
+      <c r="A2845" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2845" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:00</t>
+        </is>
+      </c>
+      <c r="C2845" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2845" s="2">
+        <v>35.3</v>
+      </c>
+      <c r="E2845" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="F2845" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2845" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2846">
+      <c r="A2846" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2846" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:10</t>
+        </is>
+      </c>
+      <c r="C2846" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2846" s="2">
+        <v>35.6</v>
+      </c>
+      <c r="E2846" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="F2846" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2846" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2847">
+      <c r="A2847" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2847" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:20</t>
+        </is>
+      </c>
+      <c r="C2847" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2847" s="2">
+        <v>35.8</v>
+      </c>
+      <c r="E2847" s="2">
+        <v>18.0</v>
+      </c>
+      <c r="F2847" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2847" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2848">
+      <c r="A2848" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2848" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:30</t>
+        </is>
+      </c>
+      <c r="C2848" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2848" s="2">
+        <v>35.6</v>
+      </c>
+      <c r="E2848" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="F2848" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2848" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2849">
+      <c r="A2849" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2849" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:40</t>
+        </is>
+      </c>
+      <c r="C2849" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2849" s="2">
+        <v>36.4</v>
+      </c>
+      <c r="E2849" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="F2849" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2849" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2850">
+      <c r="A2850" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2850" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:50</t>
+        </is>
+      </c>
+      <c r="C2850" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2850" s="2">
+        <v>36.2</v>
+      </c>
+      <c r="E2850" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="F2850" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2850" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2851">
+      <c r="A2851" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2851" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:00</t>
+        </is>
+      </c>
+      <c r="C2851" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2851" s="2">
+        <v>36.2</v>
+      </c>
+      <c r="E2851" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="F2851" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2851" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2852">
+      <c r="A2852" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2852" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:10</t>
+        </is>
+      </c>
+      <c r="C2852" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2852" s="2">
+        <v>36.5</v>
+      </c>
+      <c r="E2852" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="F2852" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2852" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2853">
+      <c r="A2853" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2853" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:20</t>
+        </is>
+      </c>
+      <c r="C2853" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2853" s="2">
+        <v>36.8</v>
+      </c>
+      <c r="E2853" s="2">
+        <v>18.0</v>
+      </c>
+      <c r="F2853" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2853" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2854">
+      <c r="A2854" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2854" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:30</t>
+        </is>
+      </c>
+      <c r="C2854" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2854" s="2">
+        <v>36.1</v>
+      </c>
+      <c r="E2854" s="2">
+        <v>17.0</v>
+      </c>
+      <c r="F2854" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2854" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2855">
+      <c r="A2855" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2855" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:40</t>
+        </is>
+      </c>
+      <c r="C2855" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2855" s="2">
+        <v>36.7</v>
+      </c>
+      <c r="E2855" s="2">
+        <v>16.0</v>
+      </c>
+      <c r="F2855" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2855" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2856">
+      <c r="A2856" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2856" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:50</t>
+        </is>
+      </c>
+      <c r="C2856" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2856" s="2">
+        <v>36.5</v>
+      </c>
+      <c r="E2856" s="2">
+        <v>18.0</v>
+      </c>
+      <c r="F2856" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2856" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2857">
+      <c r="A2857" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2857" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:00</t>
+        </is>
+      </c>
+      <c r="C2857" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2857" s="2">
+        <v>36.7</v>
+      </c>
+      <c r="E2857" s="2">
+        <v>17.0</v>
+      </c>
+      <c r="F2857" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2857" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2858">
+      <c r="A2858" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2858" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:10</t>
+        </is>
+      </c>
+      <c r="C2858" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2858" s="2">
+        <v>36.7</v>
+      </c>
+      <c r="E2858" s="2">
+        <v>17.0</v>
+      </c>
+      <c r="F2858" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2858" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2859">
+      <c r="A2859" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2859" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:20</t>
+        </is>
+      </c>
+      <c r="C2859" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2859" s="2">
+        <v>36.8</v>
+      </c>
+      <c r="E2859" s="2">
+        <v>18.0</v>
+      </c>
+      <c r="F2859" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2859" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2860">
+      <c r="A2860" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2860" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:30</t>
+        </is>
+      </c>
+      <c r="C2860" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2860" s="2">
+        <v>36.5</v>
+      </c>
+      <c r="E2860" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="F2860" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2860" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2861">
+      <c r="A2861" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2861" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:40</t>
+        </is>
+      </c>
+      <c r="C2861" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2861" s="2">
+        <v>36.6</v>
+      </c>
+      <c r="E2861" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="F2861" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2861" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2862">
+      <c r="A2862" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2862" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:50</t>
+        </is>
+      </c>
+      <c r="C2862" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2862" s="2">
+        <v>35.9</v>
+      </c>
+      <c r="E2862" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="F2862" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2862" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2863">
+      <c r="A2863" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2863" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:00</t>
+        </is>
+      </c>
+      <c r="C2863" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2863" s="2">
+        <v>36.1</v>
+      </c>
+      <c r="E2863" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="F2863" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2863" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2864">
+      <c r="A2864" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2864" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:10</t>
+        </is>
+      </c>
+      <c r="C2864" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2864" s="2">
+        <v>35.7</v>
+      </c>
+      <c r="E2864" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="F2864" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2864" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2865">
+      <c r="A2865" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2865" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:20</t>
+        </is>
+      </c>
+      <c r="C2865" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2865" s="2">
+        <v>35.4</v>
+      </c>
+      <c r="E2865" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="F2865" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2865" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2866">
+      <c r="A2866" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2866" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:30</t>
+        </is>
+      </c>
+      <c r="C2866" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2866" s="2">
+        <v>35.5</v>
+      </c>
+      <c r="E2866" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="F2866" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2866" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2867">
+      <c r="A2867" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2867" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:40</t>
+        </is>
+      </c>
+      <c r="C2867" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2867" s="2">
+        <v>35.7</v>
+      </c>
+      <c r="E2867" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="F2867" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2867" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2868">
+      <c r="A2868" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2868" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:50</t>
+        </is>
+      </c>
+      <c r="C2868" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2868" s="2">
+        <v>35.9</v>
+      </c>
+      <c r="E2868" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="F2868" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2868" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2869">
+      <c r="A2869" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2869" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:00</t>
+        </is>
+      </c>
+      <c r="C2869" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2869" s="2">
+        <v>36.2</v>
+      </c>
+      <c r="E2869" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="F2869" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2869" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2870">
+      <c r="A2870" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2870" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:10</t>
+        </is>
+      </c>
+      <c r="C2870" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2870" s="2">
+        <v>36.2</v>
+      </c>
+      <c r="E2870" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="F2870" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2870" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2871">
+      <c r="A2871" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2871" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:20</t>
+        </is>
+      </c>
+      <c r="C2871" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2871" s="2">
+        <v>36.5</v>
+      </c>
+      <c r="E2871" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="F2871" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2871" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2872">
+      <c r="A2872" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2872" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:30</t>
+        </is>
+      </c>
+      <c r="C2872" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2872" s="2">
+        <v>36.5</v>
+      </c>
+      <c r="E2872" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="F2872" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2872" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2873">
+      <c r="A2873" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2873" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:40</t>
+        </is>
+      </c>
+      <c r="C2873" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2873" s="2">
+        <v>36.7</v>
+      </c>
+      <c r="E2873" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="F2873" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2873" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2874">
+      <c r="A2874" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2874" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:50</t>
+        </is>
+      </c>
+      <c r="C2874" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2874" s="2">
+        <v>36.9</v>
+      </c>
+      <c r="E2874" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="F2874" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2874" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2875">
+      <c r="A2875" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2875" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:00</t>
+        </is>
+      </c>
+      <c r="C2875" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2875" s="2">
+        <v>36.9</v>
+      </c>
+      <c r="E2875" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="F2875" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2875" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2876">
+      <c r="A2876" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2876" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:10</t>
+        </is>
+      </c>
+      <c r="C2876" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2876" s="2">
+        <v>36.7</v>
+      </c>
+      <c r="E2876" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="F2876" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2876" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2877">
+      <c r="A2877" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2877" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:20</t>
+        </is>
+      </c>
+      <c r="C2877" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2877" s="2">
+        <v>36.5</v>
+      </c>
+      <c r="E2877" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="F2877" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2877" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2878">
+      <c r="A2878" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2878" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:30</t>
+        </is>
+      </c>
+      <c r="C2878" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2878" s="2">
+        <v>36.7</v>
+      </c>
+      <c r="E2878" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="F2878" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2878" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2879">
+      <c r="A2879" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2879" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:40</t>
+        </is>
+      </c>
+      <c r="C2879" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2879" s="2">
+        <v>36.7</v>
+      </c>
+      <c r="E2879" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="F2879" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2879" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2880">
+      <c r="A2880" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2880" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:50</t>
+        </is>
+      </c>
+      <c r="C2880" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2880" s="2">
+        <v>36.2</v>
+      </c>
+      <c r="E2880" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2880" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2880" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2881">
+      <c r="A2881" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2881" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:00</t>
+        </is>
+      </c>
+      <c r="C2881" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2881" s="2">
+        <v>35.8</v>
+      </c>
+      <c r="E2881" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2881" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2881" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2882">
+      <c r="A2882" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2882" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:10</t>
+        </is>
+      </c>
+      <c r="C2882" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2882" s="2">
+        <v>34.9</v>
+      </c>
+      <c r="E2882" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F2882" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2882" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2883">
+      <c r="A2883" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2883" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:20</t>
+        </is>
+      </c>
+      <c r="C2883" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2883" s="2">
+        <v>34.5</v>
+      </c>
+      <c r="E2883" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F2883" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2883" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2884">
+      <c r="A2884" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2884" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:30</t>
+        </is>
+      </c>
+      <c r="C2884" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2884" s="2">
+        <v>34.1</v>
+      </c>
+      <c r="E2884" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2884" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2884" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2885">
+      <c r="A2885" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2885" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:40</t>
+        </is>
+      </c>
+      <c r="C2885" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2885" s="2">
+        <v>33.8</v>
+      </c>
+      <c r="E2885" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F2885" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2885" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2886">
+      <c r="A2886" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2886" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:50</t>
+        </is>
+      </c>
+      <c r="C2886" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2886" s="2">
+        <v>33.5</v>
+      </c>
+      <c r="E2886" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2886" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2886" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2887">
+      <c r="A2887" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2887" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:00</t>
+        </is>
+      </c>
+      <c r="C2887" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2887" s="2">
+        <v>33.1</v>
+      </c>
+      <c r="E2887" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F2887" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2887" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2888">
+      <c r="A2888" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2888" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:10</t>
+        </is>
+      </c>
+      <c r="C2888" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2888" s="2">
+        <v>32.7</v>
+      </c>
+      <c r="E2888" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F2888" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2888" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2889">
+      <c r="A2889" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2889" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:20</t>
+        </is>
+      </c>
+      <c r="C2889" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2889" s="2">
+        <v>32.5</v>
+      </c>
+      <c r="E2889" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F2889" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2889" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2890">
+      <c r="A2890" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2890" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:30</t>
+        </is>
+      </c>
+      <c r="C2890" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2890" s="2">
+        <v>31.9</v>
+      </c>
+      <c r="E2890" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="F2890" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2890" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2891">
+      <c r="A2891" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2891" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:40</t>
+        </is>
+      </c>
+      <c r="C2891" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2891" s="2">
+        <v>31.2</v>
+      </c>
+      <c r="E2891" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F2891" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2891" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2892">
+      <c r="A2892" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2892" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:50</t>
+        </is>
+      </c>
+      <c r="C2892" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2892" s="2">
+        <v>30.7</v>
+      </c>
+      <c r="E2892" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F2892" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2892" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2893">
+      <c r="A2893" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2893" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:00</t>
+        </is>
+      </c>
+      <c r="C2893" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2893" s="2">
+        <v>30.4</v>
+      </c>
+      <c r="E2893" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F2893" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2893" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2894">
+      <c r="A2894" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2894" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:10</t>
+        </is>
+      </c>
+      <c r="C2894" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2894" s="2">
+        <v>29.5</v>
+      </c>
+      <c r="E2894" s="2">
+        <v>39.0</v>
+      </c>
+      <c r="F2894" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2894" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2895">
+      <c r="A2895" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2895" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:20</t>
+        </is>
+      </c>
+      <c r="C2895" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2895" s="2">
+        <v>28.8</v>
+      </c>
+      <c r="E2895" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F2895" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2895" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2896">
+      <c r="A2896" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2896" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:30</t>
+        </is>
+      </c>
+      <c r="C2896" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2896" s="2">
+        <v>28.4</v>
+      </c>
+      <c r="E2896" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F2896" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2896" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2897">
+      <c r="A2897" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2897" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:40</t>
+        </is>
+      </c>
+      <c r="C2897" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2897" s="2">
+        <v>27.7</v>
+      </c>
+      <c r="E2897" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F2897" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2897" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2898">
+      <c r="A2898" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2898" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:50</t>
+        </is>
+      </c>
+      <c r="C2898" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2898" s="2">
+        <v>27.1</v>
+      </c>
+      <c r="E2898" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F2898" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2898" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2899">
+      <c r="A2899" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2899" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:00</t>
+        </is>
+      </c>
+      <c r="C2899" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2899" s="2">
+        <v>26.9</v>
+      </c>
+      <c r="E2899" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F2899" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2899" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2900">
+      <c r="A2900" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2900" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:10</t>
+        </is>
+      </c>
+      <c r="C2900" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2900" s="2">
+        <v>26.4</v>
+      </c>
+      <c r="E2900" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F2900" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2900" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2901">
+      <c r="A2901" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2901" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:20</t>
+        </is>
+      </c>
+      <c r="C2901" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2901" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="E2901" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F2901" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2901" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2902">
+      <c r="A2902" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2902" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:30</t>
+        </is>
+      </c>
+      <c r="C2902" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2902" s="2">
+        <v>25.7</v>
+      </c>
+      <c r="E2902" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F2902" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2902" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2903">
+      <c r="A2903" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2903" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:40</t>
+        </is>
+      </c>
+      <c r="C2903" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2903" s="2">
+        <v>25.3</v>
+      </c>
+      <c r="E2903" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F2903" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2903" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2904">
+      <c r="A2904" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2904" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:50</t>
+        </is>
+      </c>
+      <c r="C2904" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2904" s="2">
+        <v>25.1</v>
+      </c>
+      <c r="E2904" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F2904" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2904" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2905">
+      <c r="A2905" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2905" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:00</t>
+        </is>
+      </c>
+      <c r="C2905" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2905" s="2">
+        <v>24.8</v>
+      </c>
+      <c r="E2905" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F2905" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2905" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2906">
+      <c r="A2906" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2906" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:10</t>
+        </is>
+      </c>
+      <c r="C2906" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2906" s="2">
+        <v>24.5</v>
+      </c>
+      <c r="E2906" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2906" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2906" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2907">
+      <c r="A2907" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2907" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:20</t>
+        </is>
+      </c>
+      <c r="C2907" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2907" s="2">
+        <v>24.1</v>
+      </c>
+      <c r="E2907" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F2907" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2907" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2908">
+      <c r="A2908" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2908" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:30</t>
+        </is>
+      </c>
+      <c r="C2908" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2908" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="E2908" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F2908" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2908" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2909">
+      <c r="A2909" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2909" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:40</t>
+        </is>
+      </c>
+      <c r="C2909" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2909" s="2">
+        <v>23.9</v>
+      </c>
+      <c r="E2909" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2909" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2909" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2910">
+      <c r="A2910" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03.08.2026</t>
+        </is>
+      </c>
+      <c r="B2910" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:50</t>
+        </is>
+      </c>
+      <c r="C2910" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2910" s="2">
+        <v>23.8</v>
+      </c>
+      <c r="E2910" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2910" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2910" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2911">
+      <c r="A2911" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2911" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:00</t>
+        </is>
+      </c>
+      <c r="C2911" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2911" s="2">
+        <v>23.7</v>
+      </c>
+      <c r="E2911" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2911" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2911" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2912">
+      <c r="A2912" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2912" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:10</t>
+        </is>
+      </c>
+      <c r="C2912" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2912" s="2">
+        <v>23.6</v>
+      </c>
+      <c r="E2912" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2912" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2912" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2913">
+      <c r="A2913" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2913" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:20</t>
+        </is>
+      </c>
+      <c r="C2913" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2913" s="2">
+        <v>23.3</v>
+      </c>
+      <c r="E2913" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F2913" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2913" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2914">
+      <c r="A2914" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2914" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:30</t>
+        </is>
+      </c>
+      <c r="C2914" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2914" s="2">
+        <v>22.9</v>
+      </c>
+      <c r="E2914" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F2914" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2914" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G2770"/>
+  <autoFilter ref="A1:G2914"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ARSO Kranj zajem 2026-08-05 00:47 Europe/Ljubljana
</commit_message>
<xml_diff>
--- a/tabela_vremena/ARSO_Kranj.xlsx
+++ b/tabela_vremena/ARSO_Kranj.xlsx
@@ -84588,7 +84588,4067 @@
         <v>0.0</v>
       </c>
     </row>
+    <row r="2915">
+      <c r="A2915" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2915" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:40</t>
+        </is>
+      </c>
+      <c r="C2915" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2915" s="2">
+        <v>22.9</v>
+      </c>
+      <c r="E2915" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F2915" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2915" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2916">
+      <c r="A2916" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2916" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:50</t>
+        </is>
+      </c>
+      <c r="C2916" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2916" s="2">
+        <v>22.8</v>
+      </c>
+      <c r="E2916" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F2916" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2916" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2917">
+      <c r="A2917" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2917" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:00</t>
+        </is>
+      </c>
+      <c r="C2917" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2917" s="2">
+        <v>22.7</v>
+      </c>
+      <c r="E2917" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F2917" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2917" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2918">
+      <c r="A2918" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2918" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:10</t>
+        </is>
+      </c>
+      <c r="C2918" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2918" s="2">
+        <v>22.7</v>
+      </c>
+      <c r="E2918" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2918" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2918" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2919">
+      <c r="A2919" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2919" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:20</t>
+        </is>
+      </c>
+      <c r="C2919" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2919" s="2">
+        <v>22.6</v>
+      </c>
+      <c r="E2919" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2919" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2919" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2920">
+      <c r="A2920" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2920" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:30</t>
+        </is>
+      </c>
+      <c r="C2920" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2920" s="2">
+        <v>22.5</v>
+      </c>
+      <c r="E2920" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F2920" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2920" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2921">
+      <c r="A2921" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2921" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:40</t>
+        </is>
+      </c>
+      <c r="C2921" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2921" s="2">
+        <v>22.6</v>
+      </c>
+      <c r="E2921" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F2921" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2921" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2922">
+      <c r="A2922" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2922" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">01:50</t>
+        </is>
+      </c>
+      <c r="C2922" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2922" s="2">
+        <v>22.3</v>
+      </c>
+      <c r="E2922" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F2922" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2922" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2923">
+      <c r="A2923" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2923" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:00</t>
+        </is>
+      </c>
+      <c r="C2923" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2923" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="E2923" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F2923" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2923" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2924">
+      <c r="A2924" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2924" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:10</t>
+        </is>
+      </c>
+      <c r="C2924" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2924" s="2">
+        <v>21.9</v>
+      </c>
+      <c r="E2924" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F2924" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2924" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2925">
+      <c r="A2925" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2925" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:20</t>
+        </is>
+      </c>
+      <c r="C2925" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2925" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="E2925" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F2925" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2925" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2926">
+      <c r="A2926" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2926" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:30</t>
+        </is>
+      </c>
+      <c r="C2926" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2926" s="2">
+        <v>21.8</v>
+      </c>
+      <c r="E2926" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F2926" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2926" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2927">
+      <c r="A2927" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2927" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:40</t>
+        </is>
+      </c>
+      <c r="C2927" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2927" s="2">
+        <v>21.6</v>
+      </c>
+      <c r="E2927" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F2927" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2927" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2928">
+      <c r="A2928" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2928" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">02:50</t>
+        </is>
+      </c>
+      <c r="C2928" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2928" s="2">
+        <v>21.3</v>
+      </c>
+      <c r="E2928" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F2928" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2928" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2929">
+      <c r="A2929" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2929" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:00</t>
+        </is>
+      </c>
+      <c r="C2929" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2929" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="E2929" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2929" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2929" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2930">
+      <c r="A2930" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2930" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:10</t>
+        </is>
+      </c>
+      <c r="C2930" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2930" s="2">
+        <v>20.8</v>
+      </c>
+      <c r="E2930" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2930" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2930" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2931">
+      <c r="A2931" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2931" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:20</t>
+        </is>
+      </c>
+      <c r="C2931" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2931" s="2">
+        <v>20.7</v>
+      </c>
+      <c r="E2931" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2931" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2931" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2932">
+      <c r="A2932" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2932" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:30</t>
+        </is>
+      </c>
+      <c r="C2932" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2932" s="2">
+        <v>20.5</v>
+      </c>
+      <c r="E2932" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2932" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2932" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2933">
+      <c r="A2933" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2933" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:40</t>
+        </is>
+      </c>
+      <c r="C2933" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2933" s="2">
+        <v>20.2</v>
+      </c>
+      <c r="E2933" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F2933" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2933" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2934">
+      <c r="A2934" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2934" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">03:50</t>
+        </is>
+      </c>
+      <c r="C2934" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2934" s="2">
+        <v>20.1</v>
+      </c>
+      <c r="E2934" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2934" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2934" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2935">
+      <c r="A2935" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2935" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:00</t>
+        </is>
+      </c>
+      <c r="C2935" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2935" s="2">
+        <v>20.2</v>
+      </c>
+      <c r="E2935" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2935" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2935" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2936">
+      <c r="A2936" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2936" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:10</t>
+        </is>
+      </c>
+      <c r="C2936" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2936" s="2">
+        <v>20.2</v>
+      </c>
+      <c r="E2936" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2936" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2936" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2937">
+      <c r="A2937" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2937" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:20</t>
+        </is>
+      </c>
+      <c r="C2937" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2937" s="2">
+        <v>20.1</v>
+      </c>
+      <c r="E2937" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2937" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2937" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2938">
+      <c r="A2938" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2938" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:30</t>
+        </is>
+      </c>
+      <c r="C2938" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2938" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="E2938" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2938" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2938" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2939">
+      <c r="A2939" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2939" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:40</t>
+        </is>
+      </c>
+      <c r="C2939" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2939" s="2">
+        <v>19.8</v>
+      </c>
+      <c r="E2939" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F2939" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2939" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2940">
+      <c r="A2940" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2940" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04:50</t>
+        </is>
+      </c>
+      <c r="C2940" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2940" s="2">
+        <v>19.6</v>
+      </c>
+      <c r="E2940" s="2">
+        <v>67.0</v>
+      </c>
+      <c r="F2940" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2940" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2941">
+      <c r="A2941" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2941" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:00</t>
+        </is>
+      </c>
+      <c r="C2941" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2941" s="2">
+        <v>19.4</v>
+      </c>
+      <c r="E2941" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F2941" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2941" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2942">
+      <c r="A2942" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2942" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:10</t>
+        </is>
+      </c>
+      <c r="C2942" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2942" s="2">
+        <v>19.2</v>
+      </c>
+      <c r="E2942" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F2942" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2942" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2943">
+      <c r="A2943" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2943" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:20</t>
+        </is>
+      </c>
+      <c r="C2943" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2943" s="2">
+        <v>19.1</v>
+      </c>
+      <c r="E2943" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F2943" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2943" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2944">
+      <c r="A2944" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2944" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:30</t>
+        </is>
+      </c>
+      <c r="C2944" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2944" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="E2944" s="2">
+        <v>69.0</v>
+      </c>
+      <c r="F2944" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2944" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2945">
+      <c r="A2945" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2945" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:40</t>
+        </is>
+      </c>
+      <c r="C2945" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2945" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="E2945" s="2">
+        <v>69.0</v>
+      </c>
+      <c r="F2945" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2945" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2946">
+      <c r="A2946" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2946" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05:50</t>
+        </is>
+      </c>
+      <c r="C2946" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2946" s="2">
+        <v>18.9</v>
+      </c>
+      <c r="E2946" s="2">
+        <v>69.0</v>
+      </c>
+      <c r="F2946" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2946" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2947">
+      <c r="A2947" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2947" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:00</t>
+        </is>
+      </c>
+      <c r="C2947" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2947" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="E2947" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F2947" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2947" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2948">
+      <c r="A2948" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2948" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:10</t>
+        </is>
+      </c>
+      <c r="C2948" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2948" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="E2948" s="2">
+        <v>68.0</v>
+      </c>
+      <c r="F2948" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2948" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2949">
+      <c r="A2949" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2949" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:20</t>
+        </is>
+      </c>
+      <c r="C2949" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2949" s="2">
+        <v>18.9</v>
+      </c>
+      <c r="E2949" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F2949" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2949" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2950">
+      <c r="A2950" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2950" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:30</t>
+        </is>
+      </c>
+      <c r="C2950" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2950" s="2">
+        <v>18.8</v>
+      </c>
+      <c r="E2950" s="2">
+        <v>70.0</v>
+      </c>
+      <c r="F2950" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2950" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2951">
+      <c r="A2951" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2951" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:40</t>
+        </is>
+      </c>
+      <c r="C2951" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2951" s="2">
+        <v>18.9</v>
+      </c>
+      <c r="E2951" s="2">
+        <v>69.0</v>
+      </c>
+      <c r="F2951" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2951" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2952">
+      <c r="A2952" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2952" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">06:50</t>
+        </is>
+      </c>
+      <c r="C2952" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2952" s="2">
+        <v>19.5</v>
+      </c>
+      <c r="E2952" s="2">
+        <v>66.0</v>
+      </c>
+      <c r="F2952" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2952" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2953">
+      <c r="A2953" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2953" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:00</t>
+        </is>
+      </c>
+      <c r="C2953" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2953" s="2">
+        <v>19.7</v>
+      </c>
+      <c r="E2953" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="F2953" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2953" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2954">
+      <c r="A2954" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2954" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:10</t>
+        </is>
+      </c>
+      <c r="C2954" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2954" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="E2954" s="2">
+        <v>64.0</v>
+      </c>
+      <c r="F2954" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2954" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2955">
+      <c r="A2955" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2955" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:20</t>
+        </is>
+      </c>
+      <c r="C2955" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2955" s="2">
+        <v>20.6</v>
+      </c>
+      <c r="E2955" s="2">
+        <v>62.0</v>
+      </c>
+      <c r="F2955" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2955" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2956">
+      <c r="A2956" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2956" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:30</t>
+        </is>
+      </c>
+      <c r="C2956" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2956" s="2">
+        <v>21.1</v>
+      </c>
+      <c r="E2956" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F2956" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2956" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2957">
+      <c r="A2957" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2957" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:40</t>
+        </is>
+      </c>
+      <c r="C2957" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2957" s="2">
+        <v>21.6</v>
+      </c>
+      <c r="E2957" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F2957" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2957" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2958">
+      <c r="A2958" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2958" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">07:50</t>
+        </is>
+      </c>
+      <c r="C2958" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2958" s="2">
+        <v>22.3</v>
+      </c>
+      <c r="E2958" s="2">
+        <v>56.0</v>
+      </c>
+      <c r="F2958" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2958" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2959">
+      <c r="A2959" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2959" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:00</t>
+        </is>
+      </c>
+      <c r="C2959" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2959" s="2">
+        <v>22.7</v>
+      </c>
+      <c r="E2959" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F2959" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2959" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2960">
+      <c r="A2960" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2960" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:10</t>
+        </is>
+      </c>
+      <c r="C2960" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2960" s="2">
+        <v>23.2</v>
+      </c>
+      <c r="E2960" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F2960" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2960" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2961">
+      <c r="A2961" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2961" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:20</t>
+        </is>
+      </c>
+      <c r="C2961" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2961" s="2">
+        <v>23.6</v>
+      </c>
+      <c r="E2961" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F2961" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2961" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2962">
+      <c r="A2962" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2962" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:30</t>
+        </is>
+      </c>
+      <c r="C2962" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2962" s="2">
+        <v>24.2</v>
+      </c>
+      <c r="E2962" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="F2962" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2962" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2963">
+      <c r="A2963" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2963" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:40</t>
+        </is>
+      </c>
+      <c r="C2963" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2963" s="2">
+        <v>24.8</v>
+      </c>
+      <c r="E2963" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F2963" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2963" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2964">
+      <c r="A2964" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2964" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">08:50</t>
+        </is>
+      </c>
+      <c r="C2964" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2964" s="2">
+        <v>25.3</v>
+      </c>
+      <c r="E2964" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F2964" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2964" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2965">
+      <c r="A2965" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2965" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:00</t>
+        </is>
+      </c>
+      <c r="C2965" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2965" s="2">
+        <v>25.9</v>
+      </c>
+      <c r="E2965" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F2965" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2965" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2966">
+      <c r="A2966" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2966" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:10</t>
+        </is>
+      </c>
+      <c r="C2966" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2966" s="2">
+        <v>26.8</v>
+      </c>
+      <c r="E2966" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F2966" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2966" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2967">
+      <c r="A2967" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2967" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:20</t>
+        </is>
+      </c>
+      <c r="C2967" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2967" s="2">
+        <v>26.8</v>
+      </c>
+      <c r="E2967" s="2">
+        <v>46.0</v>
+      </c>
+      <c r="F2967" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2967" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2968">
+      <c r="A2968" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2968" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:30</t>
+        </is>
+      </c>
+      <c r="C2968" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2968" s="2">
+        <v>27.6</v>
+      </c>
+      <c r="E2968" s="2">
+        <v>43.0</v>
+      </c>
+      <c r="F2968" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2968" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2969">
+      <c r="A2969" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2969" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:40</t>
+        </is>
+      </c>
+      <c r="C2969" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2969" s="2">
+        <v>28.2</v>
+      </c>
+      <c r="E2969" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F2969" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2969" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2970">
+      <c r="A2970" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2970" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">09:50</t>
+        </is>
+      </c>
+      <c r="C2970" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2970" s="2">
+        <v>28.4</v>
+      </c>
+      <c r="E2970" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F2970" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2970" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2971">
+      <c r="A2971" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2971" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:00</t>
+        </is>
+      </c>
+      <c r="C2971" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2971" s="2">
+        <v>29.4</v>
+      </c>
+      <c r="E2971" s="2">
+        <v>37.0</v>
+      </c>
+      <c r="F2971" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2971" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2972">
+      <c r="A2972" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2972" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:10</t>
+        </is>
+      </c>
+      <c r="C2972" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2972" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="E2972" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F2972" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2972" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2973">
+      <c r="A2973" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2973" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:20</t>
+        </is>
+      </c>
+      <c r="C2973" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2973" s="2">
+        <v>30.3</v>
+      </c>
+      <c r="E2973" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="F2973" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2973" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2974">
+      <c r="A2974" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2974" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:30</t>
+        </is>
+      </c>
+      <c r="C2974" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2974" s="2">
+        <v>30.9</v>
+      </c>
+      <c r="E2974" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F2974" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2974" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2975">
+      <c r="A2975" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2975" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:40</t>
+        </is>
+      </c>
+      <c r="C2975" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2975" s="2">
+        <v>31.7</v>
+      </c>
+      <c r="E2975" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F2975" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2975" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2976">
+      <c r="A2976" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2976" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">10:50</t>
+        </is>
+      </c>
+      <c r="C2976" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2976" s="2">
+        <v>32.3</v>
+      </c>
+      <c r="E2976" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F2976" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2976" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2977">
+      <c r="A2977" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2977" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:00</t>
+        </is>
+      </c>
+      <c r="C2977" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2977" s="2">
+        <v>32.5</v>
+      </c>
+      <c r="E2977" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="F2977" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2977" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2978">
+      <c r="A2978" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2978" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:10</t>
+        </is>
+      </c>
+      <c r="C2978" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2978" s="2">
+        <v>32.9</v>
+      </c>
+      <c r="E2978" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F2978" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2978" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2979">
+      <c r="A2979" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2979" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:20</t>
+        </is>
+      </c>
+      <c r="C2979" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2979" s="2">
+        <v>33.1</v>
+      </c>
+      <c r="E2979" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F2979" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2979" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2980">
+      <c r="A2980" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2980" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:30</t>
+        </is>
+      </c>
+      <c r="C2980" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2980" s="2">
+        <v>33.5</v>
+      </c>
+      <c r="E2980" s="2">
+        <v>32.0</v>
+      </c>
+      <c r="F2980" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2980" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2981">
+      <c r="A2981" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2981" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:40</t>
+        </is>
+      </c>
+      <c r="C2981" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2981" s="2">
+        <v>33.6</v>
+      </c>
+      <c r="E2981" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="F2981" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2981" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2982">
+      <c r="A2982" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2982" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">11:50</t>
+        </is>
+      </c>
+      <c r="C2982" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2982" s="2">
+        <v>34.0</v>
+      </c>
+      <c r="E2982" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F2982" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2982" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2983">
+      <c r="A2983" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2983" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:00</t>
+        </is>
+      </c>
+      <c r="C2983" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2983" s="2">
+        <v>34.9</v>
+      </c>
+      <c r="E2983" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F2983" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2983" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2984">
+      <c r="A2984" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2984" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:10</t>
+        </is>
+      </c>
+      <c r="C2984" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2984" s="2">
+        <v>34.9</v>
+      </c>
+      <c r="E2984" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F2984" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2984" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2985">
+      <c r="A2985" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2985" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:20</t>
+        </is>
+      </c>
+      <c r="C2985" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2985" s="2">
+        <v>35.4</v>
+      </c>
+      <c r="E2985" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="F2985" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2985" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2986">
+      <c r="A2986" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2986" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:30</t>
+        </is>
+      </c>
+      <c r="C2986" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2986" s="2">
+        <v>35.6</v>
+      </c>
+      <c r="E2986" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F2986" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2986" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2987">
+      <c r="A2987" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2987" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:40</t>
+        </is>
+      </c>
+      <c r="C2987" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2987" s="2">
+        <v>36.6</v>
+      </c>
+      <c r="E2987" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="F2987" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2987" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2988">
+      <c r="A2988" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2988" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">12:50</t>
+        </is>
+      </c>
+      <c r="C2988" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2988" s="2">
+        <v>36.9</v>
+      </c>
+      <c r="E2988" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="F2988" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2988" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2989">
+      <c r="A2989" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2989" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:00</t>
+        </is>
+      </c>
+      <c r="C2989" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2989" s="2">
+        <v>36.8</v>
+      </c>
+      <c r="E2989" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="F2989" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2989" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2990">
+      <c r="A2990" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2990" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:10</t>
+        </is>
+      </c>
+      <c r="C2990" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2990" s="2">
+        <v>36.8</v>
+      </c>
+      <c r="E2990" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="F2990" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2990" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2991">
+      <c r="A2991" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2991" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:20</t>
+        </is>
+      </c>
+      <c r="C2991" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2991" s="2">
+        <v>37.3</v>
+      </c>
+      <c r="E2991" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="F2991" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2991" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2992">
+      <c r="A2992" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2992" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:30</t>
+        </is>
+      </c>
+      <c r="C2992" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2992" s="2">
+        <v>36.8</v>
+      </c>
+      <c r="E2992" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="F2992" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2992" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2993">
+      <c r="A2993" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2993" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:40</t>
+        </is>
+      </c>
+      <c r="C2993" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2993" s="2">
+        <v>37.3</v>
+      </c>
+      <c r="E2993" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="F2993" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2993" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2994">
+      <c r="A2994" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2994" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">13:50</t>
+        </is>
+      </c>
+      <c r="C2994" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2994" s="2">
+        <v>37.6</v>
+      </c>
+      <c r="E2994" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="F2994" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2994" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2995">
+      <c r="A2995" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2995" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:00</t>
+        </is>
+      </c>
+      <c r="C2995" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2995" s="2">
+        <v>37.5</v>
+      </c>
+      <c r="E2995" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="F2995" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2995" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2996">
+      <c r="A2996" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2996" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:10</t>
+        </is>
+      </c>
+      <c r="C2996" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2996" s="2">
+        <v>37.7</v>
+      </c>
+      <c r="E2996" s="2">
+        <v>20.0</v>
+      </c>
+      <c r="F2996" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2996" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2997">
+      <c r="A2997" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2997" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:20</t>
+        </is>
+      </c>
+      <c r="C2997" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2997" s="2">
+        <v>37.8</v>
+      </c>
+      <c r="E2997" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="F2997" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2997" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2998">
+      <c r="A2998" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2998" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:30</t>
+        </is>
+      </c>
+      <c r="C2998" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2998" s="2">
+        <v>38.2</v>
+      </c>
+      <c r="E2998" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="F2998" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2998" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="2999">
+      <c r="A2999" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B2999" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:40</t>
+        </is>
+      </c>
+      <c r="C2999" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D2999" s="2">
+        <v>38.0</v>
+      </c>
+      <c r="E2999" s="2">
+        <v>18.0</v>
+      </c>
+      <c r="F2999" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G2999" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3000">
+      <c r="A3000" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3000" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">14:50</t>
+        </is>
+      </c>
+      <c r="C3000" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3000" s="2">
+        <v>38.1</v>
+      </c>
+      <c r="E3000" s="2">
+        <v>17.0</v>
+      </c>
+      <c r="F3000" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3000" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3001">
+      <c r="A3001" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3001" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:00</t>
+        </is>
+      </c>
+      <c r="C3001" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3001" s="2">
+        <v>38.0</v>
+      </c>
+      <c r="E3001" s="2">
+        <v>18.0</v>
+      </c>
+      <c r="F3001" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3001" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3002">
+      <c r="A3002" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3002" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:10</t>
+        </is>
+      </c>
+      <c r="C3002" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3002" s="2">
+        <v>37.8</v>
+      </c>
+      <c r="E3002" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="F3002" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3002" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3003">
+      <c r="A3003" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3003" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:20</t>
+        </is>
+      </c>
+      <c r="C3003" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3003" s="2">
+        <v>37.5</v>
+      </c>
+      <c r="E3003" s="2">
+        <v>19.0</v>
+      </c>
+      <c r="F3003" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3003" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3004">
+      <c r="A3004" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3004" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:30</t>
+        </is>
+      </c>
+      <c r="C3004" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3004" s="2">
+        <v>37.4</v>
+      </c>
+      <c r="E3004" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="F3004" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3004" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3005">
+      <c r="A3005" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3005" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:40</t>
+        </is>
+      </c>
+      <c r="C3005" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3005" s="2">
+        <v>36.7</v>
+      </c>
+      <c r="E3005" s="2">
+        <v>21.0</v>
+      </c>
+      <c r="F3005" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3005" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3006">
+      <c r="A3006" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3006" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">15:50</t>
+        </is>
+      </c>
+      <c r="C3006" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3006" s="2">
+        <v>36.4</v>
+      </c>
+      <c r="E3006" s="2">
+        <v>22.0</v>
+      </c>
+      <c r="F3006" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3006" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3007">
+      <c r="A3007" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3007" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:00</t>
+        </is>
+      </c>
+      <c r="C3007" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3007" s="2">
+        <v>36.2</v>
+      </c>
+      <c r="E3007" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="F3007" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3007" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3008">
+      <c r="A3008" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3008" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:10</t>
+        </is>
+      </c>
+      <c r="C3008" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3008" s="2">
+        <v>36.2</v>
+      </c>
+      <c r="E3008" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="F3008" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3008" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3009">
+      <c r="A3009" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3009" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:20</t>
+        </is>
+      </c>
+      <c r="C3009" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3009" s="2">
+        <v>36.2</v>
+      </c>
+      <c r="E3009" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="F3009" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3009" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3010">
+      <c r="A3010" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3010" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:30</t>
+        </is>
+      </c>
+      <c r="C3010" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3010" s="2">
+        <v>36.1</v>
+      </c>
+      <c r="E3010" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="F3010" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3010" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3011">
+      <c r="A3011" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3011" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:40</t>
+        </is>
+      </c>
+      <c r="C3011" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3011" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="E3011" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F3011" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3011" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3012">
+      <c r="A3012" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3012" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">16:50</t>
+        </is>
+      </c>
+      <c r="C3012" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3012" s="2">
+        <v>35.8</v>
+      </c>
+      <c r="E3012" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F3012" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3012" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3013">
+      <c r="A3013" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3013" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:00</t>
+        </is>
+      </c>
+      <c r="C3013" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3013" s="2">
+        <v>35.8</v>
+      </c>
+      <c r="E3013" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F3013" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3013" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3014">
+      <c r="A3014" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3014" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:10</t>
+        </is>
+      </c>
+      <c r="C3014" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3014" s="2">
+        <v>35.6</v>
+      </c>
+      <c r="E3014" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F3014" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3014" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3015">
+      <c r="A3015" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3015" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:20</t>
+        </is>
+      </c>
+      <c r="C3015" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3015" s="2">
+        <v>35.4</v>
+      </c>
+      <c r="E3015" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F3015" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3015" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3016">
+      <c r="A3016" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3016" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">17:30</t>
+        </is>
+      </c>
+      <c r="C3016" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3016" s="2">
+        <v>35.6</v>
+      </c>
+      <c r="E3016" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F3016" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3016" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3017">
+      <c r="A3017" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3017" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:20</t>
+        </is>
+      </c>
+      <c r="C3017" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3017" s="2">
+        <v>35.7</v>
+      </c>
+      <c r="E3017" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F3017" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3017" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3018">
+      <c r="A3018" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3018" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:30</t>
+        </is>
+      </c>
+      <c r="C3018" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3018" s="2">
+        <v>35.4</v>
+      </c>
+      <c r="E3018" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F3018" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3018" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3019">
+      <c r="A3019" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3019" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:40</t>
+        </is>
+      </c>
+      <c r="C3019" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3019" s="2">
+        <v>35.1</v>
+      </c>
+      <c r="E3019" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="F3019" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3019" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3020">
+      <c r="A3020" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3020" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">18:50</t>
+        </is>
+      </c>
+      <c r="C3020" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3020" s="2">
+        <v>35.0</v>
+      </c>
+      <c r="E3020" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F3020" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3020" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3021">
+      <c r="A3021" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3021" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:00</t>
+        </is>
+      </c>
+      <c r="C3021" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3021" s="2">
+        <v>34.8</v>
+      </c>
+      <c r="E3021" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="F3021" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3021" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3022">
+      <c r="A3022" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3022" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:10</t>
+        </is>
+      </c>
+      <c r="C3022" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3022" s="2">
+        <v>34.2</v>
+      </c>
+      <c r="E3022" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="F3022" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3022" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3023">
+      <c r="A3023" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3023" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:20</t>
+        </is>
+      </c>
+      <c r="C3023" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3023" s="2">
+        <v>33.8</v>
+      </c>
+      <c r="E3023" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="F3023" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3023" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3024">
+      <c r="A3024" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3024" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:30</t>
+        </is>
+      </c>
+      <c r="C3024" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3024" s="2">
+        <v>33.4</v>
+      </c>
+      <c r="E3024" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F3024" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3024" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3025">
+      <c r="A3025" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3025" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:40</t>
+        </is>
+      </c>
+      <c r="C3025" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3025" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="E3025" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F3025" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3025" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3026">
+      <c r="A3026" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3026" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">19:50</t>
+        </is>
+      </c>
+      <c r="C3026" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3026" s="2">
+        <v>32.8</v>
+      </c>
+      <c r="E3026" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F3026" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3026" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3027">
+      <c r="A3027" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3027" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:00</t>
+        </is>
+      </c>
+      <c r="C3027" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3027" s="2">
+        <v>32.5</v>
+      </c>
+      <c r="E3027" s="2">
+        <v>28.0</v>
+      </c>
+      <c r="F3027" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3027" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3028">
+      <c r="A3028" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3028" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:10</t>
+        </is>
+      </c>
+      <c r="C3028" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3028" s="2">
+        <v>32.2</v>
+      </c>
+      <c r="E3028" s="2">
+        <v>29.0</v>
+      </c>
+      <c r="F3028" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3028" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3029">
+      <c r="A3029" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3029" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:20</t>
+        </is>
+      </c>
+      <c r="C3029" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3029" s="2">
+        <v>31.8</v>
+      </c>
+      <c r="E3029" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F3029" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3029" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3030">
+      <c r="A3030" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3030" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:30</t>
+        </is>
+      </c>
+      <c r="C3030" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3030" s="2">
+        <v>31.4</v>
+      </c>
+      <c r="E3030" s="2">
+        <v>30.0</v>
+      </c>
+      <c r="F3030" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3030" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3031">
+      <c r="A3031" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3031" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:40</t>
+        </is>
+      </c>
+      <c r="C3031" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3031" s="2">
+        <v>30.9</v>
+      </c>
+      <c r="E3031" s="2">
+        <v>31.0</v>
+      </c>
+      <c r="F3031" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3031" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3032">
+      <c r="A3032" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3032" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">20:50</t>
+        </is>
+      </c>
+      <c r="C3032" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3032" s="2">
+        <v>30.1</v>
+      </c>
+      <c r="E3032" s="2">
+        <v>33.0</v>
+      </c>
+      <c r="F3032" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3032" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3033">
+      <c r="A3033" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3033" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:00</t>
+        </is>
+      </c>
+      <c r="C3033" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3033" s="2">
+        <v>29.5</v>
+      </c>
+      <c r="E3033" s="2">
+        <v>36.0</v>
+      </c>
+      <c r="F3033" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3033" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3034">
+      <c r="A3034" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3034" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:10</t>
+        </is>
+      </c>
+      <c r="C3034" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3034" s="2">
+        <v>28.9</v>
+      </c>
+      <c r="E3034" s="2">
+        <v>38.0</v>
+      </c>
+      <c r="F3034" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3034" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3035">
+      <c r="A3035" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3035" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:20</t>
+        </is>
+      </c>
+      <c r="C3035" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3035" s="2">
+        <v>28.3</v>
+      </c>
+      <c r="E3035" s="2">
+        <v>40.0</v>
+      </c>
+      <c r="F3035" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3035" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3036">
+      <c r="A3036" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3036" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:30</t>
+        </is>
+      </c>
+      <c r="C3036" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3036" s="2">
+        <v>27.6</v>
+      </c>
+      <c r="E3036" s="2">
+        <v>42.0</v>
+      </c>
+      <c r="F3036" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3036" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3037">
+      <c r="A3037" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3037" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:40</t>
+        </is>
+      </c>
+      <c r="C3037" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3037" s="2">
+        <v>27.0</v>
+      </c>
+      <c r="E3037" s="2">
+        <v>45.0</v>
+      </c>
+      <c r="F3037" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3037" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3038">
+      <c r="A3038" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3038" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">21:50</t>
+        </is>
+      </c>
+      <c r="C3038" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3038" s="2">
+        <v>26.5</v>
+      </c>
+      <c r="E3038" s="2">
+        <v>47.0</v>
+      </c>
+      <c r="F3038" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3038" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3039">
+      <c r="A3039" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3039" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:00</t>
+        </is>
+      </c>
+      <c r="C3039" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3039" s="2">
+        <v>26.0</v>
+      </c>
+      <c r="E3039" s="2">
+        <v>48.0</v>
+      </c>
+      <c r="F3039" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3039" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3040">
+      <c r="A3040" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3040" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:10</t>
+        </is>
+      </c>
+      <c r="C3040" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3040" s="2">
+        <v>25.7</v>
+      </c>
+      <c r="E3040" s="2">
+        <v>49.0</v>
+      </c>
+      <c r="F3040" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3040" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3041">
+      <c r="A3041" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3041" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:20</t>
+        </is>
+      </c>
+      <c r="C3041" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3041" s="2">
+        <v>25.3</v>
+      </c>
+      <c r="E3041" s="2">
+        <v>51.0</v>
+      </c>
+      <c r="F3041" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3041" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3042">
+      <c r="A3042" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3042" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:30</t>
+        </is>
+      </c>
+      <c r="C3042" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3042" s="2">
+        <v>25.0</v>
+      </c>
+      <c r="E3042" s="2">
+        <v>52.0</v>
+      </c>
+      <c r="F3042" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3042" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3043">
+      <c r="A3043" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3043" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:40</t>
+        </is>
+      </c>
+      <c r="C3043" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3043" s="2">
+        <v>24.7</v>
+      </c>
+      <c r="E3043" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F3043" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3043" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3044">
+      <c r="A3044" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3044" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">22:50</t>
+        </is>
+      </c>
+      <c r="C3044" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3044" s="2">
+        <v>24.5</v>
+      </c>
+      <c r="E3044" s="2">
+        <v>53.0</v>
+      </c>
+      <c r="F3044" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3044" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3045">
+      <c r="A3045" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3045" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:00</t>
+        </is>
+      </c>
+      <c r="C3045" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3045" s="2">
+        <v>24.4</v>
+      </c>
+      <c r="E3045" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F3045" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3045" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3046">
+      <c r="A3046" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3046" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:10</t>
+        </is>
+      </c>
+      <c r="C3046" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3046" s="2">
+        <v>24.3</v>
+      </c>
+      <c r="E3046" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F3046" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3046" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3047">
+      <c r="A3047" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3047" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:20</t>
+        </is>
+      </c>
+      <c r="C3047" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3047" s="2">
+        <v>24.1</v>
+      </c>
+      <c r="E3047" s="2">
+        <v>54.0</v>
+      </c>
+      <c r="F3047" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3047" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3048">
+      <c r="A3048" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3048" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:30</t>
+        </is>
+      </c>
+      <c r="C3048" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3048" s="2">
+        <v>24.0</v>
+      </c>
+      <c r="E3048" s="2">
+        <v>55.0</v>
+      </c>
+      <c r="F3048" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3048" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3049">
+      <c r="A3049" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3049" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:40</t>
+        </is>
+      </c>
+      <c r="C3049" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3049" s="2">
+        <v>23.6</v>
+      </c>
+      <c r="E3049" s="2">
+        <v>57.0</v>
+      </c>
+      <c r="F3049" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3049" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3050">
+      <c r="A3050" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">04.08.2026</t>
+        </is>
+      </c>
+      <c r="B3050" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">23:50</t>
+        </is>
+      </c>
+      <c r="C3050" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3050" s="2">
+        <v>23.3</v>
+      </c>
+      <c r="E3050" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F3050" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3050" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3051">
+      <c r="A3051" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05.08.2026</t>
+        </is>
+      </c>
+      <c r="B3051" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:00</t>
+        </is>
+      </c>
+      <c r="C3051" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3051" s="2">
+        <v>23.1</v>
+      </c>
+      <c r="E3051" s="2">
+        <v>58.0</v>
+      </c>
+      <c r="F3051" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3051" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3052">
+      <c r="A3052" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05.08.2026</t>
+        </is>
+      </c>
+      <c r="B3052" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:10</t>
+        </is>
+      </c>
+      <c r="C3052" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3052" s="2">
+        <v>23.0</v>
+      </c>
+      <c r="E3052" s="2">
+        <v>59.0</v>
+      </c>
+      <c r="F3052" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3052" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3053">
+      <c r="A3053" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05.08.2026</t>
+        </is>
+      </c>
+      <c r="B3053" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:20</t>
+        </is>
+      </c>
+      <c r="C3053" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3053" s="2">
+        <v>22.7</v>
+      </c>
+      <c r="E3053" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="F3053" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3053" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="3054">
+      <c r="A3054" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">05.08.2026</t>
+        </is>
+      </c>
+      <c r="B3054" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">00:30</t>
+        </is>
+      </c>
+      <c r="C3054" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Kranj</t>
+        </is>
+      </c>
+      <c r="D3054" s="2">
+        <v>22.4</v>
+      </c>
+      <c r="E3054" s="2">
+        <v>61.0</v>
+      </c>
+      <c r="F3054" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="G3054" s="2">
+        <v>0.0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G2914"/>
+  <autoFilter ref="A1:G3054"/>
 </worksheet>
 </file>
</xml_diff>